<commit_message>
Private customers in price agreements for regional tenders
</commit_message>
<xml_diff>
--- a/srv/xlsx-templates/TH - Quotation Template.xlsx
+++ b/srv/xlsx-templates/TH - Quotation Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26626"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Projects\Bayer\fastCAPv2\fastCAP-backend\srv\xlsx-templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EHQUT\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CCD3417-AF0E-4A8F-8E07-6B52F4321981}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{662F4A3F-58DB-4ADA-97CB-1B95B82C8CCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{F5CC2154-27BB-4652-B61E-D913F0CC6809}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{F5CC2154-27BB-4652-B61E-D913F0CC6809}"/>
   </bookViews>
   <sheets>
     <sheet name="Quotation" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="75">
   <si>
     <t>${offerValidation.INSTITUTENAME}</t>
   </si>
@@ -271,7 +271,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="#\.###\.###.00"/>
+    <numFmt numFmtId="164" formatCode="#\.###\.###.00"/>
   </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
@@ -434,18 +434,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -455,26 +456,25 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standaard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="7">
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="165" formatCode="#\.###\.###.00"/>
+      <numFmt numFmtId="164" formatCode="#\.###\.###.00"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="165" formatCode="#\.###\.###.00"/>
+      <numFmt numFmtId="164" formatCode="#\.###\.###.00"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="165" formatCode="#\.###\.###.00"/>
+      <numFmt numFmtId="164" formatCode="#\.###\.###.00"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="165" formatCode="#\.###\.###.00"/>
+      <numFmt numFmtId="164" formatCode="#\.###\.###.00"/>
     </dxf>
     <dxf>
       <font>
@@ -600,11 +600,11 @@
   <tableColumns count="19">
     <tableColumn id="1" xr3:uid="{6E1F8ECB-E862-46B4-998C-BE8E89C238BA}" name="PAID VOLUME"/>
     <tableColumn id="2" xr3:uid="{6497AF92-63C8-4790-818D-6E5BE819E8D6}" name="UNIT"/>
-    <tableColumn id="3" xr3:uid="{A1E59B72-B459-4BFA-9B37-9736C0F03B7E}" name="OFFER PRICE" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{A1E59B72-B459-4BFA-9B37-9736C0F03B7E}" name="OFFER PRICE" dataDxfId="4"/>
     <tableColumn id="4" xr3:uid="{1CB5E955-18ED-4738-ACA1-E270D15916F8}" name="CURRENCY"/>
-    <tableColumn id="5" xr3:uid="{77EEA9FC-8FC3-433A-9592-47B0D8B4C67B}" name="OFFER_PRICE_VAT" dataDxfId="2"/>
-    <tableColumn id="6" xr3:uid="{38030720-EDB2-473C-9CF5-2E9C926DF088}" name="GROSS SALES OFFER CURRENCY" dataDxfId="3"/>
-    <tableColumn id="7" xr3:uid="{A1EAF0A4-B4D5-428E-9D86-C12164DF9888}" name="GROSS_SALES_OFFER_CURRENCY_VAT" dataDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{77EEA9FC-8FC3-433A-9592-47B0D8B4C67B}" name="OFFER_PRICE_VAT" dataDxfId="3"/>
+    <tableColumn id="6" xr3:uid="{38030720-EDB2-473C-9CF5-2E9C926DF088}" name="GROSS SALES OFFER CURRENCY" dataDxfId="2"/>
+    <tableColumn id="7" xr3:uid="{A1EAF0A4-B4D5-428E-9D86-C12164DF9888}" name="GROSS_SALES_OFFER_CURRENCY_VAT" dataDxfId="1"/>
     <tableColumn id="8" xr3:uid="{06958303-4A18-40AA-8AD0-9A7EEFDCAF3E}" name="OFFER_ID"/>
     <tableColumn id="9" xr3:uid="{A1218AAF-0481-41A2-9C10-3038D1BF8C7D}" name="SORTER"/>
     <tableColumn id="10" xr3:uid="{5A7FFAC3-1C22-44BF-8C52-F3578967B0F3}" name="Pack Factor"/>
@@ -922,19 +922,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8F4731A-D70B-4034-AE07-DF495FD0B95B}">
   <dimension ref="C3:Q36"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="2.6640625" customWidth="1"/>
-    <col min="3" max="3" width="19.109375" customWidth="1"/>
-    <col min="4" max="4" width="24.33203125" customWidth="1"/>
-    <col min="5" max="5" width="21.88671875" customWidth="1"/>
-    <col min="6" max="6" width="15.5546875" customWidth="1"/>
-    <col min="7" max="10" width="20.6640625" customWidth="1"/>
-    <col min="16" max="17" width="20.6640625" customWidth="1"/>
-    <col min="18" max="18" width="2.6640625" customWidth="1"/>
+    <col min="1" max="2" width="2.7109375" customWidth="1"/>
+    <col min="3" max="3" width="19.140625" customWidth="1"/>
+    <col min="4" max="4" width="24.28515625" customWidth="1"/>
+    <col min="5" max="5" width="21.85546875" customWidth="1"/>
+    <col min="6" max="6" width="15.5703125" customWidth="1"/>
+    <col min="7" max="10" width="20.7109375" customWidth="1"/>
+    <col min="16" max="17" width="20.7109375" customWidth="1"/>
+    <col min="18" max="18" width="2.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="3:17" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="3:17" ht="30" x14ac:dyDescent="0.25">
       <c r="C3" s="3" t="s">
         <v>1</v>
       </c>
@@ -943,7 +943,7 @@
         <v>${offerValidation.INSTITUTENAME}</v>
       </c>
     </row>
-    <row r="5" spans="3:17" x14ac:dyDescent="0.3">
+    <row r="5" spans="3:17" ht="30" x14ac:dyDescent="0.25">
       <c r="C5" s="3" t="s">
         <v>2</v>
       </c>
@@ -953,7 +953,7 @@
       </c>
       <c r="E5" s="10"/>
     </row>
-    <row r="6" spans="3:17" x14ac:dyDescent="0.3">
+    <row r="6" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
       <c r="E6" s="5"/>
@@ -970,7 +970,7 @@
       <c r="P6" s="5"/>
       <c r="Q6" s="5"/>
     </row>
-    <row r="7" spans="3:17" x14ac:dyDescent="0.3">
+    <row r="7" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C7" s="1" t="s">
         <v>3</v>
       </c>
@@ -984,33 +984,33 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="3:17" x14ac:dyDescent="0.3">
-      <c r="C8" s="20" t="str">
+    <row r="8" spans="3:17" x14ac:dyDescent="0.25">
+      <c r="C8" s="21" t="str">
         <f>Settings!A2</f>
         <v>${offerValidation.OFFERID}</v>
       </c>
-      <c r="D8" s="20"/>
-      <c r="E8" s="20"/>
-      <c r="F8" s="19" t="str">
+      <c r="D8" s="21"/>
+      <c r="E8" s="21"/>
+      <c r="F8" s="20" t="str">
         <f>Settings!A3</f>
         <v>${offerValidation.TENDERID}</v>
       </c>
-      <c r="G8" s="19"/>
-      <c r="H8" s="19"/>
-      <c r="I8" s="19" t="str">
+      <c r="G8" s="20"/>
+      <c r="H8" s="20"/>
+      <c r="I8" s="20" t="str">
         <f>Settings!A4</f>
         <v>${offerValidation.OFFERDATE}</v>
       </c>
-      <c r="J8" s="19"/>
-      <c r="K8" s="19"/>
-      <c r="L8" s="19" t="str">
+      <c r="J8" s="20"/>
+      <c r="K8" s="20"/>
+      <c r="L8" s="20" t="str">
         <f>Settings!A5</f>
         <v>${offerValidation.OFFERVALIDITY}</v>
       </c>
-      <c r="M8" s="19"/>
-      <c r="N8" s="19"/>
-    </row>
-    <row r="9" spans="3:17" x14ac:dyDescent="0.3">
+      <c r="M8" s="20"/>
+      <c r="N8" s="20"/>
+    </row>
+    <row r="9" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C9" s="6"/>
       <c r="D9" s="6"/>
       <c r="E9" s="6"/>
@@ -1027,7 +1027,7 @@
       <c r="P9" s="5"/>
       <c r="Q9" s="5"/>
     </row>
-    <row r="10" spans="3:17" x14ac:dyDescent="0.3">
+    <row r="10" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C10" s="1" t="s">
         <v>7</v>
       </c>
@@ -1038,28 +1038,28 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="3:17" x14ac:dyDescent="0.3">
-      <c r="C11" s="21" t="str">
+    <row r="11" spans="3:17" x14ac:dyDescent="0.25">
+      <c r="C11" s="22" t="str">
         <f>Settings!A6</f>
         <v>${offerValidation.SHIPMENTTERMS}</v>
       </c>
-      <c r="D11" s="21"/>
-      <c r="E11" s="21"/>
-      <c r="F11" s="21" t="str">
+      <c r="D11" s="22"/>
+      <c r="E11" s="22"/>
+      <c r="F11" s="22" t="str">
         <f>Settings!A7</f>
         <v>${offerValidation.PAYMENTTERMS}</v>
       </c>
-      <c r="G11" s="21"/>
-      <c r="H11" s="21"/>
-      <c r="I11" s="21" t="str">
+      <c r="G11" s="22"/>
+      <c r="H11" s="22"/>
+      <c r="I11" s="22" t="str">
         <f>Settings!A8</f>
         <v>${offerValidation.DELIVERYTERMS}</v>
       </c>
-      <c r="J11" s="21"/>
-      <c r="K11" s="21"/>
-    </row>
-    <row r="12" spans="3:17" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="13" spans="3:17" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="J11" s="22"/>
+      <c r="K11" s="22"/>
+    </row>
+    <row r="12" spans="3:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="13" spans="3:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C13" s="9"/>
       <c r="D13" s="9" t="s">
         <v>10</v>
@@ -1101,7 +1101,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="14" spans="3:17" x14ac:dyDescent="0.3">
+    <row r="14" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C14" t="str">
         <f>IF(Settings!A18="","",Settings!A18)</f>
         <v>${table:offerProductValidation.SKU}</v>
@@ -1159,7 +1159,7 @@
         <v>${table:offerProductValidation.NET_PRICE} ${table:offerProductValidation.CURRENCY}</v>
       </c>
     </row>
-    <row r="15" spans="3:17" x14ac:dyDescent="0.3">
+    <row r="15" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C15" t="str">
         <f>IF(Settings!A19="","",Settings!A19)</f>
         <v/>
@@ -1217,7 +1217,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="16" spans="3:17" x14ac:dyDescent="0.3">
+    <row r="16" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C16" t="str">
         <f>IF(Settings!A20="","",Settings!A20)</f>
         <v/>
@@ -1275,7 +1275,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="17" spans="3:17" x14ac:dyDescent="0.3">
+    <row r="17" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C17" t="str">
         <f>IF(Settings!A21="","",Settings!A21)</f>
         <v/>
@@ -1333,19 +1333,12 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="18" spans="3:17" x14ac:dyDescent="0.3">
-      <c r="C18" t="str">
-        <f>IF(Settings!A22="","",Settings!A22)</f>
-        <v/>
-      </c>
-      <c r="D18" t="str">
-        <f>IF(Settings!B22="","",Settings!B22)</f>
-        <v/>
-      </c>
-      <c r="E18" t="str">
-        <f>IF(CONCATENATE(Settings!C22," ",Settings!D22,"s")=" s"," ",CONCATENATE(Settings!C22," ",Settings!D22,"s"))</f>
-        <v xml:space="preserve"> </v>
-      </c>
+    <row r="18" spans="3:17" x14ac:dyDescent="0.25">
+      <c r="C18" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="D18" s="21"/>
+      <c r="E18" s="21"/>
       <c r="F18" t="str">
         <f>IF(Settings!L22="","",Settings!L22)</f>
         <v/>
@@ -1391,7 +1384,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="19" spans="3:17" x14ac:dyDescent="0.3">
+    <row r="19" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C19" t="str">
         <f>IF(Settings!A23="","",Settings!A23)</f>
         <v/>
@@ -1449,7 +1442,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="20" spans="3:17" x14ac:dyDescent="0.3">
+    <row r="20" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C20" t="str">
         <f>IF(Settings!A24="","",Settings!A24)</f>
         <v/>
@@ -1507,7 +1500,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="21" spans="3:17" x14ac:dyDescent="0.3">
+    <row r="21" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C21" t="str">
         <f>IF(Settings!A25="","",Settings!A25)</f>
         <v/>
@@ -1565,7 +1558,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="22" spans="3:17" x14ac:dyDescent="0.3">
+    <row r="22" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C22" t="str">
         <f>IF(Settings!A26="","",Settings!A26)</f>
         <v/>
@@ -1623,7 +1616,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="23" spans="3:17" x14ac:dyDescent="0.3">
+    <row r="23" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C23" t="str">
         <f>IF(Settings!A27="","",Settings!A27)</f>
         <v/>
@@ -1681,7 +1674,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="24" spans="3:17" x14ac:dyDescent="0.3">
+    <row r="24" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C24" t="str">
         <f>IF(Settings!A28="","",Settings!A28)</f>
         <v/>
@@ -1739,7 +1732,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="25" spans="3:17" x14ac:dyDescent="0.3">
+    <row r="25" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C25" t="str">
         <f>IF(Settings!A29="","",Settings!A29)</f>
         <v/>
@@ -1797,7 +1790,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="26" spans="3:17" x14ac:dyDescent="0.3">
+    <row r="26" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C26" t="str">
         <f>IF(Settings!A30="","",Settings!A30)</f>
         <v/>
@@ -1855,7 +1848,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="27" spans="3:17" x14ac:dyDescent="0.3">
+    <row r="27" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C27" t="str">
         <f>IF(Settings!A31="","",Settings!A31)</f>
         <v/>
@@ -1913,7 +1906,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="28" spans="3:17" x14ac:dyDescent="0.3">
+    <row r="28" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C28" t="str">
         <f>IF(Settings!A32="","",Settings!A32)</f>
         <v/>
@@ -1951,7 +1944,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" spans="3:17" x14ac:dyDescent="0.3">
+    <row r="29" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C29" t="str">
         <f>IF(Settings!A33="","",Settings!A33)</f>
         <v/>
@@ -1996,7 +1989,7 @@
         <v>${offerValidation.AMOUNT_IN_NUMBERS} ${table:offerProductValidation.CURRENCY}</v>
       </c>
     </row>
-    <row r="30" spans="3:17" x14ac:dyDescent="0.3">
+    <row r="30" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C30" t="str">
         <f>IF(Settings!A34="","",Settings!A34)</f>
         <v/>
@@ -2035,7 +2028,7 @@
       </c>
       <c r="P30" s="8"/>
     </row>
-    <row r="31" spans="3:17" x14ac:dyDescent="0.3">
+    <row r="31" spans="3:17" x14ac:dyDescent="0.25">
       <c r="E31" t="str">
         <f>IF(CONCATENATE(Quotation!C83," ",Quotation!D83,"s")=" s"," ",CONCATENATE(Quotation!C83," ",Quotation!D83,"s"))</f>
         <v xml:space="preserve"> </v>
@@ -2068,7 +2061,7 @@
         <v>${offerValidation.VAT_TOTAL} ${table:offerProductValidation.CURRENCY}</v>
       </c>
     </row>
-    <row r="32" spans="3:17" x14ac:dyDescent="0.3">
+    <row r="32" spans="3:17" x14ac:dyDescent="0.25">
       <c r="E32" t="str">
         <f>IF(CONCATENATE(Quotation!C84," ",Quotation!D84,"s")=" s"," ",CONCATENATE(Quotation!C84," ",Quotation!D84,"s"))</f>
         <v xml:space="preserve"> </v>
@@ -2095,7 +2088,7 @@
       </c>
       <c r="P32" s="8"/>
     </row>
-    <row r="33" spans="5:17" x14ac:dyDescent="0.3">
+    <row r="33" spans="5:17" x14ac:dyDescent="0.25">
       <c r="E33" t="str">
         <f>IF(CONCATENATE(Quotation!C85," ",Quotation!D85,"s")=" s"," ",CONCATENATE(Quotation!C85," ",Quotation!D85,"s"))</f>
         <v xml:space="preserve"> </v>
@@ -2128,7 +2121,7 @@
         <v>${offerValidation.AMOUNT_IN_NUMBERS_VAT} ${table:offerProductValidation.CURRENCY}</v>
       </c>
     </row>
-    <row r="34" spans="5:17" x14ac:dyDescent="0.3">
+    <row r="34" spans="5:17" x14ac:dyDescent="0.25">
       <c r="E34" t="str">
         <f>IF(CONCATENATE(Quotation!C86," ",Quotation!D86,"s")=" s"," ",CONCATENATE(Quotation!C86," ",Quotation!D86,"s"))</f>
         <v xml:space="preserve"> </v>
@@ -2150,7 +2143,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="35" spans="5:17" x14ac:dyDescent="0.3">
+    <row r="35" spans="5:17" x14ac:dyDescent="0.25">
       <c r="E35" t="str">
         <f>IF(CONCATENATE(Quotation!C87," ",Quotation!D87,"s")=" s"," ",CONCATENATE(Quotation!C87," ",Quotation!D87,"s"))</f>
         <v xml:space="preserve"> </v>
@@ -2164,14 +2157,15 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="36" spans="5:17" x14ac:dyDescent="0.3">
+    <row r="36" spans="5:17" x14ac:dyDescent="0.25">
       <c r="E36" t="str">
         <f>IF(CONCATENATE(Quotation!C88," ",Quotation!D88,"s")=" s"," ",CONCATENATE(Quotation!C88," ",Quotation!D88,"s"))</f>
         <v xml:space="preserve"> </v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="8">
+    <mergeCell ref="C18:E18"/>
     <mergeCell ref="L8:N8"/>
     <mergeCell ref="C8:E8"/>
     <mergeCell ref="C11:E11"/>
@@ -2181,7 +2175,10 @@
     <mergeCell ref="I11:K11"/>
   </mergeCells>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="51" orientation="landscape" horizontalDpi="4294967294" verticalDpi="0" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="51" orientation="landscape" horizontalDpi="4294967294" r:id="rId1"/>
+  <headerFooter>
+    <oddFooter>&amp;R_x000D_&amp;1#&amp;"Calibri"&amp;22&amp;KFF8939 RESTRICTED</oddFooter>
+  </headerFooter>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
@@ -2189,32 +2186,32 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E9BADA0-6CEF-4001-8243-A13FFD1BF3BE}">
   <dimension ref="A1:U52"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="43.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="50.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="47.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="36.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="46.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="44.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="52.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="69.33203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="75.44140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="42.33203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="40.5546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="42.109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="41.77734375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="52.88671875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="36.21875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="46.6640625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="16.21875" customWidth="1"/>
-    <col min="18" max="18" width="39.5546875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="38.88671875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="27.109375" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="43.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="43.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="50.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="47.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="36.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="46.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="44.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="52.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="69.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="75.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="42.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="40.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="42.140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="41.7109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="52.85546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="36.28515625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="46.7109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="16.28515625" customWidth="1"/>
+    <col min="18" max="18" width="39.5703125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="38.85546875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="27.140625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="43.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
         <v>57</v>
       </c>
@@ -2222,7 +2219,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>23</v>
       </c>
@@ -2230,7 +2227,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>24</v>
       </c>
@@ -2238,7 +2235,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>25</v>
       </c>
@@ -2246,7 +2243,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>26</v>
       </c>
@@ -2254,7 +2251,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>29</v>
       </c>
@@ -2262,7 +2259,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>28</v>
       </c>
@@ -2270,7 +2267,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>27</v>
       </c>
@@ -2278,7 +2275,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>0</v>
       </c>
@@ -2286,7 +2283,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>71</v>
       </c>
@@ -2294,12 +2291,12 @@
         <v>72</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="11" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="17" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17" s="17" t="s">
         <v>60</v>
       </c>
@@ -2364,7 +2361,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="18" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18" s="13" t="s">
         <v>31</v>
       </c>
@@ -2377,19 +2374,19 @@
       <c r="D18" t="s">
         <v>40</v>
       </c>
-      <c r="E18" s="22" t="s">
+      <c r="E18" s="19" t="s">
         <v>43</v>
       </c>
       <c r="F18" t="s">
         <v>45</v>
       </c>
-      <c r="G18" s="22" t="s">
+      <c r="G18" s="19" t="s">
         <v>48</v>
       </c>
-      <c r="H18" s="22" t="s">
+      <c r="H18" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="I18" s="22" t="s">
+      <c r="I18" s="19" t="s">
         <v>51</v>
       </c>
       <c r="J18" t="s">
@@ -2430,409 +2427,409 @@
         <v>69</v>
       </c>
     </row>
-    <row r="19" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A19" s="13"/>
       <c r="B19" s="14"/>
-      <c r="E19" s="22"/>
-      <c r="G19" s="22"/>
-      <c r="H19" s="22"/>
-      <c r="I19" s="22"/>
+      <c r="E19" s="19"/>
+      <c r="G19" s="19"/>
+      <c r="H19" s="19"/>
+      <c r="I19" s="19"/>
       <c r="Q19" t="str">
         <f>IF(D19&gt;0,IF(D19="Unit",CONCATENATE(Settings!P19," ",Settings!D19,"s"),CONCATENATE((Settings!P19/Settings!L19)," ",Settings!D19,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="20" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20" s="13"/>
       <c r="B20" s="14"/>
-      <c r="E20" s="22"/>
-      <c r="G20" s="22"/>
-      <c r="H20" s="22"/>
-      <c r="I20" s="22"/>
+      <c r="E20" s="19"/>
+      <c r="G20" s="19"/>
+      <c r="H20" s="19"/>
+      <c r="I20" s="19"/>
       <c r="Q20" t="str">
         <f>IF(D20&gt;0,IF(D20="Unit",CONCATENATE(Settings!P20," ",Settings!D20,"s"),CONCATENATE((Settings!P20/Settings!L20)," ",Settings!D20,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="21" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21" s="13"/>
       <c r="B21" s="14"/>
-      <c r="E21" s="22"/>
-      <c r="G21" s="22"/>
-      <c r="H21" s="22"/>
-      <c r="I21" s="22"/>
+      <c r="E21" s="19"/>
+      <c r="G21" s="19"/>
+      <c r="H21" s="19"/>
+      <c r="I21" s="19"/>
       <c r="Q21" t="str">
         <f>IF(D21&gt;0,IF(D21="Unit",CONCATENATE(Settings!P21," ",Settings!D21,"s"),CONCATENATE((Settings!P21/Settings!L21)," ",Settings!D21,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="22" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A22" s="13"/>
       <c r="B22" s="14"/>
-      <c r="E22" s="22"/>
-      <c r="G22" s="22"/>
-      <c r="H22" s="22"/>
-      <c r="I22" s="22"/>
+      <c r="E22" s="19"/>
+      <c r="G22" s="19"/>
+      <c r="H22" s="19"/>
+      <c r="I22" s="19"/>
       <c r="Q22" t="str">
         <f>IF(D22&gt;0,IF(D22="Unit",CONCATENATE(Settings!P22," ",Settings!D22,"s"),CONCATENATE((Settings!P22/Settings!L22)," ",Settings!D22,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="23" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" s="13"/>
       <c r="B23" s="14"/>
-      <c r="E23" s="22"/>
-      <c r="G23" s="22"/>
-      <c r="H23" s="22"/>
-      <c r="I23" s="22"/>
+      <c r="E23" s="19"/>
+      <c r="G23" s="19"/>
+      <c r="H23" s="19"/>
+      <c r="I23" s="19"/>
       <c r="Q23" t="str">
         <f>IF(D23&gt;0,IF(D23="Unit",CONCATENATE(Settings!P23," ",Settings!D23,"s"),CONCATENATE((Settings!P23/Settings!L23)," ",Settings!D23,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="24" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" s="13"/>
       <c r="B24" s="14"/>
-      <c r="E24" s="22"/>
-      <c r="G24" s="22"/>
-      <c r="H24" s="22"/>
-      <c r="I24" s="22"/>
+      <c r="E24" s="19"/>
+      <c r="G24" s="19"/>
+      <c r="H24" s="19"/>
+      <c r="I24" s="19"/>
       <c r="Q24" t="str">
         <f>IF(D24&gt;0,IF(D24="Unit",CONCATENATE(Settings!P24," ",Settings!D24,"s"),CONCATENATE((Settings!P24/Settings!L24)," ",Settings!D24,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="25" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A25" s="13"/>
       <c r="B25" s="14"/>
-      <c r="E25" s="22"/>
-      <c r="G25" s="22"/>
-      <c r="H25" s="22"/>
-      <c r="I25" s="22"/>
+      <c r="E25" s="19"/>
+      <c r="G25" s="19"/>
+      <c r="H25" s="19"/>
+      <c r="I25" s="19"/>
       <c r="Q25" t="str">
         <f>IF(D25&gt;0,IF(D25="Unit",CONCATENATE(Settings!P25," ",Settings!D25,"s"),CONCATENATE((Settings!P25/Settings!L25)," ",Settings!D25,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="26" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26" s="13"/>
       <c r="B26" s="14"/>
-      <c r="E26" s="22"/>
-      <c r="G26" s="22"/>
-      <c r="H26" s="22"/>
-      <c r="I26" s="22"/>
+      <c r="E26" s="19"/>
+      <c r="G26" s="19"/>
+      <c r="H26" s="19"/>
+      <c r="I26" s="19"/>
       <c r="Q26" t="str">
         <f>IF(D26&gt;0,IF(D26="Unit",CONCATENATE(Settings!P26," ",Settings!D26,"s"),CONCATENATE((Settings!P26/Settings!L26)," ",Settings!D26,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="27" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27" s="13"/>
       <c r="B27" s="14"/>
-      <c r="E27" s="22"/>
-      <c r="G27" s="22"/>
-      <c r="H27" s="22"/>
-      <c r="I27" s="22"/>
+      <c r="E27" s="19"/>
+      <c r="G27" s="19"/>
+      <c r="H27" s="19"/>
+      <c r="I27" s="19"/>
       <c r="Q27" t="str">
         <f>IF(D27&gt;0,IF(D27="Unit",CONCATENATE(Settings!P27," ",Settings!D27,"s"),CONCATENATE((Settings!P27/Settings!L27)," ",Settings!D27,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="28" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A28" s="13"/>
       <c r="B28" s="14"/>
-      <c r="E28" s="22"/>
-      <c r="G28" s="22"/>
-      <c r="H28" s="22"/>
-      <c r="I28" s="22"/>
+      <c r="E28" s="19"/>
+      <c r="G28" s="19"/>
+      <c r="H28" s="19"/>
+      <c r="I28" s="19"/>
       <c r="Q28" t="str">
         <f>IF(D28&gt;0,IF(D28="Unit",CONCATENATE(Settings!P28," ",Settings!D28,"s"),CONCATENATE((Settings!P28/Settings!L28)," ",Settings!D28,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="29" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A29" s="13"/>
       <c r="B29" s="14"/>
-      <c r="E29" s="22"/>
-      <c r="G29" s="22"/>
-      <c r="H29" s="22"/>
-      <c r="I29" s="22"/>
+      <c r="E29" s="19"/>
+      <c r="G29" s="19"/>
+      <c r="H29" s="19"/>
+      <c r="I29" s="19"/>
       <c r="Q29" t="str">
         <f>IF(D29&gt;0,IF(D29="Unit",CONCATENATE(Settings!P29," ",Settings!D29,"s"),CONCATENATE((Settings!P29/Settings!L29)," ",Settings!D29,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="30" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A30" s="13"/>
       <c r="B30" s="14"/>
-      <c r="E30" s="22"/>
-      <c r="G30" s="22"/>
-      <c r="H30" s="22"/>
-      <c r="I30" s="22"/>
+      <c r="E30" s="19"/>
+      <c r="G30" s="19"/>
+      <c r="H30" s="19"/>
+      <c r="I30" s="19"/>
       <c r="Q30" t="str">
         <f>IF(D30&gt;0,IF(D30="Unit",CONCATENATE(Settings!P30," ",Settings!D30,"s"),CONCATENATE((Settings!P30/Settings!L30)," ",Settings!D30,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="31" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A31" s="13"/>
       <c r="B31" s="14"/>
-      <c r="E31" s="22"/>
-      <c r="G31" s="22"/>
-      <c r="H31" s="22"/>
-      <c r="I31" s="22"/>
+      <c r="E31" s="19"/>
+      <c r="G31" s="19"/>
+      <c r="H31" s="19"/>
+      <c r="I31" s="19"/>
       <c r="Q31" t="str">
         <f>IF(D31&gt;0,IF(D31="Unit",CONCATENATE(Settings!P31," ",Settings!D31,"s"),CONCATENATE((Settings!P31/Settings!L31)," ",Settings!D31,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="32" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A32" s="13"/>
       <c r="B32" s="14"/>
-      <c r="E32" s="22"/>
-      <c r="G32" s="22"/>
-      <c r="H32" s="22"/>
-      <c r="I32" s="22"/>
+      <c r="E32" s="19"/>
+      <c r="G32" s="19"/>
+      <c r="H32" s="19"/>
+      <c r="I32" s="19"/>
       <c r="Q32" t="str">
         <f>IF(D32&gt;0,IF(D32="Unit",CONCATENATE(Settings!P32," ",Settings!D32,"s"),CONCATENATE((Settings!P32/Settings!L32)," ",Settings!D32,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="33" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A33" s="13"/>
       <c r="B33" s="14"/>
-      <c r="E33" s="22"/>
-      <c r="G33" s="22"/>
-      <c r="H33" s="22"/>
-      <c r="I33" s="22"/>
+      <c r="E33" s="19"/>
+      <c r="G33" s="19"/>
+      <c r="H33" s="19"/>
+      <c r="I33" s="19"/>
       <c r="Q33" t="str">
         <f>IF(D33&gt;0,IF(D33="Unit",CONCATENATE(Settings!P33," ",Settings!D33,"s"),CONCATENATE((Settings!P33/Settings!L33)," ",Settings!D33,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="34" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A34" s="13"/>
       <c r="B34" s="14"/>
-      <c r="E34" s="22"/>
-      <c r="G34" s="22"/>
-      <c r="H34" s="22"/>
-      <c r="I34" s="22"/>
+      <c r="E34" s="19"/>
+      <c r="G34" s="19"/>
+      <c r="H34" s="19"/>
+      <c r="I34" s="19"/>
       <c r="Q34" t="str">
         <f>IF(D34&gt;0,IF(D34="Unit",CONCATENATE(Settings!P34," ",Settings!D34,"s"),CONCATENATE((Settings!P34/Settings!L34)," ",Settings!D34,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="35" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A35" s="13"/>
       <c r="B35" s="14"/>
-      <c r="E35" s="22"/>
-      <c r="G35" s="22"/>
-      <c r="H35" s="22"/>
-      <c r="I35" s="22"/>
+      <c r="E35" s="19"/>
+      <c r="G35" s="19"/>
+      <c r="H35" s="19"/>
+      <c r="I35" s="19"/>
       <c r="Q35" t="str">
         <f>IF(D35&gt;0,IF(D35="Unit",CONCATENATE(Settings!P35," ",Settings!D35,"s"),CONCATENATE((Settings!P35/Settings!L35)," ",Settings!D35,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="36" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A36" s="13"/>
       <c r="B36" s="14"/>
-      <c r="E36" s="22"/>
-      <c r="G36" s="22"/>
-      <c r="H36" s="22"/>
-      <c r="I36" s="22"/>
+      <c r="E36" s="19"/>
+      <c r="G36" s="19"/>
+      <c r="H36" s="19"/>
+      <c r="I36" s="19"/>
       <c r="Q36" t="str">
         <f>IF(D36&gt;0,IF(D36="Unit",CONCATENATE(Settings!P36," ",Settings!D36,"s"),CONCATENATE((Settings!P36/Settings!L36)," ",Settings!D36,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="37" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A37" s="13"/>
       <c r="B37" s="14"/>
-      <c r="E37" s="22"/>
-      <c r="G37" s="22"/>
-      <c r="H37" s="22"/>
-      <c r="I37" s="22"/>
+      <c r="E37" s="19"/>
+      <c r="G37" s="19"/>
+      <c r="H37" s="19"/>
+      <c r="I37" s="19"/>
       <c r="Q37" t="str">
         <f>IF(D37&gt;0,IF(D37="Unit",CONCATENATE(Settings!P37," ",Settings!D37,"s"),CONCATENATE((Settings!P37/Settings!L37)," ",Settings!D37,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="38" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A38" s="13"/>
       <c r="B38" s="14"/>
-      <c r="E38" s="22"/>
-      <c r="G38" s="22"/>
-      <c r="H38" s="22"/>
-      <c r="I38" s="22"/>
+      <c r="E38" s="19"/>
+      <c r="G38" s="19"/>
+      <c r="H38" s="19"/>
+      <c r="I38" s="19"/>
       <c r="Q38" t="str">
         <f>IF(D38&gt;0,IF(D38="Unit",CONCATENATE(Settings!P38," ",Settings!D38,"s"),CONCATENATE((Settings!P38/Settings!L38)," ",Settings!D38,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="39" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A39" s="13"/>
       <c r="B39" s="14"/>
-      <c r="E39" s="22"/>
-      <c r="G39" s="22"/>
-      <c r="H39" s="22"/>
-      <c r="I39" s="22"/>
+      <c r="E39" s="19"/>
+      <c r="G39" s="19"/>
+      <c r="H39" s="19"/>
+      <c r="I39" s="19"/>
       <c r="Q39" t="str">
         <f>IF(D39&gt;0,IF(D39="Unit",CONCATENATE(Settings!P39," ",Settings!D39,"s"),CONCATENATE((Settings!P39/Settings!L39)," ",Settings!D39,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="40" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A40" s="13"/>
       <c r="B40" s="14"/>
-      <c r="E40" s="22"/>
-      <c r="G40" s="22"/>
-      <c r="H40" s="22"/>
-      <c r="I40" s="22"/>
+      <c r="E40" s="19"/>
+      <c r="G40" s="19"/>
+      <c r="H40" s="19"/>
+      <c r="I40" s="19"/>
       <c r="Q40" t="str">
         <f>IF(D40&gt;0,IF(D40="Unit",CONCATENATE(Settings!P40," ",Settings!D40,"s"),CONCATENATE((Settings!P40/Settings!L40)," ",Settings!D40,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="41" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A41" s="13"/>
       <c r="B41" s="14"/>
-      <c r="E41" s="22"/>
-      <c r="G41" s="22"/>
-      <c r="H41" s="22"/>
-      <c r="I41" s="22"/>
+      <c r="E41" s="19"/>
+      <c r="G41" s="19"/>
+      <c r="H41" s="19"/>
+      <c r="I41" s="19"/>
       <c r="Q41" t="str">
         <f>IF(D41&gt;0,IF(D41="Unit",CONCATENATE(Settings!P41," ",Settings!D41,"s"),CONCATENATE((Settings!P41/Settings!L41)," ",Settings!D41,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="42" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A42" s="13"/>
       <c r="B42" s="14"/>
-      <c r="E42" s="22"/>
-      <c r="G42" s="22"/>
-      <c r="H42" s="22"/>
-      <c r="I42" s="22"/>
+      <c r="E42" s="19"/>
+      <c r="G42" s="19"/>
+      <c r="H42" s="19"/>
+      <c r="I42" s="19"/>
       <c r="Q42" t="str">
         <f>IF(D42&gt;0,IF(D42="Unit",CONCATENATE(Settings!P42," ",Settings!D42,"s"),CONCATENATE((Settings!P42/Settings!L42)," ",Settings!D42,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="43" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A43" s="13"/>
       <c r="B43" s="14"/>
-      <c r="E43" s="22"/>
-      <c r="G43" s="22"/>
-      <c r="H43" s="22"/>
-      <c r="I43" s="22"/>
+      <c r="E43" s="19"/>
+      <c r="G43" s="19"/>
+      <c r="H43" s="19"/>
+      <c r="I43" s="19"/>
       <c r="Q43" t="str">
         <f>IF(D43&gt;0,IF(D43="Unit",CONCATENATE(Settings!P43," ",Settings!D43,"s"),CONCATENATE((Settings!P43/Settings!L43)," ",Settings!D43,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="44" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A44" s="13"/>
       <c r="B44" s="14"/>
-      <c r="E44" s="22"/>
-      <c r="G44" s="22"/>
-      <c r="H44" s="22"/>
-      <c r="I44" s="22"/>
+      <c r="E44" s="19"/>
+      <c r="G44" s="19"/>
+      <c r="H44" s="19"/>
+      <c r="I44" s="19"/>
       <c r="Q44" t="str">
         <f>IF(D44&gt;0,IF(D44="Unit",CONCATENATE(Settings!P44," ",Settings!D44,"s"),CONCATENATE((Settings!P44/Settings!L44)," ",Settings!D44,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="45" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A45" s="13"/>
       <c r="B45" s="14"/>
-      <c r="E45" s="22"/>
-      <c r="G45" s="22"/>
-      <c r="H45" s="22"/>
-      <c r="I45" s="22"/>
+      <c r="E45" s="19"/>
+      <c r="G45" s="19"/>
+      <c r="H45" s="19"/>
+      <c r="I45" s="19"/>
       <c r="Q45" t="str">
         <f>IF(D45&gt;0,IF(D45="Unit",CONCATENATE(Settings!P45," ",Settings!D45,"s"),CONCATENATE((Settings!P45/Settings!L45)," ",Settings!D45,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="46" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A46" s="13"/>
       <c r="B46" s="14"/>
-      <c r="E46" s="22"/>
-      <c r="G46" s="22"/>
-      <c r="H46" s="22"/>
-      <c r="I46" s="22"/>
+      <c r="E46" s="19"/>
+      <c r="G46" s="19"/>
+      <c r="H46" s="19"/>
+      <c r="I46" s="19"/>
       <c r="Q46" t="str">
         <f>IF(D46&gt;0,IF(D46="Unit",CONCATENATE(Settings!P46," ",Settings!D46,"s"),CONCATENATE((Settings!P46/Settings!L46)," ",Settings!D46,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="47" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A47" s="13"/>
       <c r="B47" s="14"/>
-      <c r="E47" s="22"/>
-      <c r="G47" s="22"/>
-      <c r="H47" s="22"/>
-      <c r="I47" s="22"/>
+      <c r="E47" s="19"/>
+      <c r="G47" s="19"/>
+      <c r="H47" s="19"/>
+      <c r="I47" s="19"/>
       <c r="Q47" t="str">
         <f>IF(D47&gt;0,IF(D47="Unit",CONCATENATE(Settings!P47," ",Settings!D47,"s"),CONCATENATE((Settings!P47/Settings!L47)," ",Settings!D47,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="48" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A48" s="13"/>
       <c r="B48" s="14"/>
-      <c r="E48" s="22"/>
-      <c r="G48" s="22"/>
-      <c r="H48" s="22"/>
-      <c r="I48" s="22"/>
+      <c r="E48" s="19"/>
+      <c r="G48" s="19"/>
+      <c r="H48" s="19"/>
+      <c r="I48" s="19"/>
       <c r="Q48" t="str">
         <f>IF(D48&gt;0,IF(D48="Unit",CONCATENATE(Settings!P48," ",Settings!D48,"s"),CONCATENATE((Settings!P48/Settings!L48)," ",Settings!D48,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="49" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A49" s="13"/>
       <c r="B49" s="14"/>
-      <c r="E49" s="22"/>
-      <c r="G49" s="22"/>
-      <c r="H49" s="22"/>
-      <c r="I49" s="22"/>
+      <c r="E49" s="19"/>
+      <c r="G49" s="19"/>
+      <c r="H49" s="19"/>
+      <c r="I49" s="19"/>
       <c r="Q49" t="str">
         <f>IF(D49&gt;0,IF(D49="Unit",CONCATENATE(Settings!P49," ",Settings!D49,"s"),CONCATENATE((Settings!P49/Settings!L49)," ",Settings!D49,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="50" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" s="13"/>
       <c r="B50" s="14"/>
-      <c r="E50" s="22"/>
-      <c r="G50" s="22"/>
-      <c r="H50" s="22"/>
-      <c r="I50" s="22"/>
+      <c r="E50" s="19"/>
+      <c r="G50" s="19"/>
+      <c r="H50" s="19"/>
+      <c r="I50" s="19"/>
       <c r="Q50" t="str">
         <f>IF(D50&gt;0,IF(D50="Unit",CONCATENATE(Settings!P50," ",Settings!D50,"s"),CONCATENATE((Settings!P50/Settings!L50)," ",Settings!D50,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="51" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A51" s="13"/>
       <c r="B51" s="14"/>
-      <c r="E51" s="22"/>
-      <c r="G51" s="22"/>
-      <c r="H51" s="22"/>
-      <c r="I51" s="22"/>
+      <c r="E51" s="19"/>
+      <c r="G51" s="19"/>
+      <c r="H51" s="19"/>
+      <c r="I51" s="19"/>
       <c r="Q51" t="str">
         <f>IF(D51&gt;0,IF(D51="Unit",CONCATENATE(Settings!P51," ",Settings!D51,"s"),CONCATENATE((Settings!P51/Settings!L51)," ",Settings!D51,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="52" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A52" s="15"/>
       <c r="B52" s="16"/>
-      <c r="E52" s="22"/>
-      <c r="G52" s="22"/>
-      <c r="H52" s="22"/>
-      <c r="I52" s="22"/>
+      <c r="E52" s="19"/>
+      <c r="G52" s="19"/>
+      <c r="H52" s="19"/>
+      <c r="I52" s="19"/>
       <c r="Q52" t="str">
         <f>IF(D52&gt;0,IF(D52="Unit",CONCATENATE(Settings!P52," ",Settings!D52,"s"),CONCATENATE((Settings!P52/Settings!L52)," ",Settings!D52,"s")),"")</f>
         <v/>
@@ -2841,6 +2838,9 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967294" verticalDpi="0" r:id="rId1"/>
+  <headerFooter>
+    <oddFooter>&amp;R_x000D_&amp;1#&amp;"Calibri"&amp;22&amp;KFF8939 RESTRICTED</oddFooter>
+  </headerFooter>
   <tableParts count="2">
     <tablePart r:id="rId2"/>
     <tablePart r:id="rId3"/>
@@ -2863,6 +2863,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010075F372E8CCA016418A193AD921508903" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="f5e922417d740f1a527805650dc2dfa9">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="399317f3-0083-4d0b-9572-12af99626311" xmlns:ns3="1444eecc-14bb-4066-abe6-ce6de21d9439" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="078d79524add6eac9b94134ca637184e" ns2:_="" ns3:_="">
     <xsd:import namespace="399317f3-0083-4d0b-9572-12af99626311"/>
@@ -3059,15 +3068,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7EBE950A-5812-419E-B174-6A5D9B8E0414}">
   <ds:schemaRefs>
@@ -3079,6 +3079,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A00E6A9-20DD-4842-9306-307EB080AF2E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8CF88A1C-AA0D-4F8F-A0FD-6F3FAFCA9DC0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3095,12 +3103,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A00E6A9-20DD-4842-9306-307EB080AF2E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Payment terms in revised offer
</commit_message>
<xml_diff>
--- a/srv/xlsx-templates/TH - Quotation Template.xlsx
+++ b/srv/xlsx-templates/TH - Quotation Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EHQUT\Desktop\Thailand Template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80F5D0EE-04D5-4DC3-9DF3-07A3D550A529}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73333E37-04FD-4197-8192-532B6D370846}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{F5CC2154-27BB-4652-B61E-D913F0CC6809}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="115">
   <si>
     <t>${offerValidation.INSTITUTENAME}</t>
   </si>
@@ -101,9 +101,6 @@
   </si>
   <si>
     <t>${offerValidation.SHIPMENTTERMS}</t>
-  </si>
-  <si>
-    <t>${table:offerProductValidation.PRODUCT_UNIT_NAME}</t>
   </si>
   <si>
     <t>${table:offerProductValidation.SKU}</t>
@@ -291,9 +288,6 @@
 Discount</t>
   </si>
   <si>
-    <t>Total Offer Value</t>
-  </si>
-  <si>
     <t>excl. vat.</t>
   </si>
   <si>
@@ -373,10 +367,22 @@
     <t>Position</t>
   </si>
   <si>
-    <t>=Settings!A4</t>
-  </si>
-  <si>
-    <t>=Settings!A5</t>
+    <t>${offerValidation.SELLINGCOMPANY}</t>
+  </si>
+  <si>
+    <t>${offerValidation.DISTRIBUTORNAME}</t>
+  </si>
+  <si>
+    <t>${offerValidation.DISTRIBUTORADDRESS}</t>
+  </si>
+  <si>
+    <t>${table:offerProductValidation.PRODUCTNAME}</t>
+  </si>
+  <si>
+    <t>${table:offerProductValidation.PAID_VOLUME} / ${table:offerProductValidation.UNIT}</t>
+  </si>
+  <si>
+    <t>${offerValidation.CUSTOMER_CODE}</t>
   </si>
 </sst>
 </file>
@@ -754,7 +760,7 @@
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="108">
+  <cellXfs count="119">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -790,7 +796,6 @@
     <xf numFmtId="43" fontId="5" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="43" fontId="5" fillId="0" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="5" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="43" fontId="6" fillId="0" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -840,7 +845,112 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -852,55 +962,58 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -933,107 +1046,35 @@
     <xf numFmtId="0" fontId="10" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1206,8 +1247,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5B6DC07E-0020-4B51-98A2-ADA62A91E75D}" name="Tabel1" displayName="Tabel1" ref="A1:B13" totalsRowShown="0" headerRowDxfId="6">
-  <autoFilter ref="A1:B13" xr:uid="{5B6DC07E-0020-4B51-98A2-ADA62A91E75D}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5B6DC07E-0020-4B51-98A2-ADA62A91E75D}" name="Tabel1" displayName="Tabel1" ref="A1:B14" totalsRowShown="0" headerRowDxfId="6">
+  <autoFilter ref="A1:B14" xr:uid="{5B6DC07E-0020-4B51-98A2-ADA62A91E75D}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{22EAB7A2-53F9-497F-A4B5-CA34E48AC441}" name="Header fields"/>
     <tableColumn id="2" xr3:uid="{331DD14B-B263-41D9-B2C5-D198B6F2436E}" name="Description"/>
@@ -1543,7 +1584,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFBA1999-1CF9-4903-BA7D-DD523B82D6C3}">
-  <dimension ref="B2:S44"/>
+  <dimension ref="B2:T44"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="11.140625" customWidth="1"/>
@@ -1551,7 +1592,7 @@
     <col min="10" max="10" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:19" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B2" s="10"/>
       <c r="C2" s="10"/>
       <c r="D2" s="10"/>
@@ -1569,54 +1610,59 @@
       <c r="P2" s="10"/>
       <c r="Q2" s="10"/>
     </row>
-    <row r="3" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B3" s="36" t="s">
-        <v>64</v>
-      </c>
-      <c r="C3" s="59" t="str">
-        <f>Settings!A9</f>
-        <v>${offerValidation.INSTITUTENAME}</v>
-      </c>
-      <c r="D3" s="59"/>
-      <c r="E3" s="59"/>
-      <c r="F3" s="59"/>
-      <c r="G3" s="59"/>
+    <row r="3" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B3" s="35" t="s">
+        <v>63</v>
+      </c>
+      <c r="C3" s="97" t="s">
+        <v>110</v>
+      </c>
+      <c r="D3" s="97"/>
+      <c r="E3" s="97"/>
+      <c r="F3" s="97"/>
+      <c r="G3" s="97"/>
       <c r="H3" s="11"/>
       <c r="I3" s="10"/>
-      <c r="J3" s="36" t="s">
-        <v>65</v>
-      </c>
-      <c r="K3" s="59"/>
-      <c r="L3" s="59"/>
-      <c r="M3" s="59"/>
-      <c r="N3" s="59"/>
+      <c r="J3" s="35" t="s">
+        <v>64</v>
+      </c>
+      <c r="K3" s="97" t="str">
+        <f>Settings!A11</f>
+        <v>${offerValidation.SELLINGCOMPANY}</v>
+      </c>
+      <c r="L3" s="97"/>
+      <c r="M3" s="97"/>
+      <c r="N3" s="97"/>
       <c r="O3" s="10"/>
       <c r="P3" s="10"/>
       <c r="Q3" s="10"/>
     </row>
-    <row r="4" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B4" s="36" t="s">
-        <v>66</v>
-      </c>
-      <c r="C4" s="60"/>
-      <c r="D4" s="61"/>
-      <c r="E4" s="61"/>
-      <c r="F4" s="61"/>
-      <c r="G4" s="62"/>
+    <row r="4" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B4" s="35" t="s">
+        <v>65</v>
+      </c>
+      <c r="C4" s="94" t="str">
+        <f>Settings!A13</f>
+        <v>${offerValidation.DISTRIBUTORADDRESS}</v>
+      </c>
+      <c r="D4" s="95"/>
+      <c r="E4" s="95"/>
+      <c r="F4" s="95"/>
+      <c r="G4" s="96"/>
       <c r="H4" s="12"/>
       <c r="I4" s="10"/>
-      <c r="J4" s="36" t="s">
-        <v>66</v>
-      </c>
-      <c r="K4" s="63"/>
-      <c r="L4" s="64"/>
-      <c r="M4" s="64"/>
-      <c r="N4" s="65"/>
+      <c r="J4" s="35" t="s">
+        <v>65</v>
+      </c>
+      <c r="K4" s="98"/>
+      <c r="L4" s="99"/>
+      <c r="M4" s="99"/>
+      <c r="N4" s="100"/>
       <c r="O4" s="10"/>
       <c r="P4" s="10"/>
       <c r="Q4" s="10"/>
     </row>
-    <row r="5" spans="2:19" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B5" s="13"/>
       <c r="C5" s="12"/>
       <c r="D5" s="12"/>
@@ -1634,7 +1680,7 @@
       <c r="P5" s="10"/>
       <c r="Q5" s="10"/>
     </row>
-    <row r="6" spans="2:19" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B6" s="10"/>
       <c r="C6" s="10"/>
       <c r="D6" s="10"/>
@@ -1652,154 +1698,158 @@
       <c r="P6" s="10"/>
       <c r="Q6" s="10"/>
     </row>
-    <row r="7" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B7" s="67" t="s">
+    <row r="7" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B7" s="102" t="s">
+        <v>66</v>
+      </c>
+      <c r="C7" s="103"/>
+      <c r="D7" s="103"/>
+      <c r="E7" s="103"/>
+      <c r="F7" s="103"/>
+      <c r="G7" s="103"/>
+      <c r="H7" s="103"/>
+      <c r="I7" s="103"/>
+      <c r="J7" s="103"/>
+      <c r="K7" s="103"/>
+      <c r="L7" s="103"/>
+      <c r="M7" s="103"/>
+      <c r="N7" s="103"/>
+      <c r="O7" s="103"/>
+      <c r="P7" s="103"/>
+      <c r="Q7" s="103"/>
+      <c r="R7" s="103"/>
+      <c r="S7" s="104"/>
+    </row>
+    <row r="8" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B8" s="101" t="s">
         <v>67</v>
       </c>
-      <c r="C7" s="68"/>
-      <c r="D7" s="68"/>
-      <c r="E7" s="68"/>
-      <c r="F7" s="68"/>
-      <c r="G7" s="68"/>
-      <c r="H7" s="68"/>
-      <c r="I7" s="68"/>
-      <c r="J7" s="68"/>
-      <c r="K7" s="68"/>
-      <c r="L7" s="68"/>
-      <c r="M7" s="68"/>
-      <c r="N7" s="68"/>
-      <c r="O7" s="68"/>
-      <c r="P7" s="68"/>
-      <c r="Q7" s="68"/>
-      <c r="R7" s="68"/>
-      <c r="S7" s="69"/>
-    </row>
-    <row r="8" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B8" s="66" t="s">
+      <c r="C8" s="101"/>
+      <c r="D8" s="94"/>
+      <c r="E8" s="95"/>
+      <c r="F8" s="95"/>
+      <c r="G8" s="95"/>
+      <c r="H8" s="96"/>
+      <c r="I8" s="105" t="s">
         <v>68</v>
       </c>
-      <c r="C8" s="66"/>
-      <c r="D8" s="60"/>
-      <c r="E8" s="61"/>
-      <c r="F8" s="61"/>
-      <c r="G8" s="61"/>
-      <c r="H8" s="62"/>
-      <c r="I8" s="70" t="s">
+      <c r="J8" s="106"/>
+      <c r="K8" s="49"/>
+      <c r="L8" s="50"/>
+      <c r="M8" s="50"/>
+      <c r="N8" s="51"/>
+      <c r="O8" s="33" t="s">
         <v>69</v>
       </c>
-      <c r="J8" s="71"/>
-      <c r="K8" s="104"/>
-      <c r="L8" s="105"/>
-      <c r="M8" s="105"/>
-      <c r="N8" s="106"/>
-      <c r="O8" s="34" t="s">
+      <c r="P8" s="34"/>
+      <c r="Q8" s="48"/>
+      <c r="R8" s="48"/>
+      <c r="S8" s="48"/>
+    </row>
+    <row r="9" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B9" s="101" t="s">
         <v>70</v>
       </c>
-      <c r="P8" s="35"/>
-      <c r="Q8" s="103"/>
-      <c r="R8" s="103"/>
-      <c r="S8" s="103"/>
-    </row>
-    <row r="9" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B9" s="66" t="s">
+      <c r="C9" s="101"/>
+      <c r="D9" s="94" t="str">
+        <f>Settings!A14</f>
+        <v>${offerValidation.CUSTOMER_CODE}</v>
+      </c>
+      <c r="E9" s="95"/>
+      <c r="F9" s="95"/>
+      <c r="G9" s="95"/>
+      <c r="H9" s="96"/>
+      <c r="I9" s="107" t="s">
         <v>71</v>
       </c>
-      <c r="C9" s="66"/>
-      <c r="D9" s="60"/>
-      <c r="E9" s="61"/>
-      <c r="F9" s="61"/>
-      <c r="G9" s="61"/>
-      <c r="H9" s="62"/>
-      <c r="I9" s="72" t="s">
+      <c r="J9" s="108"/>
+      <c r="K9" s="52" t="s">
+        <v>17</v>
+      </c>
+      <c r="L9" s="52"/>
+      <c r="M9" s="52"/>
+      <c r="N9" s="52"/>
+      <c r="O9" s="33" t="s">
         <v>72</v>
       </c>
-      <c r="J9" s="73"/>
-      <c r="K9" s="107" t="s">
-        <v>111</v>
-      </c>
-      <c r="L9" s="107"/>
-      <c r="M9" s="107"/>
-      <c r="N9" s="107"/>
-      <c r="O9" s="34" t="s">
+      <c r="P9" s="34"/>
+      <c r="Q9" s="48"/>
+      <c r="R9" s="48"/>
+      <c r="S9" s="48"/>
+    </row>
+    <row r="10" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B10" s="101" t="s">
         <v>73</v>
       </c>
-      <c r="P9" s="35"/>
-      <c r="Q9" s="103"/>
-      <c r="R9" s="103"/>
-      <c r="S9" s="103"/>
-    </row>
-    <row r="10" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B10" s="66" t="s">
+      <c r="C10" s="101"/>
+      <c r="D10" s="94"/>
+      <c r="E10" s="95"/>
+      <c r="F10" s="95"/>
+      <c r="G10" s="95"/>
+      <c r="H10" s="96"/>
+      <c r="I10" s="92" t="s">
+        <v>5</v>
+      </c>
+      <c r="J10" s="93"/>
+      <c r="K10" s="52" t="s">
+        <v>18</v>
+      </c>
+      <c r="L10" s="52"/>
+      <c r="M10" s="52"/>
+      <c r="N10" s="52"/>
+      <c r="O10" s="33" t="s">
         <v>74</v>
       </c>
-      <c r="C10" s="66"/>
-      <c r="D10" s="60"/>
-      <c r="E10" s="61"/>
-      <c r="F10" s="61"/>
-      <c r="G10" s="61"/>
-      <c r="H10" s="62"/>
-      <c r="I10" s="74" t="s">
-        <v>5</v>
-      </c>
-      <c r="J10" s="75"/>
-      <c r="K10" s="107" t="s">
-        <v>112</v>
-      </c>
-      <c r="L10" s="107"/>
-      <c r="M10" s="107"/>
-      <c r="N10" s="107"/>
-      <c r="O10" s="34" t="s">
-        <v>75</v>
-      </c>
-      <c r="P10" s="35"/>
-      <c r="Q10" s="103"/>
-      <c r="R10" s="103"/>
-      <c r="S10" s="103"/>
-    </row>
-    <row r="11" spans="2:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="66" t="s">
+      <c r="P10" s="34"/>
+      <c r="Q10" s="48"/>
+      <c r="R10" s="48"/>
+      <c r="S10" s="48"/>
+    </row>
+    <row r="11" spans="2:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="101" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="66"/>
-      <c r="D11" s="76" t="str">
-        <f>Settings!A6</f>
-        <v>${offerValidation.SHIPMENTTERMS}</v>
-      </c>
-      <c r="E11" s="77"/>
-      <c r="F11" s="77"/>
-      <c r="G11" s="77"/>
-      <c r="H11" s="78"/>
-      <c r="I11" s="70" t="s">
+      <c r="C11" s="101"/>
+      <c r="D11" s="89" t="str">
+        <f>Settings!A12</f>
+        <v>${offerValidation.DISTRIBUTORNAME}</v>
+      </c>
+      <c r="E11" s="90"/>
+      <c r="F11" s="90"/>
+      <c r="G11" s="90"/>
+      <c r="H11" s="91"/>
+      <c r="I11" s="105" t="s">
         <v>7</v>
       </c>
-      <c r="J11" s="71"/>
-      <c r="K11" s="102" t="str">
+      <c r="J11" s="106"/>
+      <c r="K11" s="47" t="str">
         <f>Settings!A7</f>
         <v>${offerValidation.PAYMENTTERMS}</v>
       </c>
-      <c r="L11" s="102"/>
-      <c r="M11" s="102"/>
-      <c r="N11" s="102"/>
-      <c r="O11" s="34" t="s">
-        <v>73</v>
-      </c>
-      <c r="P11" s="35"/>
-      <c r="Q11" s="103"/>
-      <c r="R11" s="103"/>
-      <c r="S11" s="103"/>
-    </row>
-    <row r="12" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B12" s="66" t="s">
+      <c r="L11" s="47"/>
+      <c r="M11" s="47"/>
+      <c r="N11" s="47"/>
+      <c r="O11" s="33" t="s">
+        <v>72</v>
+      </c>
+      <c r="P11" s="34"/>
+      <c r="Q11" s="48"/>
+      <c r="R11" s="48"/>
+      <c r="S11" s="48"/>
+    </row>
+    <row r="12" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B12" s="101" t="s">
         <v>8</v>
       </c>
-      <c r="C12" s="66"/>
-      <c r="D12" s="76" t="s">
-        <v>19</v>
-      </c>
-      <c r="E12" s="77"/>
-      <c r="F12" s="77"/>
-      <c r="G12" s="77"/>
-      <c r="H12" s="78"/>
+      <c r="C12" s="101"/>
+      <c r="D12" s="89" t="str">
+        <f>Settings!A8</f>
+        <v>${offerValidation.DELIVERYTERMS}</v>
+      </c>
+      <c r="E12" s="90"/>
+      <c r="F12" s="90"/>
+      <c r="G12" s="90"/>
+      <c r="H12" s="91"/>
       <c r="I12" s="10"/>
       <c r="J12" s="10"/>
       <c r="K12" s="10"/>
@@ -1810,7 +1860,7 @@
       <c r="P12" s="10"/>
       <c r="Q12" s="10"/>
     </row>
-    <row r="13" spans="2:19" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B13" s="10"/>
       <c r="C13" s="10"/>
       <c r="D13" s="10"/>
@@ -1828,179 +1878,198 @@
       <c r="P13" s="10"/>
       <c r="Q13" s="10"/>
     </row>
-    <row r="14" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B14" s="43" t="s">
+    <row r="14" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B14" s="114" t="s">
+        <v>75</v>
+      </c>
+      <c r="C14" s="115"/>
+      <c r="D14" s="115"/>
+      <c r="E14" s="115"/>
+      <c r="F14" s="115"/>
+      <c r="G14" s="115"/>
+      <c r="H14" s="115"/>
+      <c r="I14" s="115"/>
+      <c r="J14" s="115"/>
+      <c r="K14" s="115"/>
+      <c r="L14" s="115"/>
+      <c r="M14" s="115"/>
+      <c r="N14" s="115"/>
+      <c r="O14" s="115"/>
+      <c r="P14" s="115"/>
+      <c r="Q14" s="115"/>
+      <c r="R14" s="115"/>
+    </row>
+    <row r="15" spans="2:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="78" t="s">
         <v>76</v>
       </c>
-      <c r="C14" s="43"/>
-      <c r="D14" s="43"/>
-      <c r="E14" s="43"/>
-      <c r="F14" s="43"/>
-      <c r="G14" s="43"/>
-      <c r="H14" s="43"/>
-      <c r="I14" s="43"/>
-      <c r="J14" s="43"/>
-      <c r="K14" s="43"/>
-      <c r="L14" s="43"/>
-      <c r="M14" s="43"/>
-      <c r="N14" s="43"/>
-      <c r="O14" s="43"/>
-      <c r="P14" s="43"/>
-      <c r="Q14" s="43"/>
-    </row>
-    <row r="15" spans="2:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="44" t="s">
+      <c r="C15" s="74" t="s">
         <v>77</v>
       </c>
-      <c r="C15" s="47" t="s">
+      <c r="D15" s="88" t="s">
         <v>78</v>
       </c>
-      <c r="D15" s="50" t="s">
+      <c r="E15" s="88"/>
+      <c r="F15" s="88"/>
+      <c r="G15" s="68" t="s">
         <v>79</v>
       </c>
-      <c r="E15" s="51"/>
-      <c r="F15" s="79" t="s">
+      <c r="H15" s="84"/>
+      <c r="I15" s="84"/>
+      <c r="J15" s="88" t="s">
         <v>80</v>
       </c>
-      <c r="G15" s="79"/>
-      <c r="H15" s="47" t="s">
+      <c r="K15" s="88"/>
+      <c r="L15" s="88"/>
+      <c r="M15" s="88" t="s">
+        <v>9</v>
+      </c>
+      <c r="N15" s="88"/>
+      <c r="O15" s="74" t="s">
         <v>81</v>
       </c>
-      <c r="I15" s="47" t="s">
-        <v>9</v>
-      </c>
-      <c r="J15" s="47" t="s">
+      <c r="P15" s="42" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q15" s="43"/>
+      <c r="R15" s="74" t="s">
         <v>82</v>
       </c>
-      <c r="K15" s="50" t="s">
-        <v>10</v>
-      </c>
-      <c r="L15" s="51"/>
-      <c r="M15" s="47" t="s">
+      <c r="S15" s="68" t="s">
+        <v>14</v>
+      </c>
+      <c r="T15" s="69"/>
+    </row>
+    <row r="16" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B16" s="79"/>
+      <c r="C16" s="75"/>
+      <c r="D16" s="88"/>
+      <c r="E16" s="88"/>
+      <c r="F16" s="88"/>
+      <c r="G16" s="70"/>
+      <c r="H16" s="109"/>
+      <c r="I16" s="109"/>
+      <c r="J16" s="88"/>
+      <c r="K16" s="88"/>
+      <c r="L16" s="88"/>
+      <c r="M16" s="88"/>
+      <c r="N16" s="88"/>
+      <c r="O16" s="75"/>
+      <c r="P16" s="44"/>
+      <c r="Q16" s="45"/>
+      <c r="R16" s="75"/>
+      <c r="S16" s="72"/>
+      <c r="T16" s="73"/>
+    </row>
+    <row r="17" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B17" s="80"/>
+      <c r="C17" s="76"/>
+      <c r="D17" s="88"/>
+      <c r="E17" s="88"/>
+      <c r="F17" s="88"/>
+      <c r="G17" s="70"/>
+      <c r="H17" s="109"/>
+      <c r="I17" s="109"/>
+      <c r="J17" s="88"/>
+      <c r="K17" s="88"/>
+      <c r="L17" s="88"/>
+      <c r="M17" s="88"/>
+      <c r="N17" s="88"/>
+      <c r="O17" s="76"/>
+      <c r="P17" s="15" t="s">
         <v>83</v>
       </c>
-      <c r="N15" s="50" t="s">
-        <v>14</v>
-      </c>
-      <c r="O15" s="51"/>
-      <c r="P15" s="50" t="s">
+      <c r="Q17" s="15" t="s">
         <v>84</v>
       </c>
-      <c r="Q15" s="51"/>
-    </row>
-    <row r="16" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B16" s="45"/>
-      <c r="C16" s="48"/>
-      <c r="D16" s="52"/>
-      <c r="E16" s="53"/>
-      <c r="F16" s="79"/>
-      <c r="G16" s="79"/>
-      <c r="H16" s="48"/>
-      <c r="I16" s="48"/>
-      <c r="J16" s="48"/>
-      <c r="K16" s="54"/>
-      <c r="L16" s="55"/>
-      <c r="M16" s="48"/>
-      <c r="N16" s="54"/>
-      <c r="O16" s="55"/>
-      <c r="P16" s="54"/>
-      <c r="Q16" s="55"/>
-    </row>
-    <row r="17" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B17" s="46"/>
-      <c r="C17" s="49"/>
-      <c r="D17" s="54"/>
-      <c r="E17" s="55"/>
-      <c r="F17" s="79"/>
-      <c r="G17" s="79"/>
-      <c r="H17" s="49"/>
-      <c r="I17" s="49"/>
-      <c r="J17" s="49"/>
-      <c r="K17" s="15" t="s">
-        <v>85</v>
-      </c>
-      <c r="L17" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="M17" s="49"/>
-      <c r="N17" s="15" t="s">
-        <v>85</v>
-      </c>
-      <c r="O17" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="P17" s="15" t="s">
-        <v>85</v>
-      </c>
-      <c r="Q17" s="15" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="18" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="R17" s="76"/>
+      <c r="S17" s="15" t="s">
+        <v>83</v>
+      </c>
+      <c r="T17" s="15" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="18" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B18" s="16">
         <v>1</v>
       </c>
-      <c r="C18" s="16"/>
-      <c r="D18" s="56"/>
-      <c r="E18" s="57"/>
-      <c r="F18" s="58"/>
-      <c r="G18" s="58"/>
-      <c r="H18" s="16"/>
-      <c r="I18" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="J18" s="16"/>
-      <c r="K18" s="18"/>
-      <c r="L18" s="19"/>
-      <c r="M18" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="N18" s="18"/>
-      <c r="O18" s="18"/>
+      <c r="C18" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D18" s="110" t="s">
+        <v>112</v>
+      </c>
+      <c r="E18" s="111"/>
+      <c r="F18" s="112"/>
+      <c r="G18" s="113"/>
+      <c r="H18" s="113"/>
+      <c r="I18" s="113"/>
+      <c r="J18" s="116" t="s">
+        <v>113</v>
+      </c>
+      <c r="K18" s="116"/>
+      <c r="L18" s="116"/>
+      <c r="M18" s="117" t="s">
+        <v>23</v>
+      </c>
+      <c r="N18" s="118"/>
+      <c r="O18" s="16"/>
       <c r="P18" s="18"/>
-      <c r="Q18" s="21"/>
-    </row>
-    <row r="19" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="Q18" s="19"/>
+      <c r="R18" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="S18" s="18"/>
+      <c r="T18" s="18"/>
+    </row>
+    <row r="19" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B19" s="16">
         <v>2</v>
       </c>
       <c r="C19" s="16"/>
-      <c r="D19" s="56"/>
-      <c r="E19" s="57"/>
-      <c r="F19" s="58"/>
-      <c r="G19" s="58"/>
-      <c r="H19" s="16"/>
-      <c r="I19" s="17"/>
-      <c r="J19" s="16"/>
-      <c r="K19" s="19"/>
-      <c r="L19" s="19"/>
-      <c r="M19" s="20"/>
-      <c r="N19" s="18"/>
-      <c r="O19" s="18"/>
-      <c r="P19" s="18"/>
-      <c r="Q19" s="21"/>
-    </row>
-    <row r="20" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="D19" s="87"/>
+      <c r="E19" s="87"/>
+      <c r="F19" s="87"/>
+      <c r="G19" s="113"/>
+      <c r="H19" s="113"/>
+      <c r="I19" s="113"/>
+      <c r="J19" s="87"/>
+      <c r="K19" s="87"/>
+      <c r="L19" s="87"/>
+      <c r="M19" s="17"/>
+      <c r="N19" s="17"/>
+      <c r="O19" s="16"/>
+      <c r="P19" s="19"/>
+      <c r="Q19" s="19"/>
+      <c r="R19" s="20"/>
+      <c r="S19" s="18"/>
+      <c r="T19" s="18"/>
+    </row>
+    <row r="20" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B20" s="16">
         <v>3</v>
       </c>
       <c r="C20" s="16"/>
-      <c r="D20" s="56"/>
-      <c r="E20" s="57"/>
-      <c r="F20" s="58"/>
-      <c r="G20" s="58"/>
-      <c r="H20" s="16"/>
-      <c r="I20" s="17"/>
-      <c r="J20" s="16"/>
-      <c r="K20" s="19"/>
-      <c r="L20" s="19"/>
-      <c r="M20" s="20"/>
-      <c r="N20" s="18"/>
-      <c r="O20" s="18"/>
-      <c r="P20" s="18"/>
-      <c r="Q20" s="21"/>
-    </row>
-    <row r="21" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="D20" s="87"/>
+      <c r="E20" s="87"/>
+      <c r="F20" s="87"/>
+      <c r="G20" s="113"/>
+      <c r="H20" s="113"/>
+      <c r="I20" s="113"/>
+      <c r="J20" s="87"/>
+      <c r="K20" s="87"/>
+      <c r="L20" s="87"/>
+      <c r="M20" s="16"/>
+      <c r="N20" s="16"/>
+      <c r="O20" s="16"/>
+      <c r="P20" s="19"/>
+      <c r="Q20" s="19"/>
+      <c r="R20" s="20"/>
+      <c r="S20" s="18"/>
+      <c r="T20" s="18"/>
+    </row>
+    <row r="21" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B21" s="10"/>
       <c r="C21" s="10"/>
       <c r="D21" s="10"/>
@@ -2018,165 +2087,165 @@
       <c r="P21" s="10"/>
       <c r="Q21" s="10"/>
     </row>
-    <row r="22" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B22" s="80" t="s">
-        <v>87</v>
-      </c>
-      <c r="C22" s="80"/>
-      <c r="D22" s="80"/>
-      <c r="E22" s="80"/>
-      <c r="F22" s="80"/>
-      <c r="G22" s="80"/>
-      <c r="H22" s="80"/>
-      <c r="I22" s="80"/>
-      <c r="J22" s="80"/>
-      <c r="K22" s="80"/>
-      <c r="L22" s="80"/>
-      <c r="M22" s="80"/>
+    <row r="22" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B22" s="67" t="s">
+        <v>85</v>
+      </c>
+      <c r="C22" s="67"/>
+      <c r="D22" s="67"/>
+      <c r="E22" s="67"/>
+      <c r="F22" s="67"/>
+      <c r="G22" s="67"/>
+      <c r="H22" s="67"/>
+      <c r="I22" s="67"/>
+      <c r="J22" s="67"/>
+      <c r="K22" s="67"/>
+      <c r="L22" s="67"/>
+      <c r="M22" s="67"/>
       <c r="N22" s="10"/>
       <c r="O22" s="10"/>
       <c r="P22" s="10"/>
       <c r="Q22" s="10"/>
     </row>
-    <row r="23" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B23" s="44" t="s">
+    <row r="23" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B23" s="78" t="s">
+        <v>76</v>
+      </c>
+      <c r="C23" s="74" t="s">
         <v>77</v>
       </c>
-      <c r="C23" s="47" t="s">
-        <v>78</v>
-      </c>
-      <c r="D23" s="39"/>
-      <c r="E23" s="83" t="s">
+      <c r="D23" s="38"/>
+      <c r="E23" s="81" t="s">
+        <v>86</v>
+      </c>
+      <c r="F23" s="74" t="s">
+        <v>87</v>
+      </c>
+      <c r="G23" s="74" t="s">
         <v>88</v>
       </c>
-      <c r="F23" s="47" t="s">
+      <c r="H23" s="68" t="s">
         <v>89</v>
       </c>
-      <c r="G23" s="47" t="s">
+      <c r="I23" s="84"/>
+      <c r="J23" s="69"/>
+      <c r="K23" s="68" t="s">
         <v>90</v>
       </c>
-      <c r="H23" s="50" t="s">
+      <c r="L23" s="69"/>
+      <c r="M23" s="74" t="s">
         <v>91</v>
-      </c>
-      <c r="I23" s="86"/>
-      <c r="J23" s="51"/>
-      <c r="K23" s="50" t="s">
-        <v>92</v>
-      </c>
-      <c r="L23" s="51"/>
-      <c r="M23" s="47" t="s">
-        <v>93</v>
       </c>
       <c r="N23" s="10"/>
       <c r="O23" s="10"/>
-      <c r="P23" s="42"/>
+      <c r="P23" s="41"/>
       <c r="Q23" s="10"/>
     </row>
-    <row r="24" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="45"/>
-      <c r="C24" s="48"/>
-      <c r="D24" s="40"/>
-      <c r="E24" s="84"/>
-      <c r="F24" s="48"/>
-      <c r="G24" s="48"/>
-      <c r="H24" s="52"/>
-      <c r="I24" s="87"/>
-      <c r="J24" s="53"/>
-      <c r="K24" s="52"/>
-      <c r="L24" s="53"/>
-      <c r="M24" s="48"/>
+    <row r="24" spans="2:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="79"/>
+      <c r="C24" s="75"/>
+      <c r="D24" s="39"/>
+      <c r="E24" s="82"/>
+      <c r="F24" s="75"/>
+      <c r="G24" s="75"/>
+      <c r="H24" s="70"/>
+      <c r="I24" s="85"/>
+      <c r="J24" s="71"/>
+      <c r="K24" s="70"/>
+      <c r="L24" s="71"/>
+      <c r="M24" s="75"/>
       <c r="N24" s="10"/>
       <c r="O24" s="10"/>
-      <c r="P24" s="42"/>
+      <c r="P24" s="41"/>
       <c r="Q24" s="10"/>
     </row>
-    <row r="25" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B25" s="46"/>
-      <c r="C25" s="49"/>
-      <c r="D25" s="41"/>
-      <c r="E25" s="85"/>
-      <c r="F25" s="49"/>
-      <c r="G25" s="49"/>
-      <c r="H25" s="54"/>
-      <c r="I25" s="88"/>
-      <c r="J25" s="55"/>
-      <c r="K25" s="54"/>
-      <c r="L25" s="55"/>
-      <c r="M25" s="49"/>
+    <row r="25" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B25" s="80"/>
+      <c r="C25" s="76"/>
+      <c r="D25" s="40"/>
+      <c r="E25" s="83"/>
+      <c r="F25" s="76"/>
+      <c r="G25" s="76"/>
+      <c r="H25" s="72"/>
+      <c r="I25" s="86"/>
+      <c r="J25" s="73"/>
+      <c r="K25" s="72"/>
+      <c r="L25" s="73"/>
+      <c r="M25" s="76"/>
       <c r="N25" s="10"/>
       <c r="O25" s="10"/>
       <c r="P25" s="10"/>
       <c r="Q25" s="10"/>
     </row>
-    <row r="26" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B26" s="22">
+    <row r="26" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B26" s="21">
         <v>1</v>
       </c>
-      <c r="C26" s="22"/>
-      <c r="D26" s="22"/>
-      <c r="E26" s="22"/>
-      <c r="F26" s="22"/>
-      <c r="G26" s="22"/>
-      <c r="H26" s="81"/>
-      <c r="I26" s="81"/>
-      <c r="J26" s="81"/>
-      <c r="K26" s="82"/>
-      <c r="L26" s="82"/>
-      <c r="M26" s="22"/>
+      <c r="C26" s="21"/>
+      <c r="D26" s="21"/>
+      <c r="E26" s="21"/>
+      <c r="F26" s="21"/>
+      <c r="G26" s="21"/>
+      <c r="H26" s="77"/>
+      <c r="I26" s="77"/>
+      <c r="J26" s="77"/>
+      <c r="K26" s="59"/>
+      <c r="L26" s="59"/>
+      <c r="M26" s="21"/>
       <c r="N26" s="10"/>
       <c r="O26" s="10"/>
       <c r="P26" s="10"/>
       <c r="Q26" s="10"/>
     </row>
-    <row r="27" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B27" s="22">
+    <row r="27" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B27" s="21">
         <v>2</v>
       </c>
-      <c r="C27" s="22"/>
-      <c r="D27" s="22"/>
-      <c r="E27" s="22"/>
-      <c r="F27" s="22"/>
-      <c r="G27" s="22"/>
-      <c r="H27" s="89"/>
-      <c r="I27" s="89"/>
-      <c r="J27" s="89"/>
-      <c r="K27" s="82"/>
-      <c r="L27" s="82"/>
-      <c r="M27" s="22"/>
+      <c r="C27" s="21"/>
+      <c r="D27" s="21"/>
+      <c r="E27" s="21"/>
+      <c r="F27" s="21"/>
+      <c r="G27" s="21"/>
+      <c r="H27" s="66"/>
+      <c r="I27" s="66"/>
+      <c r="J27" s="66"/>
+      <c r="K27" s="59"/>
+      <c r="L27" s="59"/>
+      <c r="M27" s="21"/>
       <c r="N27" s="10"/>
       <c r="O27" s="10"/>
       <c r="P27" s="10"/>
       <c r="Q27" s="10"/>
     </row>
-    <row r="28" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B28" s="22">
+    <row r="28" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B28" s="21">
         <v>3</v>
       </c>
-      <c r="C28" s="22"/>
-      <c r="D28" s="22"/>
-      <c r="E28" s="22"/>
-      <c r="F28" s="22"/>
-      <c r="G28" s="22"/>
-      <c r="H28" s="89"/>
-      <c r="I28" s="89"/>
-      <c r="J28" s="89"/>
-      <c r="K28" s="82"/>
-      <c r="L28" s="82"/>
-      <c r="M28" s="22"/>
+      <c r="C28" s="21"/>
+      <c r="D28" s="21"/>
+      <c r="E28" s="21"/>
+      <c r="F28" s="21"/>
+      <c r="G28" s="21"/>
+      <c r="H28" s="66"/>
+      <c r="I28" s="66"/>
+      <c r="J28" s="66"/>
+      <c r="K28" s="59"/>
+      <c r="L28" s="59"/>
+      <c r="M28" s="21"/>
       <c r="N28" s="10"/>
       <c r="O28" s="10"/>
       <c r="P28" s="10"/>
       <c r="Q28" s="10"/>
     </row>
-    <row r="29" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B29" s="10"/>
       <c r="C29" s="10"/>
       <c r="D29" s="10"/>
-      <c r="E29" s="23"/>
+      <c r="E29" s="22"/>
       <c r="F29" s="10"/>
       <c r="G29" s="10"/>
       <c r="H29" s="10"/>
-      <c r="J29" s="23"/>
+      <c r="J29" s="22"/>
       <c r="K29" s="10"/>
       <c r="L29" s="10"/>
       <c r="M29" s="10"/>
@@ -2185,130 +2254,130 @@
       <c r="P29" s="10"/>
       <c r="Q29" s="10"/>
     </row>
-    <row r="30" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B30" s="93" t="s">
+    <row r="30" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B30" s="56" t="s">
+        <v>92</v>
+      </c>
+      <c r="C30" s="56"/>
+      <c r="D30" s="56"/>
+      <c r="E30" s="56"/>
+      <c r="F30" s="56"/>
+      <c r="G30" s="23"/>
+      <c r="H30" s="36" t="s">
+        <v>93</v>
+      </c>
+      <c r="I30" s="37"/>
+      <c r="J30" s="57" t="s">
         <v>94</v>
       </c>
-      <c r="C30" s="93"/>
-      <c r="D30" s="93"/>
-      <c r="E30" s="93"/>
-      <c r="F30" s="93"/>
-      <c r="G30" s="24"/>
-      <c r="H30" s="37" t="s">
-        <v>95</v>
-      </c>
-      <c r="I30" s="38"/>
-      <c r="J30" s="94" t="s">
-        <v>96</v>
-      </c>
-      <c r="K30" s="94"/>
-      <c r="L30" s="94"/>
-      <c r="M30" s="94"/>
-      <c r="N30" s="94"/>
-      <c r="O30" s="94"/>
+      <c r="K30" s="57"/>
+      <c r="L30" s="57"/>
+      <c r="M30" s="57"/>
+      <c r="N30" s="57"/>
+      <c r="O30" s="57"/>
       <c r="P30" s="10"/>
       <c r="Q30" s="10"/>
     </row>
-    <row r="31" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B31" s="25" t="s">
-        <v>97</v>
-      </c>
-      <c r="C31" s="26"/>
-      <c r="D31" s="26"/>
-      <c r="E31" s="95"/>
-      <c r="F31" s="95"/>
+    <row r="31" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B31" s="24" t="s">
+        <v>95</v>
+      </c>
+      <c r="C31" s="25"/>
+      <c r="D31" s="25"/>
+      <c r="E31" s="58"/>
+      <c r="F31" s="58"/>
       <c r="G31" s="10"/>
-      <c r="H31" s="96" t="s">
-        <v>98</v>
-      </c>
-      <c r="I31" s="97"/>
-      <c r="J31" s="82"/>
-      <c r="K31" s="82"/>
-      <c r="L31" s="82"/>
-      <c r="M31" s="82"/>
-      <c r="N31" s="82"/>
-      <c r="O31" s="82"/>
+      <c r="H31" s="60" t="s">
+        <v>96</v>
+      </c>
+      <c r="I31" s="61"/>
+      <c r="J31" s="59"/>
+      <c r="K31" s="59"/>
+      <c r="L31" s="59"/>
+      <c r="M31" s="59"/>
+      <c r="N31" s="59"/>
+      <c r="O31" s="59"/>
       <c r="P31" s="10"/>
       <c r="Q31" s="10"/>
     </row>
-    <row r="32" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B32" s="25" t="s">
-        <v>99</v>
-      </c>
-      <c r="C32" s="26"/>
-      <c r="D32" s="26"/>
-      <c r="E32" s="82"/>
-      <c r="F32" s="82"/>
+    <row r="32" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B32" s="24" t="s">
+        <v>97</v>
+      </c>
+      <c r="C32" s="25"/>
+      <c r="D32" s="25"/>
+      <c r="E32" s="59"/>
+      <c r="F32" s="59"/>
       <c r="G32" s="10"/>
-      <c r="H32" s="98" t="s">
-        <v>100</v>
-      </c>
-      <c r="I32" s="99"/>
-      <c r="J32" s="82"/>
-      <c r="K32" s="82"/>
-      <c r="L32" s="82"/>
-      <c r="M32" s="82"/>
-      <c r="N32" s="82"/>
-      <c r="O32" s="82"/>
+      <c r="H32" s="62" t="s">
+        <v>98</v>
+      </c>
+      <c r="I32" s="63"/>
+      <c r="J32" s="59"/>
+      <c r="K32" s="59"/>
+      <c r="L32" s="59"/>
+      <c r="M32" s="59"/>
+      <c r="N32" s="59"/>
+      <c r="O32" s="59"/>
       <c r="P32" s="10"/>
       <c r="Q32" s="10"/>
     </row>
     <row r="33" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B33" s="25" t="s">
+      <c r="B33" s="24" t="s">
+        <v>99</v>
+      </c>
+      <c r="C33" s="25"/>
+      <c r="D33" s="25"/>
+      <c r="E33" s="21"/>
+      <c r="F33" s="26" t="s">
+        <v>100</v>
+      </c>
+      <c r="G33" s="10"/>
+      <c r="H33" s="62" t="s">
         <v>101</v>
       </c>
-      <c r="C33" s="26"/>
-      <c r="D33" s="26"/>
-      <c r="E33" s="22"/>
-      <c r="F33" s="27" t="s">
-        <v>102</v>
-      </c>
-      <c r="G33" s="10"/>
-      <c r="H33" s="98" t="s">
-        <v>103</v>
-      </c>
-      <c r="I33" s="99"/>
-      <c r="J33" s="82"/>
-      <c r="K33" s="82"/>
-      <c r="L33" s="82"/>
-      <c r="M33" s="82"/>
-      <c r="N33" s="82"/>
-      <c r="O33" s="82"/>
+      <c r="I33" s="63"/>
+      <c r="J33" s="59"/>
+      <c r="K33" s="59"/>
+      <c r="L33" s="59"/>
+      <c r="M33" s="59"/>
+      <c r="N33" s="59"/>
+      <c r="O33" s="59"/>
       <c r="P33" s="10"/>
       <c r="Q33" s="10"/>
     </row>
     <row r="34" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B34" s="28" t="s">
-        <v>104</v>
-      </c>
-      <c r="C34" s="29"/>
-      <c r="D34" s="29"/>
-      <c r="E34" s="22"/>
-      <c r="F34" s="27" t="s">
+      <c r="B34" s="27" t="s">
         <v>102</v>
       </c>
+      <c r="C34" s="28"/>
+      <c r="D34" s="28"/>
+      <c r="E34" s="21"/>
+      <c r="F34" s="26" t="s">
+        <v>100</v>
+      </c>
       <c r="G34" s="10"/>
-      <c r="H34" s="100" t="s">
-        <v>105</v>
-      </c>
-      <c r="I34" s="101"/>
-      <c r="J34" s="90"/>
-      <c r="K34" s="90"/>
-      <c r="L34" s="90"/>
-      <c r="M34" s="90"/>
-      <c r="N34" s="90"/>
-      <c r="O34" s="90"/>
+      <c r="H34" s="64" t="s">
+        <v>103</v>
+      </c>
+      <c r="I34" s="65"/>
+      <c r="J34" s="53"/>
+      <c r="K34" s="53"/>
+      <c r="L34" s="53"/>
+      <c r="M34" s="53"/>
+      <c r="N34" s="53"/>
+      <c r="O34" s="53"/>
       <c r="P34" s="10"/>
       <c r="Q34" s="10"/>
     </row>
     <row r="35" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B35" s="30"/>
-      <c r="C35" s="30"/>
-      <c r="D35" s="30"/>
-      <c r="E35" s="30"/>
-      <c r="F35" s="23"/>
+      <c r="B35" s="29"/>
+      <c r="C35" s="29"/>
+      <c r="D35" s="29"/>
+      <c r="E35" s="29"/>
+      <c r="F35" s="22"/>
       <c r="G35" s="10"/>
-      <c r="H35" s="31"/>
+      <c r="H35" s="30"/>
       <c r="I35" s="11"/>
       <c r="J35" s="11"/>
       <c r="K35" s="11"/>
@@ -2338,14 +2407,14 @@
       <c r="Q36" s="10"/>
     </row>
     <row r="37" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B37" s="91" t="s">
-        <v>106</v>
-      </c>
-      <c r="C37" s="91"/>
-      <c r="D37" s="91"/>
-      <c r="E37" s="91"/>
-      <c r="F37" s="91"/>
-      <c r="G37" s="91"/>
+      <c r="B37" s="54" t="s">
+        <v>104</v>
+      </c>
+      <c r="C37" s="54"/>
+      <c r="D37" s="54"/>
+      <c r="E37" s="54"/>
+      <c r="F37" s="54"/>
+      <c r="G37" s="54"/>
       <c r="H37" s="10"/>
       <c r="I37" s="10"/>
       <c r="J37" s="10"/>
@@ -2358,14 +2427,14 @@
       <c r="Q37" s="10"/>
     </row>
     <row r="38" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B38" s="92" t="s">
-        <v>107</v>
-      </c>
-      <c r="C38" s="92"/>
-      <c r="D38" s="92"/>
-      <c r="E38" s="92"/>
-      <c r="F38" s="92"/>
-      <c r="G38" s="92"/>
+      <c r="B38" s="55" t="s">
+        <v>105</v>
+      </c>
+      <c r="C38" s="55"/>
+      <c r="D38" s="55"/>
+      <c r="E38" s="55"/>
+      <c r="F38" s="55"/>
+      <c r="G38" s="55"/>
       <c r="H38" s="10"/>
       <c r="I38" s="10"/>
       <c r="J38" s="10"/>
@@ -2378,12 +2447,12 @@
       <c r="Q38" s="10"/>
     </row>
     <row r="39" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B39" s="92"/>
-      <c r="C39" s="92"/>
-      <c r="D39" s="92"/>
-      <c r="E39" s="92"/>
-      <c r="F39" s="92"/>
-      <c r="G39" s="92"/>
+      <c r="B39" s="55"/>
+      <c r="C39" s="55"/>
+      <c r="D39" s="55"/>
+      <c r="E39" s="55"/>
+      <c r="F39" s="55"/>
+      <c r="G39" s="55"/>
       <c r="H39" s="10"/>
       <c r="I39" s="10"/>
       <c r="J39" s="10"/>
@@ -2396,12 +2465,12 @@
       <c r="Q39" s="10"/>
     </row>
     <row r="40" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B40" s="92"/>
-      <c r="C40" s="92"/>
-      <c r="D40" s="92"/>
-      <c r="E40" s="92"/>
-      <c r="F40" s="92"/>
-      <c r="G40" s="92"/>
+      <c r="B40" s="55"/>
+      <c r="C40" s="55"/>
+      <c r="D40" s="55"/>
+      <c r="E40" s="55"/>
+      <c r="F40" s="55"/>
+      <c r="G40" s="55"/>
       <c r="H40" s="10"/>
       <c r="I40" s="10"/>
       <c r="J40" s="10"/>
@@ -2414,13 +2483,13 @@
       <c r="Q40" s="10"/>
     </row>
     <row r="41" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B41" s="92"/>
-      <c r="C41" s="92"/>
-      <c r="D41" s="92"/>
-      <c r="E41" s="92"/>
-      <c r="F41" s="92"/>
-      <c r="G41" s="92"/>
-      <c r="H41" s="32"/>
+      <c r="B41" s="55"/>
+      <c r="C41" s="55"/>
+      <c r="D41" s="55"/>
+      <c r="E41" s="55"/>
+      <c r="F41" s="55"/>
+      <c r="G41" s="55"/>
+      <c r="H41" s="31"/>
       <c r="I41" s="10"/>
       <c r="J41" s="10"/>
       <c r="K41" s="10"/>
@@ -2432,21 +2501,21 @@
       <c r="Q41" s="10"/>
     </row>
     <row r="42" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B42" s="92"/>
-      <c r="C42" s="92"/>
-      <c r="D42" s="92"/>
-      <c r="E42" s="92"/>
-      <c r="F42" s="92"/>
-      <c r="G42" s="92"/>
+      <c r="B42" s="55"/>
+      <c r="C42" s="55"/>
+      <c r="D42" s="55"/>
+      <c r="E42" s="55"/>
+      <c r="F42" s="55"/>
+      <c r="G42" s="55"/>
       <c r="H42" s="10"/>
-      <c r="I42" s="33" t="s">
-        <v>108</v>
+      <c r="I42" s="32" t="s">
+        <v>106</v>
       </c>
       <c r="J42" s="10"/>
       <c r="K42" s="10" t="s">
-        <v>109</v>
-      </c>
-      <c r="L42" s="23"/>
+        <v>107</v>
+      </c>
+      <c r="L42" s="22"/>
       <c r="M42" s="10"/>
       <c r="N42" s="10"/>
       <c r="O42" s="10"/>
@@ -2455,8 +2524,8 @@
     </row>
     <row r="43" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B43" s="10"/>
-      <c r="C43" s="23"/>
-      <c r="D43" s="23"/>
+      <c r="C43" s="22"/>
+      <c r="D43" s="22"/>
       <c r="E43" s="10"/>
       <c r="F43" s="10"/>
       <c r="G43" s="10"/>
@@ -2464,9 +2533,9 @@
       <c r="I43" s="10"/>
       <c r="J43" s="10"/>
       <c r="K43" s="10" t="s">
-        <v>110</v>
-      </c>
-      <c r="L43" s="23"/>
+        <v>108</v>
+      </c>
+      <c r="L43" s="22"/>
       <c r="M43" s="10"/>
       <c r="N43" s="10"/>
       <c r="O43" s="10"/>
@@ -2481,7 +2550,7 @@
       <c r="F44" s="10"/>
       <c r="G44" s="10"/>
       <c r="H44" s="10"/>
-      <c r="I44" s="23"/>
+      <c r="I44" s="22"/>
       <c r="J44" s="10"/>
       <c r="K44" s="10"/>
       <c r="L44" s="10"/>
@@ -2492,15 +2561,61 @@
       <c r="Q44" s="10"/>
     </row>
   </sheetData>
-  <mergeCells count="74">
-    <mergeCell ref="K11:N11"/>
-    <mergeCell ref="Q8:S8"/>
-    <mergeCell ref="Q9:S9"/>
-    <mergeCell ref="Q10:S10"/>
-    <mergeCell ref="Q11:S11"/>
-    <mergeCell ref="K8:N8"/>
-    <mergeCell ref="K9:N9"/>
-    <mergeCell ref="K10:N10"/>
+  <mergeCells count="75">
+    <mergeCell ref="D19:F19"/>
+    <mergeCell ref="D20:F20"/>
+    <mergeCell ref="G15:I17"/>
+    <mergeCell ref="G18:I18"/>
+    <mergeCell ref="G19:I19"/>
+    <mergeCell ref="G20:I20"/>
+    <mergeCell ref="C3:G3"/>
+    <mergeCell ref="K3:N3"/>
+    <mergeCell ref="C4:G4"/>
+    <mergeCell ref="K4:N4"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B7:S7"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="I8:J8"/>
+    <mergeCell ref="I9:J9"/>
+    <mergeCell ref="I11:J11"/>
+    <mergeCell ref="I10:J10"/>
+    <mergeCell ref="D8:H8"/>
+    <mergeCell ref="D9:H9"/>
+    <mergeCell ref="D10:H10"/>
+    <mergeCell ref="D11:H11"/>
+    <mergeCell ref="D12:H12"/>
+    <mergeCell ref="R15:R17"/>
+    <mergeCell ref="S15:T16"/>
+    <mergeCell ref="B15:B17"/>
+    <mergeCell ref="C15:C17"/>
+    <mergeCell ref="D15:F17"/>
+    <mergeCell ref="D18:F18"/>
+    <mergeCell ref="B14:R14"/>
+    <mergeCell ref="O15:O17"/>
+    <mergeCell ref="J15:L17"/>
+    <mergeCell ref="J18:L18"/>
+    <mergeCell ref="J19:L19"/>
+    <mergeCell ref="J20:L20"/>
+    <mergeCell ref="M15:N17"/>
+    <mergeCell ref="B22:M22"/>
+    <mergeCell ref="K23:L25"/>
+    <mergeCell ref="M23:M25"/>
+    <mergeCell ref="H26:J26"/>
+    <mergeCell ref="K26:L26"/>
+    <mergeCell ref="B23:B25"/>
+    <mergeCell ref="C23:C25"/>
+    <mergeCell ref="E23:E25"/>
+    <mergeCell ref="F23:F25"/>
+    <mergeCell ref="G23:G25"/>
+    <mergeCell ref="H23:J25"/>
+    <mergeCell ref="H27:J27"/>
+    <mergeCell ref="K27:L27"/>
+    <mergeCell ref="H28:J28"/>
+    <mergeCell ref="K28:L28"/>
+    <mergeCell ref="J33:O33"/>
     <mergeCell ref="J34:O34"/>
     <mergeCell ref="B37:G37"/>
     <mergeCell ref="B38:G42"/>
@@ -2514,59 +2629,14 @@
     <mergeCell ref="H32:I32"/>
     <mergeCell ref="H33:I33"/>
     <mergeCell ref="H34:I34"/>
-    <mergeCell ref="H27:J27"/>
-    <mergeCell ref="K27:L27"/>
-    <mergeCell ref="H28:J28"/>
-    <mergeCell ref="K28:L28"/>
-    <mergeCell ref="J33:O33"/>
-    <mergeCell ref="B22:M22"/>
-    <mergeCell ref="K23:L25"/>
-    <mergeCell ref="M23:M25"/>
-    <mergeCell ref="H26:J26"/>
-    <mergeCell ref="K26:L26"/>
-    <mergeCell ref="B23:B25"/>
-    <mergeCell ref="C23:C25"/>
-    <mergeCell ref="E23:E25"/>
-    <mergeCell ref="F23:F25"/>
-    <mergeCell ref="G23:G25"/>
-    <mergeCell ref="H23:J25"/>
-    <mergeCell ref="F20:G20"/>
-    <mergeCell ref="F15:G17"/>
-    <mergeCell ref="H15:H17"/>
-    <mergeCell ref="I15:I17"/>
-    <mergeCell ref="J15:J17"/>
-    <mergeCell ref="D12:H12"/>
-    <mergeCell ref="M15:M17"/>
-    <mergeCell ref="N15:O16"/>
-    <mergeCell ref="P15:Q16"/>
-    <mergeCell ref="F18:G18"/>
-    <mergeCell ref="K15:L16"/>
-    <mergeCell ref="I10:J10"/>
-    <mergeCell ref="D8:H8"/>
-    <mergeCell ref="D9:H9"/>
-    <mergeCell ref="D10:H10"/>
-    <mergeCell ref="D11:H11"/>
-    <mergeCell ref="D19:E19"/>
-    <mergeCell ref="D20:E20"/>
-    <mergeCell ref="F19:G19"/>
-    <mergeCell ref="C3:G3"/>
-    <mergeCell ref="K3:N3"/>
-    <mergeCell ref="C4:G4"/>
-    <mergeCell ref="K4:N4"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B7:S7"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="I8:J8"/>
-    <mergeCell ref="I9:J9"/>
-    <mergeCell ref="I11:J11"/>
-    <mergeCell ref="B14:Q14"/>
-    <mergeCell ref="B15:B17"/>
-    <mergeCell ref="C15:C17"/>
-    <mergeCell ref="D15:E17"/>
-    <mergeCell ref="D18:E18"/>
+    <mergeCell ref="K11:N11"/>
+    <mergeCell ref="Q8:S8"/>
+    <mergeCell ref="Q9:S9"/>
+    <mergeCell ref="Q10:S10"/>
+    <mergeCell ref="Q11:S11"/>
+    <mergeCell ref="K8:N8"/>
+    <mergeCell ref="K9:N9"/>
+    <mergeCell ref="K10:N10"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E26:E28" xr:uid="{B316A799-CF60-4C99-A88E-2204076E38E6}">
@@ -2612,15 +2682,15 @@
     <col min="21" max="21" width="43.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -2628,7 +2698,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -2636,7 +2706,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>17</v>
       </c>
@@ -2644,7 +2714,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>18</v>
       </c>
@@ -2652,7 +2722,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -2660,7 +2730,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>20</v>
       </c>
@@ -2668,7 +2738,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -2676,7 +2746,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>0</v>
       </c>
@@ -2684,52 +2754,85 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>59</v>
+      </c>
+      <c r="B10" t="s">
         <v>60</v>
       </c>
-      <c r="B10" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>109</v>
+      </c>
+      <c r="B11" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>110</v>
+      </c>
+      <c r="B12" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>111</v>
+      </c>
+      <c r="B13" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>114</v>
+      </c>
+      <c r="B14" t="s">
+        <v>70</v>
+      </c>
+      <c r="C14" s="46"/>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="B17" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="B17" s="8" t="s">
-        <v>50</v>
-      </c>
       <c r="C17" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D17" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="D17" s="2" t="s">
-        <v>31</v>
-      </c>
       <c r="E17" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F17" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G17" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="G17" s="2" t="s">
-        <v>36</v>
-      </c>
       <c r="H17" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="L17" s="2" t="s">
         <v>9</v>
@@ -2744,88 +2847,88 @@
         <v>13</v>
       </c>
       <c r="P17" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="Q17" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="Q17" s="2" t="s">
+      <c r="R17" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="R17" s="2" t="s">
-        <v>53</v>
-      </c>
       <c r="S17" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="T17" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="U17" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="C18" t="s">
+        <v>27</v>
+      </c>
+      <c r="D18" t="s">
+        <v>28</v>
+      </c>
+      <c r="E18" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="F18" t="s">
+        <v>33</v>
+      </c>
+      <c r="G18" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="H18" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="I18" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="J18" t="s">
+        <v>41</v>
+      </c>
+      <c r="K18" t="s">
+        <v>43</v>
+      </c>
+      <c r="L18" t="s">
         <v>23</v>
       </c>
-      <c r="B18" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="C18" t="s">
-        <v>28</v>
-      </c>
-      <c r="D18" t="s">
-        <v>29</v>
-      </c>
-      <c r="E18" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="F18" t="s">
-        <v>34</v>
-      </c>
-      <c r="G18" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="H18" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="I18" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="J18" t="s">
-        <v>42</v>
-      </c>
-      <c r="K18" t="s">
-        <v>44</v>
-      </c>
-      <c r="L18" t="s">
+      <c r="M18" t="s">
         <v>24</v>
       </c>
-      <c r="M18" t="s">
+      <c r="N18" t="s">
         <v>25</v>
       </c>
-      <c r="N18" t="s">
+      <c r="O18" t="s">
         <v>26</v>
       </c>
-      <c r="O18" t="s">
-        <v>27</v>
-      </c>
       <c r="P18" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="Q18" t="e">
         <f>IF(D18&gt;0,IF(D18="Unit",CONCATENATE(Settings!P18," ",Settings!D18,"s"),CONCATENATE((Settings!P18/Settings!L18)," ",Settings!D18,"s")),"")</f>
         <v>#VALUE!</v>
       </c>
       <c r="R18" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="S18" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="T18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="U18" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.25">
@@ -3250,29 +3353,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <SharedWithUsers xmlns="1444eecc-14bb-4066-abe6-ce6de21d9439">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010075F372E8CCA016418A193AD921508903" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="f5e922417d740f1a527805650dc2dfa9">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="399317f3-0083-4d0b-9572-12af99626311" xmlns:ns3="1444eecc-14bb-4066-abe6-ce6de21d9439" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="078d79524add6eac9b94134ca637184e" ns2:_="" ns3:_="">
     <xsd:import namespace="399317f3-0083-4d0b-9572-12af99626311"/>
@@ -3469,25 +3549,30 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7EBE950A-5812-419E-B174-6A5D9B8E0414}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="1444eecc-14bb-4066-abe6-ce6de21d9439"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A00E6A9-20DD-4842-9306-307EB080AF2E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <SharedWithUsers xmlns="1444eecc-14bb-4066-abe6-ce6de21d9439">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8CF88A1C-AA0D-4F8F-A0FD-6F3FAFCA9DC0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3504,4 +3589,22 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A00E6A9-20DD-4842-9306-307EB080AF2E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7EBE950A-5812-419E-B174-6A5D9B8E0414}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="1444eecc-14bb-4066-abe6-ce6de21d9439"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Payment Terms on revised Offers
</commit_message>
<xml_diff>
--- a/srv/xlsx-templates/TH - Quotation Template.xlsx
+++ b/srv/xlsx-templates/TH - Quotation Template.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26626"/>
-  <workbookPr/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EHQUT\Desktop\Thailand Template\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bayergroup-my.sharepoint.com/personal/kosal_kirthiga_ext_bayer_com/Documents/Desktop/ThailandLates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25A4229B-28F4-4104-978F-EF4BEE8B5F36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="263" documentId="8_{DE39F225-2AE1-4446-AB5F-E204FEABCD0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{36469226-B408-44E2-8967-0597E3B00D5F}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{F5CC2154-27BB-4652-B61E-D913F0CC6809}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="126">
   <si>
     <t>${offerValidation.INSTITUTENAME}</t>
   </si>
@@ -101,6 +101,9 @@
   </si>
   <si>
     <t>${offerValidation.SHIPMENTTERMS}</t>
+  </si>
+  <si>
+    <t>${table:offerProductValidation.PRODUCT_UNIT_NAME}</t>
   </si>
   <si>
     <t>${table:offerProductValidation.SKU}</t>
@@ -284,6 +287,9 @@
 Discount</t>
   </si>
   <si>
+    <t>Total Offer Value</t>
+  </si>
+  <si>
     <t>excl. vat.</t>
   </si>
   <si>
@@ -351,9 +357,6 @@
     <t>Remarks</t>
   </si>
   <si>
-    <t>With reference to the above tender, you must not on-sell the above mentioned products at a price higher than those listed above. However, you are always free to sell at a price lower, at your discretion.</t>
-  </si>
-  <si>
     <t>Approved by</t>
   </si>
   <si>
@@ -363,33 +366,56 @@
     <t>Position</t>
   </si>
   <si>
+    <t>${offerValidation.DISTRIBUTORNAME}</t>
+  </si>
+  <si>
     <t>${offerValidation.SELLINGCOMPANY}</t>
   </si>
   <si>
-    <t>${offerValidation.DISTRIBUTORNAME}</t>
-  </si>
-  <si>
     <t>${offerValidation.DISTRIBUTORADDRESS}</t>
   </si>
   <si>
+    <t>${offerValidation.CUSTOMER_CODE}</t>
+  </si>
+  <si>
     <t>${table:offerProductValidation.PRODUCTNAME}</t>
   </si>
   <si>
-    <t>${offerValidation.CUSTOMER_CODE}</t>
+    <t>UOM</t>
   </si>
   <si>
     <t xml:space="preserve">Offer QTY 
 </t>
   </si>
   <si>
-    <t xml:space="preserve">
-UoM</t>
-  </si>
-  <si>
     <t>${table:offerProductValidation.DOSAGE}</t>
   </si>
   <si>
     <t>${table:offerProductValidation.MANUFACTURER}</t>
+  </si>
+  <si>
+    <t>${offerProductValidation.NET_PRICE_UNIT_OFFER_CURRENCY_VAT}</t>
+  </si>
+  <si>
+    <t>${table:offerProductValidation.NET_PRICE_PACK_OFFER_CURRENCY_VAT}</t>
+  </si>
+  <si>
+    <t>${table:offerProductValidation.NET_PRICE_UNIT_OFFER_CURRENCY_VAT}</t>
+  </si>
+  <si>
+    <t>Net Price Pack Vat</t>
+  </si>
+  <si>
+    <t>Net Price Unit Vat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">With reference to the above tender, you must not on-sell the above mentioned products at a price higher than those listed above. However, you are always free to sell at a price lower, at your discretion. </t>
+  </si>
+  <si>
+    <t>incl. vat.(Pack)</t>
+  </si>
+  <si>
+    <t>incl. vat.(Unit)</t>
   </si>
 </sst>
 </file>
@@ -501,7 +527,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -512,12 +538,6 @@
       <patternFill patternType="solid">
         <fgColor theme="4"/>
         <bgColor theme="4"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
@@ -533,7 +553,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="18">
     <border>
       <left/>
       <right/>
@@ -641,6 +661,19 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
       <right/>
       <top style="thin">
         <color indexed="64"/>
@@ -660,11 +693,66 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left/>
       <right/>
       <top style="thin">
         <color indexed="64"/>
       </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
       <bottom/>
       <diagonal/>
     </border>
@@ -674,7 +762,7 @@
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="88">
+  <cellXfs count="126">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -689,142 +777,304 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="5" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="5" fillId="0" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="5" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="6" fillId="0" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="5" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="5" fillId="0" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="5" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="43" fontId="5" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="5" fillId="0" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -834,73 +1084,13 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -910,6 +1100,24 @@
     <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
   <dxfs count="7">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -943,24 +1151,6 @@
         <scheme val="minor"/>
       </font>
     </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -978,14 +1168,14 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>15</xdr:col>
+      <xdr:col>14</xdr:col>
       <xdr:colOff>482600</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>101600</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>458097</xdr:colOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>309931</xdr:colOff>
       <xdr:row>4</xdr:row>
       <xdr:rowOff>100462</xdr:rowOff>
     </xdr:to>
@@ -1026,75 +1216,20 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>603251</xdr:colOff>
-      <xdr:row>38</xdr:row>
-      <xdr:rowOff>74083</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>582217</xdr:colOff>
-      <xdr:row>42</xdr:row>
-      <xdr:rowOff>86342</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Picture 3">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DCAB78DC-B8BD-201A-CBFF-1F60D61D4715}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="6402918" y="7313083"/>
-          <a:ext cx="1524132" cy="774259"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5B6DC07E-0020-4B51-98A2-ADA62A91E75D}" name="Tabel1" displayName="Tabel1" ref="A1:B14" totalsRowShown="0" headerRowDxfId="6">
-  <autoFilter ref="A1:B14" xr:uid="{5B6DC07E-0020-4B51-98A2-ADA62A91E75D}"/>
-  <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{22EAB7A2-53F9-497F-A4B5-CA34E48AC441}" name="Header fields"/>
-    <tableColumn id="2" xr3:uid="{331DD14B-B263-41D9-B2C5-D198B6F2436E}" name="Description"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2EFFBCB4-83C9-46C5-9D10-EDD296E322D9}" name="Tabel2" displayName="Tabel2" ref="C17:U52" totalsRowShown="0" headerRowDxfId="5">
-  <autoFilter ref="C17:U52" xr:uid="{2EFFBCB4-83C9-46C5-9D10-EDD296E322D9}"/>
-  <tableColumns count="19">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2EFFBCB4-83C9-46C5-9D10-EDD296E322D9}" name="Tabel2" displayName="Tabel2" ref="C17:W52" totalsRowShown="0" headerRowDxfId="6">
+  <autoFilter ref="C17:W52" xr:uid="{2EFFBCB4-83C9-46C5-9D10-EDD296E322D9}"/>
+  <tableColumns count="21">
     <tableColumn id="1" xr3:uid="{6E1F8ECB-E862-46B4-998C-BE8E89C238BA}" name="PAID VOLUME"/>
     <tableColumn id="2" xr3:uid="{6497AF92-63C8-4790-818D-6E5BE819E8D6}" name="UNIT"/>
-    <tableColumn id="3" xr3:uid="{A1E59B72-B459-4BFA-9B37-9736C0F03B7E}" name="OFFER PRICE" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{A1E59B72-B459-4BFA-9B37-9736C0F03B7E}" name="OFFER PRICE" dataDxfId="5"/>
     <tableColumn id="4" xr3:uid="{1CB5E955-18ED-4738-ACA1-E270D15916F8}" name="CURRENCY"/>
-    <tableColumn id="5" xr3:uid="{77EEA9FC-8FC3-433A-9592-47B0D8B4C67B}" name="OFFER_PRICE_VAT" dataDxfId="3"/>
-    <tableColumn id="6" xr3:uid="{38030720-EDB2-473C-9CF5-2E9C926DF088}" name="GROSS SALES OFFER CURRENCY" dataDxfId="2"/>
-    <tableColumn id="7" xr3:uid="{A1EAF0A4-B4D5-428E-9D86-C12164DF9888}" name="GROSS_SALES_OFFER_CURRENCY_VAT" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{77EEA9FC-8FC3-433A-9592-47B0D8B4C67B}" name="OFFER_PRICE_VAT" dataDxfId="4"/>
+    <tableColumn id="6" xr3:uid="{38030720-EDB2-473C-9CF5-2E9C926DF088}" name="GROSS SALES OFFER CURRENCY" dataDxfId="3"/>
+    <tableColumn id="7" xr3:uid="{A1EAF0A4-B4D5-428E-9D86-C12164DF9888}" name="GROSS_SALES_OFFER_CURRENCY_VAT" dataDxfId="2"/>
     <tableColumn id="8" xr3:uid="{06958303-4A18-40AA-8AD0-9A7EEFDCAF3E}" name="OFFER_ID"/>
     <tableColumn id="9" xr3:uid="{A1218AAF-0481-41A2-9C10-3038D1BF8C7D}" name="SORTER"/>
     <tableColumn id="10" xr3:uid="{5A7FFAC3-1C22-44BF-8C52-F3578967B0F3}" name="Pack Factor"/>
@@ -1102,15 +1237,28 @@
     <tableColumn id="12" xr3:uid="{4A42B0A1-255A-4E7E-955E-674BA8AAA444}" name="Origin"/>
     <tableColumn id="13" xr3:uid="{7D1379AA-4B8F-4BC6-9726-365EBAE15341}" name="FOC"/>
     <tableColumn id="14" xr3:uid="{DF88A36E-0423-48FC-A1FC-B18BF3BA8D1A}" name="Total Quantity Units"/>
-    <tableColumn id="15" xr3:uid="{6B128E87-63EB-483B-88D7-EA33600F43AB}" name="Total QTY" dataDxfId="0">
+    <tableColumn id="15" xr3:uid="{6B128E87-63EB-483B-88D7-EA33600F43AB}" name="Total QTY" dataDxfId="1">
       <calculatedColumnFormula>IF(D18&gt;0,IF(D18="Unit",CONCATENATE(Settings!P18," ",Settings!D18,"s"),CONCATENATE((Settings!P18/Settings!L18)," ",Settings!D18,"s")),"")</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="16" xr3:uid="{E4D044B6-D053-487A-AA8C-F40FE34F30A7}" name="Net Price"/>
-    <tableColumn id="17" xr3:uid="{F95E93A8-C80D-4AC7-9526-72374F546CE7}" name="Amount in numbers"/>
-    <tableColumn id="18" xr3:uid="{2DDE85E8-6C8E-4D93-A4E8-1F80D965246B}" name="VAT total"/>
-    <tableColumn id="19" xr3:uid="{F55B5874-4E65-4E44-AEFE-7CFF114E939A}" name="Amount in numbers vat"/>
+    <tableColumn id="17" xr3:uid="{F95E93A8-C80D-4AC7-9526-72374F546CE7}" name="Net Price Pack Vat"/>
+    <tableColumn id="18" xr3:uid="{2DDE85E8-6C8E-4D93-A4E8-1F80D965246B}" name="Net Price Unit Vat"/>
+    <tableColumn id="20" xr3:uid="{CB417A4B-91CA-49CD-9B3D-699005D44488}" name="Amount in numbers"/>
+    <tableColumn id="21" xr3:uid="{07B28F29-5FC9-406A-96FC-77FFBFB88A05}" name="VAT total"/>
+    <tableColumn id="22" xr3:uid="{275B8D63-D363-4D68-BC9C-CB91FD9D0201}" name="Amount in numbers vat"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{13195211-A053-4079-8580-181B8695617E}" name="Tabel14" displayName="Tabel14" ref="A1:B15" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:B15" xr:uid="{13195211-A053-4079-8580-181B8695617E}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{04053350-A8BA-4F7A-9272-32CAE894E561}" name="Header fields"/>
+    <tableColumn id="2" xr3:uid="{91B26FA0-9378-480D-8354-6037F7FF582C}" name="Description"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -1411,16 +1559,30 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFBA1999-1CF9-4903-BA7D-DD523B82D6C3}">
-  <dimension ref="B2:Y44"/>
+  <sheetPr codeName="Sheet1"/>
+  <dimension ref="B2:Q55"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="11.140625" customWidth="1"/>
-    <col min="9" max="9" width="11.42578125" customWidth="1"/>
-    <col min="10" max="10" width="14" customWidth="1"/>
-    <col min="13" max="13" width="34.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="15.7109375" customWidth="1"/>
+    <col min="4" max="4" width="27.5703125" customWidth="1"/>
+    <col min="5" max="5" width="16.5703125" customWidth="1"/>
+    <col min="6" max="6" width="11.85546875" customWidth="1"/>
+    <col min="7" max="7" width="10.42578125" customWidth="1"/>
+    <col min="8" max="8" width="13.28515625" customWidth="1"/>
+    <col min="9" max="9" width="14.7109375" customWidth="1"/>
+    <col min="10" max="10" width="17.5703125" customWidth="1"/>
+    <col min="11" max="11" width="13.5703125" customWidth="1"/>
+    <col min="12" max="12" width="12.5703125" customWidth="1"/>
+    <col min="13" max="13" width="17.5703125" customWidth="1"/>
+    <col min="14" max="14" width="18.140625" customWidth="1"/>
+    <col min="15" max="15" width="11.42578125" customWidth="1"/>
+    <col min="16" max="16" width="15.28515625" customWidth="1"/>
+    <col min="17" max="17" width="17.85546875" customWidth="1"/>
+    <col min="18" max="18" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B2" s="10"/>
       <c r="C2" s="10"/>
       <c r="D2" s="10"/>
@@ -1436,79 +1598,73 @@
       <c r="N2" s="10"/>
       <c r="O2" s="10"/>
       <c r="P2" s="10"/>
-      <c r="Q2" s="10"/>
-    </row>
-    <row r="3" spans="2:25" x14ac:dyDescent="0.25">
-      <c r="B3" s="30" t="s">
-        <v>63</v>
-      </c>
-      <c r="C3" s="77" t="s">
+    </row>
+    <row r="3" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="B3" s="39" t="s">
+        <v>64</v>
+      </c>
+      <c r="C3" s="53" t="s">
         <v>109</v>
       </c>
-      <c r="D3" s="77"/>
-      <c r="E3" s="77"/>
-      <c r="F3" s="77"/>
-      <c r="G3" s="77"/>
-      <c r="H3" s="11"/>
-      <c r="I3" s="10"/>
-      <c r="J3" s="30" t="s">
-        <v>64</v>
-      </c>
-      <c r="K3" s="77" t="str">
-        <f>Settings!A11</f>
-        <v>${offerValidation.SELLINGCOMPANY}</v>
-      </c>
-      <c r="L3" s="77"/>
-      <c r="M3" s="77"/>
-      <c r="N3" s="77"/>
+      <c r="D3" s="54"/>
+      <c r="E3" s="54"/>
+      <c r="F3" s="54"/>
+      <c r="G3" s="55"/>
+      <c r="H3" s="10"/>
+      <c r="I3" s="39" t="s">
+        <v>65</v>
+      </c>
+      <c r="J3" s="53" t="s">
+        <v>110</v>
+      </c>
+      <c r="K3" s="54"/>
+      <c r="L3" s="54"/>
+      <c r="M3" s="55"/>
+      <c r="N3" s="10"/>
       <c r="O3" s="10"/>
       <c r="P3" s="10"/>
-      <c r="Q3" s="10"/>
-    </row>
-    <row r="4" spans="2:25" x14ac:dyDescent="0.25">
-      <c r="B4" s="30" t="s">
-        <v>65</v>
-      </c>
-      <c r="C4" s="62" t="str">
-        <f>Settings!A13</f>
-        <v>${offerValidation.DISTRIBUTORADDRESS}</v>
-      </c>
-      <c r="D4" s="63"/>
-      <c r="E4" s="63"/>
-      <c r="F4" s="63"/>
-      <c r="G4" s="64"/>
-      <c r="H4" s="12"/>
-      <c r="I4" s="10"/>
-      <c r="J4" s="30" t="s">
-        <v>65</v>
-      </c>
-      <c r="K4" s="78"/>
-      <c r="L4" s="79"/>
-      <c r="M4" s="79"/>
-      <c r="N4" s="80"/>
+    </row>
+    <row r="4" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="62" t="s">
+        <v>66</v>
+      </c>
+      <c r="C4" s="60" t="s">
+        <v>111</v>
+      </c>
+      <c r="D4" s="60"/>
+      <c r="E4" s="60"/>
+      <c r="F4" s="60"/>
+      <c r="G4" s="60"/>
+      <c r="H4" s="10"/>
+      <c r="I4" s="39" t="s">
+        <v>66</v>
+      </c>
+      <c r="J4" s="56"/>
+      <c r="K4" s="57"/>
+      <c r="L4" s="57"/>
+      <c r="M4" s="58"/>
+      <c r="N4" s="10"/>
       <c r="O4" s="10"/>
       <c r="P4" s="10"/>
-      <c r="Q4" s="10"/>
-    </row>
-    <row r="5" spans="2:25" x14ac:dyDescent="0.25">
-      <c r="B5" s="13"/>
-      <c r="C5" s="12"/>
-      <c r="D5" s="12"/>
-      <c r="E5" s="12"/>
-      <c r="F5" s="12"/>
-      <c r="G5" s="12"/>
-      <c r="H5" s="12"/>
-      <c r="I5" s="10"/>
+    </row>
+    <row r="5" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="B5" s="63"/>
+      <c r="C5" s="61"/>
+      <c r="D5" s="61"/>
+      <c r="E5" s="61"/>
+      <c r="F5" s="61"/>
+      <c r="G5" s="61"/>
+      <c r="H5" s="10"/>
+      <c r="I5" s="12"/>
       <c r="J5" s="13"/>
-      <c r="K5" s="14"/>
-      <c r="L5" s="14"/>
-      <c r="M5" s="14"/>
-      <c r="N5" s="14"/>
+      <c r="K5" s="13"/>
+      <c r="L5" s="13"/>
+      <c r="M5" s="13"/>
+      <c r="N5" s="10"/>
       <c r="O5" s="10"/>
       <c r="P5" s="10"/>
-      <c r="Q5" s="10"/>
-    </row>
-    <row r="6" spans="2:25" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B6" s="10"/>
       <c r="C6" s="10"/>
       <c r="D6" s="10"/>
@@ -1524,163 +1680,143 @@
       <c r="N6" s="10"/>
       <c r="O6" s="10"/>
       <c r="P6" s="10"/>
-      <c r="Q6" s="10"/>
-    </row>
-    <row r="7" spans="2:25" x14ac:dyDescent="0.25">
-      <c r="B7" s="81" t="s">
-        <v>66</v>
-      </c>
-      <c r="C7" s="82"/>
-      <c r="D7" s="82"/>
-      <c r="E7" s="82"/>
-      <c r="F7" s="82"/>
-      <c r="G7" s="82"/>
-      <c r="H7" s="82"/>
-      <c r="I7" s="82"/>
-      <c r="J7" s="82"/>
-      <c r="K7" s="82"/>
-      <c r="L7" s="82"/>
-      <c r="M7" s="82"/>
-      <c r="N7" s="82"/>
-      <c r="O7" s="82"/>
-      <c r="P7" s="82"/>
-      <c r="Q7" s="82"/>
-      <c r="R7" s="82"/>
-      <c r="S7" s="83"/>
-    </row>
-    <row r="8" spans="2:25" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="B7" s="123" t="s">
+        <v>67</v>
+      </c>
+      <c r="C7" s="124"/>
+      <c r="D7" s="124"/>
+      <c r="E7" s="124"/>
+      <c r="F7" s="124"/>
+      <c r="G7" s="124"/>
+      <c r="H7" s="124"/>
+      <c r="I7" s="124"/>
+      <c r="J7" s="124"/>
+      <c r="K7" s="124"/>
+      <c r="L7" s="124"/>
+      <c r="M7" s="124"/>
+      <c r="N7" s="124"/>
+      <c r="O7" s="125"/>
+    </row>
+    <row r="8" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="51" t="s">
-        <v>67</v>
-      </c>
-      <c r="C8" s="51"/>
-      <c r="D8" s="62"/>
-      <c r="E8" s="63"/>
-      <c r="F8" s="63"/>
-      <c r="G8" s="63"/>
-      <c r="H8" s="64"/>
-      <c r="I8" s="38" t="s">
         <v>68</v>
       </c>
-      <c r="J8" s="39"/>
-      <c r="K8" s="54"/>
-      <c r="L8" s="55"/>
-      <c r="M8" s="55"/>
-      <c r="N8" s="56"/>
-      <c r="O8" s="28" t="s">
+      <c r="C8" s="52"/>
+      <c r="D8" s="120"/>
+      <c r="E8" s="121"/>
+      <c r="F8" s="122"/>
+      <c r="G8" s="51" t="s">
         <v>69</v>
       </c>
-      <c r="P8" s="29"/>
-      <c r="Q8" s="46"/>
-      <c r="R8" s="46"/>
-      <c r="S8" s="46"/>
-    </row>
-    <row r="9" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="H8" s="68"/>
+      <c r="I8" s="107"/>
+      <c r="J8" s="108"/>
+      <c r="K8" s="109"/>
+      <c r="L8" s="113" t="s">
+        <v>70</v>
+      </c>
+      <c r="M8" s="114"/>
+      <c r="N8" s="105"/>
+      <c r="O8" s="106"/>
+      <c r="P8" s="32"/>
+    </row>
+    <row r="9" spans="2:17" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="51" t="s">
-        <v>70</v>
-      </c>
-      <c r="C9" s="51"/>
-      <c r="D9" s="62" t="str">
+        <v>71</v>
+      </c>
+      <c r="C9" s="52"/>
+      <c r="D9" s="120" t="str">
         <f>Settings!A14</f>
         <v>${offerValidation.CUSTOMER_CODE}</v>
       </c>
-      <c r="E9" s="63"/>
-      <c r="F9" s="63"/>
-      <c r="G9" s="63"/>
-      <c r="H9" s="64"/>
-      <c r="I9" s="40" t="s">
-        <v>71</v>
-      </c>
-      <c r="J9" s="41"/>
-      <c r="K9" s="57" t="s">
+      <c r="E9" s="121"/>
+      <c r="F9" s="122"/>
+      <c r="G9" s="69" t="s">
+        <v>72</v>
+      </c>
+      <c r="H9" s="70"/>
+      <c r="I9" s="110" t="s">
         <v>17</v>
       </c>
-      <c r="L9" s="57"/>
-      <c r="M9" s="57"/>
-      <c r="N9" s="57"/>
-      <c r="O9" s="28" t="s">
-        <v>72</v>
-      </c>
-      <c r="P9" s="29"/>
-      <c r="Q9" s="46"/>
-      <c r="R9" s="46"/>
-      <c r="S9" s="46"/>
-    </row>
-    <row r="10" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="J9" s="111"/>
+      <c r="K9" s="112"/>
+      <c r="L9" s="113" t="s">
+        <v>73</v>
+      </c>
+      <c r="M9" s="114"/>
+      <c r="N9" s="105"/>
+      <c r="O9" s="106"/>
+      <c r="P9" s="32"/>
+    </row>
+    <row r="10" spans="2:17" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="51" t="s">
-        <v>73</v>
-      </c>
-      <c r="C10" s="51"/>
-      <c r="D10" s="62" t="str">
+        <v>74</v>
+      </c>
+      <c r="C10" s="52"/>
+      <c r="D10" s="120" t="str">
         <f>Settings!A9</f>
         <v>${offerValidation.INSTITUTENAME}</v>
       </c>
-      <c r="E10" s="63"/>
-      <c r="F10" s="63"/>
-      <c r="G10" s="63"/>
-      <c r="H10" s="64"/>
-      <c r="I10" s="60" t="s">
+      <c r="E10" s="121"/>
+      <c r="F10" s="122"/>
+      <c r="G10" s="71" t="s">
         <v>5</v>
       </c>
-      <c r="J10" s="61"/>
-      <c r="K10" s="57" t="s">
+      <c r="H10" s="72"/>
+      <c r="I10" s="110" t="s">
         <v>18</v>
       </c>
-      <c r="L10" s="57"/>
-      <c r="M10" s="57"/>
-      <c r="N10" s="57"/>
-      <c r="O10" s="28" t="s">
-        <v>74</v>
-      </c>
-      <c r="P10" s="29"/>
-      <c r="Q10" s="46"/>
-      <c r="R10" s="46"/>
-      <c r="S10" s="46"/>
-    </row>
-    <row r="11" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J10" s="111"/>
+      <c r="K10" s="112"/>
+      <c r="L10" s="113" t="s">
+        <v>75</v>
+      </c>
+      <c r="M10" s="114"/>
+      <c r="N10" s="105"/>
+      <c r="O10" s="106"/>
+      <c r="P10" s="32"/>
+    </row>
+    <row r="11" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B11" s="51" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="51"/>
-      <c r="D11" s="65" t="str">
-        <f>Settings!A12</f>
-        <v>${offerValidation.DISTRIBUTORNAME}</v>
-      </c>
-      <c r="E11" s="66"/>
-      <c r="F11" s="66"/>
-      <c r="G11" s="66"/>
-      <c r="H11" s="67"/>
-      <c r="I11" s="38" t="s">
+      <c r="C11" s="52"/>
+      <c r="D11" s="97" t="s">
+        <v>21</v>
+      </c>
+      <c r="E11" s="98"/>
+      <c r="F11" s="99"/>
+      <c r="G11" s="51" t="s">
         <v>7</v>
       </c>
-      <c r="J11" s="39"/>
-      <c r="K11" s="52" t="str">
-        <f>Settings!A7</f>
-        <v>${offerValidation.PAYMENTTERMS}</v>
-      </c>
-      <c r="L11" s="52"/>
-      <c r="M11" s="52"/>
-      <c r="N11" s="52"/>
-      <c r="O11" s="28" t="s">
-        <v>72</v>
-      </c>
-      <c r="P11" s="29"/>
-      <c r="Q11" s="46"/>
-      <c r="R11" s="46"/>
-      <c r="S11" s="46"/>
-    </row>
-    <row r="12" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="H11" s="68"/>
+      <c r="I11" s="64" t="s">
+        <v>20</v>
+      </c>
+      <c r="J11" s="65"/>
+      <c r="K11" s="66"/>
+      <c r="L11" s="113" t="s">
+        <v>73</v>
+      </c>
+      <c r="M11" s="114"/>
+      <c r="N11" s="105"/>
+      <c r="O11" s="106"/>
+      <c r="P11" s="32"/>
+    </row>
+    <row r="12" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B12" s="51" t="s">
         <v>8</v>
       </c>
-      <c r="C12" s="51"/>
-      <c r="D12" s="65" t="str">
-        <f>Settings!A8</f>
-        <v>${offerValidation.DELIVERYTERMS}</v>
-      </c>
-      <c r="E12" s="66"/>
-      <c r="F12" s="66"/>
-      <c r="G12" s="66"/>
-      <c r="H12" s="67"/>
+      <c r="C12" s="52"/>
+      <c r="D12" s="97" t="s">
+        <v>19</v>
+      </c>
+      <c r="E12" s="98"/>
+      <c r="F12" s="99"/>
+      <c r="G12" s="10"/>
+      <c r="H12" s="10"/>
       <c r="I12" s="10"/>
       <c r="J12" s="10"/>
       <c r="K12" s="10"/>
@@ -1688,10 +1824,8 @@
       <c r="M12" s="10"/>
       <c r="N12" s="10"/>
       <c r="O12" s="10"/>
-      <c r="P12" s="10"/>
-      <c r="Q12" s="10"/>
-    </row>
-    <row r="13" spans="2:25" x14ac:dyDescent="0.25">
+    </row>
+    <row r="13" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B13" s="10"/>
       <c r="C13" s="10"/>
       <c r="D13" s="10"/>
@@ -1707,245 +1841,204 @@
       <c r="N13" s="10"/>
       <c r="O13" s="10"/>
       <c r="P13" s="10"/>
-      <c r="Q13" s="10"/>
-    </row>
-    <row r="14" spans="2:25" x14ac:dyDescent="0.25">
-      <c r="B14" s="85" t="s">
-        <v>75</v>
-      </c>
-      <c r="C14" s="85"/>
-      <c r="D14" s="85"/>
-      <c r="E14" s="85"/>
-      <c r="F14" s="85"/>
-      <c r="G14" s="85"/>
-      <c r="H14" s="85"/>
-      <c r="I14" s="85"/>
-      <c r="J14" s="85"/>
-      <c r="K14" s="85"/>
-      <c r="L14" s="85"/>
-      <c r="M14" s="85"/>
-      <c r="N14" s="85"/>
-      <c r="O14" s="85"/>
-      <c r="P14" s="85"/>
-      <c r="Q14" s="85"/>
-      <c r="R14" s="85"/>
-      <c r="S14" s="85"/>
-      <c r="T14" s="85"/>
-      <c r="U14" s="85"/>
-      <c r="V14" s="85"/>
-      <c r="W14" s="85"/>
-      <c r="X14" s="85"/>
-      <c r="Y14" s="85"/>
-    </row>
-    <row r="15" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="50" t="s">
+    </row>
+    <row r="14" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="B14" s="59" t="s">
         <v>76</v>
       </c>
-      <c r="C15" s="84" t="s">
+      <c r="C14" s="59"/>
+      <c r="D14" s="59"/>
+      <c r="E14" s="59"/>
+      <c r="F14" s="59"/>
+      <c r="G14" s="59"/>
+      <c r="H14" s="59"/>
+      <c r="I14" s="59"/>
+      <c r="J14" s="59"/>
+      <c r="K14" s="59"/>
+      <c r="L14" s="59"/>
+      <c r="M14" s="59"/>
+      <c r="N14" s="59"/>
+      <c r="O14" s="59"/>
+      <c r="P14" s="59"/>
+      <c r="Q14" s="59"/>
+    </row>
+    <row r="15" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="84" t="s">
         <v>77</v>
       </c>
-      <c r="D15" s="84"/>
-      <c r="E15" s="43" t="s">
+      <c r="C15" s="73" t="s">
         <v>78</v>
       </c>
-      <c r="F15" s="43"/>
-      <c r="G15" s="43"/>
-      <c r="H15" s="43" t="s">
+      <c r="D15" s="73" t="s">
         <v>79</v>
       </c>
-      <c r="I15" s="43"/>
-      <c r="J15" s="43"/>
-      <c r="K15" s="69" t="s">
+      <c r="E15" s="73" t="s">
+        <v>80</v>
+      </c>
+      <c r="F15" s="73" t="s">
+        <v>115</v>
+      </c>
+      <c r="G15" s="73" t="s">
+        <v>114</v>
+      </c>
+      <c r="H15" s="33" t="s">
+        <v>9</v>
+      </c>
+      <c r="I15" s="73" t="s">
+        <v>81</v>
+      </c>
+      <c r="J15" s="76" t="s">
+        <v>10</v>
+      </c>
+      <c r="K15" s="77"/>
+      <c r="L15" s="73" t="s">
+        <v>82</v>
+      </c>
+      <c r="M15" s="76" t="s">
+        <v>14</v>
+      </c>
+      <c r="N15" s="80"/>
+      <c r="O15" s="80"/>
+      <c r="P15" s="47" t="s">
+        <v>83</v>
+      </c>
+      <c r="Q15" s="48"/>
+    </row>
+    <row r="16" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="B16" s="85"/>
+      <c r="C16" s="74"/>
+      <c r="D16" s="74"/>
+      <c r="E16" s="74"/>
+      <c r="F16" s="74"/>
+      <c r="G16" s="74"/>
+      <c r="H16" s="35"/>
+      <c r="I16" s="74"/>
+      <c r="J16" s="78"/>
+      <c r="K16" s="79"/>
+      <c r="L16" s="74"/>
+      <c r="M16" s="81"/>
+      <c r="N16" s="82"/>
+      <c r="O16" s="82"/>
+      <c r="P16" s="49"/>
+      <c r="Q16" s="50"/>
+    </row>
+    <row r="17" spans="2:17" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B17" s="86"/>
+      <c r="C17" s="75"/>
+      <c r="D17" s="75"/>
+      <c r="E17" s="75"/>
+      <c r="F17" s="75"/>
+      <c r="G17" s="75"/>
+      <c r="H17" s="34"/>
+      <c r="I17" s="75"/>
+      <c r="J17" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="K17" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="L17" s="75"/>
+      <c r="M17" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="N17" s="14" t="s">
+        <v>125</v>
+      </c>
+      <c r="O17" s="14" t="s">
+        <v>124</v>
+      </c>
+      <c r="P17" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="Q17" s="14" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="18" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="B18" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="C18" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="D18" s="15" t="s">
         <v>113</v>
       </c>
-      <c r="L15" s="69"/>
-      <c r="M15" s="43" t="s">
-        <v>114</v>
-      </c>
-      <c r="N15" s="43" t="s">
-        <v>9</v>
-      </c>
-      <c r="O15" s="43"/>
-      <c r="P15" s="43" t="s">
-        <v>80</v>
-      </c>
-      <c r="Q15" s="43" t="s">
-        <v>10</v>
-      </c>
-      <c r="R15" s="43"/>
-      <c r="S15" s="43"/>
-      <c r="T15" s="43"/>
-      <c r="U15" s="43" t="s">
-        <v>81</v>
-      </c>
-      <c r="V15" s="43" t="s">
-        <v>14</v>
-      </c>
-      <c r="W15" s="43"/>
-      <c r="X15" s="43"/>
-      <c r="Y15" s="43"/>
-    </row>
-    <row r="16" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="50"/>
-      <c r="C16" s="84"/>
-      <c r="D16" s="84"/>
-      <c r="E16" s="43"/>
-      <c r="F16" s="43"/>
-      <c r="G16" s="43"/>
-      <c r="H16" s="43"/>
-      <c r="I16" s="43"/>
-      <c r="J16" s="43"/>
-      <c r="K16" s="69"/>
-      <c r="L16" s="69"/>
-      <c r="M16" s="43"/>
-      <c r="N16" s="43"/>
-      <c r="O16" s="43"/>
-      <c r="P16" s="43"/>
-      <c r="Q16" s="43"/>
-      <c r="R16" s="43"/>
-      <c r="S16" s="43"/>
-      <c r="T16" s="43"/>
-      <c r="U16" s="43"/>
-      <c r="V16" s="43"/>
-      <c r="W16" s="43"/>
-      <c r="X16" s="43"/>
-      <c r="Y16" s="43"/>
-    </row>
-    <row r="17" spans="2:25" x14ac:dyDescent="0.25">
-      <c r="B17" s="50"/>
-      <c r="C17" s="84"/>
-      <c r="D17" s="84"/>
-      <c r="E17" s="43"/>
-      <c r="F17" s="43"/>
-      <c r="G17" s="43"/>
-      <c r="H17" s="43"/>
-      <c r="I17" s="43"/>
-      <c r="J17" s="43"/>
-      <c r="K17" s="69"/>
-      <c r="L17" s="69"/>
-      <c r="M17" s="43"/>
-      <c r="N17" s="43"/>
-      <c r="O17" s="43"/>
-      <c r="P17" s="43"/>
-      <c r="Q17" s="44" t="s">
-        <v>82</v>
-      </c>
-      <c r="R17" s="44"/>
-      <c r="S17" s="44" t="s">
-        <v>83</v>
-      </c>
-      <c r="T17" s="44"/>
-      <c r="U17" s="43"/>
-      <c r="V17" s="44" t="s">
-        <v>82</v>
-      </c>
-      <c r="W17" s="44"/>
-      <c r="X17" s="44" t="s">
-        <v>83</v>
-      </c>
-      <c r="Y17" s="44"/>
-    </row>
-    <row r="18" spans="2:25" x14ac:dyDescent="0.25">
-      <c r="B18" s="15" t="s">
-        <v>43</v>
-      </c>
-      <c r="C18" s="52" t="s">
-        <v>22</v>
-      </c>
-      <c r="D18" s="52"/>
-      <c r="E18" s="86" t="s">
-        <v>111</v>
-      </c>
-      <c r="F18" s="86"/>
-      <c r="G18" s="86"/>
-      <c r="H18" s="53"/>
-      <c r="I18" s="53"/>
-      <c r="J18" s="53"/>
-      <c r="K18" s="46" t="s">
+      <c r="E18" s="119"/>
+      <c r="F18" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="G18" s="40" t="s">
+        <v>29</v>
+      </c>
+      <c r="H18" s="41" t="s">
+        <v>24</v>
+      </c>
+      <c r="I18" s="16" t="s">
+        <v>116</v>
+      </c>
+      <c r="J18" s="42" t="s">
+        <v>32</v>
+      </c>
+      <c r="K18" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="L18" s="41" t="s">
         <v>27</v>
       </c>
-      <c r="L18" s="46"/>
-      <c r="M18" s="36" t="s">
-        <v>28</v>
-      </c>
-      <c r="N18" s="46" t="s">
-        <v>23</v>
-      </c>
-      <c r="O18" s="46"/>
-      <c r="P18" s="37" t="s">
-        <v>115</v>
-      </c>
-      <c r="Q18" s="53" t="s">
-        <v>31</v>
-      </c>
-      <c r="R18" s="53"/>
-      <c r="S18" s="47" t="s">
-        <v>36</v>
-      </c>
-      <c r="T18" s="47"/>
-      <c r="U18" s="36" t="s">
-        <v>26</v>
-      </c>
-      <c r="V18" s="45" t="s">
-        <v>53</v>
-      </c>
-      <c r="W18" s="45"/>
-      <c r="X18" s="46"/>
-      <c r="Y18" s="46"/>
-    </row>
-    <row r="19" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="M18" s="42" t="s">
+        <v>54</v>
+      </c>
+      <c r="N18" s="17" t="s">
+        <v>120</v>
+      </c>
+      <c r="O18" s="36" t="s">
+        <v>119</v>
+      </c>
+      <c r="P18" s="45" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q18" s="18" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="19" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B19" s="15"/>
-      <c r="C19" s="48"/>
-      <c r="D19" s="48"/>
-      <c r="E19" s="53"/>
-      <c r="F19" s="53"/>
-      <c r="G19" s="53"/>
-      <c r="H19" s="53"/>
-      <c r="I19" s="53"/>
-      <c r="J19" s="53"/>
-      <c r="K19" s="53"/>
-      <c r="L19" s="53"/>
-      <c r="M19" s="37"/>
-      <c r="N19" s="46"/>
-      <c r="O19" s="46"/>
-      <c r="P19" s="37"/>
-      <c r="Q19" s="53"/>
-      <c r="R19" s="53"/>
-      <c r="S19" s="47"/>
-      <c r="T19" s="47"/>
-      <c r="U19" s="16"/>
-      <c r="V19" s="45"/>
-      <c r="W19" s="45"/>
-      <c r="X19" s="46"/>
-      <c r="Y19" s="46"/>
-    </row>
-    <row r="20" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="C19" s="15"/>
+      <c r="D19" s="15"/>
+      <c r="E19" s="119"/>
+      <c r="F19" s="15"/>
+      <c r="G19" s="36"/>
+      <c r="H19" s="16"/>
+      <c r="I19" s="15"/>
+      <c r="J19" s="18"/>
+      <c r="K19" s="18"/>
+      <c r="L19" s="19"/>
+      <c r="M19" s="17"/>
+      <c r="N19" s="17"/>
+      <c r="O19" s="36"/>
+      <c r="P19" s="17"/>
+      <c r="Q19" s="20"/>
+    </row>
+    <row r="20" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B20" s="15"/>
-      <c r="C20" s="48"/>
-      <c r="D20" s="48"/>
-      <c r="E20" s="53"/>
-      <c r="F20" s="53"/>
-      <c r="G20" s="53"/>
-      <c r="H20" s="53"/>
-      <c r="I20" s="53"/>
-      <c r="J20" s="53"/>
-      <c r="K20" s="53"/>
-      <c r="L20" s="53"/>
-      <c r="M20" s="37"/>
-      <c r="N20" s="46"/>
-      <c r="O20" s="46"/>
-      <c r="P20" s="37"/>
-      <c r="Q20" s="53"/>
-      <c r="R20" s="53"/>
-      <c r="S20" s="47"/>
-      <c r="T20" s="47"/>
-      <c r="U20" s="16"/>
-      <c r="V20" s="45"/>
-      <c r="W20" s="45"/>
-      <c r="X20" s="46"/>
-      <c r="Y20" s="46"/>
-    </row>
-    <row r="21" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="C20" s="15"/>
+      <c r="D20" s="15"/>
+      <c r="E20" s="119"/>
+      <c r="F20" s="15"/>
+      <c r="G20" s="36"/>
+      <c r="H20" s="16"/>
+      <c r="I20" s="15"/>
+      <c r="J20" s="18"/>
+      <c r="K20" s="18"/>
+      <c r="L20" s="19"/>
+      <c r="M20" s="17"/>
+      <c r="N20" s="17"/>
+      <c r="O20" s="36"/>
+      <c r="P20" s="17"/>
+      <c r="Q20" s="20"/>
+    </row>
+    <row r="21" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B21" s="10"/>
       <c r="C21" s="10"/>
       <c r="D21" s="10"/>
@@ -1961,285 +2054,258 @@
       <c r="N21" s="10"/>
       <c r="O21" s="10"/>
       <c r="P21" s="10"/>
-      <c r="Q21" s="10"/>
-    </row>
-    <row r="22" spans="2:25" x14ac:dyDescent="0.25">
-      <c r="B22" s="68" t="s">
-        <v>84</v>
-      </c>
-      <c r="C22" s="68"/>
-      <c r="D22" s="68"/>
-      <c r="E22" s="68"/>
-      <c r="F22" s="68"/>
-      <c r="G22" s="68"/>
-      <c r="H22" s="68"/>
-      <c r="I22" s="68"/>
-      <c r="J22" s="68"/>
-      <c r="K22" s="68"/>
-      <c r="L22" s="68"/>
-      <c r="M22" s="68"/>
-      <c r="N22" s="68"/>
-      <c r="O22" s="68"/>
-      <c r="P22" s="68"/>
-    </row>
-    <row r="23" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="50" t="s">
-        <v>76</v>
-      </c>
-      <c r="C23" s="43" t="s">
+    </row>
+    <row r="22" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="B22" s="59" t="s">
+        <v>86</v>
+      </c>
+      <c r="C22" s="59"/>
+      <c r="D22" s="59"/>
+      <c r="E22" s="59"/>
+      <c r="F22" s="59"/>
+      <c r="G22" s="59"/>
+      <c r="H22" s="59"/>
+      <c r="I22" s="59"/>
+      <c r="J22" s="59"/>
+      <c r="K22" s="59"/>
+      <c r="L22" s="59"/>
+      <c r="M22" s="10"/>
+    </row>
+    <row r="23" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="B23" s="87" t="s">
         <v>77</v>
       </c>
-      <c r="D23" s="43"/>
-      <c r="E23" s="43" t="s">
-        <v>85</v>
-      </c>
-      <c r="F23" s="43" t="s">
-        <v>86</v>
-      </c>
-      <c r="G23" s="43" t="s">
+      <c r="C23" s="73" t="s">
+        <v>78</v>
+      </c>
+      <c r="D23" s="88" t="s">
         <v>87</v>
       </c>
-      <c r="H23" s="43" t="s">
+      <c r="E23" s="73" t="s">
         <v>88</v>
       </c>
-      <c r="I23" s="43"/>
-      <c r="J23" s="43"/>
-      <c r="K23" s="43" t="s">
+      <c r="F23" s="73" t="s">
         <v>89</v>
       </c>
-      <c r="L23" s="43"/>
-      <c r="M23" s="43"/>
-      <c r="N23" s="43"/>
-      <c r="O23" s="43" t="s">
+      <c r="G23" s="67" t="s">
         <v>90</v>
       </c>
-      <c r="P23" s="43"/>
-    </row>
-    <row r="24" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="50"/>
-      <c r="C24" s="43"/>
-      <c r="D24" s="43"/>
-      <c r="E24" s="43"/>
-      <c r="F24" s="43"/>
-      <c r="G24" s="43"/>
-      <c r="H24" s="43"/>
-      <c r="I24" s="43"/>
-      <c r="J24" s="43"/>
-      <c r="K24" s="43"/>
-      <c r="L24" s="43"/>
-      <c r="M24" s="43"/>
-      <c r="N24" s="43"/>
-      <c r="O24" s="43"/>
-      <c r="P24" s="43"/>
-    </row>
-    <row r="25" spans="2:25" x14ac:dyDescent="0.25">
-      <c r="B25" s="50"/>
-      <c r="C25" s="43"/>
-      <c r="D25" s="43"/>
-      <c r="E25" s="43"/>
-      <c r="F25" s="43"/>
-      <c r="G25" s="43"/>
-      <c r="H25" s="43"/>
-      <c r="I25" s="43"/>
-      <c r="J25" s="43"/>
-      <c r="K25" s="43"/>
-      <c r="L25" s="43"/>
-      <c r="M25" s="43"/>
-      <c r="N25" s="43"/>
-      <c r="O25" s="43"/>
-      <c r="P25" s="43"/>
-    </row>
-    <row r="26" spans="2:25" x14ac:dyDescent="0.25">
-      <c r="B26" s="15" t="s">
-        <v>43</v>
-      </c>
-      <c r="C26" s="46" t="s">
-        <v>22</v>
-      </c>
-      <c r="D26" s="46"/>
-      <c r="E26" s="17"/>
-      <c r="F26" s="17"/>
-      <c r="G26" s="17"/>
-      <c r="H26" s="49"/>
-      <c r="I26" s="49"/>
-      <c r="J26" s="49"/>
-      <c r="K26" s="42" t="s">
-        <v>116</v>
-      </c>
-      <c r="L26" s="42"/>
-      <c r="M26" s="42"/>
-      <c r="N26" s="42"/>
-      <c r="O26" s="42" t="s">
-        <v>25</v>
-      </c>
-      <c r="P26" s="42"/>
-    </row>
-    <row r="27" spans="2:25" x14ac:dyDescent="0.25">
-      <c r="B27" s="17"/>
-      <c r="C27" s="42"/>
-      <c r="D27" s="42"/>
-      <c r="E27" s="17"/>
-      <c r="F27" s="17"/>
-      <c r="G27" s="17"/>
-      <c r="H27" s="49"/>
-      <c r="I27" s="49"/>
-      <c r="J27" s="49"/>
-      <c r="K27" s="42"/>
-      <c r="L27" s="42"/>
-      <c r="M27" s="42"/>
-      <c r="N27" s="42"/>
-      <c r="O27" s="42"/>
-      <c r="P27" s="42"/>
-    </row>
-    <row r="28" spans="2:25" x14ac:dyDescent="0.25">
-      <c r="B28" s="17"/>
-      <c r="C28" s="42"/>
-      <c r="D28" s="42"/>
-      <c r="E28" s="17"/>
-      <c r="F28" s="17"/>
-      <c r="G28" s="17"/>
-      <c r="H28" s="49"/>
-      <c r="I28" s="49"/>
-      <c r="J28" s="49"/>
-      <c r="K28" s="42"/>
-      <c r="L28" s="42"/>
-      <c r="M28" s="42"/>
-      <c r="N28" s="42"/>
-      <c r="O28" s="42"/>
-      <c r="P28" s="42"/>
-      <c r="Q28" s="10"/>
-    </row>
-    <row r="29" spans="2:25" x14ac:dyDescent="0.25">
-      <c r="B29" s="10"/>
-      <c r="C29" s="10"/>
-      <c r="D29" s="10"/>
-      <c r="E29" s="18"/>
-      <c r="F29" s="10"/>
-      <c r="G29" s="10"/>
-      <c r="H29" s="10"/>
-      <c r="J29" s="18"/>
-      <c r="K29" s="10"/>
-      <c r="L29" s="10"/>
+      <c r="H23" s="67"/>
+      <c r="I23" s="67"/>
+      <c r="J23" s="67" t="s">
+        <v>91</v>
+      </c>
+      <c r="K23" s="67"/>
+      <c r="L23" s="67" t="s">
+        <v>92</v>
+      </c>
+      <c r="M23" s="10"/>
+    </row>
+    <row r="24" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="B24" s="87"/>
+      <c r="C24" s="75"/>
+      <c r="D24" s="89"/>
+      <c r="E24" s="75"/>
+      <c r="F24" s="75"/>
+      <c r="G24" s="67"/>
+      <c r="H24" s="67"/>
+      <c r="I24" s="67"/>
+      <c r="J24" s="67"/>
+      <c r="K24" s="67"/>
+      <c r="L24" s="67"/>
+      <c r="M24" s="10"/>
+    </row>
+    <row r="25" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="B25" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="C25" s="37" t="s">
+        <v>23</v>
+      </c>
+      <c r="D25" s="38"/>
+      <c r="E25" s="21"/>
+      <c r="F25" s="21"/>
+      <c r="G25" s="116"/>
+      <c r="H25" s="116"/>
+      <c r="I25" s="116"/>
+      <c r="J25" s="105" t="s">
+        <v>117</v>
+      </c>
+      <c r="K25" s="106"/>
+      <c r="L25" s="21" t="s">
+        <v>26</v>
+      </c>
+      <c r="M25" s="10"/>
+    </row>
+    <row r="26" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="B26" s="21"/>
+      <c r="C26" s="21"/>
+      <c r="D26" s="21"/>
+      <c r="E26" s="21"/>
+      <c r="F26" s="21"/>
+      <c r="G26" s="115"/>
+      <c r="H26" s="115"/>
+      <c r="I26" s="115"/>
+      <c r="J26" s="94"/>
+      <c r="K26" s="94"/>
+      <c r="L26" s="21"/>
+      <c r="M26" s="10"/>
+    </row>
+    <row r="27" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="B27" s="21"/>
+      <c r="C27" s="21"/>
+      <c r="D27" s="21"/>
+      <c r="E27" s="21"/>
+      <c r="F27" s="21"/>
+      <c r="G27" s="115"/>
+      <c r="H27" s="115"/>
+      <c r="I27" s="115"/>
+      <c r="J27" s="94"/>
+      <c r="K27" s="94"/>
+      <c r="L27" s="21"/>
+      <c r="M27" s="10"/>
+    </row>
+    <row r="28" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="B28" s="10"/>
+      <c r="C28" s="10"/>
+      <c r="D28" s="22"/>
+      <c r="E28" s="10"/>
+      <c r="F28" s="10"/>
+      <c r="G28" s="10"/>
+      <c r="H28" s="22"/>
+      <c r="I28" s="10"/>
+      <c r="J28" s="10"/>
+      <c r="K28" s="10"/>
+      <c r="L28" s="10"/>
+      <c r="M28" s="10"/>
+      <c r="N28" s="10"/>
+      <c r="O28" s="10"/>
+      <c r="P28" s="10"/>
+    </row>
+    <row r="29" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B29" s="90" t="s">
+        <v>93</v>
+      </c>
+      <c r="C29" s="90"/>
+      <c r="D29" s="90"/>
+      <c r="E29" s="90"/>
+      <c r="F29" s="23"/>
+      <c r="G29" s="91" t="s">
+        <v>94</v>
+      </c>
+      <c r="H29" s="92"/>
+      <c r="I29" s="44" t="s">
+        <v>95</v>
+      </c>
+      <c r="J29" s="44"/>
+      <c r="K29" s="44"/>
+      <c r="L29" s="44"/>
       <c r="M29" s="10"/>
       <c r="N29" s="10"/>
-      <c r="O29" s="10"/>
-      <c r="P29" s="10"/>
-      <c r="Q29" s="10"/>
-    </row>
-    <row r="30" spans="2:25" x14ac:dyDescent="0.25">
-      <c r="B30" s="71" t="s">
-        <v>91</v>
-      </c>
-      <c r="C30" s="71"/>
-      <c r="D30" s="71"/>
-      <c r="E30" s="71"/>
-      <c r="F30" s="71"/>
-      <c r="G30" s="19"/>
-      <c r="I30" s="31" t="s">
-        <v>92</v>
-      </c>
-      <c r="J30" s="32"/>
-      <c r="K30" s="72" t="s">
-        <v>93</v>
-      </c>
-      <c r="L30" s="72"/>
-      <c r="M30" s="72"/>
-      <c r="N30" s="72"/>
-      <c r="O30" s="72"/>
-      <c r="P30" s="72"/>
-    </row>
-    <row r="31" spans="2:25" x14ac:dyDescent="0.25">
-      <c r="B31" s="20" t="s">
-        <v>94</v>
-      </c>
-      <c r="C31" s="21"/>
-      <c r="D31" s="21"/>
-      <c r="E31" s="73"/>
-      <c r="F31" s="73"/>
-      <c r="G31" s="10"/>
-      <c r="I31" s="74" t="s">
-        <v>95</v>
-      </c>
-      <c r="J31" s="75"/>
-      <c r="K31" s="42"/>
-      <c r="L31" s="42"/>
-      <c r="M31" s="42"/>
-      <c r="N31" s="42"/>
-      <c r="O31" s="42"/>
-      <c r="P31" s="42"/>
-    </row>
-    <row r="32" spans="2:25" x14ac:dyDescent="0.25">
-      <c r="B32" s="20" t="s">
+    </row>
+    <row r="30" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="B30" s="24" t="s">
         <v>96</v>
       </c>
-      <c r="C32" s="21"/>
+      <c r="C30" s="25"/>
+      <c r="D30" s="93"/>
+      <c r="E30" s="93"/>
+      <c r="F30" s="10"/>
+      <c r="G30" s="95" t="s">
+        <v>97</v>
+      </c>
+      <c r="H30" s="96"/>
+      <c r="I30" s="97"/>
+      <c r="J30" s="98"/>
+      <c r="K30" s="98"/>
+      <c r="L30" s="99"/>
+      <c r="M30" s="10"/>
+      <c r="N30" s="10"/>
+    </row>
+    <row r="31" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="B31" s="24" t="s">
+        <v>98</v>
+      </c>
+      <c r="C31" s="25"/>
+      <c r="D31" s="94"/>
+      <c r="E31" s="94"/>
+      <c r="F31" s="10"/>
+      <c r="G31" s="95" t="s">
+        <v>99</v>
+      </c>
+      <c r="H31" s="96"/>
+      <c r="I31" s="97"/>
+      <c r="J31" s="98"/>
+      <c r="K31" s="98"/>
+      <c r="L31" s="99"/>
+      <c r="M31" s="10"/>
+      <c r="N31" s="10"/>
+    </row>
+    <row r="32" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="B32" s="24" t="s">
+        <v>100</v>
+      </c>
+      <c r="C32" s="25"/>
       <c r="D32" s="21"/>
-      <c r="E32" s="42"/>
-      <c r="F32" s="42"/>
-      <c r="G32" s="10"/>
-      <c r="I32" s="74" t="s">
-        <v>97</v>
-      </c>
-      <c r="J32" s="75"/>
-      <c r="K32" s="42"/>
-      <c r="L32" s="42"/>
-      <c r="M32" s="42"/>
-      <c r="N32" s="42"/>
-      <c r="O32" s="42"/>
-      <c r="P32" s="42"/>
-    </row>
-    <row r="33" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B33" s="20" t="s">
-        <v>98</v>
-      </c>
-      <c r="C33" s="21"/>
+      <c r="E32" s="26" t="s">
+        <v>101</v>
+      </c>
+      <c r="F32" s="10"/>
+      <c r="G32" s="95" t="s">
+        <v>102</v>
+      </c>
+      <c r="H32" s="96"/>
+      <c r="I32" s="97"/>
+      <c r="J32" s="98"/>
+      <c r="K32" s="98"/>
+      <c r="L32" s="99"/>
+      <c r="M32" s="10"/>
+      <c r="N32" s="10"/>
+    </row>
+    <row r="33" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B33" s="27" t="s">
+        <v>103</v>
+      </c>
+      <c r="C33" s="28"/>
       <c r="D33" s="21"/>
-      <c r="E33" s="17"/>
-      <c r="F33" s="22" t="s">
-        <v>99</v>
-      </c>
-      <c r="G33" s="10"/>
-      <c r="I33" s="74" t="s">
-        <v>100</v>
-      </c>
-      <c r="J33" s="75"/>
-      <c r="K33" s="42"/>
-      <c r="L33" s="42"/>
-      <c r="M33" s="42"/>
-      <c r="N33" s="42"/>
-      <c r="O33" s="42"/>
-      <c r="P33" s="42"/>
-    </row>
-    <row r="34" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B34" s="23" t="s">
+      <c r="E33" s="26" t="s">
         <v>101</v>
       </c>
-      <c r="C34" s="24"/>
-      <c r="D34" s="24"/>
-      <c r="E34" s="17"/>
-      <c r="F34" s="22" t="s">
-        <v>99</v>
-      </c>
-      <c r="G34" s="10"/>
-      <c r="I34" s="34" t="s">
-        <v>102</v>
-      </c>
-      <c r="J34" s="35"/>
-      <c r="K34" s="58"/>
-      <c r="L34" s="58"/>
-      <c r="M34" s="58"/>
-      <c r="N34" s="58"/>
-      <c r="O34" s="58"/>
-      <c r="P34" s="58"/>
-    </row>
-    <row r="35" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B35" s="25"/>
-      <c r="C35" s="25"/>
-      <c r="D35" s="25"/>
-      <c r="E35" s="25"/>
-      <c r="F35" s="18"/>
-      <c r="G35" s="10"/>
-      <c r="H35" s="26"/>
+      <c r="F33" s="10"/>
+      <c r="G33" s="103" t="s">
+        <v>104</v>
+      </c>
+      <c r="H33" s="104"/>
+      <c r="I33" s="53"/>
+      <c r="J33" s="54"/>
+      <c r="K33" s="54"/>
+      <c r="L33" s="55"/>
+    </row>
+    <row r="34" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B34" s="29"/>
+      <c r="C34" s="29"/>
+      <c r="D34" s="29"/>
+      <c r="E34" s="22"/>
+      <c r="F34" s="10"/>
+      <c r="G34" s="30"/>
+      <c r="H34" s="11"/>
+      <c r="I34" s="11"/>
+      <c r="J34" s="11"/>
+      <c r="K34" s="11"/>
+      <c r="L34" s="11"/>
+      <c r="M34" s="11"/>
+      <c r="N34" s="11"/>
+      <c r="O34" s="11"/>
+      <c r="P34" s="10"/>
+    </row>
+    <row r="35" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B35" s="29"/>
+      <c r="C35" s="29"/>
+      <c r="D35" s="29"/>
+      <c r="E35" s="22"/>
+      <c r="F35" s="10"/>
+      <c r="G35" s="30"/>
+      <c r="H35" s="11"/>
       <c r="I35" s="11"/>
       <c r="J35" s="11"/>
       <c r="K35" s="11"/>
@@ -2247,303 +2313,376 @@
       <c r="M35" s="11"/>
       <c r="N35" s="11"/>
       <c r="O35" s="11"/>
-      <c r="P35" s="11"/>
-      <c r="Q35" s="10"/>
-    </row>
-    <row r="36" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B36" s="10"/>
-      <c r="C36" s="10"/>
-      <c r="D36" s="10"/>
-      <c r="E36" s="10"/>
+      <c r="P35" s="10"/>
+    </row>
+    <row r="36" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B36" s="29"/>
+      <c r="C36" s="29"/>
+      <c r="D36" s="29"/>
+      <c r="E36" s="22"/>
       <c r="F36" s="10"/>
-      <c r="G36" s="10"/>
-      <c r="H36" s="10"/>
-      <c r="I36" s="10"/>
-      <c r="J36" s="10"/>
-      <c r="K36" s="10"/>
-      <c r="L36" s="10"/>
-      <c r="M36" s="10"/>
-      <c r="N36" s="10"/>
-      <c r="O36" s="10"/>
+      <c r="G36" s="30"/>
+      <c r="H36" s="11"/>
+      <c r="I36" s="11"/>
+      <c r="J36" s="11"/>
+      <c r="K36" s="11"/>
+      <c r="L36" s="11"/>
+      <c r="M36" s="11"/>
+      <c r="N36" s="11"/>
+      <c r="O36" s="11"/>
       <c r="P36" s="10"/>
-      <c r="Q36" s="10"/>
-    </row>
-    <row r="37" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B37" s="59" t="s">
-        <v>103</v>
-      </c>
-      <c r="C37" s="59"/>
-      <c r="D37" s="59"/>
-      <c r="E37" s="59"/>
-      <c r="F37" s="59"/>
-      <c r="G37" s="59"/>
-      <c r="H37" s="10"/>
-      <c r="I37" s="10"/>
-      <c r="J37" s="10"/>
-      <c r="K37" s="10"/>
-      <c r="L37" s="10"/>
-      <c r="M37" s="10"/>
-      <c r="N37" s="10"/>
-      <c r="O37" s="10"/>
+    </row>
+    <row r="37" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="C37" s="29"/>
+      <c r="D37" s="29"/>
+      <c r="E37" s="22"/>
+      <c r="F37" s="10"/>
+      <c r="G37" s="30"/>
+      <c r="H37" s="11"/>
+      <c r="I37" s="11"/>
+      <c r="J37" s="11"/>
+      <c r="K37" s="11"/>
+      <c r="L37" s="11"/>
+      <c r="M37" s="11"/>
+      <c r="N37" s="11"/>
+      <c r="O37" s="11"/>
       <c r="P37" s="10"/>
-      <c r="Q37" s="10"/>
-    </row>
-    <row r="38" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B38" s="70" t="s">
-        <v>104</v>
-      </c>
-      <c r="C38" s="70"/>
-      <c r="D38" s="70"/>
-      <c r="E38" s="70"/>
-      <c r="F38" s="70"/>
-      <c r="G38" s="70"/>
-      <c r="H38" s="10"/>
-      <c r="I38" s="10"/>
-      <c r="J38" s="76"/>
-      <c r="K38" s="76"/>
-      <c r="L38" s="10"/>
-      <c r="M38" s="10"/>
-      <c r="N38" s="10"/>
-      <c r="O38" s="10"/>
+    </row>
+    <row r="38" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B38" s="29"/>
+      <c r="C38" s="29"/>
+      <c r="D38" s="29"/>
+      <c r="E38" s="22"/>
+      <c r="F38" s="10"/>
+      <c r="G38" s="30"/>
+      <c r="H38" s="11"/>
+      <c r="I38" s="11"/>
+      <c r="J38" s="11"/>
+      <c r="K38" s="11"/>
+      <c r="L38" s="11"/>
+      <c r="M38" s="11"/>
+      <c r="N38" s="11"/>
+      <c r="O38" s="11"/>
       <c r="P38" s="10"/>
-      <c r="Q38" s="10"/>
-    </row>
-    <row r="39" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B39" s="70"/>
-      <c r="C39" s="70"/>
-      <c r="D39" s="70"/>
-      <c r="E39" s="70"/>
-      <c r="F39" s="70"/>
-      <c r="G39" s="70"/>
+    </row>
+    <row r="39" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B39" s="10"/>
+      <c r="C39" s="10"/>
+      <c r="D39" s="10"/>
+      <c r="E39" s="10"/>
+      <c r="F39" s="10"/>
+      <c r="G39" s="10"/>
       <c r="H39" s="10"/>
       <c r="I39" s="10"/>
-      <c r="J39" s="76"/>
-      <c r="K39" s="76"/>
+      <c r="J39" s="10"/>
+      <c r="K39" s="10"/>
       <c r="L39" s="10"/>
       <c r="M39" s="10"/>
       <c r="N39" s="10"/>
       <c r="O39" s="10"/>
       <c r="P39" s="10"/>
-      <c r="Q39" s="10"/>
-    </row>
-    <row r="40" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B40" s="70"/>
-      <c r="C40" s="70"/>
-      <c r="D40" s="70"/>
-      <c r="E40" s="70"/>
-      <c r="F40" s="70"/>
-      <c r="G40" s="70"/>
+    </row>
+    <row r="40" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B40" s="100" t="s">
+        <v>105</v>
+      </c>
+      <c r="C40" s="101"/>
+      <c r="D40" s="101"/>
+      <c r="E40" s="101"/>
+      <c r="F40" s="102"/>
+      <c r="G40" s="10"/>
       <c r="H40" s="10"/>
       <c r="I40" s="10"/>
-      <c r="J40" s="76"/>
-      <c r="K40" s="76"/>
+      <c r="J40" s="10"/>
+      <c r="K40" s="10"/>
       <c r="L40" s="10"/>
       <c r="M40" s="10"/>
       <c r="N40" s="10"/>
       <c r="O40" s="10"/>
       <c r="P40" s="10"/>
-      <c r="Q40" s="10"/>
-    </row>
-    <row r="41" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B41" s="70"/>
-      <c r="C41" s="70"/>
-      <c r="D41" s="70"/>
-      <c r="E41" s="70"/>
-      <c r="F41" s="70"/>
-      <c r="G41" s="70"/>
-      <c r="H41" s="27"/>
+    </row>
+    <row r="41" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B41" s="118" t="s">
+        <v>123</v>
+      </c>
+      <c r="C41" s="118"/>
+      <c r="D41" s="118"/>
+      <c r="E41" s="118"/>
+      <c r="F41" s="118"/>
+      <c r="G41" s="117"/>
+      <c r="H41" s="10"/>
       <c r="I41" s="10"/>
-      <c r="J41" s="76"/>
-      <c r="K41" s="76"/>
+      <c r="J41" s="10"/>
+      <c r="K41" s="10"/>
       <c r="L41" s="10"/>
       <c r="M41" s="10"/>
       <c r="N41" s="10"/>
       <c r="O41" s="10"/>
       <c r="P41" s="10"/>
-      <c r="Q41" s="10"/>
-    </row>
-    <row r="42" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B42" s="70"/>
-      <c r="C42" s="70"/>
-      <c r="D42" s="70"/>
-      <c r="E42" s="70"/>
-      <c r="F42" s="70"/>
-      <c r="G42" s="70"/>
+    </row>
+    <row r="42" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B42" s="83"/>
+      <c r="C42" s="83"/>
+      <c r="D42" s="83"/>
+      <c r="E42" s="83"/>
+      <c r="F42" s="83"/>
+      <c r="G42" s="117"/>
       <c r="H42" s="10"/>
-      <c r="L42" s="87" t="s">
-        <v>105</v>
-      </c>
-      <c r="M42" s="87"/>
-      <c r="N42" s="10" t="s">
-        <v>106</v>
-      </c>
+      <c r="I42" s="10"/>
+      <c r="J42" s="10"/>
+      <c r="K42" s="10"/>
+      <c r="L42" s="10"/>
+      <c r="M42" s="10"/>
+      <c r="N42" s="10"/>
       <c r="O42" s="10"/>
       <c r="P42" s="10"/>
-      <c r="Q42" s="10"/>
-    </row>
-    <row r="43" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B43" s="10"/>
-      <c r="C43" s="18"/>
-      <c r="D43" s="18"/>
-      <c r="E43" s="10"/>
-      <c r="F43" s="10"/>
-      <c r="G43" s="10"/>
-      <c r="H43" s="10"/>
+    </row>
+    <row r="43" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B43" s="83"/>
+      <c r="C43" s="83"/>
+      <c r="D43" s="83"/>
+      <c r="E43" s="83"/>
+      <c r="F43" s="83"/>
+      <c r="G43" s="117"/>
+      <c r="H43" s="31" t="s">
+        <v>106</v>
+      </c>
+      <c r="I43" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="K43" s="10"/>
       <c r="L43" s="10"/>
       <c r="M43" s="10"/>
-      <c r="N43" s="10" t="s">
-        <v>107</v>
-      </c>
+      <c r="N43" s="10"/>
       <c r="O43" s="10"/>
       <c r="P43" s="10"/>
-      <c r="Q43" s="10"/>
-    </row>
-    <row r="44" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B44" s="10"/>
-      <c r="C44" s="10"/>
-      <c r="D44" s="10"/>
-      <c r="E44" s="10"/>
-      <c r="F44" s="10"/>
-      <c r="G44" s="10"/>
+    </row>
+    <row r="44" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B44" s="83"/>
+      <c r="C44" s="83"/>
+      <c r="D44" s="83"/>
+      <c r="E44" s="83"/>
+      <c r="F44" s="83"/>
+      <c r="G44" s="117"/>
       <c r="H44" s="10"/>
-      <c r="I44" s="18"/>
-      <c r="J44" s="10"/>
+      <c r="I44" s="10" t="s">
+        <v>108</v>
+      </c>
       <c r="K44" s="10"/>
       <c r="L44" s="10"/>
       <c r="M44" s="10"/>
       <c r="N44" s="10"/>
       <c r="O44" s="10"/>
       <c r="P44" s="10"/>
-      <c r="Q44" s="10"/>
+    </row>
+    <row r="45" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B45" s="83"/>
+      <c r="C45" s="83"/>
+      <c r="D45" s="83"/>
+      <c r="E45" s="83"/>
+      <c r="F45" s="83"/>
+      <c r="G45" s="117"/>
+      <c r="H45" s="10"/>
+      <c r="I45" s="10"/>
+      <c r="K45" s="10"/>
+      <c r="L45" s="10"/>
+      <c r="M45" s="10"/>
+      <c r="N45" s="10"/>
+      <c r="O45" s="10"/>
+      <c r="P45" s="10"/>
+    </row>
+    <row r="46" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B46" s="117"/>
+      <c r="C46" s="117"/>
+      <c r="D46" s="117"/>
+      <c r="E46" s="117"/>
+      <c r="F46" s="117"/>
+      <c r="G46" s="117"/>
+      <c r="K46" s="22"/>
+      <c r="L46" s="10"/>
+      <c r="M46" s="10"/>
+      <c r="N46" s="10"/>
+      <c r="O46" s="10"/>
+      <c r="P46" s="10"/>
+    </row>
+    <row r="47" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B47" s="117"/>
+      <c r="C47" s="117"/>
+      <c r="D47" s="117"/>
+      <c r="E47" s="117"/>
+      <c r="F47" s="117"/>
+      <c r="G47" s="117"/>
+      <c r="H47" s="22"/>
+      <c r="I47" s="10"/>
+      <c r="J47" s="10"/>
+      <c r="K47" s="22"/>
+      <c r="L47" s="10"/>
+      <c r="M47" s="10"/>
+      <c r="N47" s="10"/>
+      <c r="O47" s="10"/>
+      <c r="P47" s="10"/>
+    </row>
+    <row r="48" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B48" s="117"/>
+      <c r="C48" s="117"/>
+      <c r="D48" s="117"/>
+      <c r="E48" s="117"/>
+      <c r="F48" s="117"/>
+      <c r="G48" s="117"/>
+      <c r="K48" s="10"/>
+    </row>
+    <row r="49" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B49" s="117"/>
+      <c r="C49" s="117"/>
+      <c r="D49" s="117"/>
+      <c r="E49" s="117"/>
+      <c r="F49" s="117"/>
+      <c r="G49" s="117"/>
+    </row>
+    <row r="50" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B50" s="117"/>
+      <c r="C50" s="117"/>
+      <c r="D50" s="117"/>
+      <c r="E50" s="117"/>
+      <c r="F50" s="117"/>
+      <c r="G50" s="117"/>
+    </row>
+    <row r="51" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B51" s="117"/>
+      <c r="C51" s="117"/>
+      <c r="D51" s="117"/>
+      <c r="E51" s="117"/>
+      <c r="F51" s="117"/>
+      <c r="G51" s="117"/>
+    </row>
+    <row r="52" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B52" s="117"/>
+      <c r="C52" s="117"/>
+      <c r="D52" s="117"/>
+      <c r="E52" s="117"/>
+      <c r="F52" s="117"/>
+      <c r="G52" s="117"/>
+    </row>
+    <row r="53" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B53" s="117"/>
+      <c r="C53" s="117"/>
+      <c r="D53" s="117"/>
+      <c r="E53" s="117"/>
+      <c r="F53" s="117"/>
+      <c r="G53" s="117"/>
+    </row>
+    <row r="54" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B54" s="117"/>
+      <c r="C54" s="117"/>
+      <c r="D54" s="117"/>
+      <c r="E54" s="117"/>
+      <c r="F54" s="117"/>
+      <c r="G54" s="117"/>
+    </row>
+    <row r="55" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B55" s="117"/>
+      <c r="C55" s="117"/>
+      <c r="D55" s="117"/>
+      <c r="E55" s="117"/>
+      <c r="F55" s="117"/>
+      <c r="G55" s="117"/>
     </row>
   </sheetData>
-  <mergeCells count="106">
+  <mergeCells count="72">
+    <mergeCell ref="B7:O7"/>
+    <mergeCell ref="B41:F45"/>
+    <mergeCell ref="E15:E17"/>
+    <mergeCell ref="D8:F8"/>
+    <mergeCell ref="D9:F9"/>
+    <mergeCell ref="D10:F10"/>
+    <mergeCell ref="D11:F11"/>
+    <mergeCell ref="D12:F12"/>
+    <mergeCell ref="G26:I26"/>
+    <mergeCell ref="J26:K26"/>
+    <mergeCell ref="G27:I27"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="G25:I25"/>
+    <mergeCell ref="J25:K25"/>
+    <mergeCell ref="N11:O11"/>
+    <mergeCell ref="I8:K8"/>
+    <mergeCell ref="I9:K9"/>
+    <mergeCell ref="I10:K10"/>
+    <mergeCell ref="L8:M8"/>
+    <mergeCell ref="L9:M9"/>
+    <mergeCell ref="L10:M10"/>
+    <mergeCell ref="L11:M11"/>
+    <mergeCell ref="I31:L31"/>
+    <mergeCell ref="I32:L32"/>
+    <mergeCell ref="I33:L33"/>
+    <mergeCell ref="I30:L30"/>
+    <mergeCell ref="B40:F40"/>
+    <mergeCell ref="G33:H33"/>
+    <mergeCell ref="B29:E29"/>
+    <mergeCell ref="G29:H29"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="G32:H32"/>
+    <mergeCell ref="G30:H30"/>
+    <mergeCell ref="G31:H31"/>
+    <mergeCell ref="B15:B17"/>
+    <mergeCell ref="C15:C17"/>
+    <mergeCell ref="D15:D17"/>
+    <mergeCell ref="B22:L22"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="C23:C24"/>
+    <mergeCell ref="D23:D24"/>
+    <mergeCell ref="E23:E24"/>
+    <mergeCell ref="F23:F24"/>
+    <mergeCell ref="G23:I24"/>
+    <mergeCell ref="J23:K24"/>
+    <mergeCell ref="L23:L24"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="G9:H9"/>
+    <mergeCell ref="G10:H10"/>
+    <mergeCell ref="G11:H11"/>
+    <mergeCell ref="B14:Q14"/>
+    <mergeCell ref="G15:G17"/>
+    <mergeCell ref="L15:L17"/>
+    <mergeCell ref="J15:K16"/>
+    <mergeCell ref="I15:I17"/>
+    <mergeCell ref="F15:F17"/>
+    <mergeCell ref="M15:O16"/>
+    <mergeCell ref="N8:O8"/>
+    <mergeCell ref="N9:O9"/>
+    <mergeCell ref="N10:O10"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="J3:M3"/>
+    <mergeCell ref="J4:M4"/>
     <mergeCell ref="C3:G3"/>
-    <mergeCell ref="K3:N3"/>
-    <mergeCell ref="C4:G4"/>
-    <mergeCell ref="K4:N4"/>
+    <mergeCell ref="C4:G5"/>
+    <mergeCell ref="B4:B5"/>
     <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B7:S7"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="C23:D25"/>
-    <mergeCell ref="C15:D17"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="E15:G17"/>
-    <mergeCell ref="E19:G19"/>
-    <mergeCell ref="E20:G20"/>
-    <mergeCell ref="N15:O17"/>
-    <mergeCell ref="Q18:R18"/>
-    <mergeCell ref="Q19:R19"/>
-    <mergeCell ref="Q20:R20"/>
-    <mergeCell ref="N18:O18"/>
-    <mergeCell ref="Q15:T16"/>
-    <mergeCell ref="S17:T17"/>
-    <mergeCell ref="B14:Y14"/>
-    <mergeCell ref="K26:N26"/>
-    <mergeCell ref="B38:G42"/>
-    <mergeCell ref="B30:F30"/>
-    <mergeCell ref="K30:P30"/>
-    <mergeCell ref="E31:F31"/>
-    <mergeCell ref="K31:P31"/>
-    <mergeCell ref="E32:F32"/>
-    <mergeCell ref="K32:P32"/>
-    <mergeCell ref="K33:P33"/>
-    <mergeCell ref="I31:J31"/>
-    <mergeCell ref="I32:J32"/>
-    <mergeCell ref="J38:K41"/>
-    <mergeCell ref="I33:J33"/>
-    <mergeCell ref="L42:M42"/>
-    <mergeCell ref="Q8:S8"/>
-    <mergeCell ref="Q9:S9"/>
-    <mergeCell ref="Q10:S10"/>
-    <mergeCell ref="Q11:S11"/>
-    <mergeCell ref="K8:N8"/>
-    <mergeCell ref="K9:N9"/>
-    <mergeCell ref="K10:N10"/>
-    <mergeCell ref="K34:P34"/>
-    <mergeCell ref="B37:G37"/>
-    <mergeCell ref="O27:P27"/>
-    <mergeCell ref="O28:P28"/>
-    <mergeCell ref="I10:J10"/>
-    <mergeCell ref="D8:H8"/>
-    <mergeCell ref="D9:H9"/>
-    <mergeCell ref="D10:H10"/>
-    <mergeCell ref="D11:H11"/>
-    <mergeCell ref="D12:H12"/>
-    <mergeCell ref="B22:P22"/>
-    <mergeCell ref="O23:P25"/>
-    <mergeCell ref="O26:P26"/>
-    <mergeCell ref="K15:L17"/>
-    <mergeCell ref="K18:L18"/>
-    <mergeCell ref="K19:L19"/>
-    <mergeCell ref="K20:L20"/>
-    <mergeCell ref="H27:J27"/>
-    <mergeCell ref="H28:J28"/>
-    <mergeCell ref="H26:J26"/>
-    <mergeCell ref="H23:J25"/>
-    <mergeCell ref="P15:P17"/>
-    <mergeCell ref="B15:B17"/>
-    <mergeCell ref="Q17:R17"/>
     <mergeCell ref="B9:C9"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B23:B25"/>
-    <mergeCell ref="G23:G25"/>
-    <mergeCell ref="K11:N11"/>
-    <mergeCell ref="M15:M17"/>
-    <mergeCell ref="N19:O19"/>
-    <mergeCell ref="H15:J17"/>
-    <mergeCell ref="H18:J18"/>
-    <mergeCell ref="H19:J19"/>
-    <mergeCell ref="H20:J20"/>
-    <mergeCell ref="N20:O20"/>
-    <mergeCell ref="I8:J8"/>
-    <mergeCell ref="I9:J9"/>
-    <mergeCell ref="I11:J11"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="C28:D28"/>
-    <mergeCell ref="K23:N25"/>
-    <mergeCell ref="K28:N28"/>
-    <mergeCell ref="K27:N27"/>
-    <mergeCell ref="V15:Y16"/>
-    <mergeCell ref="V17:W17"/>
-    <mergeCell ref="V18:W18"/>
-    <mergeCell ref="V19:W19"/>
-    <mergeCell ref="V20:W20"/>
-    <mergeCell ref="X17:Y17"/>
-    <mergeCell ref="X18:Y18"/>
-    <mergeCell ref="X19:Y19"/>
-    <mergeCell ref="X20:Y20"/>
-    <mergeCell ref="S18:T18"/>
-    <mergeCell ref="S19:T19"/>
-    <mergeCell ref="S20:T20"/>
-    <mergeCell ref="U15:U17"/>
-    <mergeCell ref="E18:G18"/>
-    <mergeCell ref="E23:E25"/>
-    <mergeCell ref="F23:F25"/>
+    <mergeCell ref="I11:K11"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E26:E28" xr:uid="{B316A799-CF60-4C99-A88E-2204076E38E6}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D26:D27" xr:uid="{B316A799-CF60-4C99-A88E-2204076E38E6}">
       <formula1>"กล่อง, เม็ด, ไวอัล, แอมพูล, ขวด, box, tablet, vial, ampoul, bottle"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F33:F34" xr:uid="{2CF9FB64-438B-485F-A115-633E3AF0704D}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E32:E33" xr:uid="{2CF9FB64-438B-485F-A115-633E3AF0704D}">
       <formula1>"Days (วัน), Months (เดือน), Years (ปี)"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
   <headerFooter>
     <oddFooter>&amp;R_x000D_&amp;1#&amp;"Calibri"&amp;22&amp;KFF8939 RESTRICTED</oddFooter>
   </headerFooter>
-  <drawing r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E9BADA0-6CEF-4001-8243-A13FFD1BF3BE}">
-  <dimension ref="A1:U52"/>
+  <sheetPr codeName="Sheet2"/>
+  <dimension ref="A1:W52"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="43.5703125" bestFit="1" customWidth="1"/>
@@ -2567,17 +2706,19 @@
     <col min="19" max="19" width="38.85546875" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="27.140625" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="43.28515625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="30.42578125" customWidth="1"/>
+    <col min="23" max="23" width="35.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -2585,7 +2726,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -2593,7 +2734,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>17</v>
       </c>
@@ -2601,7 +2742,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>18</v>
       </c>
@@ -2609,7 +2750,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -2617,7 +2758,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>20</v>
       </c>
@@ -2625,7 +2766,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -2633,7 +2774,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>0</v>
       </c>
@@ -2641,85 +2782,92 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B10" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B11" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>109</v>
       </c>
       <c r="B12" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B13" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>112</v>
       </c>
       <c r="B14" t="s">
-        <v>70</v>
-      </c>
-      <c r="C14" s="33"/>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>118</v>
+      </c>
+      <c r="B15" s="46" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="17" spans="1:21" x14ac:dyDescent="0.25">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="17" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="L17" s="2" t="s">
         <v>9</v>
@@ -2734,91 +2882,103 @@
         <v>13</v>
       </c>
       <c r="P17" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q17" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="R17" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="S17" s="2" t="s">
-        <v>54</v>
+        <v>121</v>
       </c>
       <c r="T17" s="2" t="s">
-        <v>56</v>
+        <v>122</v>
       </c>
       <c r="U17" s="2" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="18" spans="1:21" x14ac:dyDescent="0.25">
+        <v>55</v>
+      </c>
+      <c r="V17" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="W17" s="2" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="18" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B18" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B18" s="4" t="s">
-        <v>111</v>
-      </c>
       <c r="C18" t="s">
+        <v>28</v>
+      </c>
+      <c r="D18" t="s">
+        <v>29</v>
+      </c>
+      <c r="E18" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="F18" t="s">
+        <v>34</v>
+      </c>
+      <c r="G18" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="H18" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="I18" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="J18" t="s">
+        <v>42</v>
+      </c>
+      <c r="K18" t="s">
+        <v>44</v>
+      </c>
+      <c r="L18" t="s">
+        <v>24</v>
+      </c>
+      <c r="M18" t="s">
+        <v>25</v>
+      </c>
+      <c r="N18" t="s">
+        <v>26</v>
+      </c>
+      <c r="O18" t="s">
         <v>27</v>
       </c>
-      <c r="D18" t="s">
-        <v>28</v>
-      </c>
-      <c r="E18" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="F18" t="s">
-        <v>33</v>
-      </c>
-      <c r="G18" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="H18" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="I18" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="J18" t="s">
-        <v>41</v>
-      </c>
-      <c r="K18" t="s">
-        <v>43</v>
-      </c>
-      <c r="L18" t="s">
-        <v>23</v>
-      </c>
-      <c r="M18" t="s">
-        <v>24</v>
-      </c>
-      <c r="N18" t="s">
-        <v>25</v>
-      </c>
-      <c r="O18" t="s">
-        <v>26</v>
-      </c>
       <c r="P18" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Q18" t="e">
         <f>IF(D18&gt;0,IF(D18="Unit",CONCATENATE(Settings!P18," ",Settings!D18,"s"),CONCATENATE((Settings!P18/Settings!L18)," ",Settings!D18,"s")),"")</f>
         <v>#VALUE!</v>
       </c>
       <c r="R18" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="S18" t="s">
-        <v>55</v>
+        <v>119</v>
       </c>
       <c r="T18" t="s">
-        <v>61</v>
+        <v>120</v>
       </c>
       <c r="U18" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="19" spans="1:21" x14ac:dyDescent="0.25">
+        <v>56</v>
+      </c>
+      <c r="V18" t="s">
+        <v>62</v>
+      </c>
+      <c r="W18" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="19" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A19" s="3"/>
       <c r="B19" s="4"/>
       <c r="E19" s="9"/>
@@ -2830,7 +2990,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A20" s="3"/>
       <c r="B20" s="4"/>
       <c r="E20" s="9"/>
@@ -2842,7 +3002,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A21" s="3"/>
       <c r="B21" s="4"/>
       <c r="E21" s="9"/>
@@ -2854,7 +3014,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A22" s="3"/>
       <c r="B22" s="4"/>
       <c r="E22" s="9"/>
@@ -2866,7 +3026,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A23" s="3"/>
       <c r="B23" s="4"/>
       <c r="E23" s="9"/>
@@ -2878,7 +3038,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A24" s="3"/>
       <c r="B24" s="4"/>
       <c r="E24" s="9"/>
@@ -2890,7 +3050,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A25" s="3"/>
       <c r="B25" s="4"/>
       <c r="E25" s="9"/>
@@ -2902,7 +3062,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A26" s="3"/>
       <c r="B26" s="4"/>
       <c r="E26" s="9"/>
@@ -2914,7 +3074,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A27" s="3"/>
       <c r="B27" s="4"/>
       <c r="E27" s="9"/>
@@ -2926,7 +3086,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A28" s="3"/>
       <c r="B28" s="4"/>
       <c r="E28" s="9"/>
@@ -2938,7 +3098,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A29" s="3"/>
       <c r="B29" s="4"/>
       <c r="E29" s="9"/>
@@ -2950,7 +3110,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A30" s="3"/>
       <c r="B30" s="4"/>
       <c r="E30" s="9"/>
@@ -2962,10 +3122,9 @@
         <v/>
       </c>
     </row>
-    <row r="31" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A31" s="3"/>
       <c r="B31" s="4"/>
-      <c r="C31" s="36"/>
       <c r="E31" s="9"/>
       <c r="G31" s="9"/>
       <c r="H31" s="9"/>
@@ -2975,10 +3134,9 @@
         <v/>
       </c>
     </row>
-    <row r="32" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A32" s="3"/>
       <c r="B32" s="4"/>
-      <c r="C32" s="36"/>
       <c r="E32" s="9"/>
       <c r="G32" s="9"/>
       <c r="H32" s="9"/>
@@ -3242,6 +3400,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010075F372E8CCA016418A193AD921508903" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="f5e922417d740f1a527805650dc2dfa9">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="399317f3-0083-4d0b-9572-12af99626311" xmlns:ns3="1444eecc-14bb-4066-abe6-ce6de21d9439" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="078d79524add6eac9b94134ca637184e" ns2:_="" ns3:_="">
     <xsd:import namespace="399317f3-0083-4d0b-9572-12af99626311"/>
@@ -3438,15 +3605,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -3462,6 +3620,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A00E6A9-20DD-4842-9306-307EB080AF2E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8CF88A1C-AA0D-4F8F-A0FD-6F3FAFCA9DC0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3480,14 +3646,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A00E6A9-20DD-4842-9306-307EB080AF2E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7EBE950A-5812-419E-B174-6A5D9B8E0414}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Template modification for thailand
</commit_message>
<xml_diff>
--- a/srv/xlsx-templates/TH - Quotation Template.xlsx
+++ b/srv/xlsx-templates/TH - Quotation Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bayergroup-my.sharepoint.com/personal/kosal_kirthiga_ext_bayer_com/Documents/Desktop/ThailandLates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="277" documentId="8_{DE39F225-2AE1-4446-AB5F-E204FEABCD0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E5C23729-F91F-43E4-9E3D-5496BB18429B}"/>
+  <xr:revisionPtr revIDLastSave="311" documentId="8_{DE39F225-2AE1-4446-AB5F-E204FEABCD0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6A39CB95-14C1-4101-B671-F581D1C814C9}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{F5CC2154-27BB-4652-B61E-D913F0CC6809}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="136">
   <si>
     <t>${offerValidation.INSTITUTENAME}</t>
   </si>
@@ -416,6 +416,36 @@
   </si>
   <si>
     <t>${table:offerProductValidation.PRESENTATION}</t>
+  </si>
+  <si>
+    <t>130/1 North Sathon Road, Silom, Bangrak, Bangkok 10500</t>
+  </si>
+  <si>
+    <t>0100</t>
+  </si>
+  <si>
+    <t xml:space="preserve">${offerValidation.TENDERID}		</t>
+  </si>
+  <si>
+    <t>${offerValidation.PRODUCT_UNIT_NAME}</t>
+  </si>
+  <si>
+    <t>ProductGenericname</t>
+  </si>
+  <si>
+    <t>ProductGenericName</t>
+  </si>
+  <si>
+    <t>${table:offerProductValidation.CODE3}</t>
+  </si>
+  <si>
+    <t>${table:offerProductValidation.CODE2}</t>
+  </si>
+  <si>
+    <t>THCC</t>
+  </si>
+  <si>
+    <t>${table:offerProductValidation.GOV_CODE}</t>
   </si>
 </sst>
 </file>
@@ -875,6 +905,11 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="43" fontId="5" fillId="0" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -931,15 +966,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -1214,14 +1240,10 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2EFFBCB4-83C9-46C5-9D10-EDD296E322D9}" name="Tabel2" displayName="Tabel2" ref="C17:W52" totalsRowShown="0" headerRowDxfId="6">
-  <autoFilter ref="C17:W52" xr:uid="{2EFFBCB4-83C9-46C5-9D10-EDD296E322D9}"/>
-  <tableColumns count="21">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2EFFBCB4-83C9-46C5-9D10-EDD296E322D9}" name="Tabel2" displayName="Tabel2" ref="D18:AA53" totalsRowShown="0" headerRowDxfId="6">
+  <autoFilter ref="D18:AA53" xr:uid="{2EFFBCB4-83C9-46C5-9D10-EDD296E322D9}"/>
+  <tableColumns count="24">
     <tableColumn id="1" xr3:uid="{6E1F8ECB-E862-46B4-998C-BE8E89C238BA}" name="PAID VOLUME"/>
     <tableColumn id="2" xr3:uid="{6497AF92-63C8-4790-818D-6E5BE819E8D6}" name="UNIT"/>
     <tableColumn id="3" xr3:uid="{A1E59B72-B459-4BFA-9B37-9736C0F03B7E}" name="OFFER PRICE" dataDxfId="5"/>
@@ -1237,13 +1259,16 @@
     <tableColumn id="13" xr3:uid="{7D1379AA-4B8F-4BC6-9726-365EBAE15341}" name="FOC"/>
     <tableColumn id="14" xr3:uid="{DF88A36E-0423-48FC-A1FC-B18BF3BA8D1A}" name="Total Quantity Units"/>
     <tableColumn id="15" xr3:uid="{6B128E87-63EB-483B-88D7-EA33600F43AB}" name="Total QTY" dataDxfId="1">
-      <calculatedColumnFormula>IF(D18&gt;0,IF(D18="Unit",CONCATENATE(Settings!P18," ",Settings!D18,"s"),CONCATENATE((Settings!P18/Settings!L18)," ",Settings!D18,"s")),"")</calculatedColumnFormula>
+      <calculatedColumnFormula>IF(E19&gt;0,IF(E19="Unit",CONCATENATE(Settings!Q19," ",Settings!E19,"s"),CONCATENATE((Settings!Q19/Settings!M19)," ",Settings!E19,"s")),"")</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="16" xr3:uid="{E4D044B6-D053-487A-AA8C-F40FE34F30A7}" name="Net Price"/>
     <tableColumn id="17" xr3:uid="{F95E93A8-C80D-4AC7-9526-72374F546CE7}" name="Net Price Pack Vat"/>
     <tableColumn id="18" xr3:uid="{2DDE85E8-6C8E-4D93-A4E8-1F80D965246B}" name="Net Price Unit Vat"/>
     <tableColumn id="20" xr3:uid="{CB417A4B-91CA-49CD-9B3D-699005D44488}" name="Amount in numbers"/>
     <tableColumn id="21" xr3:uid="{07B28F29-5FC9-406A-96FC-77FFBFB88A05}" name="VAT total"/>
+    <tableColumn id="23" xr3:uid="{6CCBAAC0-B712-4045-B8A8-11B1701BD7D7}" name="GPU"/>
+    <tableColumn id="24" xr3:uid="{CCFCD047-C7DB-493A-9963-D2A80EA567D1}" name="THCC"/>
+    <tableColumn id="19" xr3:uid="{EFC0A69B-3069-4765-A820-C00302221FA7}" name="TPU"/>
     <tableColumn id="22" xr3:uid="{275B8D63-D363-4D68-BC9C-CB91FD9D0201}" name="Amount in numbers vat"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1251,8 +1276,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{13195211-A053-4079-8580-181B8695617E}" name="Tabel14" displayName="Tabel14" ref="A1:B15" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="A1:B15" xr:uid="{13195211-A053-4079-8580-181B8695617E}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{13195211-A053-4079-8580-181B8695617E}" name="Tabel14" displayName="Tabel14" ref="A1:B16" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:B16" xr:uid="{13195211-A053-4079-8580-181B8695617E}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{04053350-A8BA-4F7A-9272-32CAE894E561}" name="Header fields"/>
     <tableColumn id="2" xr3:uid="{91B26FA0-9378-480D-8354-6037F7FF582C}" name="Description"/>
@@ -1638,7 +1663,9 @@
       <c r="I4" s="35" t="s">
         <v>66</v>
       </c>
-      <c r="J4" s="120"/>
+      <c r="J4" s="120" t="s">
+        <v>126</v>
+      </c>
       <c r="K4" s="121"/>
       <c r="L4" s="121"/>
       <c r="M4" s="122"/>
@@ -1681,44 +1708,48 @@
       <c r="P6" s="10"/>
     </row>
     <row r="7" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B7" s="54" t="s">
+      <c r="B7" s="57" t="s">
         <v>67</v>
       </c>
-      <c r="C7" s="55"/>
-      <c r="D7" s="55"/>
-      <c r="E7" s="55"/>
-      <c r="F7" s="55"/>
-      <c r="G7" s="55"/>
-      <c r="H7" s="55"/>
-      <c r="I7" s="55"/>
-      <c r="J7" s="55"/>
-      <c r="K7" s="55"/>
-      <c r="L7" s="55"/>
-      <c r="M7" s="55"/>
-      <c r="N7" s="55"/>
-      <c r="O7" s="56"/>
+      <c r="C7" s="58"/>
+      <c r="D7" s="58"/>
+      <c r="E7" s="58"/>
+      <c r="F7" s="58"/>
+      <c r="G7" s="58"/>
+      <c r="H7" s="58"/>
+      <c r="I7" s="58"/>
+      <c r="J7" s="58"/>
+      <c r="K7" s="58"/>
+      <c r="L7" s="58"/>
+      <c r="M7" s="58"/>
+      <c r="N7" s="58"/>
+      <c r="O7" s="59"/>
     </row>
     <row r="8" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="113" t="s">
         <v>68</v>
       </c>
       <c r="C8" s="119"/>
-      <c r="D8" s="62"/>
-      <c r="E8" s="63"/>
-      <c r="F8" s="64"/>
+      <c r="D8" s="65" t="s">
+        <v>128</v>
+      </c>
+      <c r="E8" s="66"/>
+      <c r="F8" s="67"/>
       <c r="G8" s="113" t="s">
         <v>69</v>
       </c>
       <c r="H8" s="114"/>
-      <c r="I8" s="73"/>
-      <c r="J8" s="74"/>
-      <c r="K8" s="75"/>
+      <c r="I8" s="76" t="s">
+        <v>127</v>
+      </c>
+      <c r="J8" s="77"/>
+      <c r="K8" s="78"/>
       <c r="L8" s="79" t="s">
         <v>70</v>
       </c>
       <c r="M8" s="80"/>
-      <c r="N8" s="71"/>
-      <c r="O8" s="72"/>
+      <c r="N8" s="74"/>
+      <c r="O8" s="75"/>
       <c r="P8" s="29"/>
     </row>
     <row r="9" spans="2:17" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1726,12 +1757,12 @@
         <v>71</v>
       </c>
       <c r="C9" s="119"/>
-      <c r="D9" s="62" t="str">
+      <c r="D9" s="65" t="str">
         <f>Settings!A14</f>
         <v>${offerValidation.CUSTOMER_CODE}</v>
       </c>
-      <c r="E9" s="63"/>
-      <c r="F9" s="64"/>
+      <c r="E9" s="66"/>
+      <c r="F9" s="67"/>
       <c r="G9" s="115" t="s">
         <v>72</v>
       </c>
@@ -1745,8 +1776,8 @@
         <v>73</v>
       </c>
       <c r="M9" s="80"/>
-      <c r="N9" s="71"/>
-      <c r="O9" s="72"/>
+      <c r="N9" s="74"/>
+      <c r="O9" s="75"/>
       <c r="P9" s="29"/>
     </row>
     <row r="10" spans="2:17" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1754,12 +1785,12 @@
         <v>74</v>
       </c>
       <c r="C10" s="119"/>
-      <c r="D10" s="62" t="str">
+      <c r="D10" s="65" t="str">
         <f>Settings!A9</f>
         <v>${offerValidation.INSTITUTENAME}</v>
       </c>
-      <c r="E10" s="63"/>
-      <c r="F10" s="64"/>
+      <c r="E10" s="66"/>
+      <c r="F10" s="67"/>
       <c r="G10" s="117" t="s">
         <v>5</v>
       </c>
@@ -1773,8 +1804,8 @@
         <v>75</v>
       </c>
       <c r="M10" s="80"/>
-      <c r="N10" s="71"/>
-      <c r="O10" s="72"/>
+      <c r="N10" s="74"/>
+      <c r="O10" s="75"/>
       <c r="P10" s="29"/>
     </row>
     <row r="11" spans="2:17" x14ac:dyDescent="0.25">
@@ -1782,11 +1813,11 @@
         <v>6</v>
       </c>
       <c r="C11" s="119"/>
-      <c r="D11" s="65" t="s">
+      <c r="D11" s="68" t="s">
         <v>21</v>
       </c>
-      <c r="E11" s="66"/>
-      <c r="F11" s="67"/>
+      <c r="E11" s="69"/>
+      <c r="F11" s="70"/>
       <c r="G11" s="113" t="s">
         <v>7</v>
       </c>
@@ -1800,8 +1831,8 @@
         <v>73</v>
       </c>
       <c r="M11" s="80"/>
-      <c r="N11" s="71"/>
-      <c r="O11" s="72"/>
+      <c r="N11" s="74"/>
+      <c r="O11" s="75"/>
       <c r="P11" s="29"/>
     </row>
     <row r="12" spans="2:17" x14ac:dyDescent="0.25">
@@ -1809,11 +1840,11 @@
         <v>8</v>
       </c>
       <c r="C12" s="119"/>
-      <c r="D12" s="65" t="s">
+      <c r="D12" s="68" t="s">
         <v>19</v>
       </c>
-      <c r="E12" s="66"/>
-      <c r="F12" s="67"/>
+      <c r="E12" s="69"/>
+      <c r="F12" s="70"/>
       <c r="G12" s="10"/>
       <c r="H12" s="10"/>
       <c r="I12" s="10"/>
@@ -1865,32 +1896,32 @@
       <c r="B15" s="95" t="s">
         <v>77</v>
       </c>
-      <c r="C15" s="59" t="s">
+      <c r="C15" s="62" t="s">
         <v>78</v>
       </c>
-      <c r="D15" s="59" t="s">
+      <c r="D15" s="62" t="s">
         <v>79</v>
       </c>
-      <c r="E15" s="59" t="s">
+      <c r="E15" s="62" t="s">
         <v>80</v>
       </c>
-      <c r="F15" s="59" t="s">
+      <c r="F15" s="62" t="s">
         <v>115</v>
       </c>
-      <c r="G15" s="59" t="s">
+      <c r="G15" s="62" t="s">
         <v>114</v>
       </c>
       <c r="H15" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="I15" s="59" t="s">
+      <c r="I15" s="62" t="s">
         <v>81</v>
       </c>
       <c r="J15" s="103" t="s">
         <v>10</v>
       </c>
       <c r="K15" s="104"/>
-      <c r="L15" s="59" t="s">
+      <c r="L15" s="62" t="s">
         <v>82</v>
       </c>
       <c r="M15" s="103" t="s">
@@ -1905,16 +1936,16 @@
     </row>
     <row r="16" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B16" s="96"/>
-      <c r="C16" s="60"/>
-      <c r="D16" s="60"/>
-      <c r="E16" s="60"/>
-      <c r="F16" s="60"/>
-      <c r="G16" s="60"/>
+      <c r="C16" s="63"/>
+      <c r="D16" s="63"/>
+      <c r="E16" s="63"/>
+      <c r="F16" s="63"/>
+      <c r="G16" s="63"/>
       <c r="H16" s="32"/>
-      <c r="I16" s="60"/>
+      <c r="I16" s="63"/>
       <c r="J16" s="105"/>
       <c r="K16" s="106"/>
-      <c r="L16" s="60"/>
+      <c r="L16" s="63"/>
       <c r="M16" s="108"/>
       <c r="N16" s="109"/>
       <c r="O16" s="109"/>
@@ -1923,20 +1954,20 @@
     </row>
     <row r="17" spans="2:19" ht="25.5" x14ac:dyDescent="0.25">
       <c r="B17" s="97"/>
-      <c r="C17" s="61"/>
-      <c r="D17" s="61"/>
-      <c r="E17" s="61"/>
-      <c r="F17" s="61"/>
-      <c r="G17" s="61"/>
+      <c r="C17" s="64"/>
+      <c r="D17" s="64"/>
+      <c r="E17" s="64"/>
+      <c r="F17" s="64"/>
+      <c r="G17" s="64"/>
       <c r="H17" s="31"/>
-      <c r="I17" s="61"/>
+      <c r="I17" s="64"/>
       <c r="J17" s="13" t="s">
         <v>84</v>
       </c>
       <c r="K17" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="L17" s="61"/>
+      <c r="L17" s="64"/>
       <c r="M17" s="13" t="s">
         <v>84</v>
       </c>
@@ -1963,7 +1994,9 @@
       <c r="D18" s="45" t="s">
         <v>113</v>
       </c>
-      <c r="E18" s="43"/>
+      <c r="E18" s="43" t="s">
+        <v>22</v>
+      </c>
       <c r="F18" s="15" t="s">
         <v>28</v>
       </c>
@@ -2076,16 +2109,16 @@
       <c r="B23" s="99" t="s">
         <v>77</v>
       </c>
-      <c r="C23" s="59" t="s">
+      <c r="C23" s="62" t="s">
         <v>78</v>
       </c>
       <c r="D23" s="100" t="s">
         <v>87</v>
       </c>
-      <c r="E23" s="59" t="s">
+      <c r="E23" s="62" t="s">
         <v>88</v>
       </c>
-      <c r="F23" s="59" t="s">
+      <c r="F23" s="62" t="s">
         <v>89</v>
       </c>
       <c r="G23" s="102" t="s">
@@ -2104,10 +2137,10 @@
     </row>
     <row r="24" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B24" s="99"/>
-      <c r="C24" s="61"/>
+      <c r="C24" s="64"/>
       <c r="D24" s="101"/>
-      <c r="E24" s="61"/>
-      <c r="F24" s="61"/>
+      <c r="E24" s="64"/>
+      <c r="F24" s="64"/>
       <c r="G24" s="102"/>
       <c r="H24" s="102"/>
       <c r="I24" s="102"/>
@@ -2124,15 +2157,21 @@
         <v>23</v>
       </c>
       <c r="D25" s="34"/>
-      <c r="E25" s="20"/>
-      <c r="F25" s="20"/>
-      <c r="G25" s="70"/>
-      <c r="H25" s="70"/>
-      <c r="I25" s="70"/>
-      <c r="J25" s="71" t="s">
+      <c r="E25" s="20" t="s">
+        <v>132</v>
+      </c>
+      <c r="F25" s="20" t="s">
+        <v>133</v>
+      </c>
+      <c r="G25" s="73" t="s">
+        <v>135</v>
+      </c>
+      <c r="H25" s="73"/>
+      <c r="I25" s="73"/>
+      <c r="J25" s="74" t="s">
         <v>116</v>
       </c>
-      <c r="K25" s="72"/>
+      <c r="K25" s="75"/>
       <c r="L25" s="20" t="s">
         <v>26</v>
       </c>
@@ -2144,11 +2183,11 @@
       <c r="D26" s="20"/>
       <c r="E26" s="20"/>
       <c r="F26" s="20"/>
-      <c r="G26" s="68"/>
-      <c r="H26" s="68"/>
-      <c r="I26" s="68"/>
-      <c r="J26" s="69"/>
-      <c r="K26" s="69"/>
+      <c r="G26" s="71"/>
+      <c r="H26" s="71"/>
+      <c r="I26" s="71"/>
+      <c r="J26" s="72"/>
+      <c r="K26" s="72"/>
       <c r="L26" s="20"/>
       <c r="M26" s="10"/>
     </row>
@@ -2158,11 +2197,11 @@
       <c r="D27" s="20"/>
       <c r="E27" s="20"/>
       <c r="F27" s="20"/>
-      <c r="G27" s="68"/>
-      <c r="H27" s="68"/>
-      <c r="I27" s="68"/>
-      <c r="J27" s="69"/>
-      <c r="K27" s="69"/>
+      <c r="G27" s="71"/>
+      <c r="H27" s="71"/>
+      <c r="I27" s="71"/>
+      <c r="J27" s="72"/>
+      <c r="K27" s="72"/>
       <c r="L27" s="20"/>
       <c r="M27" s="10"/>
     </row>
@@ -2216,10 +2255,10 @@
         <v>97</v>
       </c>
       <c r="H30" s="94"/>
-      <c r="I30" s="65"/>
-      <c r="J30" s="66"/>
-      <c r="K30" s="66"/>
-      <c r="L30" s="67"/>
+      <c r="I30" s="68"/>
+      <c r="J30" s="69"/>
+      <c r="K30" s="69"/>
+      <c r="L30" s="70"/>
       <c r="M30" s="10"/>
       <c r="N30" s="10"/>
     </row>
@@ -2228,17 +2267,17 @@
         <v>98</v>
       </c>
       <c r="C31" s="24"/>
-      <c r="D31" s="69"/>
-      <c r="E31" s="69"/>
+      <c r="D31" s="72"/>
+      <c r="E31" s="72"/>
       <c r="F31" s="10"/>
       <c r="G31" s="93" t="s">
         <v>99</v>
       </c>
       <c r="H31" s="94"/>
-      <c r="I31" s="65"/>
-      <c r="J31" s="66"/>
-      <c r="K31" s="66"/>
-      <c r="L31" s="67"/>
+      <c r="I31" s="68"/>
+      <c r="J31" s="69"/>
+      <c r="K31" s="69"/>
+      <c r="L31" s="70"/>
       <c r="M31" s="10"/>
       <c r="N31" s="10"/>
     </row>
@@ -2256,10 +2295,10 @@
         <v>102</v>
       </c>
       <c r="H32" s="94"/>
-      <c r="I32" s="65"/>
-      <c r="J32" s="66"/>
-      <c r="K32" s="66"/>
-      <c r="L32" s="67"/>
+      <c r="I32" s="68"/>
+      <c r="J32" s="69"/>
+      <c r="K32" s="69"/>
+      <c r="L32" s="70"/>
       <c r="M32" s="10"/>
       <c r="N32" s="10"/>
     </row>
@@ -2319,13 +2358,13 @@
       <c r="P35" s="10"/>
     </row>
     <row r="36" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B36" s="57" t="s">
+      <c r="B36" s="60" t="s">
         <v>122</v>
       </c>
-      <c r="C36" s="57"/>
-      <c r="D36" s="57"/>
-      <c r="E36" s="57"/>
-      <c r="F36" s="57"/>
+      <c r="C36" s="60"/>
+      <c r="D36" s="60"/>
+      <c r="E36" s="60"/>
+      <c r="F36" s="60"/>
       <c r="G36" s="42"/>
       <c r="H36" s="10"/>
       <c r="I36" s="10"/>
@@ -2338,11 +2377,11 @@
       <c r="P36" s="10"/>
     </row>
     <row r="37" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B37" s="58"/>
-      <c r="C37" s="58"/>
-      <c r="D37" s="58"/>
-      <c r="E37" s="58"/>
-      <c r="F37" s="58"/>
+      <c r="B37" s="61"/>
+      <c r="C37" s="61"/>
+      <c r="D37" s="61"/>
+      <c r="E37" s="61"/>
+      <c r="F37" s="61"/>
       <c r="G37" s="42"/>
       <c r="H37" s="10"/>
       <c r="I37" s="10"/>
@@ -2355,11 +2394,11 @@
       <c r="P37" s="10"/>
     </row>
     <row r="38" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B38" s="58"/>
-      <c r="C38" s="58"/>
-      <c r="D38" s="58"/>
-      <c r="E38" s="58"/>
-      <c r="F38" s="58"/>
+      <c r="B38" s="61"/>
+      <c r="C38" s="61"/>
+      <c r="D38" s="61"/>
+      <c r="E38" s="61"/>
+      <c r="F38" s="61"/>
       <c r="G38" s="42"/>
       <c r="H38" s="28" t="s">
         <v>106</v>
@@ -2375,11 +2414,11 @@
       <c r="P38" s="10"/>
     </row>
     <row r="39" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B39" s="58"/>
-      <c r="C39" s="58"/>
-      <c r="D39" s="58"/>
-      <c r="E39" s="58"/>
-      <c r="F39" s="58"/>
+      <c r="B39" s="61"/>
+      <c r="C39" s="61"/>
+      <c r="D39" s="61"/>
+      <c r="E39" s="61"/>
+      <c r="F39" s="61"/>
       <c r="G39" s="42"/>
       <c r="H39" s="10"/>
       <c r="I39" s="10" t="s">
@@ -2393,11 +2432,11 @@
       <c r="P39" s="10"/>
     </row>
     <row r="40" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B40" s="58"/>
-      <c r="C40" s="58"/>
-      <c r="D40" s="58"/>
-      <c r="E40" s="58"/>
-      <c r="F40" s="58"/>
+      <c r="B40" s="61"/>
+      <c r="C40" s="61"/>
+      <c r="D40" s="61"/>
+      <c r="E40" s="61"/>
+      <c r="F40" s="61"/>
       <c r="G40" s="42"/>
       <c r="H40" s="10"/>
       <c r="I40" s="10"/>
@@ -2599,43 +2638,45 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E9BADA0-6CEF-4001-8243-A13FFD1BF3BE}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:W52"/>
+  <dimension ref="A1:AA53"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="43.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="50.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="47.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="36.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="46.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="44.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="52.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="69.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="75.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="42.28515625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="40.5703125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="42.140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="41.7109375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="52.85546875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="36.28515625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="46.7109375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="16.28515625" customWidth="1"/>
-    <col min="18" max="18" width="39.5703125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="38.85546875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="27.140625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="43.28515625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="30.42578125" customWidth="1"/>
-    <col min="23" max="23" width="35.85546875" customWidth="1"/>
+    <col min="3" max="3" width="50.28515625" style="33" customWidth="1"/>
+    <col min="4" max="4" width="47.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="36.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="46.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="44.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="52.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="69.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="75.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="42.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="40.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="42.140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="41.7109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="52.85546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="36.28515625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="46.7109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="16.28515625" customWidth="1"/>
+    <col min="19" max="19" width="39.5703125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="38.85546875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="27.140625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="43.28515625" bestFit="1" customWidth="1"/>
+    <col min="23" max="26" width="30.42578125" customWidth="1"/>
+    <col min="27" max="27" width="35.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>46</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C1" s="55"/>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -2643,7 +2684,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -2651,7 +2692,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>17</v>
       </c>
@@ -2659,7 +2700,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>18</v>
       </c>
@@ -2667,7 +2708,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -2675,7 +2716,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>20</v>
       </c>
@@ -2683,7 +2724,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -2691,7 +2732,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>0</v>
       </c>
@@ -2699,7 +2740,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>60</v>
       </c>
@@ -2707,7 +2748,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>110</v>
       </c>
@@ -2715,7 +2756,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>109</v>
       </c>
@@ -2723,7 +2764,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>111</v>
       </c>
@@ -2731,7 +2772,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>112</v>
       </c>
@@ -2739,567 +2780,600 @@
         <v>71</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>129</v>
+      </c>
+      <c r="B15" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
         <v>117</v>
       </c>
-      <c r="B15" s="37" t="s">
+      <c r="B16" s="54" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
+      <c r="C16" s="37"/>
+    </row>
+    <row r="17" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A17" s="7" t="s">
+    <row r="18" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A18" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="B17" s="8" t="s">
+      <c r="B18" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="C18" s="56" t="s">
+        <v>131</v>
+      </c>
+      <c r="D18" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="D17" s="2" t="s">
+      <c r="E18" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="E17" s="2" t="s">
+      <c r="F18" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="F17" s="2" t="s">
+      <c r="G18" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="G17" s="2" t="s">
+      <c r="H18" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="H17" s="2" t="s">
+      <c r="I18" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="I17" s="2" t="s">
+      <c r="J18" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="J17" s="2" t="s">
+      <c r="K18" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="K17" s="2" t="s">
+      <c r="L18" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="L17" s="2" t="s">
+      <c r="M18" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="M17" s="2" t="s">
+      <c r="N18" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="N17" s="2" t="s">
+      <c r="O18" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="O17" s="2" t="s">
+      <c r="P18" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="P17" s="2" t="s">
+      <c r="Q18" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="Q17" s="2" t="s">
+      <c r="R18" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="R17" s="2" t="s">
+      <c r="S18" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="S17" s="2" t="s">
+      <c r="T18" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="T17" s="2" t="s">
+      <c r="U18" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="U17" s="2" t="s">
+      <c r="V18" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="V17" s="2" t="s">
+      <c r="W18" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="W17" s="2" t="s">
+      <c r="X18" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="Y18" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="Z18" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="AA18" s="2" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A18" s="3" t="s">
+    <row r="19" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="B19" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C19" s="33" t="s">
+        <v>22</v>
+      </c>
+      <c r="D19" t="s">
         <v>28</v>
       </c>
-      <c r="D18" t="s">
+      <c r="E19" t="s">
         <v>29</v>
       </c>
-      <c r="E18" s="9" t="s">
+      <c r="F19" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="F18" t="s">
+      <c r="G19" t="s">
         <v>34</v>
       </c>
-      <c r="G18" s="9" t="s">
+      <c r="H19" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="H18" s="9" t="s">
+      <c r="I19" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="I18" s="9" t="s">
+      <c r="J19" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="J18" t="s">
+      <c r="K19" t="s">
         <v>42</v>
       </c>
-      <c r="K18" t="s">
+      <c r="L19" t="s">
         <v>44</v>
       </c>
-      <c r="L18" t="s">
+      <c r="M19" t="s">
         <v>24</v>
       </c>
-      <c r="M18" t="s">
+      <c r="N19" t="s">
         <v>25</v>
       </c>
-      <c r="N18" t="s">
+      <c r="O19" t="s">
         <v>26</v>
       </c>
-      <c r="O18" t="s">
+      <c r="P19" t="s">
         <v>27</v>
       </c>
-      <c r="P18" t="s">
+      <c r="Q19" t="s">
         <v>63</v>
       </c>
-      <c r="Q18" t="e">
-        <f>IF(D18&gt;0,IF(D18="Unit",CONCATENATE(Settings!P18," ",Settings!D18,"s"),CONCATENATE((Settings!P18/Settings!L18)," ",Settings!D18,"s")),"")</f>
+      <c r="R19" t="e">
+        <f>IF(E19&gt;0,IF(E19="Unit",CONCATENATE(Settings!Q19," ",Settings!E19,"s"),CONCATENATE((Settings!Q19/Settings!M19)," ",Settings!E19,"s")),"")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="R18" t="s">
+      <c r="S19" t="s">
         <v>54</v>
       </c>
-      <c r="S18" t="s">
+      <c r="T19" t="s">
         <v>118</v>
       </c>
-      <c r="T18" t="s">
+      <c r="U19" t="s">
         <v>119</v>
       </c>
-      <c r="U18" t="s">
+      <c r="V19" t="s">
         <v>56</v>
       </c>
-      <c r="V18" t="s">
+      <c r="W19" t="s">
         <v>62</v>
       </c>
-      <c r="W18" t="s">
+      <c r="X19" t="s">
+        <v>133</v>
+      </c>
+      <c r="Y19" t="s">
+        <v>135</v>
+      </c>
+      <c r="Z19" t="s">
+        <v>132</v>
+      </c>
+      <c r="AA19" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A19" s="3"/>
-      <c r="B19" s="4"/>
-      <c r="E19" s="9"/>
-      <c r="G19" s="9"/>
-      <c r="H19" s="9"/>
-      <c r="I19" s="9"/>
-      <c r="Q19" t="str">
-        <f>IF(D19&gt;0,IF(D19="Unit",CONCATENATE(Settings!P19," ",Settings!D19,"s"),CONCATENATE((Settings!P19/Settings!L19)," ",Settings!D19,"s")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A20" s="3"/>
       <c r="B20" s="4"/>
-      <c r="E20" s="9"/>
-      <c r="G20" s="9"/>
+      <c r="F20" s="9"/>
       <c r="H20" s="9"/>
       <c r="I20" s="9"/>
-      <c r="Q20" t="str">
-        <f>IF(D20&gt;0,IF(D20="Unit",CONCATENATE(Settings!P20," ",Settings!D20,"s"),CONCATENATE((Settings!P20/Settings!L20)," ",Settings!D20,"s")),"")</f>
+      <c r="J20" s="9"/>
+      <c r="R20" t="str">
+        <f>IF(E20&gt;0,IF(E20="Unit",CONCATENATE(Settings!Q20," ",Settings!E20,"s"),CONCATENATE((Settings!Q20/Settings!M20)," ",Settings!E20,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A21" s="3"/>
       <c r="B21" s="4"/>
-      <c r="E21" s="9"/>
-      <c r="G21" s="9"/>
+      <c r="F21" s="9"/>
       <c r="H21" s="9"/>
       <c r="I21" s="9"/>
-      <c r="Q21" t="str">
-        <f>IF(D21&gt;0,IF(D21="Unit",CONCATENATE(Settings!P21," ",Settings!D21,"s"),CONCATENATE((Settings!P21/Settings!L21)," ",Settings!D21,"s")),"")</f>
+      <c r="J21" s="9"/>
+      <c r="R21" t="str">
+        <f>IF(E21&gt;0,IF(E21="Unit",CONCATENATE(Settings!Q21," ",Settings!E21,"s"),CONCATENATE((Settings!Q21/Settings!M21)," ",Settings!E21,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="22" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A22" s="3"/>
       <c r="B22" s="4"/>
-      <c r="E22" s="9"/>
-      <c r="G22" s="9"/>
+      <c r="F22" s="9"/>
       <c r="H22" s="9"/>
       <c r="I22" s="9"/>
-      <c r="Q22" t="str">
-        <f>IF(D22&gt;0,IF(D22="Unit",CONCATENATE(Settings!P22," ",Settings!D22,"s"),CONCATENATE((Settings!P22/Settings!L22)," ",Settings!D22,"s")),"")</f>
+      <c r="J22" s="9"/>
+      <c r="R22" t="str">
+        <f>IF(E22&gt;0,IF(E22="Unit",CONCATENATE(Settings!Q22," ",Settings!E22,"s"),CONCATENATE((Settings!Q22/Settings!M22)," ",Settings!E22,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="23" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A23" s="3"/>
       <c r="B23" s="4"/>
-      <c r="E23" s="9"/>
-      <c r="G23" s="9"/>
+      <c r="F23" s="9"/>
       <c r="H23" s="9"/>
       <c r="I23" s="9"/>
-      <c r="Q23" t="str">
-        <f>IF(D23&gt;0,IF(D23="Unit",CONCATENATE(Settings!P23," ",Settings!D23,"s"),CONCATENATE((Settings!P23/Settings!L23)," ",Settings!D23,"s")),"")</f>
+      <c r="J23" s="9"/>
+      <c r="R23" t="str">
+        <f>IF(E23&gt;0,IF(E23="Unit",CONCATENATE(Settings!Q23," ",Settings!E23,"s"),CONCATENATE((Settings!Q23/Settings!M23)," ",Settings!E23,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="24" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A24" s="3"/>
       <c r="B24" s="4"/>
-      <c r="E24" s="9"/>
-      <c r="G24" s="9"/>
+      <c r="F24" s="9"/>
       <c r="H24" s="9"/>
       <c r="I24" s="9"/>
-      <c r="Q24" t="str">
-        <f>IF(D24&gt;0,IF(D24="Unit",CONCATENATE(Settings!P24," ",Settings!D24,"s"),CONCATENATE((Settings!P24/Settings!L24)," ",Settings!D24,"s")),"")</f>
+      <c r="J24" s="9"/>
+      <c r="R24" t="str">
+        <f>IF(E24&gt;0,IF(E24="Unit",CONCATENATE(Settings!Q24," ",Settings!E24,"s"),CONCATENATE((Settings!Q24/Settings!M24)," ",Settings!E24,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="25" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A25" s="3"/>
       <c r="B25" s="4"/>
-      <c r="E25" s="9"/>
-      <c r="G25" s="9"/>
+      <c r="F25" s="9"/>
       <c r="H25" s="9"/>
       <c r="I25" s="9"/>
-      <c r="Q25" t="str">
-        <f>IF(D25&gt;0,IF(D25="Unit",CONCATENATE(Settings!P25," ",Settings!D25,"s"),CONCATENATE((Settings!P25/Settings!L25)," ",Settings!D25,"s")),"")</f>
+      <c r="J25" s="9"/>
+      <c r="R25" t="str">
+        <f>IF(E25&gt;0,IF(E25="Unit",CONCATENATE(Settings!Q25," ",Settings!E25,"s"),CONCATENATE((Settings!Q25/Settings!M25)," ",Settings!E25,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="26" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A26" s="3"/>
       <c r="B26" s="4"/>
-      <c r="E26" s="9"/>
-      <c r="G26" s="9"/>
+      <c r="F26" s="9"/>
       <c r="H26" s="9"/>
       <c r="I26" s="9"/>
-      <c r="Q26" t="str">
-        <f>IF(D26&gt;0,IF(D26="Unit",CONCATENATE(Settings!P26," ",Settings!D26,"s"),CONCATENATE((Settings!P26/Settings!L26)," ",Settings!D26,"s")),"")</f>
+      <c r="J26" s="9"/>
+      <c r="R26" t="str">
+        <f>IF(E26&gt;0,IF(E26="Unit",CONCATENATE(Settings!Q26," ",Settings!E26,"s"),CONCATENATE((Settings!Q26/Settings!M26)," ",Settings!E26,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="27" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A27" s="3"/>
       <c r="B27" s="4"/>
-      <c r="E27" s="9"/>
-      <c r="G27" s="9"/>
+      <c r="F27" s="9"/>
       <c r="H27" s="9"/>
       <c r="I27" s="9"/>
-      <c r="Q27" t="str">
-        <f>IF(D27&gt;0,IF(D27="Unit",CONCATENATE(Settings!P27," ",Settings!D27,"s"),CONCATENATE((Settings!P27/Settings!L27)," ",Settings!D27,"s")),"")</f>
+      <c r="J27" s="9"/>
+      <c r="R27" t="str">
+        <f>IF(E27&gt;0,IF(E27="Unit",CONCATENATE(Settings!Q27," ",Settings!E27,"s"),CONCATENATE((Settings!Q27/Settings!M27)," ",Settings!E27,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="28" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A28" s="3"/>
       <c r="B28" s="4"/>
-      <c r="E28" s="9"/>
-      <c r="G28" s="9"/>
+      <c r="F28" s="9"/>
       <c r="H28" s="9"/>
       <c r="I28" s="9"/>
-      <c r="Q28" t="str">
-        <f>IF(D28&gt;0,IF(D28="Unit",CONCATENATE(Settings!P28," ",Settings!D28,"s"),CONCATENATE((Settings!P28/Settings!L28)," ",Settings!D28,"s")),"")</f>
+      <c r="J28" s="9"/>
+      <c r="R28" t="str">
+        <f>IF(E28&gt;0,IF(E28="Unit",CONCATENATE(Settings!Q28," ",Settings!E28,"s"),CONCATENATE((Settings!Q28/Settings!M28)," ",Settings!E28,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="29" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A29" s="3"/>
       <c r="B29" s="4"/>
-      <c r="E29" s="9"/>
-      <c r="G29" s="9"/>
+      <c r="F29" s="9"/>
       <c r="H29" s="9"/>
       <c r="I29" s="9"/>
-      <c r="Q29" t="str">
-        <f>IF(D29&gt;0,IF(D29="Unit",CONCATENATE(Settings!P29," ",Settings!D29,"s"),CONCATENATE((Settings!P29/Settings!L29)," ",Settings!D29,"s")),"")</f>
+      <c r="J29" s="9"/>
+      <c r="R29" t="str">
+        <f>IF(E29&gt;0,IF(E29="Unit",CONCATENATE(Settings!Q29," ",Settings!E29,"s"),CONCATENATE((Settings!Q29/Settings!M29)," ",Settings!E29,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="30" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A30" s="3"/>
       <c r="B30" s="4"/>
-      <c r="E30" s="9"/>
-      <c r="G30" s="9"/>
+      <c r="F30" s="9"/>
       <c r="H30" s="9"/>
       <c r="I30" s="9"/>
-      <c r="Q30" t="str">
-        <f>IF(D30&gt;0,IF(D30="Unit",CONCATENATE(Settings!P30," ",Settings!D30,"s"),CONCATENATE((Settings!P30/Settings!L30)," ",Settings!D30,"s")),"")</f>
+      <c r="J30" s="9"/>
+      <c r="R30" t="str">
+        <f>IF(E30&gt;0,IF(E30="Unit",CONCATENATE(Settings!Q30," ",Settings!E30,"s"),CONCATENATE((Settings!Q30/Settings!M30)," ",Settings!E30,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="31" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A31" s="3"/>
       <c r="B31" s="4"/>
-      <c r="E31" s="9"/>
-      <c r="G31" s="9"/>
+      <c r="F31" s="9"/>
       <c r="H31" s="9"/>
       <c r="I31" s="9"/>
-      <c r="Q31" t="str">
-        <f>IF(D31&gt;0,IF(D31="Unit",CONCATENATE(Settings!P31," ",Settings!D31,"s"),CONCATENATE((Settings!P31/Settings!L31)," ",Settings!D31,"s")),"")</f>
+      <c r="J31" s="9"/>
+      <c r="R31" t="str">
+        <f>IF(E31&gt;0,IF(E31="Unit",CONCATENATE(Settings!Q31," ",Settings!E31,"s"),CONCATENATE((Settings!Q31/Settings!M31)," ",Settings!E31,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="32" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A32" s="3"/>
       <c r="B32" s="4"/>
-      <c r="E32" s="9"/>
-      <c r="G32" s="9"/>
+      <c r="F32" s="9"/>
       <c r="H32" s="9"/>
       <c r="I32" s="9"/>
-      <c r="Q32" t="str">
-        <f>IF(D32&gt;0,IF(D32="Unit",CONCATENATE(Settings!P32," ",Settings!D32,"s"),CONCATENATE((Settings!P32/Settings!L32)," ",Settings!D32,"s")),"")</f>
+      <c r="J32" s="9"/>
+      <c r="R32" t="str">
+        <f>IF(E32&gt;0,IF(E32="Unit",CONCATENATE(Settings!Q32," ",Settings!E32,"s"),CONCATENATE((Settings!Q32/Settings!M32)," ",Settings!E32,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="33" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A33" s="3"/>
       <c r="B33" s="4"/>
-      <c r="E33" s="9"/>
-      <c r="G33" s="9"/>
+      <c r="F33" s="9"/>
       <c r="H33" s="9"/>
       <c r="I33" s="9"/>
-      <c r="Q33" t="str">
-        <f>IF(D33&gt;0,IF(D33="Unit",CONCATENATE(Settings!P33," ",Settings!D33,"s"),CONCATENATE((Settings!P33/Settings!L33)," ",Settings!D33,"s")),"")</f>
+      <c r="J33" s="9"/>
+      <c r="R33" t="str">
+        <f>IF(E33&gt;0,IF(E33="Unit",CONCATENATE(Settings!Q33," ",Settings!E33,"s"),CONCATENATE((Settings!Q33/Settings!M33)," ",Settings!E33,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="34" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A34" s="3"/>
       <c r="B34" s="4"/>
-      <c r="E34" s="9"/>
-      <c r="G34" s="9"/>
+      <c r="F34" s="9"/>
       <c r="H34" s="9"/>
       <c r="I34" s="9"/>
-      <c r="Q34" t="str">
-        <f>IF(D34&gt;0,IF(D34="Unit",CONCATENATE(Settings!P34," ",Settings!D34,"s"),CONCATENATE((Settings!P34/Settings!L34)," ",Settings!D34,"s")),"")</f>
+      <c r="J34" s="9"/>
+      <c r="R34" t="str">
+        <f>IF(E34&gt;0,IF(E34="Unit",CONCATENATE(Settings!Q34," ",Settings!E34,"s"),CONCATENATE((Settings!Q34/Settings!M34)," ",Settings!E34,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="35" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A35" s="3"/>
       <c r="B35" s="4"/>
-      <c r="E35" s="9"/>
-      <c r="G35" s="9"/>
+      <c r="F35" s="9"/>
       <c r="H35" s="9"/>
       <c r="I35" s="9"/>
-      <c r="Q35" t="str">
-        <f>IF(D35&gt;0,IF(D35="Unit",CONCATENATE(Settings!P35," ",Settings!D35,"s"),CONCATENATE((Settings!P35/Settings!L35)," ",Settings!D35,"s")),"")</f>
+      <c r="J35" s="9"/>
+      <c r="R35" t="str">
+        <f>IF(E35&gt;0,IF(E35="Unit",CONCATENATE(Settings!Q35," ",Settings!E35,"s"),CONCATENATE((Settings!Q35/Settings!M35)," ",Settings!E35,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="36" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A36" s="3"/>
       <c r="B36" s="4"/>
-      <c r="E36" s="9"/>
-      <c r="G36" s="9"/>
+      <c r="F36" s="9"/>
       <c r="H36" s="9"/>
       <c r="I36" s="9"/>
-      <c r="Q36" t="str">
-        <f>IF(D36&gt;0,IF(D36="Unit",CONCATENATE(Settings!P36," ",Settings!D36,"s"),CONCATENATE((Settings!P36/Settings!L36)," ",Settings!D36,"s")),"")</f>
+      <c r="J36" s="9"/>
+      <c r="R36" t="str">
+        <f>IF(E36&gt;0,IF(E36="Unit",CONCATENATE(Settings!Q36," ",Settings!E36,"s"),CONCATENATE((Settings!Q36/Settings!M36)," ",Settings!E36,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="37" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A37" s="3"/>
       <c r="B37" s="4"/>
-      <c r="E37" s="9"/>
-      <c r="G37" s="9"/>
+      <c r="F37" s="9"/>
       <c r="H37" s="9"/>
       <c r="I37" s="9"/>
-      <c r="Q37" t="str">
-        <f>IF(D37&gt;0,IF(D37="Unit",CONCATENATE(Settings!P37," ",Settings!D37,"s"),CONCATENATE((Settings!P37/Settings!L37)," ",Settings!D37,"s")),"")</f>
+      <c r="J37" s="9"/>
+      <c r="R37" t="str">
+        <f>IF(E37&gt;0,IF(E37="Unit",CONCATENATE(Settings!Q37," ",Settings!E37,"s"),CONCATENATE((Settings!Q37/Settings!M37)," ",Settings!E37,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="38" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A38" s="3"/>
       <c r="B38" s="4"/>
-      <c r="E38" s="9"/>
-      <c r="G38" s="9"/>
+      <c r="F38" s="9"/>
       <c r="H38" s="9"/>
       <c r="I38" s="9"/>
-      <c r="Q38" t="str">
-        <f>IF(D38&gt;0,IF(D38="Unit",CONCATENATE(Settings!P38," ",Settings!D38,"s"),CONCATENATE((Settings!P38/Settings!L38)," ",Settings!D38,"s")),"")</f>
+      <c r="J38" s="9"/>
+      <c r="R38" t="str">
+        <f>IF(E38&gt;0,IF(E38="Unit",CONCATENATE(Settings!Q38," ",Settings!E38,"s"),CONCATENATE((Settings!Q38/Settings!M38)," ",Settings!E38,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="39" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A39" s="3"/>
       <c r="B39" s="4"/>
-      <c r="E39" s="9"/>
-      <c r="G39" s="9"/>
+      <c r="F39" s="9"/>
       <c r="H39" s="9"/>
       <c r="I39" s="9"/>
-      <c r="Q39" t="str">
-        <f>IF(D39&gt;0,IF(D39="Unit",CONCATENATE(Settings!P39," ",Settings!D39,"s"),CONCATENATE((Settings!P39/Settings!L39)," ",Settings!D39,"s")),"")</f>
+      <c r="J39" s="9"/>
+      <c r="R39" t="str">
+        <f>IF(E39&gt;0,IF(E39="Unit",CONCATENATE(Settings!Q39," ",Settings!E39,"s"),CONCATENATE((Settings!Q39/Settings!M39)," ",Settings!E39,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="40" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A40" s="3"/>
       <c r="B40" s="4"/>
-      <c r="E40" s="9"/>
-      <c r="G40" s="9"/>
+      <c r="F40" s="9"/>
       <c r="H40" s="9"/>
       <c r="I40" s="9"/>
-      <c r="Q40" t="str">
-        <f>IF(D40&gt;0,IF(D40="Unit",CONCATENATE(Settings!P40," ",Settings!D40,"s"),CONCATENATE((Settings!P40/Settings!L40)," ",Settings!D40,"s")),"")</f>
+      <c r="J40" s="9"/>
+      <c r="R40" t="str">
+        <f>IF(E40&gt;0,IF(E40="Unit",CONCATENATE(Settings!Q40," ",Settings!E40,"s"),CONCATENATE((Settings!Q40/Settings!M40)," ",Settings!E40,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="41" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A41" s="3"/>
       <c r="B41" s="4"/>
-      <c r="E41" s="9"/>
-      <c r="G41" s="9"/>
+      <c r="F41" s="9"/>
       <c r="H41" s="9"/>
       <c r="I41" s="9"/>
-      <c r="Q41" t="str">
-        <f>IF(D41&gt;0,IF(D41="Unit",CONCATENATE(Settings!P41," ",Settings!D41,"s"),CONCATENATE((Settings!P41/Settings!L41)," ",Settings!D41,"s")),"")</f>
+      <c r="J41" s="9"/>
+      <c r="R41" t="str">
+        <f>IF(E41&gt;0,IF(E41="Unit",CONCATENATE(Settings!Q41," ",Settings!E41,"s"),CONCATENATE((Settings!Q41/Settings!M41)," ",Settings!E41,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="42" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A42" s="3"/>
       <c r="B42" s="4"/>
-      <c r="E42" s="9"/>
-      <c r="G42" s="9"/>
+      <c r="F42" s="9"/>
       <c r="H42" s="9"/>
       <c r="I42" s="9"/>
-      <c r="Q42" t="str">
-        <f>IF(D42&gt;0,IF(D42="Unit",CONCATENATE(Settings!P42," ",Settings!D42,"s"),CONCATENATE((Settings!P42/Settings!L42)," ",Settings!D42,"s")),"")</f>
+      <c r="J42" s="9"/>
+      <c r="R42" t="str">
+        <f>IF(E42&gt;0,IF(E42="Unit",CONCATENATE(Settings!Q42," ",Settings!E42,"s"),CONCATENATE((Settings!Q42/Settings!M42)," ",Settings!E42,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="43" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A43" s="3"/>
       <c r="B43" s="4"/>
-      <c r="E43" s="9"/>
-      <c r="G43" s="9"/>
+      <c r="F43" s="9"/>
       <c r="H43" s="9"/>
       <c r="I43" s="9"/>
-      <c r="Q43" t="str">
-        <f>IF(D43&gt;0,IF(D43="Unit",CONCATENATE(Settings!P43," ",Settings!D43,"s"),CONCATENATE((Settings!P43/Settings!L43)," ",Settings!D43,"s")),"")</f>
+      <c r="J43" s="9"/>
+      <c r="R43" t="str">
+        <f>IF(E43&gt;0,IF(E43="Unit",CONCATENATE(Settings!Q43," ",Settings!E43,"s"),CONCATENATE((Settings!Q43/Settings!M43)," ",Settings!E43,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="44" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A44" s="3"/>
       <c r="B44" s="4"/>
-      <c r="E44" s="9"/>
-      <c r="G44" s="9"/>
+      <c r="F44" s="9"/>
       <c r="H44" s="9"/>
       <c r="I44" s="9"/>
-      <c r="Q44" t="str">
-        <f>IF(D44&gt;0,IF(D44="Unit",CONCATENATE(Settings!P44," ",Settings!D44,"s"),CONCATENATE((Settings!P44/Settings!L44)," ",Settings!D44,"s")),"")</f>
+      <c r="J44" s="9"/>
+      <c r="R44" t="str">
+        <f>IF(E44&gt;0,IF(E44="Unit",CONCATENATE(Settings!Q44," ",Settings!E44,"s"),CONCATENATE((Settings!Q44/Settings!M44)," ",Settings!E44,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="45" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A45" s="3"/>
       <c r="B45" s="4"/>
-      <c r="E45" s="9"/>
-      <c r="G45" s="9"/>
+      <c r="F45" s="9"/>
       <c r="H45" s="9"/>
       <c r="I45" s="9"/>
-      <c r="Q45" t="str">
-        <f>IF(D45&gt;0,IF(D45="Unit",CONCATENATE(Settings!P45," ",Settings!D45,"s"),CONCATENATE((Settings!P45/Settings!L45)," ",Settings!D45,"s")),"")</f>
+      <c r="J45" s="9"/>
+      <c r="R45" t="str">
+        <f>IF(E45&gt;0,IF(E45="Unit",CONCATENATE(Settings!Q45," ",Settings!E45,"s"),CONCATENATE((Settings!Q45/Settings!M45)," ",Settings!E45,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="46" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A46" s="3"/>
       <c r="B46" s="4"/>
-      <c r="E46" s="9"/>
-      <c r="G46" s="9"/>
+      <c r="F46" s="9"/>
       <c r="H46" s="9"/>
       <c r="I46" s="9"/>
-      <c r="Q46" t="str">
-        <f>IF(D46&gt;0,IF(D46="Unit",CONCATENATE(Settings!P46," ",Settings!D46,"s"),CONCATENATE((Settings!P46/Settings!L46)," ",Settings!D46,"s")),"")</f>
+      <c r="J46" s="9"/>
+      <c r="R46" t="str">
+        <f>IF(E46&gt;0,IF(E46="Unit",CONCATENATE(Settings!Q46," ",Settings!E46,"s"),CONCATENATE((Settings!Q46/Settings!M46)," ",Settings!E46,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="47" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A47" s="3"/>
       <c r="B47" s="4"/>
-      <c r="E47" s="9"/>
-      <c r="G47" s="9"/>
+      <c r="F47" s="9"/>
       <c r="H47" s="9"/>
       <c r="I47" s="9"/>
-      <c r="Q47" t="str">
-        <f>IF(D47&gt;0,IF(D47="Unit",CONCATENATE(Settings!P47," ",Settings!D47,"s"),CONCATENATE((Settings!P47/Settings!L47)," ",Settings!D47,"s")),"")</f>
+      <c r="J47" s="9"/>
+      <c r="R47" t="str">
+        <f>IF(E47&gt;0,IF(E47="Unit",CONCATENATE(Settings!Q47," ",Settings!E47,"s"),CONCATENATE((Settings!Q47/Settings!M47)," ",Settings!E47,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="48" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A48" s="3"/>
       <c r="B48" s="4"/>
-      <c r="E48" s="9"/>
-      <c r="G48" s="9"/>
+      <c r="F48" s="9"/>
       <c r="H48" s="9"/>
       <c r="I48" s="9"/>
-      <c r="Q48" t="str">
-        <f>IF(D48&gt;0,IF(D48="Unit",CONCATENATE(Settings!P48," ",Settings!D48,"s"),CONCATENATE((Settings!P48/Settings!L48)," ",Settings!D48,"s")),"")</f>
+      <c r="J48" s="9"/>
+      <c r="R48" t="str">
+        <f>IF(E48&gt;0,IF(E48="Unit",CONCATENATE(Settings!Q48," ",Settings!E48,"s"),CONCATENATE((Settings!Q48/Settings!M48)," ",Settings!E48,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="49" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A49" s="3"/>
       <c r="B49" s="4"/>
-      <c r="E49" s="9"/>
-      <c r="G49" s="9"/>
+      <c r="F49" s="9"/>
       <c r="H49" s="9"/>
       <c r="I49" s="9"/>
-      <c r="Q49" t="str">
-        <f>IF(D49&gt;0,IF(D49="Unit",CONCATENATE(Settings!P49," ",Settings!D49,"s"),CONCATENATE((Settings!P49/Settings!L49)," ",Settings!D49,"s")),"")</f>
+      <c r="J49" s="9"/>
+      <c r="R49" t="str">
+        <f>IF(E49&gt;0,IF(E49="Unit",CONCATENATE(Settings!Q49," ",Settings!E49,"s"),CONCATENATE((Settings!Q49/Settings!M49)," ",Settings!E49,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="50" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A50" s="3"/>
       <c r="B50" s="4"/>
-      <c r="E50" s="9"/>
-      <c r="G50" s="9"/>
+      <c r="F50" s="9"/>
       <c r="H50" s="9"/>
       <c r="I50" s="9"/>
-      <c r="Q50" t="str">
-        <f>IF(D50&gt;0,IF(D50="Unit",CONCATENATE(Settings!P50," ",Settings!D50,"s"),CONCATENATE((Settings!P50/Settings!L50)," ",Settings!D50,"s")),"")</f>
+      <c r="J50" s="9"/>
+      <c r="R50" t="str">
+        <f>IF(E50&gt;0,IF(E50="Unit",CONCATENATE(Settings!Q50," ",Settings!E50,"s"),CONCATENATE((Settings!Q50/Settings!M50)," ",Settings!E50,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="51" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A51" s="3"/>
       <c r="B51" s="4"/>
-      <c r="E51" s="9"/>
-      <c r="G51" s="9"/>
+      <c r="F51" s="9"/>
       <c r="H51" s="9"/>
       <c r="I51" s="9"/>
-      <c r="Q51" t="str">
-        <f>IF(D51&gt;0,IF(D51="Unit",CONCATENATE(Settings!P51," ",Settings!D51,"s"),CONCATENATE((Settings!P51/Settings!L51)," ",Settings!D51,"s")),"")</f>
+      <c r="J51" s="9"/>
+      <c r="R51" t="str">
+        <f>IF(E51&gt;0,IF(E51="Unit",CONCATENATE(Settings!Q51," ",Settings!E51,"s"),CONCATENATE((Settings!Q51/Settings!M51)," ",Settings!E51,"s")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="52" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A52" s="5"/>
-      <c r="B52" s="6"/>
-      <c r="E52" s="9"/>
-      <c r="G52" s="9"/>
+    <row r="52" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A52" s="3"/>
+      <c r="B52" s="4"/>
+      <c r="F52" s="9"/>
       <c r="H52" s="9"/>
       <c r="I52" s="9"/>
-      <c r="Q52" t="str">
-        <f>IF(D52&gt;0,IF(D52="Unit",CONCATENATE(Settings!P52," ",Settings!D52,"s"),CONCATENATE((Settings!P52/Settings!L52)," ",Settings!D52,"s")),"")</f>
+      <c r="J52" s="9"/>
+      <c r="R52" t="str">
+        <f>IF(E52&gt;0,IF(E52="Unit",CONCATENATE(Settings!Q52," ",Settings!E52,"s"),CONCATENATE((Settings!Q52/Settings!M52)," ",Settings!E52,"s")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A53" s="5"/>
+      <c r="B53" s="6"/>
+      <c r="F53" s="9"/>
+      <c r="H53" s="9"/>
+      <c r="I53" s="9"/>
+      <c r="J53" s="9"/>
+      <c r="R53" t="str">
+        <f>IF(E53&gt;0,IF(E53="Unit",CONCATENATE(Settings!Q53," ",Settings!E53,"s"),CONCATENATE((Settings!Q53/Settings!M53)," ",Settings!E53,"s")),"")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Updated TH Quotation Template
</commit_message>
<xml_diff>
--- a/srv/xlsx-templates/TH - Quotation Template.xlsx
+++ b/srv/xlsx-templates/TH - Quotation Template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EHMHV\OneDrive\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EHMHV\Documents\WordQuotationDocuments\TH\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC81B2CC-B30A-42AE-9400-9AD510750D3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4CE1E7B0-2788-42EB-ADF7-DEE2724BEF50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="18975" windowHeight="9195" xr2:uid="{F5CC2154-27BB-4652-B61E-D913F0CC6809}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="18735" windowHeight="9240" xr2:uid="{F5CC2154-27BB-4652-B61E-D913F0CC6809}"/>
   </bookViews>
   <sheets>
     <sheet name="Quotation" sheetId="3" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="143">
   <si>
     <t>Offered Party</t>
   </si>
@@ -56,9 +56,6 @@
   </si>
   <si>
     <t>130/1 North Sathon Road, Silom, Bangrak, Bangkok 10500</t>
-  </si>
-  <si>
-    <t>Quotation Request Information</t>
   </si>
   <si>
     <t>FAST Request ID</t>
@@ -430,6 +427,45 @@
   </si>
   <si>
     <t>${table:offerProductValidation.CODE1}</t>
+  </si>
+  <si>
+    <t>Job Type</t>
+  </si>
+  <si>
+    <t>Tender Announcement Reference</t>
+  </si>
+  <si>
+    <t>Tender Item Number</t>
+  </si>
+  <si>
+    <t>Bank gaurantee - Start date</t>
+  </si>
+  <si>
+    <t>Bank gaurantee - End date</t>
+  </si>
+  <si>
+    <t>Bank gaurantee value (THB)</t>
+  </si>
+  <si>
+    <t>${offerValidation.TenderAnnouncementReference}</t>
+  </si>
+  <si>
+    <t>${offerValidation.ItemNumber}</t>
+  </si>
+  <si>
+    <t>${offerValidation.PeriodOfBankGauranteeStart}</t>
+  </si>
+  <si>
+    <t>${offerValidation.PeriodOfBankGauranteeEnd}</t>
+  </si>
+  <si>
+    <t>${offerValidation.BGValueBaht}</t>
+  </si>
+  <si>
+    <t>Offer Request Information</t>
+  </si>
+  <si>
+    <t>${offerValidation.CLASSIFICATION} ${offerValidation.PROCUREMENT_REASON}</t>
   </si>
 </sst>
 </file>
@@ -573,7 +609,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="15">
+  <borders count="20">
     <border>
       <left/>
       <right/>
@@ -745,12 +781,61 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="113">
+  <cellXfs count="123">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -914,6 +999,15 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -962,21 +1056,12 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -1010,18 +1095,6 @@
     <xf numFmtId="49" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -1045,6 +1118,48 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1578,8 +1693,8 @@
     <col min="4" max="4" width="33.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="52.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11.85546875" customWidth="1"/>
-    <col min="7" max="7" width="10.42578125" customWidth="1"/>
-    <col min="8" max="8" width="15.85546875" customWidth="1"/>
+    <col min="7" max="7" width="17" customWidth="1"/>
+    <col min="8" max="8" width="24.5703125" customWidth="1"/>
     <col min="9" max="9" width="14.7109375" customWidth="1"/>
     <col min="10" max="10" width="21.28515625" customWidth="1"/>
     <col min="11" max="11" width="14.85546875" customWidth="1"/>
@@ -1630,23 +1745,23 @@
       <c r="B4" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="69" t="s">
+      <c r="C4" s="72" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="70"/>
-      <c r="E4" s="70"/>
-      <c r="F4" s="70"/>
-      <c r="G4" s="71"/>
+      <c r="D4" s="73"/>
+      <c r="E4" s="73"/>
+      <c r="F4" s="73"/>
+      <c r="G4" s="74"/>
       <c r="H4" s="10"/>
       <c r="I4" s="26" t="s">
         <v>4</v>
       </c>
-      <c r="J4" s="77" t="s">
+      <c r="J4" s="80" t="s">
         <v>6</v>
       </c>
-      <c r="K4" s="78"/>
-      <c r="L4" s="78"/>
-      <c r="M4" s="79"/>
+      <c r="K4" s="81"/>
+      <c r="L4" s="81"/>
+      <c r="M4" s="82"/>
       <c r="N4" s="10"/>
     </row>
     <row r="5" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1695,52 +1810,52 @@
       <c r="N7" s="10"/>
     </row>
     <row r="8" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B8" s="72" t="s">
+      <c r="B8" s="75" t="s">
+        <v>141</v>
+      </c>
+      <c r="C8" s="76"/>
+      <c r="D8" s="76"/>
+      <c r="E8" s="76"/>
+      <c r="F8" s="76"/>
+      <c r="G8" s="76"/>
+      <c r="H8" s="76"/>
+      <c r="I8" s="76"/>
+      <c r="J8" s="76"/>
+      <c r="K8" s="76"/>
+      <c r="L8" s="76"/>
+      <c r="M8" s="76"/>
+      <c r="N8" s="77"/>
+    </row>
+    <row r="9" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B9" s="83" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="73"/>
-      <c r="D8" s="73"/>
-      <c r="E8" s="73"/>
-      <c r="F8" s="73"/>
-      <c r="G8" s="73"/>
-      <c r="H8" s="73"/>
-      <c r="I8" s="73"/>
-      <c r="J8" s="73"/>
-      <c r="K8" s="73"/>
-      <c r="L8" s="73"/>
-      <c r="M8" s="73"/>
-      <c r="N8" s="74"/>
-    </row>
-    <row r="9" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B9" s="80" t="s">
+      <c r="C9" s="84"/>
+      <c r="D9" s="94" t="s">
         <v>8</v>
-      </c>
-      <c r="C9" s="81"/>
-      <c r="D9" s="94" t="s">
-        <v>9</v>
       </c>
       <c r="E9" s="94"/>
       <c r="F9" s="40"/>
       <c r="G9" s="42" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H9" s="42"/>
       <c r="I9" s="90" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="J9" s="90"/>
       <c r="K9" s="91"/>
-      <c r="L9" s="75" t="s">
+      <c r="L9" s="78" t="s">
+        <v>11</v>
+      </c>
+      <c r="M9" s="79"/>
+      <c r="N9" s="43"/>
+    </row>
+    <row r="10" spans="2:14" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="85" t="s">
         <v>12</v>
       </c>
-      <c r="M9" s="76"/>
-      <c r="N9" s="43"/>
-    </row>
-    <row r="10" spans="2:14" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="82" t="s">
-        <v>13</v>
-      </c>
-      <c r="C10" s="83"/>
+      <c r="C10" s="86"/>
       <c r="D10" s="95" t="str">
         <f>Settings!A14</f>
         <v>${offerValidation.CUSTOMER_CODE}</v>
@@ -1748,89 +1863,90 @@
       <c r="E10" s="95"/>
       <c r="F10" s="40"/>
       <c r="G10" s="96" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H10" s="96"/>
       <c r="I10" s="92" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J10" s="92"/>
       <c r="K10" s="93"/>
       <c r="L10" s="48" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="M10" s="49"/>
       <c r="N10" s="38"/>
     </row>
     <row r="11" spans="2:14" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="82" t="s">
-        <v>17</v>
-      </c>
-      <c r="C11" s="83"/>
-      <c r="D11" s="69" t="str">
+      <c r="B11" s="85" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11" s="86"/>
+      <c r="D11" s="72" t="str">
         <f>Settings!A9</f>
         <v>${offerValidation.INSTITUTENAME}</v>
       </c>
-      <c r="E11" s="71"/>
+      <c r="E11" s="74"/>
       <c r="F11" s="40"/>
       <c r="G11" s="97" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H11" s="97"/>
       <c r="I11" s="92" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J11" s="92"/>
       <c r="K11" s="93"/>
       <c r="L11" s="48" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="M11" s="49"/>
       <c r="N11" s="38"/>
     </row>
     <row r="12" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B12" s="82" t="s">
+      <c r="B12" s="85" t="s">
+        <v>20</v>
+      </c>
+      <c r="C12" s="86"/>
+      <c r="D12" s="56" t="s">
         <v>21</v>
-      </c>
-      <c r="C12" s="83"/>
-      <c r="D12" s="56" t="s">
-        <v>22</v>
       </c>
       <c r="E12" s="58"/>
       <c r="F12" s="10"/>
-      <c r="G12" s="89" t="s">
+      <c r="G12" s="69" t="s">
+        <v>22</v>
+      </c>
+      <c r="H12" s="69"/>
+      <c r="I12" s="70" t="s">
         <v>23</v>
       </c>
-      <c r="H12" s="89"/>
-      <c r="I12" s="85" t="s">
-        <v>24</v>
-      </c>
-      <c r="J12" s="85"/>
-      <c r="K12" s="86"/>
+      <c r="J12" s="70"/>
+      <c r="K12" s="71"/>
       <c r="L12" s="48" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="M12" s="49"/>
       <c r="N12" s="38"/>
     </row>
     <row r="13" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B13" s="82" t="s">
+      <c r="B13" s="85" t="s">
+        <v>24</v>
+      </c>
+      <c r="C13" s="86"/>
+      <c r="D13" s="56" t="s">
         <v>25</v>
-      </c>
-      <c r="C13" s="83"/>
-      <c r="D13" s="56" t="s">
-        <v>26</v>
       </c>
       <c r="E13" s="58"/>
       <c r="F13" s="10"/>
-      <c r="G13" s="10"/>
-      <c r="H13" s="10"/>
-      <c r="I13" s="10"/>
-      <c r="J13" s="10"/>
-      <c r="K13" s="10"/>
-      <c r="L13" s="10"/>
-      <c r="M13" s="10"/>
-      <c r="N13" s="10"/>
+      <c r="G13" s="69" t="s">
+        <v>130</v>
+      </c>
+      <c r="H13" s="69"/>
+      <c r="I13" s="70" t="s">
+        <v>142</v>
+      </c>
+      <c r="J13" s="70"/>
+      <c r="K13" s="71"/>
     </row>
     <row r="14" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B14" s="10"/>
@@ -1843,64 +1959,61 @@
       <c r="I14" s="10"/>
       <c r="J14" s="10"/>
       <c r="K14" s="10"/>
-      <c r="L14" s="10"/>
-      <c r="M14" s="10"/>
-      <c r="N14" s="10"/>
     </row>
     <row r="15" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B15" s="87" t="s">
+      <c r="B15" s="88" t="s">
+        <v>26</v>
+      </c>
+      <c r="C15" s="88"/>
+      <c r="D15" s="88"/>
+      <c r="E15" s="88"/>
+      <c r="F15" s="88"/>
+      <c r="G15" s="88"/>
+      <c r="H15" s="88"/>
+      <c r="I15" s="88"/>
+      <c r="J15" s="88"/>
+      <c r="K15" s="88"/>
+      <c r="L15" s="88"/>
+      <c r="M15" s="88"/>
+      <c r="N15" s="88"/>
+    </row>
+    <row r="16" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B16" s="87" t="s">
         <v>27</v>
       </c>
-      <c r="C15" s="87"/>
-      <c r="D15" s="87"/>
-      <c r="E15" s="87"/>
-      <c r="F15" s="87"/>
-      <c r="G15" s="87"/>
-      <c r="H15" s="87"/>
-      <c r="I15" s="87"/>
-      <c r="J15" s="87"/>
-      <c r="K15" s="87"/>
-      <c r="L15" s="87"/>
-      <c r="M15" s="87"/>
-      <c r="N15" s="87"/>
-    </row>
-    <row r="16" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B16" s="84" t="s">
+      <c r="C16" s="68" t="s">
         <v>28</v>
       </c>
-      <c r="C16" s="68" t="s">
+      <c r="D16" s="68" t="s">
         <v>29</v>
       </c>
-      <c r="D16" s="68" t="s">
+      <c r="E16" s="68" t="s">
         <v>30</v>
       </c>
-      <c r="E16" s="68" t="s">
+      <c r="F16" s="68" t="s">
         <v>31</v>
       </c>
-      <c r="F16" s="68" t="s">
+      <c r="G16" s="68" t="s">
         <v>32</v>
       </c>
-      <c r="G16" s="68" t="s">
+      <c r="H16" s="50" t="s">
         <v>33</v>
       </c>
-      <c r="H16" s="50" t="s">
+      <c r="I16" s="68" t="s">
         <v>34</v>
       </c>
-      <c r="I16" s="68" t="s">
+      <c r="J16" s="68" t="s">
         <v>35</v>
-      </c>
-      <c r="J16" s="68" t="s">
-        <v>36</v>
       </c>
       <c r="K16" s="68"/>
       <c r="L16" s="68"/>
       <c r="M16" s="68" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="N16" s="68"/>
     </row>
     <row r="17" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B17" s="84"/>
+      <c r="B17" s="87"/>
       <c r="C17" s="68"/>
       <c r="D17" s="68"/>
       <c r="E17" s="68"/>
@@ -1915,7 +2028,7 @@
       <c r="N17" s="68"/>
     </row>
     <row r="18" spans="2:15" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="84"/>
+      <c r="B18" s="87"/>
       <c r="C18" s="68"/>
       <c r="D18" s="68"/>
       <c r="E18" s="68"/>
@@ -1924,56 +2037,56 @@
       <c r="H18" s="52"/>
       <c r="I18" s="68"/>
       <c r="J18" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="K18" s="89" t="s">
         <v>38</v>
       </c>
-      <c r="K18" s="88" t="s">
-        <v>39</v>
-      </c>
-      <c r="L18" s="88"/>
+      <c r="L18" s="89"/>
       <c r="M18" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="N18" s="11" t="s">
         <v>38</v>
-      </c>
-      <c r="N18" s="11" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="19" spans="2:15" ht="30" x14ac:dyDescent="0.25">
       <c r="B19" s="25" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C19" s="25" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D19" s="39" t="s">
+        <v>41</v>
+      </c>
+      <c r="E19" s="39" t="s">
         <v>42</v>
       </c>
-      <c r="E19" s="39" t="s">
+      <c r="F19" s="37" t="s">
         <v>43</v>
       </c>
-      <c r="F19" s="37" t="s">
+      <c r="G19" s="37" t="s">
         <v>44</v>
       </c>
-      <c r="G19" s="37" t="s">
+      <c r="H19" s="37" t="s">
         <v>45</v>
       </c>
-      <c r="H19" s="37" t="s">
+      <c r="I19" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="I19" s="37" t="s">
+      <c r="J19" s="37" t="s">
         <v>47</v>
       </c>
-      <c r="J19" s="37" t="s">
+      <c r="K19" s="59" t="s">
         <v>48</v>
-      </c>
-      <c r="K19" s="59" t="s">
-        <v>49</v>
       </c>
       <c r="L19" s="59"/>
       <c r="M19" s="41" t="s">
+        <v>49</v>
+      </c>
+      <c r="N19" s="41" t="s">
         <v>50</v>
-      </c>
-      <c r="N19" s="41" t="s">
-        <v>51</v>
       </c>
       <c r="O19" s="31"/>
     </row>
@@ -2003,14 +2116,14 @@
       <c r="I21" s="12"/>
       <c r="J21" s="15"/>
       <c r="K21" s="67" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="L21" s="67"/>
       <c r="M21" s="37" t="s">
+        <v>52</v>
+      </c>
+      <c r="N21" s="37" t="s">
         <v>53</v>
-      </c>
-      <c r="N21" s="37" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="22" spans="2:15" x14ac:dyDescent="0.25">
@@ -2030,7 +2143,7 @@
     </row>
     <row r="23" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B23" s="99" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C23" s="99"/>
       <c r="D23" s="99"/>
@@ -2045,37 +2158,37 @@
       <c r="M23" s="10"/>
     </row>
     <row r="24" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B24" s="84" t="s">
+      <c r="B24" s="87" t="s">
+        <v>27</v>
+      </c>
+      <c r="C24" s="68" t="s">
         <v>28</v>
       </c>
-      <c r="C24" s="68" t="s">
-        <v>29</v>
-      </c>
       <c r="D24" s="68" t="s">
+        <v>55</v>
+      </c>
+      <c r="E24" s="68" t="s">
         <v>56</v>
       </c>
-      <c r="E24" s="68" t="s">
+      <c r="F24" s="68" t="s">
         <v>57</v>
       </c>
-      <c r="F24" s="68" t="s">
+      <c r="G24" s="68" t="s">
         <v>58</v>
-      </c>
-      <c r="G24" s="68" t="s">
-        <v>59</v>
       </c>
       <c r="H24" s="68"/>
       <c r="I24" s="68"/>
       <c r="J24" s="68" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K24" s="68"/>
       <c r="L24" s="68" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="M24" s="10"/>
     </row>
     <row r="25" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B25" s="84"/>
+      <c r="B25" s="87"/>
       <c r="C25" s="68"/>
       <c r="D25" s="68"/>
       <c r="E25" s="68"/>
@@ -2090,29 +2203,29 @@
     </row>
     <row r="26" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C26" s="37" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D26" s="44"/>
       <c r="E26" s="38" t="s">
+        <v>61</v>
+      </c>
+      <c r="F26" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="F26" s="16" t="s">
+      <c r="G26" s="64" t="s">
         <v>63</v>
-      </c>
-      <c r="G26" s="64" t="s">
-        <v>64</v>
       </c>
       <c r="H26" s="64"/>
       <c r="I26" s="64"/>
       <c r="J26" s="64" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="K26" s="64"/>
       <c r="L26" s="16" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="M26" s="10"/>
     </row>
@@ -2161,18 +2274,18 @@
     </row>
     <row r="30" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="98" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C30" s="98"/>
       <c r="D30" s="98"/>
       <c r="E30" s="98"/>
       <c r="F30" s="18"/>
       <c r="G30" s="65" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H30" s="66"/>
       <c r="I30" s="27" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="J30" s="27"/>
       <c r="K30" s="27"/>
@@ -2182,16 +2295,16 @@
     </row>
     <row r="31" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B31" s="19" t="s">
+        <v>69</v>
+      </c>
+      <c r="C31" s="20"/>
+      <c r="D31" s="103"/>
+      <c r="E31" s="103"/>
+      <c r="F31" s="10"/>
+      <c r="G31" s="104" t="s">
         <v>70</v>
       </c>
-      <c r="C31" s="20"/>
-      <c r="D31" s="107"/>
-      <c r="E31" s="107"/>
-      <c r="F31" s="10"/>
-      <c r="G31" s="108" t="s">
-        <v>71</v>
-      </c>
-      <c r="H31" s="109"/>
+      <c r="H31" s="105"/>
       <c r="I31" s="56"/>
       <c r="J31" s="57"/>
       <c r="K31" s="57"/>
@@ -2201,16 +2314,16 @@
     </row>
     <row r="32" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B32" s="19" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C32" s="20"/>
       <c r="D32" s="64"/>
       <c r="E32" s="64"/>
       <c r="F32" s="10"/>
-      <c r="G32" s="108" t="s">
-        <v>73</v>
-      </c>
-      <c r="H32" s="109"/>
+      <c r="G32" s="104" t="s">
+        <v>72</v>
+      </c>
+      <c r="H32" s="105"/>
       <c r="I32" s="56"/>
       <c r="J32" s="57"/>
       <c r="K32" s="57"/>
@@ -2220,18 +2333,18 @@
     </row>
     <row r="33" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B33" s="19" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C33" s="20"/>
       <c r="D33" s="16"/>
       <c r="E33" s="21" t="s">
+        <v>74</v>
+      </c>
+      <c r="F33" s="10"/>
+      <c r="G33" s="104" t="s">
         <v>75</v>
       </c>
-      <c r="F33" s="10"/>
-      <c r="G33" s="108" t="s">
-        <v>76</v>
-      </c>
-      <c r="H33" s="109"/>
+      <c r="H33" s="105"/>
       <c r="I33" s="56"/>
       <c r="J33" s="57"/>
       <c r="K33" s="57"/>
@@ -2241,18 +2354,18 @@
     </row>
     <row r="34" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B34" s="22" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C34" s="23"/>
       <c r="D34" s="16"/>
       <c r="E34" s="21" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F34" s="10"/>
-      <c r="G34" s="105" t="s">
-        <v>78</v>
-      </c>
-      <c r="H34" s="106"/>
+      <c r="G34" s="101" t="s">
+        <v>77</v>
+      </c>
+      <c r="H34" s="102"/>
       <c r="I34" s="53"/>
       <c r="J34" s="54"/>
       <c r="K34" s="54"/>
@@ -2273,71 +2386,91 @@
       <c r="M35" s="10"/>
       <c r="N35" s="10"/>
     </row>
-    <row r="36" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B36" s="102" t="s">
-        <v>79</v>
-      </c>
-      <c r="C36" s="103"/>
-      <c r="D36" s="103"/>
-      <c r="E36" s="103"/>
-      <c r="F36" s="104"/>
-      <c r="G36" s="29"/>
-      <c r="H36" s="29"/>
+    <row r="36" spans="2:14" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B36" s="109" t="s">
+        <v>78</v>
+      </c>
+      <c r="C36" s="110"/>
+      <c r="D36" s="110"/>
+      <c r="E36" s="111"/>
+      <c r="F36" s="29"/>
+      <c r="G36" s="121" t="s">
+        <v>131</v>
+      </c>
+      <c r="H36" s="122" t="s">
+        <v>136</v>
+      </c>
       <c r="I36" s="29"/>
       <c r="J36" s="29"/>
     </row>
     <row r="37" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B37" s="101" t="s">
-        <v>80</v>
-      </c>
-      <c r="C37" s="101"/>
-      <c r="D37" s="101"/>
-      <c r="E37" s="101"/>
-      <c r="F37" s="101"/>
-      <c r="G37" s="29"/>
-      <c r="H37" s="29"/>
+      <c r="B37" s="112" t="s">
+        <v>79</v>
+      </c>
+      <c r="C37" s="113"/>
+      <c r="D37" s="113"/>
+      <c r="E37" s="114"/>
+      <c r="F37" s="29"/>
+      <c r="G37" s="121" t="s">
+        <v>132</v>
+      </c>
+      <c r="H37" s="122" t="s">
+        <v>137</v>
+      </c>
       <c r="I37" s="29"/>
       <c r="J37" s="29"/>
     </row>
-    <row r="38" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B38" s="101"/>
-      <c r="C38" s="101"/>
-      <c r="D38" s="101"/>
-      <c r="E38" s="101"/>
-      <c r="F38" s="101"/>
-      <c r="G38" s="29"/>
-      <c r="H38" s="29"/>
+    <row r="38" spans="2:14" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B38" s="115"/>
+      <c r="C38" s="116"/>
+      <c r="D38" s="116"/>
+      <c r="E38" s="117"/>
+      <c r="F38" s="29"/>
+      <c r="G38" s="121" t="s">
+        <v>133</v>
+      </c>
+      <c r="H38" s="122" t="s">
+        <v>138</v>
+      </c>
       <c r="I38" s="29"/>
       <c r="J38" s="29"/>
     </row>
-    <row r="39" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B39" s="101"/>
-      <c r="C39" s="101"/>
-      <c r="D39" s="101"/>
-      <c r="E39" s="101"/>
-      <c r="F39" s="101"/>
-      <c r="G39" s="29"/>
-      <c r="H39" s="29"/>
+    <row r="39" spans="2:14" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B39" s="115"/>
+      <c r="C39" s="116"/>
+      <c r="D39" s="116"/>
+      <c r="E39" s="117"/>
+      <c r="F39" s="29"/>
+      <c r="G39" s="121" t="s">
+        <v>134</v>
+      </c>
+      <c r="H39" s="122" t="s">
+        <v>139</v>
+      </c>
       <c r="I39" s="29"/>
       <c r="J39" s="29"/>
     </row>
-    <row r="40" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B40" s="101"/>
-      <c r="C40" s="101"/>
-      <c r="D40" s="101"/>
-      <c r="E40" s="101"/>
-      <c r="F40" s="101"/>
-      <c r="G40" s="29"/>
-      <c r="H40" s="29"/>
+    <row r="40" spans="2:14" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B40" s="115"/>
+      <c r="C40" s="116"/>
+      <c r="D40" s="116"/>
+      <c r="E40" s="117"/>
+      <c r="F40" s="29"/>
+      <c r="G40" s="121" t="s">
+        <v>135</v>
+      </c>
+      <c r="H40" s="122" t="s">
+        <v>140</v>
+      </c>
       <c r="I40" s="29"/>
       <c r="J40" s="29"/>
     </row>
     <row r="41" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B41" s="101"/>
-      <c r="C41" s="101"/>
-      <c r="D41" s="101"/>
-      <c r="E41" s="101"/>
-      <c r="F41" s="101"/>
+      <c r="B41" s="118"/>
+      <c r="C41" s="119"/>
+      <c r="D41" s="119"/>
+      <c r="E41" s="120"/>
+      <c r="F41" s="29"/>
       <c r="G41" s="29"/>
       <c r="H41" s="29"/>
       <c r="I41" s="29"/>
@@ -2441,13 +2574,12 @@
       <c r="J53" s="45"/>
     </row>
   </sheetData>
-  <mergeCells count="70">
-    <mergeCell ref="B37:F41"/>
+  <mergeCells count="71">
+    <mergeCell ref="B37:E41"/>
     <mergeCell ref="I33:L33"/>
     <mergeCell ref="G16:G18"/>
     <mergeCell ref="I16:I18"/>
     <mergeCell ref="J16:L17"/>
-    <mergeCell ref="B36:F36"/>
     <mergeCell ref="G34:H34"/>
     <mergeCell ref="D31:E31"/>
     <mergeCell ref="D32:E32"/>
@@ -2512,6 +2644,8 @@
     <mergeCell ref="K21:L21"/>
     <mergeCell ref="L24:L25"/>
     <mergeCell ref="G24:I25"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="I13:K13"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D27:D28 D26" xr:uid="{B316A799-CF60-4C99-A88E-2204076E38E6}">
@@ -2564,88 +2698,88 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>81</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>82</v>
       </c>
       <c r="C1" s="33"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B2" t="s">
         <v>83</v>
       </c>
-      <c r="B2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C2" s="110"/>
+      <c r="C2" s="106"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B3" t="s">
         <v>85</v>
       </c>
-      <c r="B3" t="s">
-        <v>86</v>
-      </c>
-      <c r="C3" s="111"/>
+      <c r="C3" s="107"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B4" t="s">
-        <v>87</v>
-      </c>
-      <c r="C4" s="111"/>
+        <v>86</v>
+      </c>
+      <c r="C4" s="107"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B5" t="s">
-        <v>18</v>
-      </c>
-      <c r="C5" s="111"/>
+        <v>17</v>
+      </c>
+      <c r="C5" s="107"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C6" s="112"/>
+        <v>20</v>
+      </c>
+      <c r="C6" s="108"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B8" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>87</v>
+      </c>
+      <c r="B9" t="s">
         <v>88</v>
-      </c>
-      <c r="B9" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>89</v>
+      </c>
+      <c r="B10" t="s">
         <v>90</v>
-      </c>
-      <c r="B10" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -2674,18 +2808,18 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>92</v>
+      </c>
+      <c r="B15" t="s">
         <v>93</v>
-      </c>
-      <c r="B15" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="17" spans="1:27" x14ac:dyDescent="0.25">
@@ -2694,174 +2828,174 @@
     </row>
     <row r="18" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="19" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="B19" s="8" t="s">
         <v>96</v>
       </c>
-      <c r="B19" s="8" t="s">
+      <c r="C19" s="34" t="s">
         <v>97</v>
       </c>
-      <c r="C19" s="34" t="s">
+      <c r="D19" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="D19" s="2" t="s">
+      <c r="E19" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="E19" s="2" t="s">
+      <c r="F19" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="F19" s="2" t="s">
+      <c r="G19" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="G19" s="2" t="s">
+      <c r="H19" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="H19" s="2" t="s">
+      <c r="I19" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="I19" s="2" t="s">
+      <c r="J19" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="J19" s="2" t="s">
+      <c r="K19" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="K19" s="2" t="s">
+      <c r="L19" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="L19" s="2" t="s">
+      <c r="M19" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="N19" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="M19" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="N19" s="2" t="s">
+      <c r="O19" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="O19" s="2" t="s">
+      <c r="P19" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="P19" s="2" t="s">
+      <c r="Q19" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="Q19" s="2" t="s">
+      <c r="R19" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="R19" s="2" t="s">
+      <c r="S19" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="S19" s="2" t="s">
+      <c r="T19" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="T19" s="2" t="s">
+      <c r="U19" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="U19" s="2" t="s">
+      <c r="V19" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="V19" s="2" t="s">
+      <c r="W19" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="W19" s="2" t="s">
+      <c r="X19" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="Y19" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="X19" s="2" t="s">
+      <c r="Z19" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="Y19" s="2" t="s">
+      <c r="AA19" s="2" t="s">
         <v>118</v>
-      </c>
-      <c r="Z19" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="AA19" s="2" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="20" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B20" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="C20" s="25" t="s">
+        <v>42</v>
+      </c>
+      <c r="D20" t="s">
+        <v>43</v>
+      </c>
+      <c r="E20" t="s">
+        <v>44</v>
+      </c>
+      <c r="F20" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="G20" t="s">
         <v>120</v>
       </c>
-      <c r="C20" s="25" t="s">
-        <v>43</v>
-      </c>
-      <c r="D20" t="s">
-        <v>44</v>
-      </c>
-      <c r="E20" t="s">
+      <c r="H20" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="I20" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="J20" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="K20" t="s">
+        <v>121</v>
+      </c>
+      <c r="L20" t="s">
+        <v>39</v>
+      </c>
+      <c r="M20" t="s">
         <v>45</v>
       </c>
-      <c r="F20" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="G20" t="s">
-        <v>121</v>
-      </c>
-      <c r="H20" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="I20" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="J20" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="K20" t="s">
+      <c r="N20" t="s">
         <v>122</v>
       </c>
-      <c r="L20" t="s">
-        <v>40</v>
-      </c>
-      <c r="M20" t="s">
-        <v>46</v>
-      </c>
-      <c r="N20" t="s">
+      <c r="O20" t="s">
+        <v>65</v>
+      </c>
+      <c r="P20" t="s">
         <v>123</v>
       </c>
-      <c r="O20" t="s">
-        <v>66</v>
-      </c>
-      <c r="P20" t="s">
+      <c r="Q20" t="s">
         <v>124</v>
-      </c>
-      <c r="Q20" t="s">
-        <v>125</v>
       </c>
       <c r="R20" t="e">
         <f>IF(E20&gt;0,IF(E20="Unit",CONCATENATE(Settings!Q20," ",Settings!E20,"s"),CONCATENATE((Settings!Q20/Settings!M20)," ",Settings!E20,"s")),"")</f>
         <v>#VALUE!</v>
       </c>
       <c r="S20" s="35" t="s">
+        <v>125</v>
+      </c>
+      <c r="T20" s="35" t="s">
         <v>126</v>
       </c>
-      <c r="T20" s="35" t="s">
+      <c r="U20" s="35" t="s">
         <v>127</v>
       </c>
-      <c r="U20" s="35" t="s">
+      <c r="V20" t="s">
+        <v>52</v>
+      </c>
+      <c r="W20" t="s">
         <v>128</v>
       </c>
-      <c r="V20" t="s">
+      <c r="X20" t="s">
+        <v>62</v>
+      </c>
+      <c r="Y20" t="s">
+        <v>61</v>
+      </c>
+      <c r="Z20" t="s">
+        <v>63</v>
+      </c>
+      <c r="AA20" t="s">
         <v>53</v>
-      </c>
-      <c r="W20" t="s">
-        <v>129</v>
-      </c>
-      <c r="X20" t="s">
-        <v>63</v>
-      </c>
-      <c r="Y20" t="s">
-        <v>62</v>
-      </c>
-      <c r="Z20" t="s">
-        <v>64</v>
-      </c>
-      <c r="AA20" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="21" spans="1:27" x14ac:dyDescent="0.25">
@@ -3291,15 +3425,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010075F372E8CCA016418A193AD921508903" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="f5e922417d740f1a527805650dc2dfa9">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="399317f3-0083-4d0b-9572-12af99626311" xmlns:ns3="1444eecc-14bb-4066-abe6-ce6de21d9439" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="078d79524add6eac9b94134ca637184e" ns2:_="" ns3:_="">
     <xsd:import namespace="399317f3-0083-4d0b-9572-12af99626311"/>
@@ -3496,7 +3621,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <SharedWithUsers xmlns="1444eecc-14bb-4066-abe6-ce6de21d9439">
@@ -3510,15 +3635,16 @@
 </p:properties>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A00E6A9-20DD-4842-9306-307EB080AF2E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8CF88A1C-AA0D-4F8F-A0FD-6F3FAFCA9DC0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3537,7 +3663,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7EBE950A-5812-419E-B174-6A5D9B8E0414}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -3545,4 +3671,12 @@
     <ds:schemaRef ds:uri="1444eecc-14bb-4066-abe6-ce6de21d9439"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A00E6A9-20DD-4842-9306-307EB080AF2E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Changes in tender application fields
</commit_message>
<xml_diff>
--- a/srv/xlsx-templates/TH - Quotation Template.xlsx
+++ b/srv/xlsx-templates/TH - Quotation Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24931"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EHQUT\Desktop\WordTemplate\Spain LatestChange-08082023\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EHMHV\Documents\WordQuotationDocuments\TH\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B523AEF-0582-486B-B8A0-975D0F558720}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4CE1E7B0-2788-42EB-ADF7-DEE2724BEF50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{F5CC2154-27BB-4652-B61E-D913F0CC6809}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="18735" windowHeight="9240" xr2:uid="{F5CC2154-27BB-4652-B61E-D913F0CC6809}"/>
   </bookViews>
   <sheets>
     <sheet name="Quotation" sheetId="3" r:id="rId1"/>
@@ -28,8 +28,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -37,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="143">
   <si>
     <t>Offered Party</t>
   </si>
@@ -58,9 +56,6 @@
   </si>
   <si>
     <t>130/1 North Sathon Road, Silom, Bangrak, Bangkok 10500</t>
-  </si>
-  <si>
-    <t>Quotation Request Information</t>
   </si>
   <si>
     <t>FAST Request ID</t>
@@ -432,6 +427,45 @@
   </si>
   <si>
     <t>${table:offerProductValidation.CODE1}</t>
+  </si>
+  <si>
+    <t>Job Type</t>
+  </si>
+  <si>
+    <t>Tender Announcement Reference</t>
+  </si>
+  <si>
+    <t>Tender Item Number</t>
+  </si>
+  <si>
+    <t>Bank gaurantee - Start date</t>
+  </si>
+  <si>
+    <t>Bank gaurantee - End date</t>
+  </si>
+  <si>
+    <t>Bank gaurantee value (THB)</t>
+  </si>
+  <si>
+    <t>${offerValidation.TenderAnnouncementReference}</t>
+  </si>
+  <si>
+    <t>${offerValidation.ItemNumber}</t>
+  </si>
+  <si>
+    <t>${offerValidation.PeriodOfBankGauranteeStart}</t>
+  </si>
+  <si>
+    <t>${offerValidation.PeriodOfBankGauranteeEnd}</t>
+  </si>
+  <si>
+    <t>${offerValidation.BGValueBaht}</t>
+  </si>
+  <si>
+    <t>Offer Request Information</t>
+  </si>
+  <si>
+    <t>${offerValidation.CLASSIFICATION} ${offerValidation.PROCUREMENT_REASON}</t>
   </si>
 </sst>
 </file>
@@ -575,7 +609,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="15">
+  <borders count="20">
     <border>
       <left/>
       <right/>
@@ -747,12 +781,61 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="113">
+  <cellXfs count="123">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -916,6 +999,15 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -964,21 +1056,12 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -1012,18 +1095,6 @@
     <xf numFmtId="49" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -1047,6 +1118,48 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1580,8 +1693,8 @@
     <col min="4" max="4" width="33.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="52.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11.85546875" customWidth="1"/>
-    <col min="7" max="7" width="10.42578125" customWidth="1"/>
-    <col min="8" max="8" width="15.85546875" customWidth="1"/>
+    <col min="7" max="7" width="17" customWidth="1"/>
+    <col min="8" max="8" width="24.5703125" customWidth="1"/>
     <col min="9" max="9" width="14.7109375" customWidth="1"/>
     <col min="10" max="10" width="21.28515625" customWidth="1"/>
     <col min="11" max="11" width="14.85546875" customWidth="1"/>
@@ -1632,23 +1745,23 @@
       <c r="B4" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="69" t="s">
+      <c r="C4" s="72" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="70"/>
-      <c r="E4" s="70"/>
-      <c r="F4" s="70"/>
-      <c r="G4" s="71"/>
+      <c r="D4" s="73"/>
+      <c r="E4" s="73"/>
+      <c r="F4" s="73"/>
+      <c r="G4" s="74"/>
       <c r="H4" s="10"/>
       <c r="I4" s="26" t="s">
         <v>4</v>
       </c>
-      <c r="J4" s="77" t="s">
+      <c r="J4" s="80" t="s">
         <v>6</v>
       </c>
-      <c r="K4" s="78"/>
-      <c r="L4" s="78"/>
-      <c r="M4" s="79"/>
+      <c r="K4" s="81"/>
+      <c r="L4" s="81"/>
+      <c r="M4" s="82"/>
       <c r="N4" s="10"/>
     </row>
     <row r="5" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1697,52 +1810,52 @@
       <c r="N7" s="10"/>
     </row>
     <row r="8" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B8" s="72" t="s">
+      <c r="B8" s="75" t="s">
+        <v>141</v>
+      </c>
+      <c r="C8" s="76"/>
+      <c r="D8" s="76"/>
+      <c r="E8" s="76"/>
+      <c r="F8" s="76"/>
+      <c r="G8" s="76"/>
+      <c r="H8" s="76"/>
+      <c r="I8" s="76"/>
+      <c r="J8" s="76"/>
+      <c r="K8" s="76"/>
+      <c r="L8" s="76"/>
+      <c r="M8" s="76"/>
+      <c r="N8" s="77"/>
+    </row>
+    <row r="9" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B9" s="83" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="73"/>
-      <c r="D8" s="73"/>
-      <c r="E8" s="73"/>
-      <c r="F8" s="73"/>
-      <c r="G8" s="73"/>
-      <c r="H8" s="73"/>
-      <c r="I8" s="73"/>
-      <c r="J8" s="73"/>
-      <c r="K8" s="73"/>
-      <c r="L8" s="73"/>
-      <c r="M8" s="73"/>
-      <c r="N8" s="74"/>
-    </row>
-    <row r="9" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B9" s="80" t="s">
+      <c r="C9" s="84"/>
+      <c r="D9" s="94" t="s">
         <v>8</v>
-      </c>
-      <c r="C9" s="81"/>
-      <c r="D9" s="94" t="s">
-        <v>9</v>
       </c>
       <c r="E9" s="94"/>
       <c r="F9" s="40"/>
       <c r="G9" s="42" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H9" s="42"/>
       <c r="I9" s="90" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="J9" s="90"/>
       <c r="K9" s="91"/>
-      <c r="L9" s="75" t="s">
+      <c r="L9" s="78" t="s">
+        <v>11</v>
+      </c>
+      <c r="M9" s="79"/>
+      <c r="N9" s="43"/>
+    </row>
+    <row r="10" spans="2:14" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="85" t="s">
         <v>12</v>
       </c>
-      <c r="M9" s="76"/>
-      <c r="N9" s="43"/>
-    </row>
-    <row r="10" spans="2:14" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="82" t="s">
-        <v>13</v>
-      </c>
-      <c r="C10" s="83"/>
+      <c r="C10" s="86"/>
       <c r="D10" s="95" t="str">
         <f>Settings!A14</f>
         <v>${offerValidation.CUSTOMER_CODE}</v>
@@ -1750,89 +1863,90 @@
       <c r="E10" s="95"/>
       <c r="F10" s="40"/>
       <c r="G10" s="96" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H10" s="96"/>
       <c r="I10" s="92" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J10" s="92"/>
       <c r="K10" s="93"/>
       <c r="L10" s="48" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="M10" s="49"/>
       <c r="N10" s="38"/>
     </row>
     <row r="11" spans="2:14" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="82" t="s">
-        <v>17</v>
-      </c>
-      <c r="C11" s="83"/>
-      <c r="D11" s="69" t="str">
+      <c r="B11" s="85" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11" s="86"/>
+      <c r="D11" s="72" t="str">
         <f>Settings!A9</f>
         <v>${offerValidation.INSTITUTENAME}</v>
       </c>
-      <c r="E11" s="71"/>
+      <c r="E11" s="74"/>
       <c r="F11" s="40"/>
       <c r="G11" s="97" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H11" s="97"/>
       <c r="I11" s="92" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J11" s="92"/>
       <c r="K11" s="93"/>
       <c r="L11" s="48" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="M11" s="49"/>
       <c r="N11" s="38"/>
     </row>
     <row r="12" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B12" s="82" t="s">
+      <c r="B12" s="85" t="s">
+        <v>20</v>
+      </c>
+      <c r="C12" s="86"/>
+      <c r="D12" s="56" t="s">
         <v>21</v>
-      </c>
-      <c r="C12" s="83"/>
-      <c r="D12" s="56" t="s">
-        <v>22</v>
       </c>
       <c r="E12" s="58"/>
       <c r="F12" s="10"/>
-      <c r="G12" s="89" t="s">
+      <c r="G12" s="69" t="s">
+        <v>22</v>
+      </c>
+      <c r="H12" s="69"/>
+      <c r="I12" s="70" t="s">
         <v>23</v>
       </c>
-      <c r="H12" s="89"/>
-      <c r="I12" s="85" t="s">
-        <v>24</v>
-      </c>
-      <c r="J12" s="85"/>
-      <c r="K12" s="86"/>
+      <c r="J12" s="70"/>
+      <c r="K12" s="71"/>
       <c r="L12" s="48" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="M12" s="49"/>
       <c r="N12" s="38"/>
     </row>
     <row r="13" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B13" s="82" t="s">
+      <c r="B13" s="85" t="s">
+        <v>24</v>
+      </c>
+      <c r="C13" s="86"/>
+      <c r="D13" s="56" t="s">
         <v>25</v>
-      </c>
-      <c r="C13" s="83"/>
-      <c r="D13" s="56" t="s">
-        <v>26</v>
       </c>
       <c r="E13" s="58"/>
       <c r="F13" s="10"/>
-      <c r="G13" s="10"/>
-      <c r="H13" s="10"/>
-      <c r="I13" s="10"/>
-      <c r="J13" s="10"/>
-      <c r="K13" s="10"/>
-      <c r="L13" s="10"/>
-      <c r="M13" s="10"/>
-      <c r="N13" s="10"/>
+      <c r="G13" s="69" t="s">
+        <v>130</v>
+      </c>
+      <c r="H13" s="69"/>
+      <c r="I13" s="70" t="s">
+        <v>142</v>
+      </c>
+      <c r="J13" s="70"/>
+      <c r="K13" s="71"/>
     </row>
     <row r="14" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B14" s="10"/>
@@ -1845,64 +1959,61 @@
       <c r="I14" s="10"/>
       <c r="J14" s="10"/>
       <c r="K14" s="10"/>
-      <c r="L14" s="10"/>
-      <c r="M14" s="10"/>
-      <c r="N14" s="10"/>
     </row>
     <row r="15" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B15" s="87" t="s">
+      <c r="B15" s="88" t="s">
+        <v>26</v>
+      </c>
+      <c r="C15" s="88"/>
+      <c r="D15" s="88"/>
+      <c r="E15" s="88"/>
+      <c r="F15" s="88"/>
+      <c r="G15" s="88"/>
+      <c r="H15" s="88"/>
+      <c r="I15" s="88"/>
+      <c r="J15" s="88"/>
+      <c r="K15" s="88"/>
+      <c r="L15" s="88"/>
+      <c r="M15" s="88"/>
+      <c r="N15" s="88"/>
+    </row>
+    <row r="16" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B16" s="87" t="s">
         <v>27</v>
       </c>
-      <c r="C15" s="87"/>
-      <c r="D15" s="87"/>
-      <c r="E15" s="87"/>
-      <c r="F15" s="87"/>
-      <c r="G15" s="87"/>
-      <c r="H15" s="87"/>
-      <c r="I15" s="87"/>
-      <c r="J15" s="87"/>
-      <c r="K15" s="87"/>
-      <c r="L15" s="87"/>
-      <c r="M15" s="87"/>
-      <c r="N15" s="87"/>
-    </row>
-    <row r="16" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B16" s="84" t="s">
+      <c r="C16" s="68" t="s">
         <v>28</v>
       </c>
-      <c r="C16" s="68" t="s">
+      <c r="D16" s="68" t="s">
         <v>29</v>
       </c>
-      <c r="D16" s="68" t="s">
+      <c r="E16" s="68" t="s">
         <v>30</v>
       </c>
-      <c r="E16" s="68" t="s">
+      <c r="F16" s="68" t="s">
         <v>31</v>
       </c>
-      <c r="F16" s="68" t="s">
+      <c r="G16" s="68" t="s">
         <v>32</v>
       </c>
-      <c r="G16" s="68" t="s">
+      <c r="H16" s="50" t="s">
         <v>33</v>
       </c>
-      <c r="H16" s="50" t="s">
+      <c r="I16" s="68" t="s">
         <v>34</v>
       </c>
-      <c r="I16" s="68" t="s">
+      <c r="J16" s="68" t="s">
         <v>35</v>
-      </c>
-      <c r="J16" s="68" t="s">
-        <v>36</v>
       </c>
       <c r="K16" s="68"/>
       <c r="L16" s="68"/>
       <c r="M16" s="68" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="N16" s="68"/>
     </row>
     <row r="17" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B17" s="84"/>
+      <c r="B17" s="87"/>
       <c r="C17" s="68"/>
       <c r="D17" s="68"/>
       <c r="E17" s="68"/>
@@ -1917,7 +2028,7 @@
       <c r="N17" s="68"/>
     </row>
     <row r="18" spans="2:15" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="84"/>
+      <c r="B18" s="87"/>
       <c r="C18" s="68"/>
       <c r="D18" s="68"/>
       <c r="E18" s="68"/>
@@ -1926,56 +2037,56 @@
       <c r="H18" s="52"/>
       <c r="I18" s="68"/>
       <c r="J18" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="K18" s="89" t="s">
         <v>38</v>
       </c>
-      <c r="K18" s="88" t="s">
-        <v>39</v>
-      </c>
-      <c r="L18" s="88"/>
+      <c r="L18" s="89"/>
       <c r="M18" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="N18" s="11" t="s">
         <v>38</v>
-      </c>
-      <c r="N18" s="11" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="19" spans="2:15" ht="30" x14ac:dyDescent="0.25">
       <c r="B19" s="25" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C19" s="25" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D19" s="39" t="s">
+        <v>41</v>
+      </c>
+      <c r="E19" s="39" t="s">
         <v>42</v>
       </c>
-      <c r="E19" s="39" t="s">
+      <c r="F19" s="37" t="s">
         <v>43</v>
       </c>
-      <c r="F19" s="37" t="s">
+      <c r="G19" s="37" t="s">
         <v>44</v>
       </c>
-      <c r="G19" s="37" t="s">
+      <c r="H19" s="37" t="s">
         <v>45</v>
       </c>
-      <c r="H19" s="37" t="s">
+      <c r="I19" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="I19" s="37" t="s">
+      <c r="J19" s="37" t="s">
         <v>47</v>
       </c>
-      <c r="J19" s="37" t="s">
+      <c r="K19" s="59" t="s">
         <v>48</v>
-      </c>
-      <c r="K19" s="59" t="s">
-        <v>49</v>
       </c>
       <c r="L19" s="59"/>
       <c r="M19" s="41" t="s">
+        <v>49</v>
+      </c>
+      <c r="N19" s="41" t="s">
         <v>50</v>
-      </c>
-      <c r="N19" s="41" t="s">
-        <v>51</v>
       </c>
       <c r="O19" s="31"/>
     </row>
@@ -2005,14 +2116,14 @@
       <c r="I21" s="12"/>
       <c r="J21" s="15"/>
       <c r="K21" s="67" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="L21" s="67"/>
       <c r="M21" s="37" t="s">
+        <v>52</v>
+      </c>
+      <c r="N21" s="37" t="s">
         <v>53</v>
-      </c>
-      <c r="N21" s="37" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="22" spans="2:15" x14ac:dyDescent="0.25">
@@ -2032,7 +2143,7 @@
     </row>
     <row r="23" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B23" s="99" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C23" s="99"/>
       <c r="D23" s="99"/>
@@ -2047,37 +2158,37 @@
       <c r="M23" s="10"/>
     </row>
     <row r="24" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B24" s="84" t="s">
+      <c r="B24" s="87" t="s">
+        <v>27</v>
+      </c>
+      <c r="C24" s="68" t="s">
         <v>28</v>
       </c>
-      <c r="C24" s="68" t="s">
-        <v>29</v>
-      </c>
       <c r="D24" s="68" t="s">
+        <v>55</v>
+      </c>
+      <c r="E24" s="68" t="s">
         <v>56</v>
       </c>
-      <c r="E24" s="68" t="s">
+      <c r="F24" s="68" t="s">
         <v>57</v>
       </c>
-      <c r="F24" s="68" t="s">
+      <c r="G24" s="68" t="s">
         <v>58</v>
-      </c>
-      <c r="G24" s="68" t="s">
-        <v>59</v>
       </c>
       <c r="H24" s="68"/>
       <c r="I24" s="68"/>
       <c r="J24" s="68" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K24" s="68"/>
       <c r="L24" s="68" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="M24" s="10"/>
     </row>
     <row r="25" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B25" s="84"/>
+      <c r="B25" s="87"/>
       <c r="C25" s="68"/>
       <c r="D25" s="68"/>
       <c r="E25" s="68"/>
@@ -2092,29 +2203,29 @@
     </row>
     <row r="26" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C26" s="37" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D26" s="44"/>
       <c r="E26" s="38" t="s">
+        <v>61</v>
+      </c>
+      <c r="F26" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="F26" s="16" t="s">
+      <c r="G26" s="64" t="s">
         <v>63</v>
-      </c>
-      <c r="G26" s="64" t="s">
-        <v>64</v>
       </c>
       <c r="H26" s="64"/>
       <c r="I26" s="64"/>
       <c r="J26" s="64" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="K26" s="64"/>
       <c r="L26" s="16" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="M26" s="10"/>
     </row>
@@ -2163,18 +2274,18 @@
     </row>
     <row r="30" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="98" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C30" s="98"/>
       <c r="D30" s="98"/>
       <c r="E30" s="98"/>
       <c r="F30" s="18"/>
       <c r="G30" s="65" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H30" s="66"/>
       <c r="I30" s="27" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="J30" s="27"/>
       <c r="K30" s="27"/>
@@ -2184,16 +2295,16 @@
     </row>
     <row r="31" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B31" s="19" t="s">
+        <v>69</v>
+      </c>
+      <c r="C31" s="20"/>
+      <c r="D31" s="103"/>
+      <c r="E31" s="103"/>
+      <c r="F31" s="10"/>
+      <c r="G31" s="104" t="s">
         <v>70</v>
       </c>
-      <c r="C31" s="20"/>
-      <c r="D31" s="107"/>
-      <c r="E31" s="107"/>
-      <c r="F31" s="10"/>
-      <c r="G31" s="108" t="s">
-        <v>71</v>
-      </c>
-      <c r="H31" s="109"/>
+      <c r="H31" s="105"/>
       <c r="I31" s="56"/>
       <c r="J31" s="57"/>
       <c r="K31" s="57"/>
@@ -2203,16 +2314,16 @@
     </row>
     <row r="32" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B32" s="19" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C32" s="20"/>
       <c r="D32" s="64"/>
       <c r="E32" s="64"/>
       <c r="F32" s="10"/>
-      <c r="G32" s="108" t="s">
-        <v>73</v>
-      </c>
-      <c r="H32" s="109"/>
+      <c r="G32" s="104" t="s">
+        <v>72</v>
+      </c>
+      <c r="H32" s="105"/>
       <c r="I32" s="56"/>
       <c r="J32" s="57"/>
       <c r="K32" s="57"/>
@@ -2222,18 +2333,18 @@
     </row>
     <row r="33" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B33" s="19" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C33" s="20"/>
       <c r="D33" s="16"/>
       <c r="E33" s="21" t="s">
+        <v>74</v>
+      </c>
+      <c r="F33" s="10"/>
+      <c r="G33" s="104" t="s">
         <v>75</v>
       </c>
-      <c r="F33" s="10"/>
-      <c r="G33" s="108" t="s">
-        <v>76</v>
-      </c>
-      <c r="H33" s="109"/>
+      <c r="H33" s="105"/>
       <c r="I33" s="56"/>
       <c r="J33" s="57"/>
       <c r="K33" s="57"/>
@@ -2243,18 +2354,18 @@
     </row>
     <row r="34" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B34" s="22" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C34" s="23"/>
       <c r="D34" s="16"/>
       <c r="E34" s="21" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F34" s="10"/>
-      <c r="G34" s="105" t="s">
-        <v>78</v>
-      </c>
-      <c r="H34" s="106"/>
+      <c r="G34" s="101" t="s">
+        <v>77</v>
+      </c>
+      <c r="H34" s="102"/>
       <c r="I34" s="53"/>
       <c r="J34" s="54"/>
       <c r="K34" s="54"/>
@@ -2275,71 +2386,91 @@
       <c r="M35" s="10"/>
       <c r="N35" s="10"/>
     </row>
-    <row r="36" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B36" s="102" t="s">
-        <v>79</v>
-      </c>
-      <c r="C36" s="103"/>
-      <c r="D36" s="103"/>
-      <c r="E36" s="103"/>
-      <c r="F36" s="104"/>
-      <c r="G36" s="29"/>
-      <c r="H36" s="29"/>
+    <row r="36" spans="2:14" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B36" s="109" t="s">
+        <v>78</v>
+      </c>
+      <c r="C36" s="110"/>
+      <c r="D36" s="110"/>
+      <c r="E36" s="111"/>
+      <c r="F36" s="29"/>
+      <c r="G36" s="121" t="s">
+        <v>131</v>
+      </c>
+      <c r="H36" s="122" t="s">
+        <v>136</v>
+      </c>
       <c r="I36" s="29"/>
       <c r="J36" s="29"/>
     </row>
     <row r="37" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B37" s="101" t="s">
-        <v>80</v>
-      </c>
-      <c r="C37" s="101"/>
-      <c r="D37" s="101"/>
-      <c r="E37" s="101"/>
-      <c r="F37" s="101"/>
-      <c r="G37" s="29"/>
-      <c r="H37" s="29"/>
+      <c r="B37" s="112" t="s">
+        <v>79</v>
+      </c>
+      <c r="C37" s="113"/>
+      <c r="D37" s="113"/>
+      <c r="E37" s="114"/>
+      <c r="F37" s="29"/>
+      <c r="G37" s="121" t="s">
+        <v>132</v>
+      </c>
+      <c r="H37" s="122" t="s">
+        <v>137</v>
+      </c>
       <c r="I37" s="29"/>
       <c r="J37" s="29"/>
     </row>
-    <row r="38" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B38" s="101"/>
-      <c r="C38" s="101"/>
-      <c r="D38" s="101"/>
-      <c r="E38" s="101"/>
-      <c r="F38" s="101"/>
-      <c r="G38" s="29"/>
-      <c r="H38" s="29"/>
+    <row r="38" spans="2:14" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B38" s="115"/>
+      <c r="C38" s="116"/>
+      <c r="D38" s="116"/>
+      <c r="E38" s="117"/>
+      <c r="F38" s="29"/>
+      <c r="G38" s="121" t="s">
+        <v>133</v>
+      </c>
+      <c r="H38" s="122" t="s">
+        <v>138</v>
+      </c>
       <c r="I38" s="29"/>
       <c r="J38" s="29"/>
     </row>
-    <row r="39" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B39" s="101"/>
-      <c r="C39" s="101"/>
-      <c r="D39" s="101"/>
-      <c r="E39" s="101"/>
-      <c r="F39" s="101"/>
-      <c r="G39" s="29"/>
-      <c r="H39" s="29"/>
+    <row r="39" spans="2:14" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B39" s="115"/>
+      <c r="C39" s="116"/>
+      <c r="D39" s="116"/>
+      <c r="E39" s="117"/>
+      <c r="F39" s="29"/>
+      <c r="G39" s="121" t="s">
+        <v>134</v>
+      </c>
+      <c r="H39" s="122" t="s">
+        <v>139</v>
+      </c>
       <c r="I39" s="29"/>
       <c r="J39" s="29"/>
     </row>
-    <row r="40" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B40" s="101"/>
-      <c r="C40" s="101"/>
-      <c r="D40" s="101"/>
-      <c r="E40" s="101"/>
-      <c r="F40" s="101"/>
-      <c r="G40" s="29"/>
-      <c r="H40" s="29"/>
+    <row r="40" spans="2:14" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B40" s="115"/>
+      <c r="C40" s="116"/>
+      <c r="D40" s="116"/>
+      <c r="E40" s="117"/>
+      <c r="F40" s="29"/>
+      <c r="G40" s="121" t="s">
+        <v>135</v>
+      </c>
+      <c r="H40" s="122" t="s">
+        <v>140</v>
+      </c>
       <c r="I40" s="29"/>
       <c r="J40" s="29"/>
     </row>
     <row r="41" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B41" s="101"/>
-      <c r="C41" s="101"/>
-      <c r="D41" s="101"/>
-      <c r="E41" s="101"/>
-      <c r="F41" s="101"/>
+      <c r="B41" s="118"/>
+      <c r="C41" s="119"/>
+      <c r="D41" s="119"/>
+      <c r="E41" s="120"/>
+      <c r="F41" s="29"/>
       <c r="G41" s="29"/>
       <c r="H41" s="29"/>
       <c r="I41" s="29"/>
@@ -2443,13 +2574,12 @@
       <c r="J53" s="45"/>
     </row>
   </sheetData>
-  <mergeCells count="70">
-    <mergeCell ref="B37:F41"/>
+  <mergeCells count="71">
+    <mergeCell ref="B37:E41"/>
     <mergeCell ref="I33:L33"/>
     <mergeCell ref="G16:G18"/>
     <mergeCell ref="I16:I18"/>
     <mergeCell ref="J16:L17"/>
-    <mergeCell ref="B36:F36"/>
     <mergeCell ref="G34:H34"/>
     <mergeCell ref="D31:E31"/>
     <mergeCell ref="D32:E32"/>
@@ -2514,6 +2644,8 @@
     <mergeCell ref="K21:L21"/>
     <mergeCell ref="L24:L25"/>
     <mergeCell ref="G24:I25"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="I13:K13"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D27:D28 D26" xr:uid="{B316A799-CF60-4C99-A88E-2204076E38E6}">
@@ -2566,88 +2698,88 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>81</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>82</v>
       </c>
       <c r="C1" s="33"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B2" t="s">
         <v>83</v>
       </c>
-      <c r="B2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C2" s="110"/>
+      <c r="C2" s="106"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B3" t="s">
         <v>85</v>
       </c>
-      <c r="B3" t="s">
-        <v>86</v>
-      </c>
-      <c r="C3" s="111"/>
+      <c r="C3" s="107"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B4" t="s">
-        <v>87</v>
-      </c>
-      <c r="C4" s="111"/>
+        <v>86</v>
+      </c>
+      <c r="C4" s="107"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B5" t="s">
-        <v>18</v>
-      </c>
-      <c r="C5" s="111"/>
+        <v>17</v>
+      </c>
+      <c r="C5" s="107"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C6" s="112"/>
+        <v>20</v>
+      </c>
+      <c r="C6" s="108"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B8" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>87</v>
+      </c>
+      <c r="B9" t="s">
         <v>88</v>
-      </c>
-      <c r="B9" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>89</v>
+      </c>
+      <c r="B10" t="s">
         <v>90</v>
-      </c>
-      <c r="B10" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -2676,18 +2808,18 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>92</v>
+      </c>
+      <c r="B15" t="s">
         <v>93</v>
-      </c>
-      <c r="B15" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="17" spans="1:27" x14ac:dyDescent="0.25">
@@ -2696,174 +2828,174 @@
     </row>
     <row r="18" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="19" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="B19" s="8" t="s">
         <v>96</v>
       </c>
-      <c r="B19" s="8" t="s">
+      <c r="C19" s="34" t="s">
         <v>97</v>
       </c>
-      <c r="C19" s="34" t="s">
+      <c r="D19" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="D19" s="2" t="s">
+      <c r="E19" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="E19" s="2" t="s">
+      <c r="F19" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="F19" s="2" t="s">
+      <c r="G19" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="G19" s="2" t="s">
+      <c r="H19" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="H19" s="2" t="s">
+      <c r="I19" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="I19" s="2" t="s">
+      <c r="J19" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="J19" s="2" t="s">
+      <c r="K19" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="K19" s="2" t="s">
+      <c r="L19" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="L19" s="2" t="s">
+      <c r="M19" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="N19" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="M19" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="N19" s="2" t="s">
+      <c r="O19" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="O19" s="2" t="s">
+      <c r="P19" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="P19" s="2" t="s">
+      <c r="Q19" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="Q19" s="2" t="s">
+      <c r="R19" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="R19" s="2" t="s">
+      <c r="S19" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="S19" s="2" t="s">
+      <c r="T19" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="T19" s="2" t="s">
+      <c r="U19" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="U19" s="2" t="s">
+      <c r="V19" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="V19" s="2" t="s">
+      <c r="W19" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="W19" s="2" t="s">
+      <c r="X19" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="Y19" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="X19" s="2" t="s">
+      <c r="Z19" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="Y19" s="2" t="s">
+      <c r="AA19" s="2" t="s">
         <v>118</v>
-      </c>
-      <c r="Z19" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="AA19" s="2" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="20" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B20" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="C20" s="25" t="s">
+        <v>42</v>
+      </c>
+      <c r="D20" t="s">
+        <v>43</v>
+      </c>
+      <c r="E20" t="s">
+        <v>44</v>
+      </c>
+      <c r="F20" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="G20" t="s">
         <v>120</v>
       </c>
-      <c r="C20" s="25" t="s">
-        <v>43</v>
-      </c>
-      <c r="D20" t="s">
-        <v>44</v>
-      </c>
-      <c r="E20" t="s">
+      <c r="H20" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="I20" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="J20" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="K20" t="s">
+        <v>121</v>
+      </c>
+      <c r="L20" t="s">
+        <v>39</v>
+      </c>
+      <c r="M20" t="s">
         <v>45</v>
       </c>
-      <c r="F20" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="G20" t="s">
-        <v>121</v>
-      </c>
-      <c r="H20" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="I20" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="J20" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="K20" t="s">
+      <c r="N20" t="s">
         <v>122</v>
       </c>
-      <c r="L20" t="s">
-        <v>40</v>
-      </c>
-      <c r="M20" t="s">
-        <v>46</v>
-      </c>
-      <c r="N20" t="s">
+      <c r="O20" t="s">
+        <v>65</v>
+      </c>
+      <c r="P20" t="s">
         <v>123</v>
       </c>
-      <c r="O20" t="s">
-        <v>66</v>
-      </c>
-      <c r="P20" t="s">
+      <c r="Q20" t="s">
         <v>124</v>
-      </c>
-      <c r="Q20" t="s">
-        <v>125</v>
       </c>
       <c r="R20" t="e">
         <f>IF(E20&gt;0,IF(E20="Unit",CONCATENATE(Settings!Q20," ",Settings!E20,"s"),CONCATENATE((Settings!Q20/Settings!M20)," ",Settings!E20,"s")),"")</f>
         <v>#VALUE!</v>
       </c>
       <c r="S20" s="35" t="s">
+        <v>125</v>
+      </c>
+      <c r="T20" s="35" t="s">
         <v>126</v>
       </c>
-      <c r="T20" s="35" t="s">
+      <c r="U20" s="35" t="s">
         <v>127</v>
       </c>
-      <c r="U20" s="35" t="s">
+      <c r="V20" t="s">
+        <v>52</v>
+      </c>
+      <c r="W20" t="s">
         <v>128</v>
       </c>
-      <c r="V20" t="s">
+      <c r="X20" t="s">
+        <v>62</v>
+      </c>
+      <c r="Y20" t="s">
+        <v>61</v>
+      </c>
+      <c r="Z20" t="s">
+        <v>63</v>
+      </c>
+      <c r="AA20" t="s">
         <v>53</v>
-      </c>
-      <c r="W20" t="s">
-        <v>129</v>
-      </c>
-      <c r="X20" t="s">
-        <v>63</v>
-      </c>
-      <c r="Y20" t="s">
-        <v>62</v>
-      </c>
-      <c r="Z20" t="s">
-        <v>64</v>
-      </c>
-      <c r="AA20" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="21" spans="1:27" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Add few missing fields into Thailand Quotation Template
</commit_message>
<xml_diff>
--- a/srv/xlsx-templates/TH - Quotation Template.xlsx
+++ b/srv/xlsx-templates/TH - Quotation Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EHMHV\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6246CB4C-31EC-4625-88D7-A3F32C8EC385}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F63A248-C45E-45EF-B0F8-F57C0B341C6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19200" windowHeight="9020" xr2:uid="{F5CC2154-27BB-4652-B61E-D913F0CC6809}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="19170" windowHeight="8520" xr2:uid="{F5CC2154-27BB-4652-B61E-D913F0CC6809}"/>
   </bookViews>
   <sheets>
     <sheet name="Quotation" sheetId="3" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="147">
   <si>
     <t>Offered Party</t>
   </si>
@@ -243,9 +243,6 @@
     <t>Quotation Delivery Channels</t>
   </si>
   <si>
-    <t>Receiver Information (Name, Phone, Address and/or Email)</t>
-  </si>
-  <si>
     <t>Quotation Date (วันที่)</t>
   </si>
   <si>
@@ -438,9 +435,6 @@
     <t>${offerValidation.TenderAnnouncementReference}</t>
   </si>
   <si>
-    <t>${offerValidation.ItemNumber}</t>
-  </si>
-  <si>
     <t>${offerValidation.PeriodOfBankGauranteeStart}</t>
   </si>
   <si>
@@ -471,10 +465,19 @@
     <t>${offerValidation.QuotationDeliverymethod}</t>
   </si>
   <si>
-    <t>${offerValidation.QuotationRecipientname} , ${offerValidation.QuotationRecipientcontact}</t>
-  </si>
-  <si>
     <t>${offerValidation.TENDER_SUBMITTED_BY}</t>
+  </si>
+  <si>
+    <t>${offerValidation.QuotationRecipientcontact}</t>
+  </si>
+  <si>
+    <t>${offerValidation.QuotationRecipientname}</t>
+  </si>
+  <si>
+    <t>Receiver Information (Name)</t>
+  </si>
+  <si>
+    <t>${table:offerProductValidation.ItemNumber}</t>
   </si>
 </sst>
 </file>
@@ -844,7 +847,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="121">
+  <cellXfs count="124">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -960,6 +963,162 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="6" fillId="0" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="43" fontId="5" fillId="0" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -987,172 +1146,25 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="6" fillId="0" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="5" fillId="0" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1689,24 +1701,24 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFBA1999-1CF9-4903-BA7D-DD523B82D6C3}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="B2:O53"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="12" customWidth="1"/>
-    <col min="3" max="3" width="15.7265625" customWidth="1"/>
-    <col min="4" max="4" width="33.26953125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="52.453125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.81640625" customWidth="1"/>
+    <col min="3" max="3" width="15.7109375" customWidth="1"/>
+    <col min="4" max="4" width="33.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="52.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.85546875" customWidth="1"/>
     <col min="7" max="7" width="17" customWidth="1"/>
-    <col min="8" max="8" width="24.54296875" customWidth="1"/>
-    <col min="9" max="9" width="14.7265625" customWidth="1"/>
-    <col min="10" max="10" width="21.26953125" customWidth="1"/>
-    <col min="11" max="11" width="14.81640625" customWidth="1"/>
-    <col min="12" max="12" width="12.54296875" customWidth="1"/>
+    <col min="8" max="8" width="24.5703125" customWidth="1"/>
+    <col min="9" max="9" width="14.7109375" customWidth="1"/>
+    <col min="10" max="10" width="21.28515625" customWidth="1"/>
+    <col min="11" max="11" width="14.85546875" customWidth="1"/>
+    <col min="12" max="12" width="12.5703125" customWidth="1"/>
     <col min="13" max="13" width="27" customWidth="1"/>
-    <col min="14" max="14" width="34.08984375" customWidth="1"/>
+    <col min="14" max="14" width="34.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B2" s="10"/>
       <c r="C2" s="10"/>
       <c r="D2" s="10"/>
@@ -1721,53 +1733,53 @@
       <c r="M2" s="10"/>
       <c r="N2" s="10"/>
     </row>
-    <row r="3" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B3" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="88" t="s">
+      <c r="C3" s="75" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="89"/>
-      <c r="E3" s="89"/>
-      <c r="F3" s="89"/>
-      <c r="G3" s="90"/>
+      <c r="D3" s="76"/>
+      <c r="E3" s="76"/>
+      <c r="F3" s="76"/>
+      <c r="G3" s="77"/>
       <c r="H3" s="10"/>
       <c r="I3" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="J3" s="88" t="s">
+      <c r="J3" s="75" t="s">
         <v>3</v>
       </c>
-      <c r="K3" s="89"/>
-      <c r="L3" s="89"/>
-      <c r="M3" s="90"/>
+      <c r="K3" s="76"/>
+      <c r="L3" s="76"/>
+      <c r="M3" s="77"/>
       <c r="N3" s="10"/>
     </row>
-    <row r="4" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="79" t="s">
+      <c r="C4" s="78" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="91"/>
-      <c r="E4" s="91"/>
-      <c r="F4" s="91"/>
+      <c r="D4" s="79"/>
+      <c r="E4" s="79"/>
+      <c r="F4" s="79"/>
       <c r="G4" s="80"/>
       <c r="H4" s="10"/>
       <c r="I4" s="26" t="s">
         <v>4</v>
       </c>
-      <c r="J4" s="97" t="s">
+      <c r="J4" s="86" t="s">
         <v>6</v>
       </c>
-      <c r="K4" s="98"/>
-      <c r="L4" s="98"/>
-      <c r="M4" s="99"/>
+      <c r="K4" s="87"/>
+      <c r="L4" s="87"/>
+      <c r="M4" s="88"/>
       <c r="N4" s="10"/>
     </row>
-    <row r="5" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="45"/>
       <c r="C5" s="45"/>
       <c r="D5" s="45"/>
@@ -1782,7 +1794,7 @@
       <c r="M5" s="46"/>
       <c r="N5" s="10"/>
     </row>
-    <row r="6" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="45"/>
       <c r="C6" s="45"/>
       <c r="D6" s="45"/>
@@ -1797,7 +1809,7 @@
       <c r="M6" s="46"/>
       <c r="N6" s="10"/>
     </row>
-    <row r="7" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B7" s="10"/>
       <c r="C7" s="10"/>
       <c r="D7" s="10"/>
@@ -1812,154 +1824,154 @@
       <c r="M7" s="10"/>
       <c r="N7" s="10"/>
     </row>
-    <row r="8" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B8" s="92" t="s">
-        <v>137</v>
-      </c>
-      <c r="C8" s="93"/>
-      <c r="D8" s="93"/>
-      <c r="E8" s="93"/>
-      <c r="F8" s="93"/>
-      <c r="G8" s="93"/>
-      <c r="H8" s="93"/>
-      <c r="I8" s="93"/>
-      <c r="J8" s="93"/>
-      <c r="K8" s="93"/>
-      <c r="L8" s="93"/>
-      <c r="M8" s="93"/>
-      <c r="N8" s="94"/>
-    </row>
-    <row r="9" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B9" s="100" t="s">
+    <row r="8" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B8" s="81" t="s">
+        <v>135</v>
+      </c>
+      <c r="C8" s="82"/>
+      <c r="D8" s="82"/>
+      <c r="E8" s="82"/>
+      <c r="F8" s="82"/>
+      <c r="G8" s="82"/>
+      <c r="H8" s="82"/>
+      <c r="I8" s="82"/>
+      <c r="J8" s="82"/>
+      <c r="K8" s="82"/>
+      <c r="L8" s="82"/>
+      <c r="M8" s="82"/>
+      <c r="N8" s="83"/>
+    </row>
+    <row r="9" spans="2:14" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B9" s="89" t="s">
         <v>7</v>
       </c>
-      <c r="C9" s="101"/>
-      <c r="D9" s="77" t="s">
+      <c r="C9" s="90"/>
+      <c r="D9" s="99" t="s">
         <v>8</v>
       </c>
-      <c r="E9" s="77"/>
+      <c r="E9" s="99"/>
       <c r="F9" s="40"/>
       <c r="G9" s="42" t="s">
         <v>9</v>
       </c>
       <c r="H9" s="42"/>
-      <c r="I9" s="71" t="s">
+      <c r="I9" s="94" t="s">
         <v>10</v>
       </c>
-      <c r="J9" s="71"/>
-      <c r="K9" s="72"/>
-      <c r="L9" s="95" t="s">
+      <c r="J9" s="94"/>
+      <c r="K9" s="95"/>
+      <c r="L9" s="84" t="s">
         <v>11</v>
       </c>
-      <c r="M9" s="96"/>
+      <c r="M9" s="85"/>
       <c r="N9" s="52" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="10" spans="2:14" ht="26.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="102" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="10" spans="2:14" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="91" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="103"/>
-      <c r="D10" s="78" t="str">
+      <c r="C10" s="92"/>
+      <c r="D10" s="100" t="str">
         <f>Settings!A14</f>
         <v>${offerValidation.CUSTOMER_CODE}</v>
       </c>
-      <c r="E10" s="78"/>
+      <c r="E10" s="100"/>
       <c r="F10" s="40"/>
-      <c r="G10" s="81" t="s">
+      <c r="G10" s="101" t="s">
         <v>13</v>
       </c>
-      <c r="H10" s="81"/>
-      <c r="I10" s="73" t="s">
+      <c r="H10" s="101"/>
+      <c r="I10" s="96" t="s">
         <v>14</v>
       </c>
-      <c r="J10" s="73"/>
-      <c r="K10" s="74"/>
-      <c r="L10" s="84" t="s">
+      <c r="J10" s="96"/>
+      <c r="K10" s="97"/>
+      <c r="L10" s="68" t="s">
         <v>15</v>
       </c>
-      <c r="M10" s="85"/>
+      <c r="M10" s="69"/>
       <c r="N10" s="52" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="11" spans="2:14" ht="26.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="102" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="11" spans="2:14" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="91" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="103"/>
-      <c r="D11" s="79" t="str">
+      <c r="C11" s="92"/>
+      <c r="D11" s="78" t="str">
         <f>Settings!A9</f>
         <v>${offerValidation.INSTITUTENAME}</v>
       </c>
       <c r="E11" s="80"/>
       <c r="F11" s="40"/>
-      <c r="G11" s="82" t="s">
+      <c r="G11" s="102" t="s">
         <v>17</v>
       </c>
-      <c r="H11" s="82"/>
-      <c r="I11" s="73" t="s">
+      <c r="H11" s="102"/>
+      <c r="I11" s="96" t="s">
         <v>18</v>
       </c>
-      <c r="J11" s="73"/>
-      <c r="K11" s="74"/>
-      <c r="L11" s="84" t="s">
+      <c r="J11" s="96"/>
+      <c r="K11" s="97"/>
+      <c r="L11" s="68" t="s">
         <v>19</v>
       </c>
-      <c r="M11" s="85"/>
+      <c r="M11" s="69"/>
       <c r="N11" s="52" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="12" spans="2:14" ht="26" x14ac:dyDescent="0.35">
-      <c r="B12" s="102" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="12" spans="2:14" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B12" s="91" t="s">
         <v>20</v>
       </c>
-      <c r="C12" s="103"/>
-      <c r="D12" s="67" t="s">
+      <c r="C12" s="92"/>
+      <c r="D12" s="103" t="s">
         <v>21</v>
       </c>
-      <c r="E12" s="69"/>
+      <c r="E12" s="59"/>
       <c r="F12" s="10"/>
-      <c r="G12" s="87" t="s">
+      <c r="G12" s="53" t="s">
         <v>22</v>
       </c>
-      <c r="H12" s="87"/>
-      <c r="I12" s="104" t="s">
+      <c r="H12" s="53"/>
+      <c r="I12" s="54" t="s">
         <v>23</v>
       </c>
-      <c r="J12" s="104"/>
-      <c r="K12" s="105"/>
-      <c r="L12" s="84" t="s">
+      <c r="J12" s="54"/>
+      <c r="K12" s="55"/>
+      <c r="L12" s="68" t="s">
         <v>15</v>
       </c>
-      <c r="M12" s="85"/>
+      <c r="M12" s="69"/>
       <c r="N12" s="52" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="13" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B13" s="102" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="13" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B13" s="91" t="s">
         <v>24</v>
       </c>
-      <c r="C13" s="103"/>
-      <c r="D13" s="67" t="s">
+      <c r="C13" s="92"/>
+      <c r="D13" s="103" t="s">
         <v>25</v>
       </c>
-      <c r="E13" s="69"/>
+      <c r="E13" s="59"/>
       <c r="F13" s="10"/>
-      <c r="G13" s="87" t="s">
-        <v>126</v>
-      </c>
-      <c r="H13" s="87"/>
-      <c r="I13" s="104" t="s">
-        <v>138</v>
-      </c>
-      <c r="J13" s="104"/>
-      <c r="K13" s="105"/>
-    </row>
-    <row r="14" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="G13" s="53" t="s">
+        <v>125</v>
+      </c>
+      <c r="H13" s="53"/>
+      <c r="I13" s="54" t="s">
+        <v>136</v>
+      </c>
+      <c r="J13" s="54"/>
+      <c r="K13" s="55"/>
+    </row>
+    <row r="14" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B14" s="10"/>
       <c r="C14" s="10"/>
       <c r="D14" s="10"/>
@@ -1971,89 +1983,89 @@
       <c r="J14" s="10"/>
       <c r="K14" s="10"/>
     </row>
-    <row r="15" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B15" s="83" t="s">
+    <row r="15" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B15" s="67" t="s">
         <v>26</v>
       </c>
-      <c r="C15" s="83"/>
-      <c r="D15" s="83"/>
-      <c r="E15" s="83"/>
-      <c r="F15" s="83"/>
-      <c r="G15" s="83"/>
-      <c r="H15" s="83"/>
-      <c r="I15" s="83"/>
-      <c r="J15" s="83"/>
-      <c r="K15" s="83"/>
-      <c r="L15" s="83"/>
-      <c r="M15" s="83"/>
-      <c r="N15" s="83"/>
-    </row>
-    <row r="16" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B16" s="76" t="s">
+      <c r="C15" s="67"/>
+      <c r="D15" s="67"/>
+      <c r="E15" s="67"/>
+      <c r="F15" s="67"/>
+      <c r="G15" s="67"/>
+      <c r="H15" s="67"/>
+      <c r="I15" s="67"/>
+      <c r="J15" s="67"/>
+      <c r="K15" s="67"/>
+      <c r="L15" s="67"/>
+      <c r="M15" s="67"/>
+      <c r="N15" s="67"/>
+    </row>
+    <row r="16" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B16" s="93" t="s">
         <v>27</v>
       </c>
-      <c r="C16" s="62" t="s">
+      <c r="C16" s="61" t="s">
         <v>28</v>
       </c>
-      <c r="D16" s="62" t="s">
+      <c r="D16" s="61" t="s">
         <v>29</v>
       </c>
-      <c r="E16" s="62" t="s">
+      <c r="E16" s="61" t="s">
         <v>30</v>
       </c>
-      <c r="F16" s="62" t="s">
+      <c r="F16" s="61" t="s">
         <v>31</v>
       </c>
-      <c r="G16" s="62" t="s">
+      <c r="G16" s="61" t="s">
         <v>32</v>
       </c>
-      <c r="H16" s="113" t="s">
+      <c r="H16" s="71" t="s">
         <v>33</v>
       </c>
-      <c r="I16" s="62" t="s">
+      <c r="I16" s="61" t="s">
         <v>34</v>
       </c>
-      <c r="J16" s="62" t="s">
+      <c r="J16" s="61" t="s">
         <v>35</v>
       </c>
-      <c r="K16" s="62"/>
-      <c r="L16" s="62"/>
-      <c r="M16" s="62" t="s">
+      <c r="K16" s="61"/>
+      <c r="L16" s="61"/>
+      <c r="M16" s="61" t="s">
         <v>36</v>
       </c>
-      <c r="N16" s="62"/>
-    </row>
-    <row r="17" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="B17" s="76"/>
-      <c r="C17" s="62"/>
-      <c r="D17" s="62"/>
-      <c r="E17" s="62"/>
-      <c r="F17" s="62"/>
-      <c r="G17" s="62"/>
-      <c r="H17" s="114"/>
-      <c r="I17" s="62"/>
-      <c r="J17" s="62"/>
-      <c r="K17" s="62"/>
-      <c r="L17" s="62"/>
-      <c r="M17" s="62"/>
-      <c r="N17" s="62"/>
-    </row>
-    <row r="18" spans="2:15" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="76"/>
-      <c r="C18" s="62"/>
-      <c r="D18" s="62"/>
-      <c r="E18" s="62"/>
-      <c r="F18" s="62"/>
-      <c r="G18" s="62"/>
-      <c r="H18" s="115"/>
-      <c r="I18" s="62"/>
+      <c r="N16" s="61"/>
+    </row>
+    <row r="17" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B17" s="93"/>
+      <c r="C17" s="61"/>
+      <c r="D17" s="61"/>
+      <c r="E17" s="61"/>
+      <c r="F17" s="61"/>
+      <c r="G17" s="61"/>
+      <c r="H17" s="72"/>
+      <c r="I17" s="61"/>
+      <c r="J17" s="61"/>
+      <c r="K17" s="61"/>
+      <c r="L17" s="61"/>
+      <c r="M17" s="61"/>
+      <c r="N17" s="61"/>
+    </row>
+    <row r="18" spans="2:15" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="93"/>
+      <c r="C18" s="61"/>
+      <c r="D18" s="61"/>
+      <c r="E18" s="61"/>
+      <c r="F18" s="61"/>
+      <c r="G18" s="61"/>
+      <c r="H18" s="73"/>
+      <c r="I18" s="61"/>
       <c r="J18" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="K18" s="86" t="s">
+      <c r="K18" s="70" t="s">
         <v>38</v>
       </c>
-      <c r="L18" s="86"/>
+      <c r="L18" s="70"/>
       <c r="M18" s="11" t="s">
         <v>37</v>
       </c>
@@ -2061,12 +2073,12 @@
         <v>38</v>
       </c>
     </row>
-    <row r="19" spans="2:15" ht="29" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:15" ht="30" x14ac:dyDescent="0.25">
       <c r="B19" s="25" t="s">
         <v>39</v>
       </c>
       <c r="C19" s="25" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D19" s="39" t="s">
         <v>41</v>
@@ -2089,10 +2101,10 @@
       <c r="J19" s="37" t="s">
         <v>47</v>
       </c>
-      <c r="K19" s="116" t="s">
+      <c r="K19" s="74" t="s">
         <v>48</v>
       </c>
-      <c r="L19" s="116"/>
+      <c r="L19" s="74"/>
       <c r="M19" s="41" t="s">
         <v>49</v>
       </c>
@@ -2101,7 +2113,7 @@
       </c>
       <c r="O19" s="31"/>
     </row>
-    <row r="20" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B20" s="12"/>
       <c r="C20" s="12"/>
       <c r="D20" s="12"/>
@@ -2111,12 +2123,12 @@
       <c r="H20" s="13"/>
       <c r="I20" s="12"/>
       <c r="J20" s="15"/>
-      <c r="K20" s="117"/>
-      <c r="L20" s="117"/>
+      <c r="K20" s="104"/>
+      <c r="L20" s="104"/>
       <c r="M20" s="14"/>
       <c r="N20" s="36"/>
     </row>
-    <row r="21" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B21" s="12"/>
       <c r="C21" s="12"/>
       <c r="D21" s="12"/>
@@ -2126,10 +2138,10 @@
       <c r="H21" s="13"/>
       <c r="I21" s="12"/>
       <c r="J21" s="15"/>
-      <c r="K21" s="111" t="s">
+      <c r="K21" s="66" t="s">
         <v>51</v>
       </c>
-      <c r="L21" s="111"/>
+      <c r="L21" s="66"/>
       <c r="M21" s="37" t="s">
         <v>52</v>
       </c>
@@ -2137,7 +2149,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="22" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B22" s="10"/>
       <c r="C22" s="10"/>
       <c r="D22" s="10"/>
@@ -2152,123 +2164,132 @@
       <c r="M22" s="10"/>
       <c r="N22" s="10"/>
     </row>
-    <row r="23" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="B23" s="75" t="s">
+    <row r="23" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B23" s="98" t="s">
         <v>54</v>
       </c>
-      <c r="C23" s="75"/>
-      <c r="D23" s="75"/>
-      <c r="E23" s="75"/>
-      <c r="F23" s="75"/>
-      <c r="G23" s="75"/>
-      <c r="H23" s="75"/>
-      <c r="I23" s="75"/>
-      <c r="J23" s="75"/>
-      <c r="K23" s="75"/>
-      <c r="L23" s="75"/>
+      <c r="C23" s="98"/>
+      <c r="D23" s="98"/>
+      <c r="E23" s="98"/>
+      <c r="F23" s="98"/>
+      <c r="G23" s="98"/>
+      <c r="H23" s="98"/>
+      <c r="I23" s="98"/>
+      <c r="J23" s="98"/>
+      <c r="K23" s="98"/>
+      <c r="L23" s="98"/>
       <c r="M23" s="10"/>
     </row>
-    <row r="24" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="B24" s="76" t="s">
+    <row r="24" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B24" s="93" t="s">
         <v>27</v>
       </c>
-      <c r="C24" s="62" t="s">
+      <c r="C24" s="61" t="s">
         <v>28</v>
       </c>
-      <c r="D24" s="62" t="s">
+      <c r="D24" s="71" t="s">
+        <v>127</v>
+      </c>
+      <c r="E24" s="61" t="s">
         <v>55</v>
       </c>
-      <c r="E24" s="62" t="s">
+      <c r="F24" s="61" t="s">
         <v>56</v>
       </c>
-      <c r="F24" s="62" t="s">
+      <c r="G24" s="61" t="s">
         <v>57</v>
       </c>
-      <c r="G24" s="62" t="s">
+      <c r="H24" s="61" t="s">
         <v>58</v>
       </c>
-      <c r="H24" s="62"/>
-      <c r="I24" s="62"/>
-      <c r="J24" s="62" t="s">
+      <c r="I24" s="61"/>
+      <c r="J24" s="61"/>
+      <c r="K24" s="61" t="s">
         <v>59</v>
       </c>
-      <c r="K24" s="62"/>
-      <c r="L24" s="62" t="s">
+      <c r="L24" s="61"/>
+      <c r="M24" s="61" t="s">
         <v>60</v>
       </c>
-      <c r="M24" s="10"/>
-    </row>
-    <row r="25" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="B25" s="76"/>
-      <c r="C25" s="62"/>
-      <c r="D25" s="62"/>
-      <c r="E25" s="62"/>
-      <c r="F25" s="62"/>
-      <c r="G25" s="62"/>
-      <c r="H25" s="62"/>
-      <c r="I25" s="62"/>
-      <c r="J25" s="62"/>
-      <c r="K25" s="62"/>
-      <c r="L25" s="62"/>
-      <c r="M25" s="10"/>
-    </row>
-    <row r="26" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="N24" s="10"/>
+    </row>
+    <row r="25" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B25" s="93"/>
+      <c r="C25" s="61"/>
+      <c r="D25" s="73"/>
+      <c r="E25" s="61"/>
+      <c r="F25" s="61"/>
+      <c r="G25" s="61"/>
+      <c r="H25" s="61"/>
+      <c r="I25" s="61"/>
+      <c r="J25" s="61"/>
+      <c r="K25" s="61"/>
+      <c r="L25" s="61"/>
+      <c r="M25" s="61"/>
+      <c r="N25" s="10"/>
+    </row>
+    <row r="26" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="12" t="s">
         <v>39</v>
       </c>
       <c r="C26" s="37" t="s">
-        <v>125</v>
-      </c>
-      <c r="D26" s="43"/>
-      <c r="E26" s="38" t="s">
+        <v>124</v>
+      </c>
+      <c r="D26" s="37" t="s">
+        <v>146</v>
+      </c>
+      <c r="E26" s="43"/>
+      <c r="F26" s="38" t="s">
         <v>61</v>
       </c>
-      <c r="F26" s="16" t="s">
+      <c r="G26" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="G26" s="64" t="s">
+      <c r="H26" s="65" t="s">
         <v>63</v>
       </c>
-      <c r="H26" s="64"/>
-      <c r="I26" s="64"/>
-      <c r="J26" s="64" t="s">
+      <c r="I26" s="65"/>
+      <c r="J26" s="65"/>
+      <c r="K26" s="65" t="s">
         <v>64</v>
       </c>
-      <c r="K26" s="64"/>
-      <c r="L26" s="16" t="s">
+      <c r="L26" s="65"/>
+      <c r="M26" s="16" t="s">
         <v>65</v>
       </c>
-      <c r="M26" s="10"/>
-    </row>
-    <row r="27" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="N26" s="10"/>
+    </row>
+    <row r="27" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B27" s="16"/>
       <c r="C27" s="16"/>
       <c r="D27" s="16"/>
       <c r="E27" s="16"/>
       <c r="F27" s="16"/>
-      <c r="G27" s="106"/>
-      <c r="H27" s="107"/>
-      <c r="I27" s="108"/>
+      <c r="G27" s="16"/>
+      <c r="H27" s="62"/>
+      <c r="I27" s="63"/>
       <c r="J27" s="64"/>
-      <c r="K27" s="64"/>
-      <c r="L27" s="16"/>
-      <c r="M27" s="10"/>
-    </row>
-    <row r="28" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="K27" s="65"/>
+      <c r="L27" s="65"/>
+      <c r="M27" s="16"/>
+      <c r="N27" s="10"/>
+    </row>
+    <row r="28" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B28" s="16"/>
       <c r="C28" s="16"/>
       <c r="D28" s="16"/>
       <c r="E28" s="16"/>
       <c r="F28" s="16"/>
-      <c r="G28" s="112"/>
-      <c r="H28" s="112"/>
-      <c r="I28" s="112"/>
-      <c r="J28" s="64"/>
-      <c r="K28" s="64"/>
-      <c r="L28" s="16"/>
-      <c r="M28" s="10"/>
-    </row>
-    <row r="29" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="G28" s="16"/>
+      <c r="H28" s="120"/>
+      <c r="I28" s="120"/>
+      <c r="J28" s="120"/>
+      <c r="K28" s="65"/>
+      <c r="L28" s="65"/>
+      <c r="M28" s="16"/>
+      <c r="N28" s="10"/>
+    </row>
+    <row r="29" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B29" s="10"/>
       <c r="C29" s="10"/>
       <c r="D29" s="17"/>
@@ -2283,55 +2304,59 @@
       <c r="M29" s="10"/>
       <c r="N29" s="10"/>
     </row>
-    <row r="30" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B30" s="70" t="s">
+    <row r="30" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B30" s="117" t="s">
         <v>66</v>
       </c>
-      <c r="C30" s="70"/>
-      <c r="D30" s="70"/>
-      <c r="E30" s="70"/>
+      <c r="C30" s="117"/>
+      <c r="D30" s="117"/>
+      <c r="E30" s="117"/>
       <c r="F30" s="18"/>
-      <c r="G30" s="109" t="s">
+      <c r="G30" s="118" t="s">
         <v>67</v>
       </c>
-      <c r="H30" s="110"/>
-      <c r="I30" s="27" t="s">
-        <v>68</v>
-      </c>
-      <c r="J30" s="27"/>
-      <c r="K30" s="27"/>
+      <c r="H30" s="119"/>
+      <c r="I30" s="56" t="s">
+        <v>145</v>
+      </c>
+      <c r="J30" s="57"/>
+      <c r="K30" s="27" t="s">
+        <v>15</v>
+      </c>
       <c r="L30" s="27"/>
       <c r="M30" s="10"/>
       <c r="N30" s="10"/>
     </row>
-    <row r="31" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B31" s="19" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C31" s="20"/>
-      <c r="D31" s="63"/>
-      <c r="E31" s="63"/>
+      <c r="D31" s="114"/>
+      <c r="E31" s="114"/>
       <c r="F31" s="10"/>
-      <c r="G31" s="65" t="s">
+      <c r="G31" s="115" t="s">
+        <v>141</v>
+      </c>
+      <c r="H31" s="116"/>
+      <c r="I31" s="60" t="s">
+        <v>144</v>
+      </c>
+      <c r="J31" s="60"/>
+      <c r="K31" s="58" t="s">
         <v>143</v>
       </c>
-      <c r="H31" s="66"/>
-      <c r="I31" s="67" t="s">
-        <v>144</v>
-      </c>
-      <c r="J31" s="68"/>
-      <c r="K31" s="68"/>
-      <c r="L31" s="69"/>
+      <c r="L31" s="59"/>
       <c r="M31" s="10"/>
       <c r="N31" s="10"/>
     </row>
-    <row r="32" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B32" s="19" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C32" s="20"/>
-      <c r="D32" s="64"/>
-      <c r="E32" s="64"/>
+      <c r="D32" s="65"/>
+      <c r="E32" s="65"/>
       <c r="F32" s="10"/>
       <c r="G32" s="10"/>
       <c r="H32" s="10"/>
@@ -2342,14 +2367,14 @@
       <c r="M32" s="10"/>
       <c r="N32" s="10"/>
     </row>
-    <row r="33" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B33" s="19" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C33" s="20"/>
       <c r="D33" s="16"/>
       <c r="E33" s="21" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F33" s="10"/>
       <c r="G33" s="10"/>
@@ -2361,16 +2386,16 @@
       <c r="M33" s="10"/>
       <c r="N33" s="10"/>
     </row>
-    <row r="34" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B34" s="22" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C34" s="23"/>
       <c r="D34" s="16" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="E34" s="21" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F34" s="10"/>
       <c r="G34" s="10"/>
@@ -2380,7 +2405,7 @@
       <c r="K34" s="10"/>
       <c r="L34" s="10"/>
     </row>
-    <row r="35" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B35" s="10"/>
       <c r="C35" s="10"/>
       <c r="D35" s="10"/>
@@ -2395,97 +2420,93 @@
       <c r="M35" s="10"/>
       <c r="N35" s="10"/>
     </row>
-    <row r="36" spans="2:14" ht="39" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:14" ht="38.25" x14ac:dyDescent="0.25">
       <c r="B36" s="47" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C36" s="48"/>
       <c r="D36" s="48"/>
       <c r="E36" s="49"/>
       <c r="F36" s="29"/>
       <c r="G36" s="50" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="H36" s="51" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="I36" s="29"/>
       <c r="J36" s="29"/>
     </row>
-    <row r="37" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B37" s="53" t="s">
-        <v>75</v>
-      </c>
-      <c r="C37" s="54"/>
-      <c r="D37" s="54"/>
-      <c r="E37" s="55"/>
+    <row r="37" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B37" s="105" t="s">
+        <v>74</v>
+      </c>
+      <c r="C37" s="106"/>
+      <c r="D37" s="106"/>
+      <c r="E37" s="107"/>
       <c r="F37" s="29"/>
       <c r="G37" s="50" t="s">
         <v>128</v>
       </c>
       <c r="H37" s="51" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="I37" s="29"/>
       <c r="J37" s="29"/>
     </row>
-    <row r="38" spans="2:14" ht="26" x14ac:dyDescent="0.35">
-      <c r="B38" s="56"/>
-      <c r="C38" s="57"/>
-      <c r="D38" s="57"/>
-      <c r="E38" s="58"/>
+    <row r="38" spans="2:14" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B38" s="108"/>
+      <c r="C38" s="109"/>
+      <c r="D38" s="109"/>
+      <c r="E38" s="110"/>
       <c r="F38" s="29"/>
       <c r="G38" s="50" t="s">
         <v>129</v>
       </c>
       <c r="H38" s="51" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="I38" s="29"/>
       <c r="J38" s="29"/>
     </row>
-    <row r="39" spans="2:14" ht="26" x14ac:dyDescent="0.35">
-      <c r="B39" s="56"/>
-      <c r="C39" s="57"/>
-      <c r="D39" s="57"/>
-      <c r="E39" s="58"/>
+    <row r="39" spans="2:14" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B39" s="108"/>
+      <c r="C39" s="109"/>
+      <c r="D39" s="109"/>
+      <c r="E39" s="110"/>
       <c r="F39" s="29"/>
       <c r="G39" s="50" t="s">
         <v>130</v>
       </c>
       <c r="H39" s="51" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="I39" s="29"/>
       <c r="J39" s="29"/>
     </row>
-    <row r="40" spans="2:14" ht="26" x14ac:dyDescent="0.35">
-      <c r="B40" s="56"/>
-      <c r="C40" s="57"/>
-      <c r="D40" s="57"/>
-      <c r="E40" s="58"/>
+    <row r="40" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B40" s="108"/>
+      <c r="C40" s="109"/>
+      <c r="D40" s="109"/>
+      <c r="E40" s="110"/>
       <c r="F40" s="29"/>
-      <c r="G40" s="50" t="s">
-        <v>131</v>
-      </c>
-      <c r="H40" s="51" t="s">
-        <v>136</v>
-      </c>
+      <c r="G40" s="29"/>
+      <c r="H40" s="29"/>
       <c r="I40" s="29"/>
       <c r="J40" s="29"/>
     </row>
-    <row r="41" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B41" s="59"/>
-      <c r="C41" s="60"/>
-      <c r="D41" s="60"/>
-      <c r="E41" s="61"/>
+    <row r="41" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B41" s="111"/>
+      <c r="C41" s="112"/>
+      <c r="D41" s="112"/>
+      <c r="E41" s="113"/>
       <c r="F41" s="29"/>
       <c r="G41" s="29"/>
-      <c r="H41" s="29"/>
+      <c r="H41" s="10"/>
       <c r="I41" s="29"/>
       <c r="J41" s="29"/>
     </row>
-    <row r="42" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B42" s="29"/>
       <c r="C42" s="29"/>
       <c r="D42" s="29"/>
@@ -2496,18 +2517,17 @@
       <c r="I42" s="10"/>
       <c r="J42" s="10"/>
     </row>
-    <row r="43" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B43" s="29"/>
       <c r="C43" s="29"/>
       <c r="D43" s="29"/>
       <c r="E43" s="29"/>
       <c r="F43" s="29"/>
-      <c r="G43" s="29"/>
       <c r="H43" s="10"/>
       <c r="I43" s="10"/>
       <c r="J43" s="10"/>
     </row>
-    <row r="44" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="44" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B44" s="29"/>
       <c r="C44" s="29"/>
       <c r="D44" s="29"/>
@@ -2517,17 +2537,17 @@
       <c r="J44" s="10"/>
       <c r="K44" s="10"/>
     </row>
-    <row r="45" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="45" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B45" s="29"/>
       <c r="C45" s="29"/>
       <c r="D45" s="29"/>
       <c r="E45" s="29"/>
-      <c r="H45" s="10"/>
+      <c r="H45" s="24"/>
       <c r="I45" s="10"/>
       <c r="J45" s="10"/>
       <c r="K45" s="10"/>
     </row>
-    <row r="46" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="46" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B46" s="29"/>
       <c r="C46" s="29"/>
       <c r="D46" s="29"/>
@@ -2536,7 +2556,7 @@
       <c r="I46" s="24"/>
       <c r="J46" s="24"/>
     </row>
-    <row r="47" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B47" s="29"/>
       <c r="C47" s="29"/>
       <c r="D47" s="29"/>
@@ -2545,25 +2565,25 @@
       <c r="I47" s="24"/>
       <c r="J47" s="24"/>
     </row>
-    <row r="48" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="48" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B48" s="29"/>
       <c r="C48" s="29"/>
       <c r="D48" s="29"/>
       <c r="E48" s="29"/>
-      <c r="H48" s="24"/>
+      <c r="H48" s="17"/>
       <c r="I48" s="24"/>
       <c r="J48" s="24"/>
     </row>
-    <row r="49" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="49" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B49" s="29"/>
       <c r="C49" s="29"/>
       <c r="D49" s="29"/>
       <c r="E49" s="29"/>
-      <c r="H49" s="17"/>
+      <c r="G49" s="29"/>
       <c r="I49" s="10"/>
       <c r="J49" s="10"/>
     </row>
-    <row r="50" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="50" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B50" s="29"/>
       <c r="C50" s="29"/>
       <c r="D50" s="29"/>
@@ -2571,41 +2591,44 @@
       <c r="F50" s="29"/>
       <c r="G50" s="29"/>
     </row>
-    <row r="51" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="51" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B51" s="29"/>
       <c r="C51" s="29"/>
       <c r="D51" s="29"/>
       <c r="E51" s="29"/>
       <c r="F51" s="29"/>
-      <c r="G51" s="29"/>
-    </row>
-    <row r="53" spans="2:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="53" spans="2:10" x14ac:dyDescent="0.25">
       <c r="J53" s="44"/>
     </row>
   </sheetData>
-  <mergeCells count="65">
+  <mergeCells count="68">
     <mergeCell ref="L10:M10"/>
     <mergeCell ref="L11:M11"/>
-    <mergeCell ref="H16:H18"/>
-    <mergeCell ref="K19:L19"/>
     <mergeCell ref="K20:L20"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="I13:K13"/>
+    <mergeCell ref="B37:E41"/>
+    <mergeCell ref="G16:G18"/>
+    <mergeCell ref="I16:I18"/>
+    <mergeCell ref="J16:L17"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="G31:H31"/>
+    <mergeCell ref="C24:C25"/>
+    <mergeCell ref="E24:E25"/>
+    <mergeCell ref="F24:F25"/>
+    <mergeCell ref="B30:E30"/>
+    <mergeCell ref="G30:H30"/>
+    <mergeCell ref="H28:J28"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="C16:C18"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B13:C13"/>
-    <mergeCell ref="M16:N17"/>
-    <mergeCell ref="I12:K12"/>
-    <mergeCell ref="G27:I27"/>
-    <mergeCell ref="J27:K27"/>
-    <mergeCell ref="K21:L21"/>
-    <mergeCell ref="L24:L25"/>
-    <mergeCell ref="G24:I25"/>
-    <mergeCell ref="G26:I26"/>
-    <mergeCell ref="J26:K26"/>
-    <mergeCell ref="B15:N15"/>
-    <mergeCell ref="L12:M12"/>
-    <mergeCell ref="K18:L18"/>
-    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="G10:H10"/>
+    <mergeCell ref="G11:H11"/>
     <mergeCell ref="C3:G3"/>
     <mergeCell ref="C4:G4"/>
     <mergeCell ref="F16:F18"/>
@@ -2621,37 +2644,36 @@
     <mergeCell ref="I9:K9"/>
     <mergeCell ref="I10:K10"/>
     <mergeCell ref="I11:K11"/>
-    <mergeCell ref="F24:F25"/>
     <mergeCell ref="D16:D18"/>
+    <mergeCell ref="M16:N17"/>
+    <mergeCell ref="I12:K12"/>
+    <mergeCell ref="H27:J27"/>
+    <mergeCell ref="K27:L27"/>
+    <mergeCell ref="K21:L21"/>
+    <mergeCell ref="M24:M25"/>
+    <mergeCell ref="H24:J25"/>
+    <mergeCell ref="H26:J26"/>
+    <mergeCell ref="K26:L26"/>
+    <mergeCell ref="B15:N15"/>
+    <mergeCell ref="L12:M12"/>
+    <mergeCell ref="K18:L18"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="G24:G25"/>
+    <mergeCell ref="H16:H18"/>
+    <mergeCell ref="K19:L19"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="I13:K13"/>
+    <mergeCell ref="I30:J30"/>
+    <mergeCell ref="K31:L31"/>
+    <mergeCell ref="I31:J31"/>
     <mergeCell ref="B23:L23"/>
     <mergeCell ref="B24:B25"/>
-    <mergeCell ref="J24:K25"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="G10:H10"/>
-    <mergeCell ref="G11:H11"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="C16:C18"/>
-    <mergeCell ref="B37:E41"/>
-    <mergeCell ref="G16:G18"/>
-    <mergeCell ref="I16:I18"/>
-    <mergeCell ref="J16:L17"/>
-    <mergeCell ref="D31:E31"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="G31:H31"/>
-    <mergeCell ref="C24:C25"/>
+    <mergeCell ref="K24:L25"/>
+    <mergeCell ref="K28:L28"/>
     <mergeCell ref="D24:D25"/>
-    <mergeCell ref="E24:E25"/>
-    <mergeCell ref="I31:L31"/>
-    <mergeCell ref="B30:E30"/>
-    <mergeCell ref="G30:H30"/>
-    <mergeCell ref="G28:I28"/>
-    <mergeCell ref="J28:K28"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D26:D28" xr:uid="{B316A799-CF60-4C99-A88E-2204076E38E6}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E26:E28" xr:uid="{B316A799-CF60-4C99-A88E-2204076E38E6}">
       <formula1>"กล่อง, เม็ด, ไวอัล, แอมพูล, ขวด, box, tablet, vial, ampoul, bottle"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E33:E34" xr:uid="{2CF9FB64-438B-485F-A115-633E3AF0704D}">
@@ -2671,89 +2693,89 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E9BADA0-6CEF-4001-8243-A13FFD1BF3BE}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:AA54"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="43.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="50.26953125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="50.26953125" style="25" customWidth="1"/>
-    <col min="4" max="4" width="47.26953125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="36.7265625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="46.7265625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="44.26953125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="52.26953125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="69.26953125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="75.453125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="42.26953125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="40.54296875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="42.1796875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="41.7265625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="52.81640625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="36.26953125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="46.7265625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="16.26953125" customWidth="1"/>
-    <col min="19" max="19" width="39.54296875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="38.81640625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="27.1796875" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="43.26953125" bestFit="1" customWidth="1"/>
-    <col min="23" max="26" width="30.453125" customWidth="1"/>
-    <col min="27" max="27" width="35.81640625" customWidth="1"/>
+    <col min="1" max="1" width="43.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="50.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="50.28515625" style="25" customWidth="1"/>
+    <col min="4" max="4" width="47.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="36.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="46.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="44.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="52.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="69.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="75.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="42.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="40.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="42.140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="41.7109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="52.85546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="36.28515625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="46.7109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="16.28515625" customWidth="1"/>
+    <col min="19" max="19" width="39.5703125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="38.85546875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="27.140625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="43.28515625" bestFit="1" customWidth="1"/>
+    <col min="23" max="26" width="30.42578125" customWidth="1"/>
+    <col min="27" max="27" width="35.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="33"/>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>77</v>
       </c>
-      <c r="C1" s="33"/>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="B2" t="s">
         <v>78</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" s="121"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>79</v>
       </c>
-      <c r="C2" s="118"/>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
+      <c r="B3" t="s">
         <v>80</v>
       </c>
-      <c r="B3" t="s">
-        <v>81</v>
-      </c>
-      <c r="C3" s="119"/>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="C3" s="122"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>14</v>
       </c>
       <c r="B4" t="s">
-        <v>82</v>
-      </c>
-      <c r="C4" s="119"/>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+        <v>81</v>
+      </c>
+      <c r="C4" s="122"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>18</v>
       </c>
       <c r="B5" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="119"/>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="C5" s="122"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>21</v>
       </c>
       <c r="B6" t="s">
         <v>20</v>
       </c>
-      <c r="C6" s="120"/>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="C6" s="123"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>23</v>
       </c>
@@ -2761,7 +2783,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>25</v>
       </c>
@@ -2769,23 +2791,23 @@
         <v>24</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>82</v>
+      </c>
+      <c r="B9" t="s">
         <v>83</v>
       </c>
-      <c r="B9" t="s">
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
+      <c r="B10" t="s">
         <v>85</v>
       </c>
-      <c r="B10" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -2793,7 +2815,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>1</v>
       </c>
@@ -2801,7 +2823,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>5</v>
       </c>
@@ -2809,120 +2831,120 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B14" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>87</v>
+      </c>
+      <c r="B15" t="s">
         <v>88</v>
       </c>
-      <c r="B15" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="17" spans="1:27" x14ac:dyDescent="0.35">
+    </row>
+    <row r="17" spans="1:27" x14ac:dyDescent="0.25">
       <c r="B17" s="32"/>
       <c r="C17" s="28"/>
     </row>
-    <row r="18" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="19" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A19" s="7" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="19" spans="1:27" x14ac:dyDescent="0.35">
-      <c r="A19" s="7" t="s">
+      <c r="B19" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="B19" s="8" t="s">
+      <c r="C19" s="34" t="s">
         <v>92</v>
       </c>
-      <c r="C19" s="34" t="s">
+      <c r="D19" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="D19" s="2" t="s">
+      <c r="E19" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="E19" s="2" t="s">
+      <c r="F19" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="F19" s="2" t="s">
+      <c r="G19" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="G19" s="2" t="s">
+      <c r="H19" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="H19" s="2" t="s">
+      <c r="I19" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="I19" s="2" t="s">
+      <c r="J19" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="J19" s="2" t="s">
+      <c r="K19" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="K19" s="2" t="s">
+      <c r="L19" s="2" t="s">
         <v>101</v>
-      </c>
-      <c r="L19" s="2" t="s">
-        <v>102</v>
       </c>
       <c r="M19" s="2" t="s">
         <v>33</v>
       </c>
       <c r="N19" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="O19" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="O19" s="2" t="s">
+      <c r="P19" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="P19" s="2" t="s">
+      <c r="Q19" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="Q19" s="2" t="s">
+      <c r="R19" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="R19" s="2" t="s">
+      <c r="S19" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="S19" s="2" t="s">
+      <c r="T19" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="T19" s="2" t="s">
+      <c r="U19" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="U19" s="2" t="s">
+      <c r="V19" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="V19" s="2" t="s">
+      <c r="W19" s="2" t="s">
         <v>111</v>
-      </c>
-      <c r="W19" s="2" t="s">
-        <v>112</v>
       </c>
       <c r="X19" s="2" t="s">
         <v>57</v>
       </c>
       <c r="Y19" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="Z19" s="2" t="s">
         <v>58</v>
       </c>
       <c r="AA19" s="2" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="20" spans="1:27" x14ac:dyDescent="0.35">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="20" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>40</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C20" s="25" t="s">
         <v>42</v>
@@ -2937,7 +2959,7 @@
         <v>47</v>
       </c>
       <c r="G20" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="H20" s="9" t="s">
         <v>48</v>
@@ -2949,7 +2971,7 @@
         <v>50</v>
       </c>
       <c r="K20" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="L20" t="s">
         <v>39</v>
@@ -2958,35 +2980,35 @@
         <v>45</v>
       </c>
       <c r="N20" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="O20" t="s">
         <v>65</v>
       </c>
       <c r="P20" t="s">
+        <v>118</v>
+      </c>
+      <c r="Q20" t="s">
         <v>119</v>
-      </c>
-      <c r="Q20" t="s">
-        <v>120</v>
       </c>
       <c r="R20" t="e">
         <f>IF(E20&gt;0,IF(E20="Unit",CONCATENATE(Settings!Q20," ",Settings!E20,"s"),CONCATENATE((Settings!Q20/Settings!M20)," ",Settings!E20,"s")),"")</f>
         <v>#VALUE!</v>
       </c>
       <c r="S20" s="35" t="s">
+        <v>120</v>
+      </c>
+      <c r="T20" s="35" t="s">
         <v>121</v>
       </c>
-      <c r="T20" s="35" t="s">
+      <c r="U20" s="35" t="s">
         <v>122</v>
-      </c>
-      <c r="U20" s="35" t="s">
-        <v>123</v>
       </c>
       <c r="V20" t="s">
         <v>52</v>
       </c>
       <c r="W20" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="X20" t="s">
         <v>62</v>
@@ -3001,7 +3023,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="21" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A21" s="3"/>
       <c r="B21" s="4"/>
       <c r="F21" s="9"/>
@@ -3013,7 +3035,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A22" s="3"/>
       <c r="B22" s="4"/>
       <c r="F22" s="9"/>
@@ -3025,7 +3047,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A23" s="3"/>
       <c r="B23" s="4"/>
       <c r="F23" s="9"/>
@@ -3037,7 +3059,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A24" s="3"/>
       <c r="B24" s="4"/>
       <c r="F24" s="9"/>
@@ -3049,7 +3071,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A25" s="3"/>
       <c r="B25" s="4"/>
       <c r="F25" s="9"/>
@@ -3061,7 +3083,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A26" s="3"/>
       <c r="B26" s="4"/>
       <c r="F26" s="9"/>
@@ -3073,7 +3095,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A27" s="3"/>
       <c r="B27" s="4"/>
       <c r="F27" s="9"/>
@@ -3085,7 +3107,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A28" s="3"/>
       <c r="B28" s="4"/>
       <c r="F28" s="9"/>
@@ -3097,7 +3119,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A29" s="3"/>
       <c r="B29" s="4"/>
       <c r="F29" s="9"/>
@@ -3109,7 +3131,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A30" s="3"/>
       <c r="B30" s="4"/>
       <c r="F30" s="9"/>
@@ -3121,7 +3143,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A31" s="3"/>
       <c r="B31" s="4"/>
       <c r="F31" s="9"/>
@@ -3133,7 +3155,7 @@
         <v/>
       </c>
     </row>
-    <row r="32" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A32" s="3"/>
       <c r="B32" s="4"/>
       <c r="F32" s="9"/>
@@ -3145,7 +3167,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A33" s="3"/>
       <c r="B33" s="4"/>
       <c r="F33" s="9"/>
@@ -3157,7 +3179,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A34" s="3"/>
       <c r="B34" s="4"/>
       <c r="F34" s="9"/>
@@ -3169,7 +3191,7 @@
         <v/>
       </c>
     </row>
-    <row r="35" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A35" s="3"/>
       <c r="B35" s="4"/>
       <c r="F35" s="9"/>
@@ -3181,7 +3203,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A36" s="3"/>
       <c r="B36" s="4"/>
       <c r="F36" s="9"/>
@@ -3193,7 +3215,7 @@
         <v/>
       </c>
     </row>
-    <row r="37" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A37" s="3"/>
       <c r="B37" s="4"/>
       <c r="F37" s="9"/>
@@ -3205,7 +3227,7 @@
         <v/>
       </c>
     </row>
-    <row r="38" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A38" s="3"/>
       <c r="B38" s="4"/>
       <c r="F38" s="9"/>
@@ -3217,7 +3239,7 @@
         <v/>
       </c>
     </row>
-    <row r="39" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A39" s="3"/>
       <c r="B39" s="4"/>
       <c r="F39" s="9"/>
@@ -3229,7 +3251,7 @@
         <v/>
       </c>
     </row>
-    <row r="40" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A40" s="3"/>
       <c r="B40" s="4"/>
       <c r="F40" s="9"/>
@@ -3241,7 +3263,7 @@
         <v/>
       </c>
     </row>
-    <row r="41" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A41" s="3"/>
       <c r="B41" s="4"/>
       <c r="F41" s="9"/>
@@ -3253,7 +3275,7 @@
         <v/>
       </c>
     </row>
-    <row r="42" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A42" s="3"/>
       <c r="B42" s="4"/>
       <c r="F42" s="9"/>
@@ -3265,7 +3287,7 @@
         <v/>
       </c>
     </row>
-    <row r="43" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A43" s="3"/>
       <c r="B43" s="4"/>
       <c r="F43" s="9"/>
@@ -3277,7 +3299,7 @@
         <v/>
       </c>
     </row>
-    <row r="44" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A44" s="3"/>
       <c r="B44" s="4"/>
       <c r="F44" s="9"/>
@@ -3289,7 +3311,7 @@
         <v/>
       </c>
     </row>
-    <row r="45" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A45" s="3"/>
       <c r="B45" s="4"/>
       <c r="F45" s="9"/>
@@ -3301,7 +3323,7 @@
         <v/>
       </c>
     </row>
-    <row r="46" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A46" s="3"/>
       <c r="B46" s="4"/>
       <c r="F46" s="9"/>
@@ -3313,7 +3335,7 @@
         <v/>
       </c>
     </row>
-    <row r="47" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A47" s="3"/>
       <c r="B47" s="4"/>
       <c r="F47" s="9"/>
@@ -3325,7 +3347,7 @@
         <v/>
       </c>
     </row>
-    <row r="48" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A48" s="3"/>
       <c r="B48" s="4"/>
       <c r="F48" s="9"/>
@@ -3337,7 +3359,7 @@
         <v/>
       </c>
     </row>
-    <row r="49" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A49" s="3"/>
       <c r="B49" s="4"/>
       <c r="F49" s="9"/>
@@ -3349,7 +3371,7 @@
         <v/>
       </c>
     </row>
-    <row r="50" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A50" s="3"/>
       <c r="B50" s="4"/>
       <c r="F50" s="9"/>
@@ -3361,7 +3383,7 @@
         <v/>
       </c>
     </row>
-    <row r="51" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A51" s="3"/>
       <c r="B51" s="4"/>
       <c r="F51" s="9"/>
@@ -3373,7 +3395,7 @@
         <v/>
       </c>
     </row>
-    <row r="52" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A52" s="3"/>
       <c r="B52" s="4"/>
       <c r="F52" s="9"/>
@@ -3385,7 +3407,7 @@
         <v/>
       </c>
     </row>
-    <row r="53" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A53" s="3"/>
       <c r="B53" s="4"/>
       <c r="F53" s="9"/>
@@ -3397,7 +3419,7 @@
         <v/>
       </c>
     </row>
-    <row r="54" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A54" s="5"/>
       <c r="B54" s="6"/>
       <c r="F54" s="9"/>
@@ -3428,17 +3450,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <SharedWithUsers xmlns="1444eecc-14bb-4066-abe6-ce6de21d9439">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3639,20 +3656,23 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <SharedWithUsers xmlns="1444eecc-14bb-4066-abe6-ce6de21d9439">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7EBE950A-5812-419E-B174-6A5D9B8E0414}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A00E6A9-20DD-4842-9306-307EB080AF2E}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="1444eecc-14bb-4066-abe6-ce6de21d9439"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -3677,9 +3697,11 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A00E6A9-20DD-4842-9306-307EB080AF2E}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7EBE950A-5812-419E-B174-6A5D9B8E0414}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="1444eecc-14bb-4066-abe6-ce6de21d9439"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Updated Thailand template with new data
</commit_message>
<xml_diff>
--- a/srv/xlsx-templates/TH - Quotation Template.xlsx
+++ b/srv/xlsx-templates/TH - Quotation Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27531"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EHMHV\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F63A248-C45E-45EF-B0F8-F57C0B341C6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA20D76F-F558-4467-BD1E-506ADB44BDCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="19170" windowHeight="8520" xr2:uid="{F5CC2154-27BB-4652-B61E-D913F0CC6809}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{F5CC2154-27BB-4652-B61E-D913F0CC6809}"/>
   </bookViews>
   <sheets>
     <sheet name="Quotation" sheetId="3" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="149">
   <si>
     <t>Offered Party</t>
   </si>
@@ -252,9 +252,6 @@
     <t>Validity Period (กำหนดยืนราคา)</t>
   </si>
   <si>
-    <t>years (ปี)</t>
-  </si>
-  <si>
     <t>Delivery Due (กำหนดส่งสินค้า)</t>
   </si>
   <si>
@@ -478,6 +475,15 @@
   </si>
   <si>
     <t>${table:offerProductValidation.ItemNumber}</t>
+  </si>
+  <si>
+    <t>${offerValidation.ContractLength}</t>
+  </si>
+  <si>
+    <t>${offerValidation.ContractLenghtUnit}</t>
+  </si>
+  <si>
+    <t>${offerValidation.Unitofdeliverydue}</t>
   </si>
 </sst>
 </file>
@@ -881,7 +887,6 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -963,6 +968,9 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="4" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -987,9 +995,24 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -999,9 +1022,6 @@
     <xf numFmtId="49" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="43" fontId="6" fillId="0" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1017,15 +1037,9 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1083,9 +1097,6 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -1097,9 +1108,6 @@
     </xf>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -1701,24 +1709,24 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFBA1999-1CF9-4903-BA7D-DD523B82D6C3}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="B2:O53"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="12" customWidth="1"/>
-    <col min="3" max="3" width="15.7109375" customWidth="1"/>
-    <col min="4" max="4" width="33.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="52.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.85546875" customWidth="1"/>
+    <col min="3" max="3" width="15.7265625" customWidth="1"/>
+    <col min="4" max="4" width="33.26953125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="52.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.81640625" customWidth="1"/>
     <col min="7" max="7" width="17" customWidth="1"/>
-    <col min="8" max="8" width="24.5703125" customWidth="1"/>
-    <col min="9" max="9" width="14.7109375" customWidth="1"/>
-    <col min="10" max="10" width="21.28515625" customWidth="1"/>
-    <col min="11" max="11" width="14.85546875" customWidth="1"/>
-    <col min="12" max="12" width="12.5703125" customWidth="1"/>
+    <col min="8" max="8" width="24.54296875" customWidth="1"/>
+    <col min="9" max="9" width="14.7265625" customWidth="1"/>
+    <col min="10" max="10" width="21.26953125" customWidth="1"/>
+    <col min="11" max="11" width="14.81640625" customWidth="1"/>
+    <col min="12" max="12" width="12.54296875" customWidth="1"/>
     <col min="13" max="13" width="27" customWidth="1"/>
-    <col min="14" max="14" width="34.140625" customWidth="1"/>
+    <col min="14" max="14" width="34.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B2" s="10"/>
       <c r="C2" s="10"/>
       <c r="D2" s="10"/>
@@ -1733,83 +1741,83 @@
       <c r="M2" s="10"/>
       <c r="N2" s="10"/>
     </row>
-    <row r="3" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B3" s="26" t="s">
+    <row r="3" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B3" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="75" t="s">
+      <c r="C3" s="77" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="76"/>
-      <c r="E3" s="76"/>
-      <c r="F3" s="76"/>
-      <c r="G3" s="77"/>
+      <c r="D3" s="78"/>
+      <c r="E3" s="78"/>
+      <c r="F3" s="78"/>
+      <c r="G3" s="79"/>
       <c r="H3" s="10"/>
-      <c r="I3" s="26" t="s">
+      <c r="I3" s="25" t="s">
         <v>2</v>
       </c>
-      <c r="J3" s="75" t="s">
+      <c r="J3" s="77" t="s">
         <v>3</v>
       </c>
-      <c r="K3" s="76"/>
-      <c r="L3" s="76"/>
-      <c r="M3" s="77"/>
+      <c r="K3" s="78"/>
+      <c r="L3" s="78"/>
+      <c r="M3" s="79"/>
       <c r="N3" s="10"/>
     </row>
-    <row r="4" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="27" t="s">
+    <row r="4" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B4" s="26" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="78" t="s">
+      <c r="C4" s="80" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="79"/>
-      <c r="E4" s="79"/>
-      <c r="F4" s="79"/>
-      <c r="G4" s="80"/>
+      <c r="D4" s="81"/>
+      <c r="E4" s="81"/>
+      <c r="F4" s="81"/>
+      <c r="G4" s="82"/>
       <c r="H4" s="10"/>
-      <c r="I4" s="26" t="s">
+      <c r="I4" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="J4" s="86" t="s">
+      <c r="J4" s="88" t="s">
         <v>6</v>
       </c>
-      <c r="K4" s="87"/>
-      <c r="L4" s="87"/>
-      <c r="M4" s="88"/>
+      <c r="K4" s="89"/>
+      <c r="L4" s="89"/>
+      <c r="M4" s="90"/>
       <c r="N4" s="10"/>
     </row>
-    <row r="5" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="45"/>
-      <c r="C5" s="45"/>
-      <c r="D5" s="45"/>
-      <c r="E5" s="45"/>
-      <c r="F5" s="45"/>
-      <c r="G5" s="45"/>
+    <row r="5" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B5" s="44"/>
+      <c r="C5" s="44"/>
+      <c r="D5" s="44"/>
+      <c r="E5" s="44"/>
+      <c r="F5" s="44"/>
+      <c r="G5" s="44"/>
       <c r="H5" s="10"/>
       <c r="I5" s="10"/>
-      <c r="J5" s="46"/>
-      <c r="K5" s="46"/>
-      <c r="L5" s="46"/>
-      <c r="M5" s="46"/>
+      <c r="J5" s="45"/>
+      <c r="K5" s="45"/>
+      <c r="L5" s="45"/>
+      <c r="M5" s="45"/>
       <c r="N5" s="10"/>
     </row>
-    <row r="6" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="45"/>
-      <c r="C6" s="45"/>
-      <c r="D6" s="45"/>
-      <c r="E6" s="45"/>
-      <c r="F6" s="45"/>
-      <c r="G6" s="45"/>
+    <row r="6" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B6" s="44"/>
+      <c r="C6" s="44"/>
+      <c r="D6" s="44"/>
+      <c r="E6" s="44"/>
+      <c r="F6" s="44"/>
+      <c r="G6" s="44"/>
       <c r="H6" s="10"/>
       <c r="I6" s="10"/>
-      <c r="J6" s="46"/>
-      <c r="K6" s="46"/>
-      <c r="L6" s="46"/>
-      <c r="M6" s="46"/>
+      <c r="J6" s="45"/>
+      <c r="K6" s="45"/>
+      <c r="L6" s="45"/>
+      <c r="M6" s="45"/>
       <c r="N6" s="10"/>
     </row>
-    <row r="7" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B7" s="10"/>
       <c r="C7" s="10"/>
       <c r="D7" s="10"/>
@@ -1824,111 +1832,111 @@
       <c r="M7" s="10"/>
       <c r="N7" s="10"/>
     </row>
-    <row r="8" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B8" s="81" t="s">
-        <v>135</v>
-      </c>
-      <c r="C8" s="82"/>
-      <c r="D8" s="82"/>
-      <c r="E8" s="82"/>
-      <c r="F8" s="82"/>
-      <c r="G8" s="82"/>
-      <c r="H8" s="82"/>
-      <c r="I8" s="82"/>
-      <c r="J8" s="82"/>
-      <c r="K8" s="82"/>
-      <c r="L8" s="82"/>
-      <c r="M8" s="82"/>
-      <c r="N8" s="83"/>
-    </row>
-    <row r="9" spans="2:14" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="B9" s="89" t="s">
+    <row r="8" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B8" s="83" t="s">
+        <v>134</v>
+      </c>
+      <c r="C8" s="84"/>
+      <c r="D8" s="84"/>
+      <c r="E8" s="84"/>
+      <c r="F8" s="84"/>
+      <c r="G8" s="84"/>
+      <c r="H8" s="84"/>
+      <c r="I8" s="84"/>
+      <c r="J8" s="84"/>
+      <c r="K8" s="84"/>
+      <c r="L8" s="84"/>
+      <c r="M8" s="84"/>
+      <c r="N8" s="85"/>
+    </row>
+    <row r="9" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B9" s="91" t="s">
         <v>7</v>
       </c>
-      <c r="C9" s="90"/>
+      <c r="C9" s="92"/>
       <c r="D9" s="99" t="s">
         <v>8</v>
       </c>
       <c r="E9" s="99"/>
-      <c r="F9" s="40"/>
-      <c r="G9" s="42" t="s">
+      <c r="F9" s="39"/>
+      <c r="G9" s="41" t="s">
         <v>9</v>
       </c>
-      <c r="H9" s="42"/>
-      <c r="I9" s="94" t="s">
+      <c r="H9" s="41"/>
+      <c r="I9" s="95" t="s">
         <v>10</v>
       </c>
-      <c r="J9" s="94"/>
-      <c r="K9" s="95"/>
-      <c r="L9" s="84" t="s">
+      <c r="J9" s="95"/>
+      <c r="K9" s="96"/>
+      <c r="L9" s="86" t="s">
         <v>11</v>
       </c>
-      <c r="M9" s="85"/>
-      <c r="N9" s="52" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="10" spans="2:14" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="91" t="s">
+      <c r="M9" s="87"/>
+      <c r="N9" s="51" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="10" spans="2:14" ht="26.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B10" s="93" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="92"/>
+      <c r="C10" s="94"/>
       <c r="D10" s="100" t="str">
         <f>Settings!A14</f>
         <v>${offerValidation.CUSTOMER_CODE}</v>
       </c>
       <c r="E10" s="100"/>
-      <c r="F10" s="40"/>
+      <c r="F10" s="39"/>
       <c r="G10" s="101" t="s">
         <v>13</v>
       </c>
       <c r="H10" s="101"/>
-      <c r="I10" s="96" t="s">
+      <c r="I10" s="97" t="s">
         <v>14</v>
       </c>
-      <c r="J10" s="96"/>
-      <c r="K10" s="97"/>
-      <c r="L10" s="68" t="s">
+      <c r="J10" s="97"/>
+      <c r="K10" s="98"/>
+      <c r="L10" s="72" t="s">
         <v>15</v>
       </c>
-      <c r="M10" s="69"/>
-      <c r="N10" s="52" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="11" spans="2:14" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="91" t="s">
+      <c r="M10" s="73"/>
+      <c r="N10" s="51" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="11" spans="2:14" ht="26.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B11" s="93" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="92"/>
-      <c r="D11" s="78" t="str">
+      <c r="C11" s="94"/>
+      <c r="D11" s="80" t="str">
         <f>Settings!A9</f>
         <v>${offerValidation.INSTITUTENAME}</v>
       </c>
-      <c r="E11" s="80"/>
-      <c r="F11" s="40"/>
+      <c r="E11" s="82"/>
+      <c r="F11" s="39"/>
       <c r="G11" s="102" t="s">
         <v>17</v>
       </c>
       <c r="H11" s="102"/>
-      <c r="I11" s="96" t="s">
+      <c r="I11" s="97" t="s">
         <v>18</v>
       </c>
-      <c r="J11" s="96"/>
-      <c r="K11" s="97"/>
-      <c r="L11" s="68" t="s">
+      <c r="J11" s="97"/>
+      <c r="K11" s="98"/>
+      <c r="L11" s="72" t="s">
         <v>19</v>
       </c>
-      <c r="M11" s="69"/>
-      <c r="N11" s="52" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="12" spans="2:14" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="B12" s="91" t="s">
+      <c r="M11" s="73"/>
+      <c r="N11" s="51" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="12" spans="2:14" ht="26" x14ac:dyDescent="0.35">
+      <c r="B12" s="93" t="s">
         <v>20</v>
       </c>
-      <c r="C12" s="92"/>
+      <c r="C12" s="94"/>
       <c r="D12" s="103" t="s">
         <v>21</v>
       </c>
@@ -1943,35 +1951,35 @@
       </c>
       <c r="J12" s="54"/>
       <c r="K12" s="55"/>
-      <c r="L12" s="68" t="s">
+      <c r="L12" s="72" t="s">
         <v>15</v>
       </c>
-      <c r="M12" s="69"/>
-      <c r="N12" s="52" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="13" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B13" s="91" t="s">
+      <c r="M12" s="73"/>
+      <c r="N12" s="51" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="13" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B13" s="93" t="s">
         <v>24</v>
       </c>
-      <c r="C13" s="92"/>
+      <c r="C13" s="94"/>
       <c r="D13" s="103" t="s">
         <v>25</v>
       </c>
       <c r="E13" s="59"/>
       <c r="F13" s="10"/>
       <c r="G13" s="53" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="H13" s="53"/>
       <c r="I13" s="54" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="J13" s="54"/>
       <c r="K13" s="55"/>
     </row>
-    <row r="14" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B14" s="10"/>
       <c r="C14" s="10"/>
       <c r="D14" s="10"/>
@@ -1983,89 +1991,89 @@
       <c r="J14" s="10"/>
       <c r="K14" s="10"/>
     </row>
-    <row r="15" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B15" s="67" t="s">
+    <row r="15" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B15" s="71" t="s">
         <v>26</v>
       </c>
-      <c r="C15" s="67"/>
-      <c r="D15" s="67"/>
-      <c r="E15" s="67"/>
-      <c r="F15" s="67"/>
-      <c r="G15" s="67"/>
-      <c r="H15" s="67"/>
-      <c r="I15" s="67"/>
-      <c r="J15" s="67"/>
-      <c r="K15" s="67"/>
-      <c r="L15" s="67"/>
-      <c r="M15" s="67"/>
-      <c r="N15" s="67"/>
-    </row>
-    <row r="16" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B16" s="93" t="s">
+      <c r="C15" s="71"/>
+      <c r="D15" s="71"/>
+      <c r="E15" s="71"/>
+      <c r="F15" s="71"/>
+      <c r="G15" s="71"/>
+      <c r="H15" s="71"/>
+      <c r="I15" s="71"/>
+      <c r="J15" s="71"/>
+      <c r="K15" s="71"/>
+      <c r="L15" s="71"/>
+      <c r="M15" s="71"/>
+      <c r="N15" s="71"/>
+    </row>
+    <row r="16" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B16" s="62" t="s">
         <v>27</v>
       </c>
-      <c r="C16" s="61" t="s">
+      <c r="C16" s="63" t="s">
         <v>28</v>
       </c>
-      <c r="D16" s="61" t="s">
+      <c r="D16" s="63" t="s">
         <v>29</v>
       </c>
-      <c r="E16" s="61" t="s">
+      <c r="E16" s="63" t="s">
         <v>30</v>
       </c>
-      <c r="F16" s="61" t="s">
+      <c r="F16" s="63" t="s">
         <v>31</v>
       </c>
-      <c r="G16" s="61" t="s">
+      <c r="G16" s="63" t="s">
         <v>32</v>
       </c>
-      <c r="H16" s="71" t="s">
+      <c r="H16" s="65" t="s">
         <v>33</v>
       </c>
-      <c r="I16" s="61" t="s">
+      <c r="I16" s="63" t="s">
         <v>34</v>
       </c>
-      <c r="J16" s="61" t="s">
+      <c r="J16" s="63" t="s">
         <v>35</v>
       </c>
-      <c r="K16" s="61"/>
-      <c r="L16" s="61"/>
-      <c r="M16" s="61" t="s">
+      <c r="K16" s="63"/>
+      <c r="L16" s="63"/>
+      <c r="M16" s="63" t="s">
         <v>36</v>
       </c>
-      <c r="N16" s="61"/>
-    </row>
-    <row r="17" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B17" s="93"/>
-      <c r="C17" s="61"/>
-      <c r="D17" s="61"/>
-      <c r="E17" s="61"/>
-      <c r="F17" s="61"/>
-      <c r="G17" s="61"/>
-      <c r="H17" s="72"/>
-      <c r="I17" s="61"/>
-      <c r="J17" s="61"/>
-      <c r="K17" s="61"/>
-      <c r="L17" s="61"/>
-      <c r="M17" s="61"/>
-      <c r="N17" s="61"/>
-    </row>
-    <row r="18" spans="2:15" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="93"/>
-      <c r="C18" s="61"/>
-      <c r="D18" s="61"/>
-      <c r="E18" s="61"/>
-      <c r="F18" s="61"/>
-      <c r="G18" s="61"/>
-      <c r="H18" s="73"/>
-      <c r="I18" s="61"/>
+      <c r="N16" s="63"/>
+    </row>
+    <row r="17" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="B17" s="62"/>
+      <c r="C17" s="63"/>
+      <c r="D17" s="63"/>
+      <c r="E17" s="63"/>
+      <c r="F17" s="63"/>
+      <c r="G17" s="63"/>
+      <c r="H17" s="75"/>
+      <c r="I17" s="63"/>
+      <c r="J17" s="63"/>
+      <c r="K17" s="63"/>
+      <c r="L17" s="63"/>
+      <c r="M17" s="63"/>
+      <c r="N17" s="63"/>
+    </row>
+    <row r="18" spans="2:15" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B18" s="62"/>
+      <c r="C18" s="63"/>
+      <c r="D18" s="63"/>
+      <c r="E18" s="63"/>
+      <c r="F18" s="63"/>
+      <c r="G18" s="63"/>
+      <c r="H18" s="66"/>
+      <c r="I18" s="63"/>
       <c r="J18" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="K18" s="70" t="s">
+      <c r="K18" s="74" t="s">
         <v>38</v>
       </c>
-      <c r="L18" s="70"/>
+      <c r="L18" s="74"/>
       <c r="M18" s="11" t="s">
         <v>37</v>
       </c>
@@ -2073,83 +2081,83 @@
         <v>38</v>
       </c>
     </row>
-    <row r="19" spans="2:15" ht="30" x14ac:dyDescent="0.25">
-      <c r="B19" s="25" t="s">
+    <row r="19" spans="2:15" ht="29" x14ac:dyDescent="0.35">
+      <c r="B19" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="C19" s="25" t="s">
-        <v>124</v>
-      </c>
-      <c r="D19" s="39" t="s">
+      <c r="C19" s="24" t="s">
+        <v>123</v>
+      </c>
+      <c r="D19" s="38" t="s">
         <v>41</v>
       </c>
-      <c r="E19" s="39" t="s">
+      <c r="E19" s="38" t="s">
         <v>42</v>
       </c>
-      <c r="F19" s="37" t="s">
+      <c r="F19" s="36" t="s">
         <v>43</v>
       </c>
-      <c r="G19" s="37" t="s">
+      <c r="G19" s="36" t="s">
         <v>44</v>
       </c>
-      <c r="H19" s="37" t="s">
+      <c r="H19" s="36" t="s">
         <v>45</v>
       </c>
-      <c r="I19" s="37" t="s">
+      <c r="I19" s="36" t="s">
         <v>46</v>
       </c>
-      <c r="J19" s="37" t="s">
+      <c r="J19" s="36" t="s">
         <v>47</v>
       </c>
-      <c r="K19" s="74" t="s">
+      <c r="K19" s="76" t="s">
         <v>48</v>
       </c>
-      <c r="L19" s="74"/>
-      <c r="M19" s="41" t="s">
+      <c r="L19" s="76"/>
+      <c r="M19" s="40" t="s">
         <v>49</v>
       </c>
-      <c r="N19" s="41" t="s">
+      <c r="N19" s="40" t="s">
         <v>50</v>
       </c>
-      <c r="O19" s="31"/>
-    </row>
-    <row r="20" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="O19" s="30"/>
+    </row>
+    <row r="20" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B20" s="12"/>
       <c r="C20" s="12"/>
       <c r="D20" s="12"/>
-      <c r="E20" s="30"/>
+      <c r="E20" s="29"/>
       <c r="F20" s="12"/>
-      <c r="G20" s="25"/>
+      <c r="G20" s="24"/>
       <c r="H20" s="13"/>
       <c r="I20" s="12"/>
       <c r="J20" s="15"/>
       <c r="K20" s="104"/>
       <c r="L20" s="104"/>
       <c r="M20" s="14"/>
-      <c r="N20" s="36"/>
-    </row>
-    <row r="21" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="N20" s="35"/>
+    </row>
+    <row r="21" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B21" s="12"/>
       <c r="C21" s="12"/>
       <c r="D21" s="12"/>
-      <c r="E21" s="30"/>
+      <c r="E21" s="29"/>
       <c r="F21" s="12"/>
-      <c r="G21" s="25"/>
+      <c r="G21" s="24"/>
       <c r="H21" s="13"/>
       <c r="I21" s="12"/>
       <c r="J21" s="15"/>
-      <c r="K21" s="66" t="s">
+      <c r="K21" s="70" t="s">
         <v>51</v>
       </c>
-      <c r="L21" s="66"/>
-      <c r="M21" s="37" t="s">
+      <c r="L21" s="70"/>
+      <c r="M21" s="36" t="s">
         <v>52</v>
       </c>
-      <c r="N21" s="37" t="s">
+      <c r="N21" s="36" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="22" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B22" s="10"/>
       <c r="C22" s="10"/>
       <c r="D22" s="10"/>
@@ -2164,117 +2172,117 @@
       <c r="M22" s="10"/>
       <c r="N22" s="10"/>
     </row>
-    <row r="23" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B23" s="98" t="s">
+    <row r="23" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="B23" s="61" t="s">
         <v>54</v>
       </c>
-      <c r="C23" s="98"/>
-      <c r="D23" s="98"/>
-      <c r="E23" s="98"/>
-      <c r="F23" s="98"/>
-      <c r="G23" s="98"/>
-      <c r="H23" s="98"/>
-      <c r="I23" s="98"/>
-      <c r="J23" s="98"/>
-      <c r="K23" s="98"/>
-      <c r="L23" s="98"/>
+      <c r="C23" s="61"/>
+      <c r="D23" s="61"/>
+      <c r="E23" s="61"/>
+      <c r="F23" s="61"/>
+      <c r="G23" s="61"/>
+      <c r="H23" s="61"/>
+      <c r="I23" s="61"/>
+      <c r="J23" s="61"/>
+      <c r="K23" s="61"/>
+      <c r="L23" s="61"/>
       <c r="M23" s="10"/>
     </row>
-    <row r="24" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B24" s="93" t="s">
+    <row r="24" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="B24" s="62" t="s">
         <v>27</v>
       </c>
-      <c r="C24" s="61" t="s">
+      <c r="C24" s="63" t="s">
         <v>28</v>
       </c>
-      <c r="D24" s="71" t="s">
-        <v>127</v>
-      </c>
-      <c r="E24" s="61" t="s">
+      <c r="D24" s="65" t="s">
+        <v>126</v>
+      </c>
+      <c r="E24" s="63" t="s">
         <v>55</v>
       </c>
-      <c r="F24" s="61" t="s">
+      <c r="F24" s="63" t="s">
         <v>56</v>
       </c>
-      <c r="G24" s="61" t="s">
+      <c r="G24" s="63" t="s">
         <v>57</v>
       </c>
-      <c r="H24" s="61" t="s">
+      <c r="H24" s="63" t="s">
         <v>58</v>
       </c>
-      <c r="I24" s="61"/>
-      <c r="J24" s="61"/>
-      <c r="K24" s="61" t="s">
+      <c r="I24" s="63"/>
+      <c r="J24" s="63"/>
+      <c r="K24" s="63" t="s">
         <v>59</v>
       </c>
-      <c r="L24" s="61"/>
-      <c r="M24" s="61" t="s">
+      <c r="L24" s="63"/>
+      <c r="M24" s="63" t="s">
         <v>60</v>
       </c>
       <c r="N24" s="10"/>
     </row>
-    <row r="25" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B25" s="93"/>
-      <c r="C25" s="61"/>
-      <c r="D25" s="73"/>
-      <c r="E25" s="61"/>
-      <c r="F25" s="61"/>
-      <c r="G25" s="61"/>
-      <c r="H25" s="61"/>
-      <c r="I25" s="61"/>
-      <c r="J25" s="61"/>
-      <c r="K25" s="61"/>
-      <c r="L25" s="61"/>
-      <c r="M25" s="61"/>
+    <row r="25" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="B25" s="62"/>
+      <c r="C25" s="63"/>
+      <c r="D25" s="66"/>
+      <c r="E25" s="63"/>
+      <c r="F25" s="63"/>
+      <c r="G25" s="63"/>
+      <c r="H25" s="63"/>
+      <c r="I25" s="63"/>
+      <c r="J25" s="63"/>
+      <c r="K25" s="63"/>
+      <c r="L25" s="63"/>
+      <c r="M25" s="63"/>
       <c r="N25" s="10"/>
     </row>
-    <row r="26" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B26" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="C26" s="37" t="s">
-        <v>124</v>
-      </c>
-      <c r="D26" s="37" t="s">
-        <v>146</v>
-      </c>
-      <c r="E26" s="43"/>
-      <c r="F26" s="38" t="s">
+      <c r="C26" s="36" t="s">
+        <v>123</v>
+      </c>
+      <c r="D26" s="36" t="s">
+        <v>145</v>
+      </c>
+      <c r="E26" s="42"/>
+      <c r="F26" s="37" t="s">
         <v>61</v>
       </c>
       <c r="G26" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="H26" s="65" t="s">
+      <c r="H26" s="64" t="s">
         <v>63</v>
       </c>
-      <c r="I26" s="65"/>
-      <c r="J26" s="65"/>
-      <c r="K26" s="65" t="s">
+      <c r="I26" s="64"/>
+      <c r="J26" s="64"/>
+      <c r="K26" s="64" t="s">
         <v>64</v>
       </c>
-      <c r="L26" s="65"/>
+      <c r="L26" s="64"/>
       <c r="M26" s="16" t="s">
         <v>65</v>
       </c>
       <c r="N26" s="10"/>
     </row>
-    <row r="27" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B27" s="16"/>
       <c r="C27" s="16"/>
       <c r="D27" s="16"/>
       <c r="E27" s="16"/>
       <c r="F27" s="16"/>
       <c r="G27" s="16"/>
-      <c r="H27" s="62"/>
-      <c r="I27" s="63"/>
-      <c r="J27" s="64"/>
-      <c r="K27" s="65"/>
-      <c r="L27" s="65"/>
+      <c r="H27" s="67"/>
+      <c r="I27" s="68"/>
+      <c r="J27" s="69"/>
+      <c r="K27" s="64"/>
+      <c r="L27" s="64"/>
       <c r="M27" s="16"/>
       <c r="N27" s="10"/>
     </row>
-    <row r="28" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B28" s="16"/>
       <c r="C28" s="16"/>
       <c r="D28" s="16"/>
@@ -2284,12 +2292,12 @@
       <c r="H28" s="120"/>
       <c r="I28" s="120"/>
       <c r="J28" s="120"/>
-      <c r="K28" s="65"/>
-      <c r="L28" s="65"/>
+      <c r="K28" s="64"/>
+      <c r="L28" s="64"/>
       <c r="M28" s="16"/>
       <c r="N28" s="10"/>
     </row>
-    <row r="29" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B29" s="10"/>
       <c r="C29" s="10"/>
       <c r="D29" s="17"/>
@@ -2304,7 +2312,7 @@
       <c r="M29" s="10"/>
       <c r="N29" s="10"/>
     </row>
-    <row r="30" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B30" s="117" t="s">
         <v>66</v>
       </c>
@@ -2317,17 +2325,17 @@
       </c>
       <c r="H30" s="119"/>
       <c r="I30" s="56" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="J30" s="57"/>
-      <c r="K30" s="27" t="s">
+      <c r="K30" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="L30" s="27"/>
+      <c r="L30" s="26"/>
       <c r="M30" s="10"/>
       <c r="N30" s="10"/>
     </row>
-    <row r="31" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B31" s="19" t="s">
         <v>68</v>
       </c>
@@ -2336,27 +2344,27 @@
       <c r="E31" s="114"/>
       <c r="F31" s="10"/>
       <c r="G31" s="115" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="H31" s="116"/>
       <c r="I31" s="60" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="J31" s="60"/>
       <c r="K31" s="58" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="L31" s="59"/>
       <c r="M31" s="10"/>
       <c r="N31" s="10"/>
     </row>
-    <row r="32" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B32" s="19" t="s">
         <v>69</v>
       </c>
       <c r="C32" s="20"/>
-      <c r="D32" s="65"/>
-      <c r="E32" s="65"/>
+      <c r="D32" s="64"/>
+      <c r="E32" s="64"/>
       <c r="F32" s="10"/>
       <c r="G32" s="10"/>
       <c r="H32" s="10"/>
@@ -2367,14 +2375,16 @@
       <c r="M32" s="10"/>
       <c r="N32" s="10"/>
     </row>
-    <row r="33" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B33" s="19" t="s">
         <v>70</v>
       </c>
       <c r="C33" s="20"/>
-      <c r="D33" s="16"/>
-      <c r="E33" s="21" t="s">
-        <v>71</v>
+      <c r="D33" s="16" t="s">
+        <v>146</v>
+      </c>
+      <c r="E33" s="16" t="s">
+        <v>147</v>
       </c>
       <c r="F33" s="10"/>
       <c r="G33" s="10"/>
@@ -2386,16 +2396,16 @@
       <c r="M33" s="10"/>
       <c r="N33" s="10"/>
     </row>
-    <row r="34" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B34" s="22" t="s">
-        <v>72</v>
-      </c>
-      <c r="C34" s="23"/>
+    <row r="34" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B34" s="21" t="s">
+        <v>71</v>
+      </c>
+      <c r="C34" s="22"/>
       <c r="D34" s="16" t="s">
-        <v>140</v>
-      </c>
-      <c r="E34" s="21" t="s">
-        <v>71</v>
+        <v>139</v>
+      </c>
+      <c r="E34" s="16" t="s">
+        <v>148</v>
       </c>
       <c r="F34" s="10"/>
       <c r="G34" s="10"/>
@@ -2405,7 +2415,7 @@
       <c r="K34" s="10"/>
       <c r="L34" s="10"/>
     </row>
-    <row r="35" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B35" s="10"/>
       <c r="C35" s="10"/>
       <c r="D35" s="10"/>
@@ -2420,186 +2430,186 @@
       <c r="M35" s="10"/>
       <c r="N35" s="10"/>
     </row>
-    <row r="36" spans="2:14" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="B36" s="47" t="s">
+    <row r="36" spans="2:14" ht="39" x14ac:dyDescent="0.35">
+      <c r="B36" s="46" t="s">
+        <v>72</v>
+      </c>
+      <c r="C36" s="47"/>
+      <c r="D36" s="47"/>
+      <c r="E36" s="48"/>
+      <c r="F36" s="28"/>
+      <c r="G36" s="49" t="s">
+        <v>125</v>
+      </c>
+      <c r="H36" s="50" t="s">
+        <v>130</v>
+      </c>
+      <c r="I36" s="28"/>
+      <c r="J36" s="28"/>
+    </row>
+    <row r="37" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B37" s="105" t="s">
         <v>73</v>
-      </c>
-      <c r="C36" s="48"/>
-      <c r="D36" s="48"/>
-      <c r="E36" s="49"/>
-      <c r="F36" s="29"/>
-      <c r="G36" s="50" t="s">
-        <v>126</v>
-      </c>
-      <c r="H36" s="51" t="s">
-        <v>131</v>
-      </c>
-      <c r="I36" s="29"/>
-      <c r="J36" s="29"/>
-    </row>
-    <row r="37" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B37" s="105" t="s">
-        <v>74</v>
       </c>
       <c r="C37" s="106"/>
       <c r="D37" s="106"/>
       <c r="E37" s="107"/>
-      <c r="F37" s="29"/>
-      <c r="G37" s="50" t="s">
-        <v>128</v>
-      </c>
-      <c r="H37" s="51" t="s">
-        <v>132</v>
-      </c>
-      <c r="I37" s="29"/>
-      <c r="J37" s="29"/>
-    </row>
-    <row r="38" spans="2:14" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="F37" s="28"/>
+      <c r="G37" s="49" t="s">
+        <v>127</v>
+      </c>
+      <c r="H37" s="50" t="s">
+        <v>131</v>
+      </c>
+      <c r="I37" s="28"/>
+      <c r="J37" s="28"/>
+    </row>
+    <row r="38" spans="2:14" ht="26" x14ac:dyDescent="0.35">
       <c r="B38" s="108"/>
       <c r="C38" s="109"/>
       <c r="D38" s="109"/>
       <c r="E38" s="110"/>
-      <c r="F38" s="29"/>
-      <c r="G38" s="50" t="s">
-        <v>129</v>
-      </c>
-      <c r="H38" s="51" t="s">
-        <v>133</v>
-      </c>
-      <c r="I38" s="29"/>
-      <c r="J38" s="29"/>
-    </row>
-    <row r="39" spans="2:14" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="F38" s="28"/>
+      <c r="G38" s="49" t="s">
+        <v>128</v>
+      </c>
+      <c r="H38" s="50" t="s">
+        <v>132</v>
+      </c>
+      <c r="I38" s="28"/>
+      <c r="J38" s="28"/>
+    </row>
+    <row r="39" spans="2:14" ht="26" x14ac:dyDescent="0.35">
       <c r="B39" s="108"/>
       <c r="C39" s="109"/>
       <c r="D39" s="109"/>
       <c r="E39" s="110"/>
-      <c r="F39" s="29"/>
-      <c r="G39" s="50" t="s">
-        <v>130</v>
-      </c>
-      <c r="H39" s="51" t="s">
-        <v>134</v>
-      </c>
-      <c r="I39" s="29"/>
-      <c r="J39" s="29"/>
-    </row>
-    <row r="40" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="F39" s="28"/>
+      <c r="G39" s="49" t="s">
+        <v>129</v>
+      </c>
+      <c r="H39" s="52" t="s">
+        <v>133</v>
+      </c>
+      <c r="I39" s="28"/>
+      <c r="J39" s="28"/>
+    </row>
+    <row r="40" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B40" s="108"/>
       <c r="C40" s="109"/>
       <c r="D40" s="109"/>
       <c r="E40" s="110"/>
-      <c r="F40" s="29"/>
-      <c r="G40" s="29"/>
-      <c r="H40" s="29"/>
-      <c r="I40" s="29"/>
-      <c r="J40" s="29"/>
-    </row>
-    <row r="41" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="F40" s="28"/>
+      <c r="G40" s="28"/>
+      <c r="H40" s="28"/>
+      <c r="I40" s="28"/>
+      <c r="J40" s="28"/>
+    </row>
+    <row r="41" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B41" s="111"/>
       <c r="C41" s="112"/>
       <c r="D41" s="112"/>
       <c r="E41" s="113"/>
-      <c r="F41" s="29"/>
-      <c r="G41" s="29"/>
+      <c r="F41" s="28"/>
+      <c r="G41" s="28"/>
       <c r="H41" s="10"/>
-      <c r="I41" s="29"/>
-      <c r="J41" s="29"/>
-    </row>
-    <row r="42" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B42" s="29"/>
-      <c r="C42" s="29"/>
-      <c r="D42" s="29"/>
-      <c r="E42" s="29"/>
-      <c r="F42" s="29"/>
-      <c r="G42" s="29"/>
+      <c r="I41" s="28"/>
+      <c r="J41" s="28"/>
+    </row>
+    <row r="42" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B42" s="28"/>
+      <c r="C42" s="28"/>
+      <c r="D42" s="28"/>
+      <c r="E42" s="28"/>
+      <c r="F42" s="28"/>
+      <c r="G42" s="28"/>
       <c r="H42" s="10"/>
       <c r="I42" s="10"/>
       <c r="J42" s="10"/>
     </row>
-    <row r="43" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B43" s="29"/>
-      <c r="C43" s="29"/>
-      <c r="D43" s="29"/>
-      <c r="E43" s="29"/>
-      <c r="F43" s="29"/>
+    <row r="43" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B43" s="28"/>
+      <c r="C43" s="28"/>
+      <c r="D43" s="28"/>
+      <c r="E43" s="28"/>
+      <c r="F43" s="28"/>
       <c r="H43" s="10"/>
       <c r="I43" s="10"/>
       <c r="J43" s="10"/>
     </row>
-    <row r="44" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B44" s="29"/>
-      <c r="C44" s="29"/>
-      <c r="D44" s="29"/>
-      <c r="E44" s="29"/>
+    <row r="44" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B44" s="28"/>
+      <c r="C44" s="28"/>
+      <c r="D44" s="28"/>
+      <c r="E44" s="28"/>
       <c r="H44" s="10"/>
       <c r="I44" s="10"/>
       <c r="J44" s="10"/>
       <c r="K44" s="10"/>
     </row>
-    <row r="45" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B45" s="29"/>
-      <c r="C45" s="29"/>
-      <c r="D45" s="29"/>
-      <c r="E45" s="29"/>
-      <c r="H45" s="24"/>
+    <row r="45" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B45" s="28"/>
+      <c r="C45" s="28"/>
+      <c r="D45" s="28"/>
+      <c r="E45" s="28"/>
+      <c r="H45" s="23"/>
       <c r="I45" s="10"/>
       <c r="J45" s="10"/>
       <c r="K45" s="10"/>
     </row>
-    <row r="46" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B46" s="29"/>
-      <c r="C46" s="29"/>
-      <c r="D46" s="29"/>
-      <c r="E46" s="29"/>
-      <c r="H46" s="24"/>
-      <c r="I46" s="24"/>
-      <c r="J46" s="24"/>
-    </row>
-    <row r="47" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B47" s="29"/>
-      <c r="C47" s="29"/>
-      <c r="D47" s="29"/>
-      <c r="E47" s="29"/>
-      <c r="H47" s="24"/>
-      <c r="I47" s="24"/>
-      <c r="J47" s="24"/>
-    </row>
-    <row r="48" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B48" s="29"/>
-      <c r="C48" s="29"/>
-      <c r="D48" s="29"/>
-      <c r="E48" s="29"/>
+    <row r="46" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B46" s="28"/>
+      <c r="C46" s="28"/>
+      <c r="D46" s="28"/>
+      <c r="E46" s="28"/>
+      <c r="H46" s="23"/>
+      <c r="I46" s="23"/>
+      <c r="J46" s="23"/>
+    </row>
+    <row r="47" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B47" s="28"/>
+      <c r="C47" s="28"/>
+      <c r="D47" s="28"/>
+      <c r="E47" s="28"/>
+      <c r="H47" s="23"/>
+      <c r="I47" s="23"/>
+      <c r="J47" s="23"/>
+    </row>
+    <row r="48" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B48" s="28"/>
+      <c r="C48" s="28"/>
+      <c r="D48" s="28"/>
+      <c r="E48" s="28"/>
       <c r="H48" s="17"/>
-      <c r="I48" s="24"/>
-      <c r="J48" s="24"/>
-    </row>
-    <row r="49" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B49" s="29"/>
-      <c r="C49" s="29"/>
-      <c r="D49" s="29"/>
-      <c r="E49" s="29"/>
-      <c r="G49" s="29"/>
+      <c r="I48" s="23"/>
+      <c r="J48" s="23"/>
+    </row>
+    <row r="49" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B49" s="28"/>
+      <c r="C49" s="28"/>
+      <c r="D49" s="28"/>
+      <c r="E49" s="28"/>
+      <c r="G49" s="28"/>
       <c r="I49" s="10"/>
       <c r="J49" s="10"/>
     </row>
-    <row r="50" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B50" s="29"/>
-      <c r="C50" s="29"/>
-      <c r="D50" s="29"/>
-      <c r="E50" s="29"/>
-      <c r="F50" s="29"/>
-      <c r="G50" s="29"/>
-    </row>
-    <row r="51" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B51" s="29"/>
-      <c r="C51" s="29"/>
-      <c r="D51" s="29"/>
-      <c r="E51" s="29"/>
-      <c r="F51" s="29"/>
-    </row>
-    <row r="53" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="J53" s="44"/>
+    <row r="50" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B50" s="28"/>
+      <c r="C50" s="28"/>
+      <c r="D50" s="28"/>
+      <c r="E50" s="28"/>
+      <c r="F50" s="28"/>
+      <c r="G50" s="28"/>
+    </row>
+    <row r="51" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B51" s="28"/>
+      <c r="C51" s="28"/>
+      <c r="D51" s="28"/>
+      <c r="E51" s="28"/>
+      <c r="F51" s="28"/>
+    </row>
+    <row r="53" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="J53" s="43"/>
     </row>
   </sheetData>
   <mergeCells count="68">
@@ -2672,12 +2682,9 @@
     <mergeCell ref="K28:L28"/>
     <mergeCell ref="D24:D25"/>
   </mergeCells>
-  <dataValidations count="2">
+  <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E26:E28" xr:uid="{B316A799-CF60-4C99-A88E-2204076E38E6}">
       <formula1>"กล่อง, เม็ด, ไวอัล, แอมพูล, ขวด, box, tablet, vial, ampoul, bottle"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E33:E34" xr:uid="{2CF9FB64-438B-485F-A115-633E3AF0704D}">
-      <formula1>"Days (วัน), Months (เดือน), Years (ปี)"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2693,71 +2700,71 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E9BADA0-6CEF-4001-8243-A13FFD1BF3BE}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:AA54"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="43.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="50.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="50.28515625" style="25" customWidth="1"/>
-    <col min="4" max="4" width="47.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="36.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="46.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="44.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="52.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="69.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="75.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="42.28515625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="40.5703125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="42.140625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="41.7109375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="52.85546875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="36.28515625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="46.7109375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="16.28515625" customWidth="1"/>
-    <col min="19" max="19" width="39.5703125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="38.85546875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="27.140625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="43.28515625" bestFit="1" customWidth="1"/>
-    <col min="23" max="26" width="30.42578125" customWidth="1"/>
-    <col min="27" max="27" width="35.85546875" customWidth="1"/>
+    <col min="1" max="1" width="43.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="50.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="50.26953125" style="24" customWidth="1"/>
+    <col min="4" max="4" width="47.26953125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="36.7265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="46.7265625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="44.26953125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="52.26953125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="69.26953125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="75.453125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="42.26953125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="40.54296875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="42.1796875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="41.7265625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="52.81640625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="36.26953125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="46.7265625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="16.26953125" customWidth="1"/>
+    <col min="19" max="19" width="39.54296875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="38.81640625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="27.1796875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="43.26953125" bestFit="1" customWidth="1"/>
+    <col min="23" max="26" width="30.453125" customWidth="1"/>
+    <col min="27" max="27" width="35.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="32"/>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>76</v>
       </c>
-      <c r="C1" s="33"/>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="B2" t="s">
         <v>77</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" s="121"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
         <v>78</v>
       </c>
-      <c r="C2" s="121"/>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="B3" t="s">
         <v>79</v>
       </c>
-      <c r="B3" t="s">
-        <v>80</v>
-      </c>
       <c r="C3" s="122"/>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>14</v>
       </c>
       <c r="B4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C4" s="122"/>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>18</v>
       </c>
@@ -2766,7 +2773,7 @@
       </c>
       <c r="C5" s="122"/>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -2775,7 +2782,7 @@
       </c>
       <c r="C6" s="123"/>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>23</v>
       </c>
@@ -2783,7 +2790,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>25</v>
       </c>
@@ -2791,23 +2798,23 @@
         <v>24</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
+        <v>81</v>
+      </c>
+      <c r="B9" t="s">
         <v>82</v>
       </c>
-      <c r="B9" t="s">
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+      <c r="B10" t="s">
         <v>84</v>
       </c>
-      <c r="B10" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -2815,7 +2822,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>1</v>
       </c>
@@ -2823,7 +2830,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>5</v>
       </c>
@@ -2831,122 +2838,122 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B14" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
+        <v>86</v>
+      </c>
+      <c r="B15" t="s">
         <v>87</v>
       </c>
-      <c r="B15" t="s">
+    </row>
+    <row r="17" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="B17" s="31"/>
+      <c r="C17" s="27"/>
+    </row>
+    <row r="18" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="A18" s="1" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="17" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="B17" s="32"/>
-      <c r="C17" s="28"/>
-    </row>
-    <row r="18" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
+    <row r="19" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="A19" s="7" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="19" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A19" s="7" t="s">
+      <c r="B19" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="B19" s="8" t="s">
+      <c r="C19" s="33" t="s">
         <v>91</v>
       </c>
-      <c r="C19" s="34" t="s">
+      <c r="D19" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="D19" s="2" t="s">
+      <c r="E19" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="E19" s="2" t="s">
+      <c r="F19" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="F19" s="2" t="s">
+      <c r="G19" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="G19" s="2" t="s">
+      <c r="H19" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="H19" s="2" t="s">
+      <c r="I19" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="I19" s="2" t="s">
+      <c r="J19" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="J19" s="2" t="s">
+      <c r="K19" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="K19" s="2" t="s">
+      <c r="L19" s="2" t="s">
         <v>100</v>
-      </c>
-      <c r="L19" s="2" t="s">
-        <v>101</v>
       </c>
       <c r="M19" s="2" t="s">
         <v>33</v>
       </c>
       <c r="N19" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="O19" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="O19" s="2" t="s">
+      <c r="P19" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="P19" s="2" t="s">
+      <c r="Q19" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="Q19" s="2" t="s">
+      <c r="R19" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="R19" s="2" t="s">
+      <c r="S19" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="S19" s="2" t="s">
+      <c r="T19" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="T19" s="2" t="s">
+      <c r="U19" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="U19" s="2" t="s">
+      <c r="V19" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="V19" s="2" t="s">
+      <c r="W19" s="2" t="s">
         <v>110</v>
-      </c>
-      <c r="W19" s="2" t="s">
-        <v>111</v>
       </c>
       <c r="X19" s="2" t="s">
         <v>57</v>
       </c>
       <c r="Y19" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="Z19" s="2" t="s">
         <v>58</v>
       </c>
       <c r="AA19" s="2" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="20" spans="1:27" x14ac:dyDescent="0.25">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="20" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A20" s="3" t="s">
         <v>40</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="C20" s="25" t="s">
+        <v>113</v>
+      </c>
+      <c r="C20" s="24" t="s">
         <v>42</v>
       </c>
       <c r="D20" t="s">
@@ -2959,7 +2966,7 @@
         <v>47</v>
       </c>
       <c r="G20" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="H20" s="9" t="s">
         <v>48</v>
@@ -2971,7 +2978,7 @@
         <v>50</v>
       </c>
       <c r="K20" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="L20" t="s">
         <v>39</v>
@@ -2980,35 +2987,35 @@
         <v>45</v>
       </c>
       <c r="N20" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="O20" t="s">
         <v>65</v>
       </c>
       <c r="P20" t="s">
+        <v>117</v>
+      </c>
+      <c r="Q20" t="s">
         <v>118</v>
-      </c>
-      <c r="Q20" t="s">
-        <v>119</v>
       </c>
       <c r="R20" t="e">
         <f>IF(E20&gt;0,IF(E20="Unit",CONCATENATE(Settings!Q20," ",Settings!E20,"s"),CONCATENATE((Settings!Q20/Settings!M20)," ",Settings!E20,"s")),"")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="S20" s="35" t="s">
+      <c r="S20" s="34" t="s">
+        <v>119</v>
+      </c>
+      <c r="T20" s="34" t="s">
         <v>120</v>
       </c>
-      <c r="T20" s="35" t="s">
+      <c r="U20" s="34" t="s">
         <v>121</v>
-      </c>
-      <c r="U20" s="35" t="s">
-        <v>122</v>
       </c>
       <c r="V20" t="s">
         <v>52</v>
       </c>
       <c r="W20" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="X20" t="s">
         <v>62</v>
@@ -3023,7 +3030,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="21" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A21" s="3"/>
       <c r="B21" s="4"/>
       <c r="F21" s="9"/>
@@ -3035,7 +3042,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A22" s="3"/>
       <c r="B22" s="4"/>
       <c r="F22" s="9"/>
@@ -3047,7 +3054,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A23" s="3"/>
       <c r="B23" s="4"/>
       <c r="F23" s="9"/>
@@ -3059,7 +3066,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A24" s="3"/>
       <c r="B24" s="4"/>
       <c r="F24" s="9"/>
@@ -3071,7 +3078,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A25" s="3"/>
       <c r="B25" s="4"/>
       <c r="F25" s="9"/>
@@ -3083,7 +3090,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A26" s="3"/>
       <c r="B26" s="4"/>
       <c r="F26" s="9"/>
@@ -3095,7 +3102,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A27" s="3"/>
       <c r="B27" s="4"/>
       <c r="F27" s="9"/>
@@ -3107,7 +3114,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A28" s="3"/>
       <c r="B28" s="4"/>
       <c r="F28" s="9"/>
@@ -3119,7 +3126,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A29" s="3"/>
       <c r="B29" s="4"/>
       <c r="F29" s="9"/>
@@ -3131,7 +3138,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A30" s="3"/>
       <c r="B30" s="4"/>
       <c r="F30" s="9"/>
@@ -3143,7 +3150,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A31" s="3"/>
       <c r="B31" s="4"/>
       <c r="F31" s="9"/>
@@ -3155,7 +3162,7 @@
         <v/>
       </c>
     </row>
-    <row r="32" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A32" s="3"/>
       <c r="B32" s="4"/>
       <c r="F32" s="9"/>
@@ -3167,7 +3174,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A33" s="3"/>
       <c r="B33" s="4"/>
       <c r="F33" s="9"/>
@@ -3179,7 +3186,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A34" s="3"/>
       <c r="B34" s="4"/>
       <c r="F34" s="9"/>
@@ -3191,7 +3198,7 @@
         <v/>
       </c>
     </row>
-    <row r="35" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A35" s="3"/>
       <c r="B35" s="4"/>
       <c r="F35" s="9"/>
@@ -3203,7 +3210,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A36" s="3"/>
       <c r="B36" s="4"/>
       <c r="F36" s="9"/>
@@ -3215,7 +3222,7 @@
         <v/>
       </c>
     </row>
-    <row r="37" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A37" s="3"/>
       <c r="B37" s="4"/>
       <c r="F37" s="9"/>
@@ -3227,7 +3234,7 @@
         <v/>
       </c>
     </row>
-    <row r="38" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A38" s="3"/>
       <c r="B38" s="4"/>
       <c r="F38" s="9"/>
@@ -3239,7 +3246,7 @@
         <v/>
       </c>
     </row>
-    <row r="39" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A39" s="3"/>
       <c r="B39" s="4"/>
       <c r="F39" s="9"/>
@@ -3251,7 +3258,7 @@
         <v/>
       </c>
     </row>
-    <row r="40" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A40" s="3"/>
       <c r="B40" s="4"/>
       <c r="F40" s="9"/>
@@ -3263,7 +3270,7 @@
         <v/>
       </c>
     </row>
-    <row r="41" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A41" s="3"/>
       <c r="B41" s="4"/>
       <c r="F41" s="9"/>
@@ -3275,7 +3282,7 @@
         <v/>
       </c>
     </row>
-    <row r="42" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A42" s="3"/>
       <c r="B42" s="4"/>
       <c r="F42" s="9"/>
@@ -3287,7 +3294,7 @@
         <v/>
       </c>
     </row>
-    <row r="43" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A43" s="3"/>
       <c r="B43" s="4"/>
       <c r="F43" s="9"/>
@@ -3299,7 +3306,7 @@
         <v/>
       </c>
     </row>
-    <row r="44" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A44" s="3"/>
       <c r="B44" s="4"/>
       <c r="F44" s="9"/>
@@ -3311,7 +3318,7 @@
         <v/>
       </c>
     </row>
-    <row r="45" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A45" s="3"/>
       <c r="B45" s="4"/>
       <c r="F45" s="9"/>
@@ -3323,7 +3330,7 @@
         <v/>
       </c>
     </row>
-    <row r="46" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A46" s="3"/>
       <c r="B46" s="4"/>
       <c r="F46" s="9"/>
@@ -3335,7 +3342,7 @@
         <v/>
       </c>
     </row>
-    <row r="47" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A47" s="3"/>
       <c r="B47" s="4"/>
       <c r="F47" s="9"/>
@@ -3347,7 +3354,7 @@
         <v/>
       </c>
     </row>
-    <row r="48" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A48" s="3"/>
       <c r="B48" s="4"/>
       <c r="F48" s="9"/>
@@ -3359,7 +3366,7 @@
         <v/>
       </c>
     </row>
-    <row r="49" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A49" s="3"/>
       <c r="B49" s="4"/>
       <c r="F49" s="9"/>
@@ -3371,7 +3378,7 @@
         <v/>
       </c>
     </row>
-    <row r="50" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A50" s="3"/>
       <c r="B50" s="4"/>
       <c r="F50" s="9"/>
@@ -3383,7 +3390,7 @@
         <v/>
       </c>
     </row>
-    <row r="51" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A51" s="3"/>
       <c r="B51" s="4"/>
       <c r="F51" s="9"/>
@@ -3395,7 +3402,7 @@
         <v/>
       </c>
     </row>
-    <row r="52" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A52" s="3"/>
       <c r="B52" s="4"/>
       <c r="F52" s="9"/>
@@ -3407,7 +3414,7 @@
         <v/>
       </c>
     </row>
-    <row r="53" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A53" s="3"/>
       <c r="B53" s="4"/>
       <c r="F53" s="9"/>
@@ -3419,7 +3426,7 @@
         <v/>
       </c>
     </row>
-    <row r="54" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A54" s="5"/>
       <c r="B54" s="6"/>
       <c r="F54" s="9"/>

</xml_diff>

<commit_message>
Map Quotation due date and Attention to fields in Excel quotation template and Format the date
</commit_message>
<xml_diff>
--- a/srv/xlsx-templates/TH - Quotation Template.xlsx
+++ b/srv/xlsx-templates/TH - Quotation Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EHMHV\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA20D76F-F558-4467-BD1E-506ADB44BDCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B41CFE0A-EBA5-4221-AC56-E2D6D5F5A116}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{F5CC2154-27BB-4652-B61E-D913F0CC6809}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19200" windowHeight="9020" xr2:uid="{F5CC2154-27BB-4652-B61E-D913F0CC6809}"/>
   </bookViews>
   <sheets>
     <sheet name="Quotation" sheetId="3" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="151">
   <si>
     <t>Offered Party</t>
   </si>
@@ -484,6 +484,12 @@
   </si>
   <si>
     <t>${offerValidation.Unitofdeliverydue}</t>
+  </si>
+  <si>
+    <t>${offerValidation.QuotationDate}</t>
+  </si>
+  <si>
+    <t>${offerValidation.AttentionTo}</t>
   </si>
 </sst>
 </file>
@@ -853,7 +859,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="124">
+  <cellXfs count="123">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -971,14 +977,191 @@
     <xf numFmtId="4" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="43" fontId="5" fillId="0" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="6" fillId="0" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -989,190 +1172,10 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="6" fillId="0" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="43" fontId="5" fillId="0" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1745,46 +1748,46 @@
       <c r="B3" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="77" t="s">
+      <c r="C3" s="83" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="78"/>
-      <c r="E3" s="78"/>
-      <c r="F3" s="78"/>
-      <c r="G3" s="79"/>
+      <c r="D3" s="84"/>
+      <c r="E3" s="84"/>
+      <c r="F3" s="84"/>
+      <c r="G3" s="85"/>
       <c r="H3" s="10"/>
       <c r="I3" s="25" t="s">
         <v>2</v>
       </c>
-      <c r="J3" s="77" t="s">
+      <c r="J3" s="83" t="s">
         <v>3</v>
       </c>
-      <c r="K3" s="78"/>
-      <c r="L3" s="78"/>
-      <c r="M3" s="79"/>
+      <c r="K3" s="84"/>
+      <c r="L3" s="84"/>
+      <c r="M3" s="85"/>
       <c r="N3" s="10"/>
     </row>
     <row r="4" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B4" s="26" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="80" t="s">
+      <c r="C4" s="79" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="81"/>
-      <c r="E4" s="81"/>
-      <c r="F4" s="81"/>
-      <c r="G4" s="82"/>
+      <c r="D4" s="86"/>
+      <c r="E4" s="86"/>
+      <c r="F4" s="86"/>
+      <c r="G4" s="80"/>
       <c r="H4" s="10"/>
       <c r="I4" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="J4" s="88" t="s">
+      <c r="J4" s="92" t="s">
         <v>6</v>
       </c>
-      <c r="K4" s="89"/>
-      <c r="L4" s="89"/>
-      <c r="M4" s="90"/>
+      <c r="K4" s="93"/>
+      <c r="L4" s="93"/>
+      <c r="M4" s="94"/>
       <c r="N4" s="10"/>
     </row>
     <row r="5" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -1833,151 +1836,151 @@
       <c r="N7" s="10"/>
     </row>
     <row r="8" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B8" s="83" t="s">
+      <c r="B8" s="87" t="s">
         <v>134</v>
       </c>
-      <c r="C8" s="84"/>
-      <c r="D8" s="84"/>
-      <c r="E8" s="84"/>
-      <c r="F8" s="84"/>
-      <c r="G8" s="84"/>
-      <c r="H8" s="84"/>
-      <c r="I8" s="84"/>
-      <c r="J8" s="84"/>
-      <c r="K8" s="84"/>
-      <c r="L8" s="84"/>
-      <c r="M8" s="84"/>
-      <c r="N8" s="85"/>
+      <c r="C8" s="88"/>
+      <c r="D8" s="88"/>
+      <c r="E8" s="88"/>
+      <c r="F8" s="88"/>
+      <c r="G8" s="88"/>
+      <c r="H8" s="88"/>
+      <c r="I8" s="88"/>
+      <c r="J8" s="88"/>
+      <c r="K8" s="88"/>
+      <c r="L8" s="88"/>
+      <c r="M8" s="88"/>
+      <c r="N8" s="89"/>
     </row>
     <row r="9" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B9" s="91" t="s">
+      <c r="B9" s="95" t="s">
         <v>7</v>
       </c>
-      <c r="C9" s="92"/>
-      <c r="D9" s="99" t="s">
+      <c r="C9" s="96"/>
+      <c r="D9" s="77" t="s">
         <v>8</v>
       </c>
-      <c r="E9" s="99"/>
+      <c r="E9" s="77"/>
       <c r="F9" s="39"/>
       <c r="G9" s="41" t="s">
         <v>9</v>
       </c>
       <c r="H9" s="41"/>
-      <c r="I9" s="95" t="s">
+      <c r="I9" s="98" t="s">
         <v>10</v>
       </c>
-      <c r="J9" s="95"/>
-      <c r="K9" s="96"/>
-      <c r="L9" s="86" t="s">
+      <c r="J9" s="98"/>
+      <c r="K9" s="99"/>
+      <c r="L9" s="90" t="s">
         <v>11</v>
       </c>
-      <c r="M9" s="87"/>
+      <c r="M9" s="91"/>
       <c r="N9" s="51" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="10" spans="2:14" ht="26.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="93" t="s">
+      <c r="B10" s="75" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="94"/>
-      <c r="D10" s="100" t="str">
+      <c r="C10" s="76"/>
+      <c r="D10" s="78" t="str">
         <f>Settings!A14</f>
         <v>${offerValidation.CUSTOMER_CODE}</v>
       </c>
-      <c r="E10" s="100"/>
+      <c r="E10" s="78"/>
       <c r="F10" s="39"/>
-      <c r="G10" s="101" t="s">
+      <c r="G10" s="81" t="s">
         <v>13</v>
       </c>
-      <c r="H10" s="101"/>
-      <c r="I10" s="97" t="s">
+      <c r="H10" s="81"/>
+      <c r="I10" s="100" t="s">
         <v>14</v>
       </c>
-      <c r="J10" s="97"/>
-      <c r="K10" s="98"/>
-      <c r="L10" s="72" t="s">
+      <c r="J10" s="100"/>
+      <c r="K10" s="101"/>
+      <c r="L10" s="53" t="s">
         <v>15</v>
       </c>
-      <c r="M10" s="73"/>
+      <c r="M10" s="54"/>
       <c r="N10" s="51" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="11" spans="2:14" ht="26.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="93" t="s">
+      <c r="B11" s="75" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="94"/>
-      <c r="D11" s="80" t="str">
+      <c r="C11" s="76"/>
+      <c r="D11" s="79" t="str">
         <f>Settings!A9</f>
         <v>${offerValidation.INSTITUTENAME}</v>
       </c>
-      <c r="E11" s="82"/>
+      <c r="E11" s="80"/>
       <c r="F11" s="39"/>
-      <c r="G11" s="102" t="s">
+      <c r="G11" s="82" t="s">
         <v>17</v>
       </c>
-      <c r="H11" s="102"/>
-      <c r="I11" s="97" t="s">
+      <c r="H11" s="82"/>
+      <c r="I11" s="100" t="s">
         <v>18</v>
       </c>
-      <c r="J11" s="97"/>
-      <c r="K11" s="98"/>
-      <c r="L11" s="72" t="s">
+      <c r="J11" s="100"/>
+      <c r="K11" s="101"/>
+      <c r="L11" s="53" t="s">
         <v>19</v>
       </c>
-      <c r="M11" s="73"/>
+      <c r="M11" s="54"/>
       <c r="N11" s="51" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="12" spans="2:14" ht="26" x14ac:dyDescent="0.35">
-      <c r="B12" s="93" t="s">
+      <c r="B12" s="75" t="s">
         <v>20</v>
       </c>
-      <c r="C12" s="94"/>
-      <c r="D12" s="103" t="s">
+      <c r="C12" s="76"/>
+      <c r="D12" s="73" t="s">
         <v>21</v>
       </c>
-      <c r="E12" s="59"/>
+      <c r="E12" s="74"/>
       <c r="F12" s="10"/>
-      <c r="G12" s="53" t="s">
+      <c r="G12" s="110" t="s">
         <v>22</v>
       </c>
-      <c r="H12" s="53"/>
-      <c r="I12" s="54" t="s">
+      <c r="H12" s="110"/>
+      <c r="I12" s="102" t="s">
         <v>23</v>
       </c>
-      <c r="J12" s="54"/>
-      <c r="K12" s="55"/>
-      <c r="L12" s="72" t="s">
+      <c r="J12" s="102"/>
+      <c r="K12" s="103"/>
+      <c r="L12" s="53" t="s">
         <v>15</v>
       </c>
-      <c r="M12" s="73"/>
+      <c r="M12" s="54"/>
       <c r="N12" s="51" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="13" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B13" s="93" t="s">
+      <c r="B13" s="75" t="s">
         <v>24</v>
       </c>
-      <c r="C13" s="94"/>
-      <c r="D13" s="103" t="s">
+      <c r="C13" s="76"/>
+      <c r="D13" s="73" t="s">
         <v>25</v>
       </c>
-      <c r="E13" s="59"/>
+      <c r="E13" s="74"/>
       <c r="F13" s="10"/>
-      <c r="G13" s="53" t="s">
+      <c r="G13" s="110" t="s">
         <v>124</v>
       </c>
-      <c r="H13" s="53"/>
-      <c r="I13" s="54" t="s">
+      <c r="H13" s="110"/>
+      <c r="I13" s="102" t="s">
         <v>135</v>
       </c>
-      <c r="J13" s="54"/>
-      <c r="K13" s="55"/>
+      <c r="J13" s="102"/>
+      <c r="K13" s="103"/>
     </row>
     <row r="14" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B14" s="10"/>
@@ -1992,88 +1995,88 @@
       <c r="K14" s="10"/>
     </row>
     <row r="15" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B15" s="71" t="s">
+      <c r="B15" s="108" t="s">
         <v>26</v>
       </c>
-      <c r="C15" s="71"/>
-      <c r="D15" s="71"/>
-      <c r="E15" s="71"/>
-      <c r="F15" s="71"/>
-      <c r="G15" s="71"/>
-      <c r="H15" s="71"/>
-      <c r="I15" s="71"/>
-      <c r="J15" s="71"/>
-      <c r="K15" s="71"/>
-      <c r="L15" s="71"/>
-      <c r="M15" s="71"/>
-      <c r="N15" s="71"/>
+      <c r="C15" s="108"/>
+      <c r="D15" s="108"/>
+      <c r="E15" s="108"/>
+      <c r="F15" s="108"/>
+      <c r="G15" s="108"/>
+      <c r="H15" s="108"/>
+      <c r="I15" s="108"/>
+      <c r="J15" s="108"/>
+      <c r="K15" s="108"/>
+      <c r="L15" s="108"/>
+      <c r="M15" s="108"/>
+      <c r="N15" s="108"/>
     </row>
     <row r="16" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B16" s="62" t="s">
+      <c r="B16" s="97" t="s">
         <v>27</v>
       </c>
-      <c r="C16" s="63" t="s">
+      <c r="C16" s="65" t="s">
         <v>28</v>
       </c>
-      <c r="D16" s="63" t="s">
+      <c r="D16" s="65" t="s">
         <v>29</v>
       </c>
-      <c r="E16" s="63" t="s">
+      <c r="E16" s="65" t="s">
         <v>30</v>
       </c>
-      <c r="F16" s="63" t="s">
+      <c r="F16" s="65" t="s">
         <v>31</v>
       </c>
-      <c r="G16" s="63" t="s">
+      <c r="G16" s="65" t="s">
         <v>32</v>
       </c>
-      <c r="H16" s="65" t="s">
+      <c r="H16" s="111" t="s">
         <v>33</v>
       </c>
-      <c r="I16" s="63" t="s">
+      <c r="I16" s="65" t="s">
         <v>34</v>
       </c>
-      <c r="J16" s="63" t="s">
+      <c r="J16" s="65" t="s">
         <v>35</v>
       </c>
-      <c r="K16" s="63"/>
-      <c r="L16" s="63"/>
-      <c r="M16" s="63" t="s">
+      <c r="K16" s="65"/>
+      <c r="L16" s="65"/>
+      <c r="M16" s="65" t="s">
         <v>36</v>
       </c>
-      <c r="N16" s="63"/>
+      <c r="N16" s="65"/>
     </row>
     <row r="17" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="B17" s="62"/>
-      <c r="C17" s="63"/>
-      <c r="D17" s="63"/>
-      <c r="E17" s="63"/>
-      <c r="F17" s="63"/>
-      <c r="G17" s="63"/>
-      <c r="H17" s="75"/>
-      <c r="I17" s="63"/>
-      <c r="J17" s="63"/>
-      <c r="K17" s="63"/>
-      <c r="L17" s="63"/>
-      <c r="M17" s="63"/>
-      <c r="N17" s="63"/>
+      <c r="B17" s="97"/>
+      <c r="C17" s="65"/>
+      <c r="D17" s="65"/>
+      <c r="E17" s="65"/>
+      <c r="F17" s="65"/>
+      <c r="G17" s="65"/>
+      <c r="H17" s="112"/>
+      <c r="I17" s="65"/>
+      <c r="J17" s="65"/>
+      <c r="K17" s="65"/>
+      <c r="L17" s="65"/>
+      <c r="M17" s="65"/>
+      <c r="N17" s="65"/>
     </row>
     <row r="18" spans="2:15" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="62"/>
-      <c r="C18" s="63"/>
-      <c r="D18" s="63"/>
-      <c r="E18" s="63"/>
-      <c r="F18" s="63"/>
-      <c r="G18" s="63"/>
-      <c r="H18" s="66"/>
-      <c r="I18" s="63"/>
+      <c r="B18" s="97"/>
+      <c r="C18" s="65"/>
+      <c r="D18" s="65"/>
+      <c r="E18" s="65"/>
+      <c r="F18" s="65"/>
+      <c r="G18" s="65"/>
+      <c r="H18" s="113"/>
+      <c r="I18" s="65"/>
       <c r="J18" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="K18" s="74" t="s">
+      <c r="K18" s="109" t="s">
         <v>38</v>
       </c>
-      <c r="L18" s="74"/>
+      <c r="L18" s="109"/>
       <c r="M18" s="11" t="s">
         <v>37</v>
       </c>
@@ -2109,10 +2112,10 @@
       <c r="J19" s="36" t="s">
         <v>47</v>
       </c>
-      <c r="K19" s="76" t="s">
+      <c r="K19" s="114" t="s">
         <v>48</v>
       </c>
-      <c r="L19" s="76"/>
+      <c r="L19" s="114"/>
       <c r="M19" s="40" t="s">
         <v>49</v>
       </c>
@@ -2131,8 +2134,8 @@
       <c r="H20" s="13"/>
       <c r="I20" s="12"/>
       <c r="J20" s="15"/>
-      <c r="K20" s="104"/>
-      <c r="L20" s="104"/>
+      <c r="K20" s="55"/>
+      <c r="L20" s="55"/>
       <c r="M20" s="14"/>
       <c r="N20" s="35"/>
     </row>
@@ -2146,10 +2149,10 @@
       <c r="H21" s="13"/>
       <c r="I21" s="12"/>
       <c r="J21" s="15"/>
-      <c r="K21" s="70" t="s">
+      <c r="K21" s="107" t="s">
         <v>51</v>
       </c>
-      <c r="L21" s="70"/>
+      <c r="L21" s="107"/>
       <c r="M21" s="36" t="s">
         <v>52</v>
       </c>
@@ -2173,67 +2176,67 @@
       <c r="N22" s="10"/>
     </row>
     <row r="23" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="B23" s="61" t="s">
+      <c r="B23" s="119" t="s">
         <v>54</v>
       </c>
-      <c r="C23" s="61"/>
-      <c r="D23" s="61"/>
-      <c r="E23" s="61"/>
-      <c r="F23" s="61"/>
-      <c r="G23" s="61"/>
-      <c r="H23" s="61"/>
-      <c r="I23" s="61"/>
-      <c r="J23" s="61"/>
-      <c r="K23" s="61"/>
-      <c r="L23" s="61"/>
+      <c r="C23" s="119"/>
+      <c r="D23" s="119"/>
+      <c r="E23" s="119"/>
+      <c r="F23" s="119"/>
+      <c r="G23" s="119"/>
+      <c r="H23" s="119"/>
+      <c r="I23" s="119"/>
+      <c r="J23" s="119"/>
+      <c r="K23" s="119"/>
+      <c r="L23" s="119"/>
       <c r="M23" s="10"/>
     </row>
     <row r="24" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="B24" s="62" t="s">
+      <c r="B24" s="97" t="s">
         <v>27</v>
       </c>
-      <c r="C24" s="63" t="s">
+      <c r="C24" s="65" t="s">
         <v>28</v>
       </c>
-      <c r="D24" s="65" t="s">
+      <c r="D24" s="111" t="s">
         <v>126</v>
       </c>
-      <c r="E24" s="63" t="s">
+      <c r="E24" s="65" t="s">
         <v>55</v>
       </c>
-      <c r="F24" s="63" t="s">
+      <c r="F24" s="65" t="s">
         <v>56</v>
       </c>
-      <c r="G24" s="63" t="s">
+      <c r="G24" s="65" t="s">
         <v>57</v>
       </c>
-      <c r="H24" s="63" t="s">
+      <c r="H24" s="65" t="s">
         <v>58</v>
       </c>
-      <c r="I24" s="63"/>
-      <c r="J24" s="63"/>
-      <c r="K24" s="63" t="s">
+      <c r="I24" s="65"/>
+      <c r="J24" s="65"/>
+      <c r="K24" s="65" t="s">
         <v>59</v>
       </c>
-      <c r="L24" s="63"/>
-      <c r="M24" s="63" t="s">
+      <c r="L24" s="65"/>
+      <c r="M24" s="65" t="s">
         <v>60</v>
       </c>
       <c r="N24" s="10"/>
     </row>
     <row r="25" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="B25" s="62"/>
-      <c r="C25" s="63"/>
-      <c r="D25" s="66"/>
-      <c r="E25" s="63"/>
-      <c r="F25" s="63"/>
-      <c r="G25" s="63"/>
-      <c r="H25" s="63"/>
-      <c r="I25" s="63"/>
-      <c r="J25" s="63"/>
-      <c r="K25" s="63"/>
-      <c r="L25" s="63"/>
-      <c r="M25" s="63"/>
+      <c r="B25" s="97"/>
+      <c r="C25" s="65"/>
+      <c r="D25" s="113"/>
+      <c r="E25" s="65"/>
+      <c r="F25" s="65"/>
+      <c r="G25" s="65"/>
+      <c r="H25" s="65"/>
+      <c r="I25" s="65"/>
+      <c r="J25" s="65"/>
+      <c r="K25" s="65"/>
+      <c r="L25" s="65"/>
+      <c r="M25" s="65"/>
       <c r="N25" s="10"/>
     </row>
     <row r="26" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -2253,15 +2256,15 @@
       <c r="G26" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="H26" s="64" t="s">
+      <c r="H26" s="66" t="s">
         <v>63</v>
       </c>
-      <c r="I26" s="64"/>
-      <c r="J26" s="64"/>
-      <c r="K26" s="64" t="s">
+      <c r="I26" s="66"/>
+      <c r="J26" s="66"/>
+      <c r="K26" s="66" t="s">
         <v>64</v>
       </c>
-      <c r="L26" s="64"/>
+      <c r="L26" s="66"/>
       <c r="M26" s="16" t="s">
         <v>65</v>
       </c>
@@ -2274,11 +2277,11 @@
       <c r="E27" s="16"/>
       <c r="F27" s="16"/>
       <c r="G27" s="16"/>
-      <c r="H27" s="67"/>
-      <c r="I27" s="68"/>
-      <c r="J27" s="69"/>
-      <c r="K27" s="64"/>
-      <c r="L27" s="64"/>
+      <c r="H27" s="104"/>
+      <c r="I27" s="105"/>
+      <c r="J27" s="106"/>
+      <c r="K27" s="66"/>
+      <c r="L27" s="66"/>
       <c r="M27" s="16"/>
       <c r="N27" s="10"/>
     </row>
@@ -2289,11 +2292,11 @@
       <c r="E28" s="16"/>
       <c r="F28" s="16"/>
       <c r="G28" s="16"/>
-      <c r="H28" s="120"/>
-      <c r="I28" s="120"/>
-      <c r="J28" s="120"/>
-      <c r="K28" s="64"/>
-      <c r="L28" s="64"/>
+      <c r="H28" s="72"/>
+      <c r="I28" s="72"/>
+      <c r="J28" s="72"/>
+      <c r="K28" s="66"/>
+      <c r="L28" s="66"/>
       <c r="M28" s="16"/>
       <c r="N28" s="10"/>
     </row>
@@ -2313,21 +2316,21 @@
       <c r="N29" s="10"/>
     </row>
     <row r="30" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B30" s="117" t="s">
+      <c r="B30" s="69" t="s">
         <v>66</v>
       </c>
-      <c r="C30" s="117"/>
-      <c r="D30" s="117"/>
-      <c r="E30" s="117"/>
+      <c r="C30" s="69"/>
+      <c r="D30" s="69"/>
+      <c r="E30" s="69"/>
       <c r="F30" s="18"/>
-      <c r="G30" s="118" t="s">
+      <c r="G30" s="70" t="s">
         <v>67</v>
       </c>
-      <c r="H30" s="119"/>
-      <c r="I30" s="56" t="s">
+      <c r="H30" s="71"/>
+      <c r="I30" s="115" t="s">
         <v>144</v>
       </c>
-      <c r="J30" s="57"/>
+      <c r="J30" s="116"/>
       <c r="K30" s="26" t="s">
         <v>15</v>
       </c>
@@ -2340,21 +2343,23 @@
         <v>68</v>
       </c>
       <c r="C31" s="20"/>
-      <c r="D31" s="114"/>
-      <c r="E31" s="114"/>
+      <c r="D31" s="66" t="s">
+        <v>149</v>
+      </c>
+      <c r="E31" s="66"/>
       <c r="F31" s="10"/>
-      <c r="G31" s="115" t="s">
+      <c r="G31" s="67" t="s">
         <v>140</v>
       </c>
-      <c r="H31" s="116"/>
-      <c r="I31" s="60" t="s">
+      <c r="H31" s="68"/>
+      <c r="I31" s="118" t="s">
         <v>143</v>
       </c>
-      <c r="J31" s="60"/>
-      <c r="K31" s="58" t="s">
+      <c r="J31" s="118"/>
+      <c r="K31" s="117" t="s">
         <v>142</v>
       </c>
-      <c r="L31" s="59"/>
+      <c r="L31" s="74"/>
       <c r="M31" s="10"/>
       <c r="N31" s="10"/>
     </row>
@@ -2363,8 +2368,10 @@
         <v>69</v>
       </c>
       <c r="C32" s="20"/>
-      <c r="D32" s="64"/>
-      <c r="E32" s="64"/>
+      <c r="D32" s="66" t="s">
+        <v>150</v>
+      </c>
+      <c r="E32" s="66"/>
       <c r="F32" s="10"/>
       <c r="G32" s="10"/>
       <c r="H32" s="10"/>
@@ -2448,12 +2455,12 @@
       <c r="J36" s="28"/>
     </row>
     <row r="37" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B37" s="105" t="s">
+      <c r="B37" s="56" t="s">
         <v>73</v>
       </c>
-      <c r="C37" s="106"/>
-      <c r="D37" s="106"/>
-      <c r="E37" s="107"/>
+      <c r="C37" s="57"/>
+      <c r="D37" s="57"/>
+      <c r="E37" s="58"/>
       <c r="F37" s="28"/>
       <c r="G37" s="49" t="s">
         <v>127</v>
@@ -2465,10 +2472,10 @@
       <c r="J37" s="28"/>
     </row>
     <row r="38" spans="2:14" ht="26" x14ac:dyDescent="0.35">
-      <c r="B38" s="108"/>
-      <c r="C38" s="109"/>
-      <c r="D38" s="109"/>
-      <c r="E38" s="110"/>
+      <c r="B38" s="59"/>
+      <c r="C38" s="60"/>
+      <c r="D38" s="60"/>
+      <c r="E38" s="61"/>
       <c r="F38" s="28"/>
       <c r="G38" s="49" t="s">
         <v>128</v>
@@ -2480,10 +2487,10 @@
       <c r="J38" s="28"/>
     </row>
     <row r="39" spans="2:14" ht="26" x14ac:dyDescent="0.35">
-      <c r="B39" s="108"/>
-      <c r="C39" s="109"/>
-      <c r="D39" s="109"/>
-      <c r="E39" s="110"/>
+      <c r="B39" s="59"/>
+      <c r="C39" s="60"/>
+      <c r="D39" s="60"/>
+      <c r="E39" s="61"/>
       <c r="F39" s="28"/>
       <c r="G39" s="49" t="s">
         <v>129</v>
@@ -2495,10 +2502,10 @@
       <c r="J39" s="28"/>
     </row>
     <row r="40" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B40" s="108"/>
-      <c r="C40" s="109"/>
-      <c r="D40" s="109"/>
-      <c r="E40" s="110"/>
+      <c r="B40" s="59"/>
+      <c r="C40" s="60"/>
+      <c r="D40" s="60"/>
+      <c r="E40" s="61"/>
       <c r="F40" s="28"/>
       <c r="G40" s="28"/>
       <c r="H40" s="28"/>
@@ -2506,10 +2513,10 @@
       <c r="J40" s="28"/>
     </row>
     <row r="41" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B41" s="111"/>
-      <c r="C41" s="112"/>
-      <c r="D41" s="112"/>
-      <c r="E41" s="113"/>
+      <c r="B41" s="62"/>
+      <c r="C41" s="63"/>
+      <c r="D41" s="63"/>
+      <c r="E41" s="64"/>
       <c r="F41" s="28"/>
       <c r="G41" s="28"/>
       <c r="H41" s="10"/>
@@ -2613,6 +2620,58 @@
     </row>
   </sheetData>
   <mergeCells count="68">
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="I13:K13"/>
+    <mergeCell ref="I30:J30"/>
+    <mergeCell ref="K31:L31"/>
+    <mergeCell ref="I31:J31"/>
+    <mergeCell ref="B23:L23"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="K24:L25"/>
+    <mergeCell ref="K28:L28"/>
+    <mergeCell ref="D24:D25"/>
+    <mergeCell ref="M16:N17"/>
+    <mergeCell ref="I12:K12"/>
+    <mergeCell ref="H27:J27"/>
+    <mergeCell ref="K27:L27"/>
+    <mergeCell ref="K21:L21"/>
+    <mergeCell ref="M24:M25"/>
+    <mergeCell ref="H24:J25"/>
+    <mergeCell ref="H26:J26"/>
+    <mergeCell ref="K26:L26"/>
+    <mergeCell ref="B15:N15"/>
+    <mergeCell ref="L12:M12"/>
+    <mergeCell ref="K18:L18"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="G24:G25"/>
+    <mergeCell ref="H16:H18"/>
+    <mergeCell ref="K19:L19"/>
+    <mergeCell ref="C3:G3"/>
+    <mergeCell ref="C4:G4"/>
+    <mergeCell ref="F16:F18"/>
+    <mergeCell ref="B8:N8"/>
+    <mergeCell ref="L9:M9"/>
+    <mergeCell ref="E16:E18"/>
+    <mergeCell ref="J3:M3"/>
+    <mergeCell ref="J4:M4"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B16:B18"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="I9:K9"/>
+    <mergeCell ref="I10:K10"/>
+    <mergeCell ref="I11:K11"/>
+    <mergeCell ref="D16:D18"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="G10:H10"/>
+    <mergeCell ref="G11:H11"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="C16:C18"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B13:C13"/>
     <mergeCell ref="L10:M10"/>
     <mergeCell ref="L11:M11"/>
     <mergeCell ref="K20:L20"/>
@@ -2629,58 +2688,6 @@
     <mergeCell ref="B30:E30"/>
     <mergeCell ref="G30:H30"/>
     <mergeCell ref="H28:J28"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="C16:C18"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="G10:H10"/>
-    <mergeCell ref="G11:H11"/>
-    <mergeCell ref="C3:G3"/>
-    <mergeCell ref="C4:G4"/>
-    <mergeCell ref="F16:F18"/>
-    <mergeCell ref="B8:N8"/>
-    <mergeCell ref="L9:M9"/>
-    <mergeCell ref="E16:E18"/>
-    <mergeCell ref="J3:M3"/>
-    <mergeCell ref="J4:M4"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B16:B18"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="I9:K9"/>
-    <mergeCell ref="I10:K10"/>
-    <mergeCell ref="I11:K11"/>
-    <mergeCell ref="D16:D18"/>
-    <mergeCell ref="M16:N17"/>
-    <mergeCell ref="I12:K12"/>
-    <mergeCell ref="H27:J27"/>
-    <mergeCell ref="K27:L27"/>
-    <mergeCell ref="K21:L21"/>
-    <mergeCell ref="M24:M25"/>
-    <mergeCell ref="H24:J25"/>
-    <mergeCell ref="H26:J26"/>
-    <mergeCell ref="K26:L26"/>
-    <mergeCell ref="B15:N15"/>
-    <mergeCell ref="L12:M12"/>
-    <mergeCell ref="K18:L18"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="G24:G25"/>
-    <mergeCell ref="H16:H18"/>
-    <mergeCell ref="K19:L19"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="I13:K13"/>
-    <mergeCell ref="I30:J30"/>
-    <mergeCell ref="K31:L31"/>
-    <mergeCell ref="I31:J31"/>
-    <mergeCell ref="B23:L23"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="K24:L25"/>
-    <mergeCell ref="K28:L28"/>
-    <mergeCell ref="D24:D25"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E26:E28" xr:uid="{B316A799-CF60-4C99-A88E-2204076E38E6}">
@@ -2744,7 +2751,7 @@
       <c r="B2" t="s">
         <v>77</v>
       </c>
-      <c r="C2" s="121"/>
+      <c r="C2" s="120"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
@@ -2753,7 +2760,7 @@
       <c r="B3" t="s">
         <v>79</v>
       </c>
-      <c r="C3" s="122"/>
+      <c r="C3" s="121"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
@@ -2762,7 +2769,7 @@
       <c r="B4" t="s">
         <v>80</v>
       </c>
-      <c r="C4" s="122"/>
+      <c r="C4" s="121"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
@@ -2771,7 +2778,7 @@
       <c r="B5" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="122"/>
+      <c r="C5" s="121"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
@@ -2780,7 +2787,7 @@
       <c r="B6" t="s">
         <v>20</v>
       </c>
-      <c r="C6" s="123"/>
+      <c r="C6" s="122"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
@@ -3457,12 +3464,17 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <SharedWithUsers xmlns="1444eecc-14bb-4066-abe6-ce6de21d9439">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3663,23 +3675,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <SharedWithUsers xmlns="1444eecc-14bb-4066-abe6-ce6de21d9439">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A00E6A9-20DD-4842-9306-307EB080AF2E}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7EBE950A-5812-419E-B174-6A5D9B8E0414}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="1444eecc-14bb-4066-abe6-ce6de21d9439"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -3704,11 +3713,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7EBE950A-5812-419E-B174-6A5D9B8E0414}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A00E6A9-20DD-4842-9306-307EB080AF2E}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="1444eecc-14bb-4066-abe6-ce6de21d9439"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Thailand quotation template changes
</commit_message>
<xml_diff>
--- a/srv/xlsx-templates/TH - Quotation Template.xlsx
+++ b/srv/xlsx-templates/TH - Quotation Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EHMHV\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B41CFE0A-EBA5-4221-AC56-E2D6D5F5A116}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{714FDFF9-E09B-48C9-B3AA-07421092CB2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19200" windowHeight="9020" xr2:uid="{F5CC2154-27BB-4652-B61E-D913F0CC6809}"/>
   </bookViews>
@@ -601,7 +601,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -623,12 +623,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="2" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.14999847407452621"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -859,7 +853,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="123">
+  <cellXfs count="125">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -929,53 +923,101 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="43" fontId="6" fillId="0" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -983,6 +1025,96 @@
     <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="43" fontId="5" fillId="0" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1013,12 +1145,6 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1037,147 +1163,6 @@
     <xf numFmtId="49" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="6" fillId="0" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1186,6 +1171,21 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1719,8 +1719,8 @@
     <col min="4" max="4" width="33.26953125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="52.453125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11.81640625" customWidth="1"/>
-    <col min="7" max="7" width="17" customWidth="1"/>
-    <col min="8" max="8" width="24.54296875" customWidth="1"/>
+    <col min="7" max="7" width="22" customWidth="1"/>
+    <col min="8" max="8" width="19" customWidth="1"/>
     <col min="9" max="9" width="14.7265625" customWidth="1"/>
     <col min="10" max="10" width="21.26953125" customWidth="1"/>
     <col min="11" max="11" width="14.81640625" customWidth="1"/>
@@ -1748,76 +1748,76 @@
       <c r="B3" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="83" t="s">
+      <c r="C3" s="74" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="84"/>
-      <c r="E3" s="84"/>
-      <c r="F3" s="84"/>
-      <c r="G3" s="85"/>
+      <c r="D3" s="75"/>
+      <c r="E3" s="75"/>
+      <c r="F3" s="75"/>
+      <c r="G3" s="76"/>
       <c r="H3" s="10"/>
       <c r="I3" s="25" t="s">
         <v>2</v>
       </c>
-      <c r="J3" s="83" t="s">
+      <c r="J3" s="74" t="s">
         <v>3</v>
       </c>
-      <c r="K3" s="84"/>
-      <c r="L3" s="84"/>
-      <c r="M3" s="85"/>
+      <c r="K3" s="75"/>
+      <c r="L3" s="75"/>
+      <c r="M3" s="76"/>
       <c r="N3" s="10"/>
     </row>
     <row r="4" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B4" s="26" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="79" t="s">
+      <c r="C4" s="77" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="86"/>
-      <c r="E4" s="86"/>
-      <c r="F4" s="86"/>
-      <c r="G4" s="80"/>
+      <c r="D4" s="78"/>
+      <c r="E4" s="78"/>
+      <c r="F4" s="78"/>
+      <c r="G4" s="79"/>
       <c r="H4" s="10"/>
       <c r="I4" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="J4" s="92" t="s">
+      <c r="J4" s="85" t="s">
         <v>6</v>
       </c>
-      <c r="K4" s="93"/>
-      <c r="L4" s="93"/>
-      <c r="M4" s="94"/>
+      <c r="K4" s="86"/>
+      <c r="L4" s="86"/>
+      <c r="M4" s="87"/>
       <c r="N4" s="10"/>
     </row>
     <row r="5" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="44"/>
-      <c r="C5" s="44"/>
-      <c r="D5" s="44"/>
-      <c r="E5" s="44"/>
-      <c r="F5" s="44"/>
-      <c r="G5" s="44"/>
+      <c r="B5" s="42"/>
+      <c r="C5" s="42"/>
+      <c r="D5" s="42"/>
+      <c r="E5" s="42"/>
+      <c r="F5" s="42"/>
+      <c r="G5" s="42"/>
       <c r="H5" s="10"/>
       <c r="I5" s="10"/>
-      <c r="J5" s="45"/>
-      <c r="K5" s="45"/>
-      <c r="L5" s="45"/>
-      <c r="M5" s="45"/>
+      <c r="J5" s="43"/>
+      <c r="K5" s="43"/>
+      <c r="L5" s="43"/>
+      <c r="M5" s="43"/>
       <c r="N5" s="10"/>
     </row>
     <row r="6" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="44"/>
-      <c r="C6" s="44"/>
-      <c r="D6" s="44"/>
-      <c r="E6" s="44"/>
-      <c r="F6" s="44"/>
-      <c r="G6" s="44"/>
+      <c r="B6" s="42"/>
+      <c r="C6" s="42"/>
+      <c r="D6" s="42"/>
+      <c r="E6" s="42"/>
+      <c r="F6" s="42"/>
+      <c r="G6" s="42"/>
       <c r="H6" s="10"/>
       <c r="I6" s="10"/>
-      <c r="J6" s="45"/>
-      <c r="K6" s="45"/>
-      <c r="L6" s="45"/>
-      <c r="M6" s="45"/>
+      <c r="J6" s="43"/>
+      <c r="K6" s="43"/>
+      <c r="L6" s="43"/>
+      <c r="M6" s="43"/>
       <c r="N6" s="10"/>
     </row>
     <row r="7" spans="2:14" x14ac:dyDescent="0.35">
@@ -1836,151 +1836,151 @@
       <c r="N7" s="10"/>
     </row>
     <row r="8" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B8" s="87" t="s">
+      <c r="B8" s="80" t="s">
         <v>134</v>
       </c>
-      <c r="C8" s="88"/>
-      <c r="D8" s="88"/>
-      <c r="E8" s="88"/>
-      <c r="F8" s="88"/>
-      <c r="G8" s="88"/>
-      <c r="H8" s="88"/>
-      <c r="I8" s="88"/>
-      <c r="J8" s="88"/>
-      <c r="K8" s="88"/>
-      <c r="L8" s="88"/>
-      <c r="M8" s="88"/>
-      <c r="N8" s="89"/>
+      <c r="C8" s="81"/>
+      <c r="D8" s="81"/>
+      <c r="E8" s="81"/>
+      <c r="F8" s="81"/>
+      <c r="G8" s="81"/>
+      <c r="H8" s="81"/>
+      <c r="I8" s="81"/>
+      <c r="J8" s="81"/>
+      <c r="K8" s="81"/>
+      <c r="L8" s="81"/>
+      <c r="M8" s="81"/>
+      <c r="N8" s="82"/>
     </row>
     <row r="9" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B9" s="95" t="s">
+      <c r="B9" s="88" t="s">
         <v>7</v>
       </c>
-      <c r="C9" s="96"/>
-      <c r="D9" s="77" t="s">
+      <c r="C9" s="89"/>
+      <c r="D9" s="96" t="s">
         <v>8</v>
       </c>
-      <c r="E9" s="77"/>
-      <c r="F9" s="39"/>
-      <c r="G9" s="41" t="s">
+      <c r="E9" s="96"/>
+      <c r="F9" s="38"/>
+      <c r="G9" s="120" t="s">
         <v>9</v>
       </c>
-      <c r="H9" s="41"/>
-      <c r="I9" s="98" t="s">
+      <c r="H9" s="121"/>
+      <c r="I9" s="92" t="s">
         <v>10</v>
       </c>
-      <c r="J9" s="98"/>
-      <c r="K9" s="99"/>
-      <c r="L9" s="90" t="s">
+      <c r="J9" s="92"/>
+      <c r="K9" s="93"/>
+      <c r="L9" s="83" t="s">
         <v>11</v>
       </c>
-      <c r="M9" s="91"/>
-      <c r="N9" s="51" t="s">
+      <c r="M9" s="84"/>
+      <c r="N9" s="48" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="10" spans="2:14" ht="26.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="75" t="s">
+      <c r="B10" s="90" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="76"/>
-      <c r="D10" s="78" t="str">
+      <c r="C10" s="91"/>
+      <c r="D10" s="97" t="str">
         <f>Settings!A14</f>
         <v>${offerValidation.CUSTOMER_CODE}</v>
       </c>
-      <c r="E10" s="78"/>
-      <c r="F10" s="39"/>
-      <c r="G10" s="81" t="s">
+      <c r="E10" s="97"/>
+      <c r="F10" s="38"/>
+      <c r="G10" s="98" t="s">
         <v>13</v>
       </c>
-      <c r="H10" s="81"/>
-      <c r="I10" s="100" t="s">
+      <c r="H10" s="98"/>
+      <c r="I10" s="94" t="s">
         <v>14</v>
       </c>
-      <c r="J10" s="100"/>
-      <c r="K10" s="101"/>
-      <c r="L10" s="53" t="s">
+      <c r="J10" s="94"/>
+      <c r="K10" s="95"/>
+      <c r="L10" s="69" t="s">
         <v>15</v>
       </c>
-      <c r="M10" s="54"/>
-      <c r="N10" s="51" t="s">
+      <c r="M10" s="70"/>
+      <c r="N10" s="48" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="11" spans="2:14" ht="26.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="75" t="s">
+      <c r="B11" s="90" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="76"/>
-      <c r="D11" s="79" t="str">
+      <c r="C11" s="91"/>
+      <c r="D11" s="77" t="str">
         <f>Settings!A9</f>
         <v>${offerValidation.INSTITUTENAME}</v>
       </c>
-      <c r="E11" s="80"/>
-      <c r="F11" s="39"/>
-      <c r="G11" s="82" t="s">
+      <c r="E11" s="79"/>
+      <c r="F11" s="38"/>
+      <c r="G11" s="99" t="s">
         <v>17</v>
       </c>
-      <c r="H11" s="82"/>
-      <c r="I11" s="100" t="s">
+      <c r="H11" s="99"/>
+      <c r="I11" s="94" t="s">
         <v>18</v>
       </c>
-      <c r="J11" s="100"/>
-      <c r="K11" s="101"/>
-      <c r="L11" s="53" t="s">
+      <c r="J11" s="94"/>
+      <c r="K11" s="95"/>
+      <c r="L11" s="69" t="s">
         <v>19</v>
       </c>
-      <c r="M11" s="54"/>
-      <c r="N11" s="51" t="s">
+      <c r="M11" s="70"/>
+      <c r="N11" s="48" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="12" spans="2:14" ht="26" x14ac:dyDescent="0.35">
-      <c r="B12" s="75" t="s">
+      <c r="B12" s="90" t="s">
         <v>20</v>
       </c>
-      <c r="C12" s="76"/>
-      <c r="D12" s="73" t="s">
+      <c r="C12" s="91"/>
+      <c r="D12" s="100" t="s">
         <v>21</v>
       </c>
-      <c r="E12" s="74"/>
+      <c r="E12" s="57"/>
       <c r="F12" s="10"/>
-      <c r="G12" s="110" t="s">
+      <c r="G12" s="51" t="s">
         <v>22</v>
       </c>
-      <c r="H12" s="110"/>
-      <c r="I12" s="102" t="s">
+      <c r="H12" s="51"/>
+      <c r="I12" s="52" t="s">
         <v>23</v>
       </c>
-      <c r="J12" s="102"/>
-      <c r="K12" s="103"/>
-      <c r="L12" s="53" t="s">
+      <c r="J12" s="52"/>
+      <c r="K12" s="53"/>
+      <c r="L12" s="69" t="s">
         <v>15</v>
       </c>
-      <c r="M12" s="54"/>
-      <c r="N12" s="51" t="s">
+      <c r="M12" s="70"/>
+      <c r="N12" s="48" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="13" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B13" s="75" t="s">
+      <c r="B13" s="90" t="s">
         <v>24</v>
       </c>
-      <c r="C13" s="76"/>
-      <c r="D13" s="73" t="s">
+      <c r="C13" s="91"/>
+      <c r="D13" s="100" t="s">
         <v>25</v>
       </c>
-      <c r="E13" s="74"/>
+      <c r="E13" s="57"/>
       <c r="F13" s="10"/>
-      <c r="G13" s="110" t="s">
+      <c r="G13" s="51" t="s">
         <v>124</v>
       </c>
-      <c r="H13" s="110"/>
-      <c r="I13" s="102" t="s">
+      <c r="H13" s="51"/>
+      <c r="I13" s="52" t="s">
         <v>135</v>
       </c>
-      <c r="J13" s="102"/>
-      <c r="K13" s="103"/>
+      <c r="J13" s="52"/>
+      <c r="K13" s="53"/>
     </row>
     <row r="14" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B14" s="10"/>
@@ -1995,88 +1995,88 @@
       <c r="K14" s="10"/>
     </row>
     <row r="15" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B15" s="108" t="s">
+      <c r="B15" s="80" t="s">
         <v>26</v>
       </c>
-      <c r="C15" s="108"/>
-      <c r="D15" s="108"/>
-      <c r="E15" s="108"/>
-      <c r="F15" s="108"/>
-      <c r="G15" s="108"/>
-      <c r="H15" s="108"/>
-      <c r="I15" s="108"/>
-      <c r="J15" s="108"/>
-      <c r="K15" s="108"/>
-      <c r="L15" s="108"/>
-      <c r="M15" s="108"/>
-      <c r="N15" s="108"/>
+      <c r="C15" s="81"/>
+      <c r="D15" s="81"/>
+      <c r="E15" s="81"/>
+      <c r="F15" s="81"/>
+      <c r="G15" s="81"/>
+      <c r="H15" s="81"/>
+      <c r="I15" s="81"/>
+      <c r="J15" s="81"/>
+      <c r="K15" s="81"/>
+      <c r="L15" s="81"/>
+      <c r="M15" s="81"/>
+      <c r="N15" s="82"/>
     </row>
     <row r="16" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B16" s="97" t="s">
+      <c r="B16" s="60" t="s">
         <v>27</v>
       </c>
-      <c r="C16" s="65" t="s">
+      <c r="C16" s="61" t="s">
         <v>28</v>
       </c>
-      <c r="D16" s="65" t="s">
+      <c r="D16" s="61" t="s">
         <v>29</v>
       </c>
-      <c r="E16" s="65" t="s">
+      <c r="E16" s="61" t="s">
         <v>30</v>
       </c>
-      <c r="F16" s="65" t="s">
+      <c r="F16" s="61" t="s">
         <v>31</v>
       </c>
-      <c r="G16" s="65" t="s">
+      <c r="G16" s="61" t="s">
         <v>32</v>
       </c>
-      <c r="H16" s="111" t="s">
+      <c r="H16" s="63" t="s">
         <v>33</v>
       </c>
-      <c r="I16" s="65" t="s">
+      <c r="I16" s="61" t="s">
         <v>34</v>
       </c>
-      <c r="J16" s="65" t="s">
+      <c r="J16" s="61" t="s">
         <v>35</v>
       </c>
-      <c r="K16" s="65"/>
-      <c r="L16" s="65"/>
-      <c r="M16" s="65" t="s">
+      <c r="K16" s="61"/>
+      <c r="L16" s="61"/>
+      <c r="M16" s="61" t="s">
         <v>36</v>
       </c>
-      <c r="N16" s="65"/>
+      <c r="N16" s="61"/>
     </row>
     <row r="17" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="B17" s="97"/>
-      <c r="C17" s="65"/>
-      <c r="D17" s="65"/>
-      <c r="E17" s="65"/>
-      <c r="F17" s="65"/>
-      <c r="G17" s="65"/>
-      <c r="H17" s="112"/>
-      <c r="I17" s="65"/>
-      <c r="J17" s="65"/>
-      <c r="K17" s="65"/>
-      <c r="L17" s="65"/>
-      <c r="M17" s="65"/>
-      <c r="N17" s="65"/>
+      <c r="B17" s="60"/>
+      <c r="C17" s="61"/>
+      <c r="D17" s="61"/>
+      <c r="E17" s="61"/>
+      <c r="F17" s="61"/>
+      <c r="G17" s="61"/>
+      <c r="H17" s="72"/>
+      <c r="I17" s="61"/>
+      <c r="J17" s="61"/>
+      <c r="K17" s="61"/>
+      <c r="L17" s="61"/>
+      <c r="M17" s="61"/>
+      <c r="N17" s="61"/>
     </row>
     <row r="18" spans="2:15" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="97"/>
-      <c r="C18" s="65"/>
-      <c r="D18" s="65"/>
-      <c r="E18" s="65"/>
-      <c r="F18" s="65"/>
-      <c r="G18" s="65"/>
-      <c r="H18" s="113"/>
-      <c r="I18" s="65"/>
+      <c r="B18" s="60"/>
+      <c r="C18" s="61"/>
+      <c r="D18" s="61"/>
+      <c r="E18" s="61"/>
+      <c r="F18" s="61"/>
+      <c r="G18" s="61"/>
+      <c r="H18" s="64"/>
+      <c r="I18" s="61"/>
       <c r="J18" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="K18" s="109" t="s">
+      <c r="K18" s="71" t="s">
         <v>38</v>
       </c>
-      <c r="L18" s="109"/>
+      <c r="L18" s="71"/>
       <c r="M18" s="11" t="s">
         <v>37</v>
       </c>
@@ -2091,10 +2091,10 @@
       <c r="C19" s="24" t="s">
         <v>123</v>
       </c>
-      <c r="D19" s="38" t="s">
+      <c r="D19" s="37" t="s">
         <v>41</v>
       </c>
-      <c r="E19" s="38" t="s">
+      <c r="E19" s="37" t="s">
         <v>42</v>
       </c>
       <c r="F19" s="36" t="s">
@@ -2112,14 +2112,14 @@
       <c r="J19" s="36" t="s">
         <v>47</v>
       </c>
-      <c r="K19" s="114" t="s">
+      <c r="K19" s="73" t="s">
         <v>48</v>
       </c>
-      <c r="L19" s="114"/>
-      <c r="M19" s="40" t="s">
+      <c r="L19" s="73"/>
+      <c r="M19" s="39" t="s">
         <v>49</v>
       </c>
-      <c r="N19" s="40" t="s">
+      <c r="N19" s="39" t="s">
         <v>50</v>
       </c>
       <c r="O19" s="30"/>
@@ -2134,8 +2134,8 @@
       <c r="H20" s="13"/>
       <c r="I20" s="12"/>
       <c r="J20" s="15"/>
-      <c r="K20" s="55"/>
-      <c r="L20" s="55"/>
+      <c r="K20" s="101"/>
+      <c r="L20" s="101"/>
       <c r="M20" s="14"/>
       <c r="N20" s="35"/>
     </row>
@@ -2149,10 +2149,10 @@
       <c r="H21" s="13"/>
       <c r="I21" s="12"/>
       <c r="J21" s="15"/>
-      <c r="K21" s="107" t="s">
+      <c r="K21" s="68" t="s">
         <v>51</v>
       </c>
-      <c r="L21" s="107"/>
+      <c r="L21" s="68"/>
       <c r="M21" s="36" t="s">
         <v>52</v>
       </c>
@@ -2176,68 +2176,73 @@
       <c r="N22" s="10"/>
     </row>
     <row r="23" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="B23" s="119" t="s">
+      <c r="B23" s="59" t="s">
         <v>54</v>
       </c>
-      <c r="C23" s="119"/>
-      <c r="D23" s="119"/>
-      <c r="E23" s="119"/>
-      <c r="F23" s="119"/>
-      <c r="G23" s="119"/>
-      <c r="H23" s="119"/>
-      <c r="I23" s="119"/>
-      <c r="J23" s="119"/>
-      <c r="K23" s="119"/>
-      <c r="L23" s="119"/>
-      <c r="M23" s="10"/>
+      <c r="C23" s="59"/>
+      <c r="D23" s="59"/>
+      <c r="E23" s="59"/>
+      <c r="F23" s="59"/>
+      <c r="G23" s="59"/>
+      <c r="H23" s="59"/>
+      <c r="I23" s="59"/>
+      <c r="J23" s="59"/>
+      <c r="K23" s="59"/>
+      <c r="L23" s="59"/>
+      <c r="M23" s="59"/>
+      <c r="N23" s="59"/>
     </row>
     <row r="24" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="B24" s="97" t="s">
+      <c r="B24" s="122" t="s">
         <v>27</v>
       </c>
-      <c r="C24" s="65" t="s">
+      <c r="C24" s="64" t="s">
         <v>28</v>
       </c>
-      <c r="D24" s="111" t="s">
+      <c r="D24" s="72" t="s">
+        <v>125</v>
+      </c>
+      <c r="E24" s="72" t="s">
         <v>126</v>
       </c>
-      <c r="E24" s="65" t="s">
+      <c r="F24" s="64" t="s">
         <v>55</v>
       </c>
-      <c r="F24" s="65" t="s">
+      <c r="G24" s="64" t="s">
+        <v>57</v>
+      </c>
+      <c r="H24" s="64" t="s">
+        <v>58</v>
+      </c>
+      <c r="I24" s="64" t="s">
         <v>56</v>
       </c>
-      <c r="G24" s="65" t="s">
-        <v>57</v>
-      </c>
-      <c r="H24" s="65" t="s">
-        <v>58</v>
-      </c>
-      <c r="I24" s="65"/>
-      <c r="J24" s="65"/>
-      <c r="K24" s="65" t="s">
+      <c r="J24" s="64"/>
+      <c r="K24" s="64"/>
+      <c r="L24" s="64" t="s">
         <v>59</v>
       </c>
-      <c r="L24" s="65"/>
-      <c r="M24" s="65" t="s">
+      <c r="M24" s="64"/>
+      <c r="N24" s="64" t="s">
         <v>60</v>
       </c>
-      <c r="N24" s="10"/>
+      <c r="O24" s="10"/>
     </row>
     <row r="25" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="B25" s="97"/>
-      <c r="C25" s="65"/>
-      <c r="D25" s="113"/>
-      <c r="E25" s="65"/>
-      <c r="F25" s="65"/>
-      <c r="G25" s="65"/>
-      <c r="H25" s="65"/>
-      <c r="I25" s="65"/>
-      <c r="J25" s="65"/>
-      <c r="K25" s="65"/>
-      <c r="L25" s="65"/>
-      <c r="M25" s="65"/>
-      <c r="N25" s="10"/>
+      <c r="B25" s="60"/>
+      <c r="C25" s="61"/>
+      <c r="D25" s="64"/>
+      <c r="E25" s="64"/>
+      <c r="F25" s="61"/>
+      <c r="G25" s="61"/>
+      <c r="H25" s="61"/>
+      <c r="I25" s="61"/>
+      <c r="J25" s="61"/>
+      <c r="K25" s="61"/>
+      <c r="L25" s="61"/>
+      <c r="M25" s="61"/>
+      <c r="N25" s="61"/>
+      <c r="O25" s="10"/>
     </row>
     <row r="26" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B26" s="12" t="s">
@@ -2247,28 +2252,31 @@
         <v>123</v>
       </c>
       <c r="D26" s="36" t="s">
+        <v>130</v>
+      </c>
+      <c r="E26" s="36" t="s">
         <v>145</v>
       </c>
-      <c r="E26" s="42"/>
-      <c r="F26" s="37" t="s">
+      <c r="F26" s="40"/>
+      <c r="G26" s="50" t="s">
+        <v>62</v>
+      </c>
+      <c r="H26" s="50" t="s">
+        <v>63</v>
+      </c>
+      <c r="I26" s="62" t="s">
         <v>61</v>
       </c>
-      <c r="G26" s="16" t="s">
-        <v>62</v>
-      </c>
-      <c r="H26" s="66" t="s">
-        <v>63</v>
-      </c>
-      <c r="I26" s="66"/>
-      <c r="J26" s="66"/>
-      <c r="K26" s="66" t="s">
+      <c r="J26" s="62"/>
+      <c r="K26" s="62"/>
+      <c r="L26" s="62" t="s">
         <v>64</v>
       </c>
-      <c r="L26" s="66"/>
-      <c r="M26" s="16" t="s">
+      <c r="M26" s="62"/>
+      <c r="N26" s="16" t="s">
         <v>65</v>
       </c>
-      <c r="N26" s="10"/>
+      <c r="O26" s="10"/>
     </row>
     <row r="27" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B27" s="16"/>
@@ -2277,13 +2285,14 @@
       <c r="E27" s="16"/>
       <c r="F27" s="16"/>
       <c r="G27" s="16"/>
-      <c r="H27" s="104"/>
-      <c r="I27" s="105"/>
-      <c r="J27" s="106"/>
-      <c r="K27" s="66"/>
-      <c r="L27" s="66"/>
-      <c r="M27" s="16"/>
-      <c r="N27" s="10"/>
+      <c r="H27" s="16"/>
+      <c r="I27" s="65"/>
+      <c r="J27" s="66"/>
+      <c r="K27" s="67"/>
+      <c r="L27" s="62"/>
+      <c r="M27" s="62"/>
+      <c r="N27" s="16"/>
+      <c r="O27" s="10"/>
     </row>
     <row r="28" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B28" s="16"/>
@@ -2292,13 +2301,14 @@
       <c r="E28" s="16"/>
       <c r="F28" s="16"/>
       <c r="G28" s="16"/>
-      <c r="H28" s="72"/>
-      <c r="I28" s="72"/>
-      <c r="J28" s="72"/>
-      <c r="K28" s="66"/>
-      <c r="L28" s="66"/>
-      <c r="M28" s="16"/>
-      <c r="N28" s="10"/>
+      <c r="H28" s="16"/>
+      <c r="I28" s="116"/>
+      <c r="J28" s="116"/>
+      <c r="K28" s="116"/>
+      <c r="L28" s="62"/>
+      <c r="M28" s="62"/>
+      <c r="N28" s="16"/>
+      <c r="O28" s="10"/>
     </row>
     <row r="29" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B29" s="10"/>
@@ -2316,21 +2326,21 @@
       <c r="N29" s="10"/>
     </row>
     <row r="30" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B30" s="69" t="s">
+      <c r="B30" s="113" t="s">
         <v>66</v>
       </c>
-      <c r="C30" s="69"/>
-      <c r="D30" s="69"/>
-      <c r="E30" s="69"/>
+      <c r="C30" s="113"/>
+      <c r="D30" s="113"/>
+      <c r="E30" s="113"/>
       <c r="F30" s="18"/>
-      <c r="G30" s="70" t="s">
+      <c r="G30" s="114" t="s">
         <v>67</v>
       </c>
-      <c r="H30" s="71"/>
-      <c r="I30" s="115" t="s">
+      <c r="H30" s="115"/>
+      <c r="I30" s="54" t="s">
         <v>144</v>
       </c>
-      <c r="J30" s="116"/>
+      <c r="J30" s="55"/>
       <c r="K30" s="26" t="s">
         <v>15</v>
       </c>
@@ -2343,23 +2353,23 @@
         <v>68</v>
       </c>
       <c r="C31" s="20"/>
-      <c r="D31" s="66" t="s">
+      <c r="D31" s="62" t="s">
         <v>149</v>
       </c>
-      <c r="E31" s="66"/>
+      <c r="E31" s="62"/>
       <c r="F31" s="10"/>
-      <c r="G31" s="67" t="s">
+      <c r="G31" s="111" t="s">
         <v>140</v>
       </c>
-      <c r="H31" s="68"/>
-      <c r="I31" s="118" t="s">
+      <c r="H31" s="112"/>
+      <c r="I31" s="58" t="s">
         <v>143</v>
       </c>
-      <c r="J31" s="118"/>
-      <c r="K31" s="117" t="s">
+      <c r="J31" s="58"/>
+      <c r="K31" s="56" t="s">
         <v>142</v>
       </c>
-      <c r="L31" s="74"/>
+      <c r="L31" s="57"/>
       <c r="M31" s="10"/>
       <c r="N31" s="10"/>
     </row>
@@ -2368,10 +2378,10 @@
         <v>69</v>
       </c>
       <c r="C32" s="20"/>
-      <c r="D32" s="66" t="s">
+      <c r="D32" s="62" t="s">
         <v>150</v>
       </c>
-      <c r="E32" s="66"/>
+      <c r="E32" s="62"/>
       <c r="F32" s="10"/>
       <c r="G32" s="10"/>
       <c r="H32" s="10"/>
@@ -2437,86 +2447,82 @@
       <c r="M35" s="10"/>
       <c r="N35" s="10"/>
     </row>
-    <row r="36" spans="2:14" ht="39" x14ac:dyDescent="0.35">
-      <c r="B36" s="46" t="s">
+    <row r="36" spans="2:14" ht="21" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B36" s="44" t="s">
         <v>72</v>
       </c>
-      <c r="C36" s="47"/>
-      <c r="D36" s="47"/>
-      <c r="E36" s="48"/>
+      <c r="C36" s="45"/>
+      <c r="D36" s="45"/>
+      <c r="E36" s="46"/>
       <c r="F36" s="28"/>
-      <c r="G36" s="49" t="s">
-        <v>125</v>
-      </c>
-      <c r="H36" s="50" t="s">
-        <v>130</v>
-      </c>
-      <c r="I36" s="28"/>
+      <c r="G36" s="123" t="s">
+        <v>127</v>
+      </c>
+      <c r="H36" s="124"/>
+      <c r="I36" s="47" t="s">
+        <v>131</v>
+      </c>
       <c r="J36" s="28"/>
     </row>
     <row r="37" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B37" s="56" t="s">
+      <c r="B37" s="102" t="s">
         <v>73</v>
       </c>
-      <c r="C37" s="57"/>
-      <c r="D37" s="57"/>
-      <c r="E37" s="58"/>
+      <c r="C37" s="103"/>
+      <c r="D37" s="103"/>
+      <c r="E37" s="104"/>
       <c r="F37" s="28"/>
-      <c r="G37" s="49" t="s">
-        <v>127</v>
-      </c>
-      <c r="H37" s="50" t="s">
-        <v>131</v>
-      </c>
-      <c r="I37" s="28"/>
+      <c r="G37" s="123" t="s">
+        <v>128</v>
+      </c>
+      <c r="H37" s="124"/>
+      <c r="I37" s="47" t="s">
+        <v>132</v>
+      </c>
       <c r="J37" s="28"/>
     </row>
     <row r="38" spans="2:14" ht="26" x14ac:dyDescent="0.35">
-      <c r="B38" s="59"/>
-      <c r="C38" s="60"/>
-      <c r="D38" s="60"/>
-      <c r="E38" s="61"/>
+      <c r="B38" s="105"/>
+      <c r="C38" s="106"/>
+      <c r="D38" s="106"/>
+      <c r="E38" s="107"/>
       <c r="F38" s="28"/>
-      <c r="G38" s="49" t="s">
-        <v>128</v>
-      </c>
-      <c r="H38" s="50" t="s">
-        <v>132</v>
-      </c>
-      <c r="I38" s="28"/>
+      <c r="G38" s="123" t="s">
+        <v>129</v>
+      </c>
+      <c r="H38" s="124"/>
+      <c r="I38" s="49" t="s">
+        <v>133</v>
+      </c>
       <c r="J38" s="28"/>
     </row>
-    <row r="39" spans="2:14" ht="26" x14ac:dyDescent="0.35">
-      <c r="B39" s="59"/>
-      <c r="C39" s="60"/>
-      <c r="D39" s="60"/>
-      <c r="E39" s="61"/>
+    <row r="39" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B39" s="105"/>
+      <c r="C39" s="106"/>
+      <c r="D39" s="106"/>
+      <c r="E39" s="107"/>
       <c r="F39" s="28"/>
-      <c r="G39" s="49" t="s">
-        <v>129</v>
-      </c>
-      <c r="H39" s="52" t="s">
-        <v>133</v>
-      </c>
+      <c r="G39" s="28"/>
+      <c r="H39" s="28"/>
       <c r="I39" s="28"/>
       <c r="J39" s="28"/>
     </row>
     <row r="40" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B40" s="59"/>
-      <c r="C40" s="60"/>
-      <c r="D40" s="60"/>
-      <c r="E40" s="61"/>
+      <c r="B40" s="105"/>
+      <c r="C40" s="106"/>
+      <c r="D40" s="106"/>
+      <c r="E40" s="107"/>
       <c r="F40" s="28"/>
       <c r="G40" s="28"/>
-      <c r="H40" s="28"/>
+      <c r="H40" s="10"/>
       <c r="I40" s="28"/>
       <c r="J40" s="28"/>
     </row>
     <row r="41" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B41" s="62"/>
-      <c r="C41" s="63"/>
-      <c r="D41" s="63"/>
-      <c r="E41" s="64"/>
+      <c r="B41" s="108"/>
+      <c r="C41" s="109"/>
+      <c r="D41" s="109"/>
+      <c r="E41" s="110"/>
       <c r="F41" s="28"/>
       <c r="G41" s="28"/>
       <c r="H41" s="10"/>
@@ -2529,7 +2535,6 @@
       <c r="D42" s="28"/>
       <c r="E42" s="28"/>
       <c r="F42" s="28"/>
-      <c r="G42" s="28"/>
       <c r="H42" s="10"/>
       <c r="I42" s="10"/>
       <c r="J42" s="10"/>
@@ -2549,7 +2554,7 @@
       <c r="C44" s="28"/>
       <c r="D44" s="28"/>
       <c r="E44" s="28"/>
-      <c r="H44" s="10"/>
+      <c r="H44" s="23"/>
       <c r="I44" s="10"/>
       <c r="J44" s="10"/>
       <c r="K44" s="10"/>
@@ -2578,7 +2583,7 @@
       <c r="C47" s="28"/>
       <c r="D47" s="28"/>
       <c r="E47" s="28"/>
-      <c r="H47" s="23"/>
+      <c r="H47" s="17"/>
       <c r="I47" s="23"/>
       <c r="J47" s="23"/>
     </row>
@@ -2587,7 +2592,7 @@
       <c r="C48" s="28"/>
       <c r="D48" s="28"/>
       <c r="E48" s="28"/>
-      <c r="H48" s="17"/>
+      <c r="G48" s="28"/>
       <c r="I48" s="23"/>
       <c r="J48" s="23"/>
     </row>
@@ -2606,7 +2611,6 @@
       <c r="D50" s="28"/>
       <c r="E50" s="28"/>
       <c r="F50" s="28"/>
-      <c r="G50" s="28"/>
     </row>
     <row r="51" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B51" s="28"/>
@@ -2616,36 +2620,40 @@
       <c r="F51" s="28"/>
     </row>
     <row r="53" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="J53" s="43"/>
+      <c r="J53" s="41"/>
     </row>
   </sheetData>
-  <mergeCells count="68">
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="I13:K13"/>
-    <mergeCell ref="I30:J30"/>
-    <mergeCell ref="K31:L31"/>
-    <mergeCell ref="I31:J31"/>
-    <mergeCell ref="B23:L23"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="K24:L25"/>
-    <mergeCell ref="K28:L28"/>
-    <mergeCell ref="D24:D25"/>
-    <mergeCell ref="M16:N17"/>
-    <mergeCell ref="I12:K12"/>
-    <mergeCell ref="H27:J27"/>
-    <mergeCell ref="K27:L27"/>
-    <mergeCell ref="K21:L21"/>
-    <mergeCell ref="M24:M25"/>
-    <mergeCell ref="H24:J25"/>
-    <mergeCell ref="H26:J26"/>
-    <mergeCell ref="K26:L26"/>
-    <mergeCell ref="B15:N15"/>
-    <mergeCell ref="L12:M12"/>
-    <mergeCell ref="K18:L18"/>
-    <mergeCell ref="G12:H12"/>
+  <mergeCells count="73">
+    <mergeCell ref="G36:H36"/>
+    <mergeCell ref="G37:H37"/>
+    <mergeCell ref="G38:H38"/>
+    <mergeCell ref="L10:M10"/>
+    <mergeCell ref="L11:M11"/>
+    <mergeCell ref="K20:L20"/>
+    <mergeCell ref="B37:E41"/>
+    <mergeCell ref="G16:G18"/>
+    <mergeCell ref="I16:I18"/>
+    <mergeCell ref="J16:L17"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="G31:H31"/>
+    <mergeCell ref="C24:C25"/>
+    <mergeCell ref="F24:F25"/>
     <mergeCell ref="G24:G25"/>
-    <mergeCell ref="H16:H18"/>
-    <mergeCell ref="K19:L19"/>
+    <mergeCell ref="B30:E30"/>
+    <mergeCell ref="G30:H30"/>
+    <mergeCell ref="I28:K28"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="C16:C18"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="G10:H10"/>
+    <mergeCell ref="G11:H11"/>
+    <mergeCell ref="G9:H9"/>
     <mergeCell ref="C3:G3"/>
     <mergeCell ref="C4:G4"/>
     <mergeCell ref="F16:F18"/>
@@ -2662,35 +2670,36 @@
     <mergeCell ref="I10:K10"/>
     <mergeCell ref="I11:K11"/>
     <mergeCell ref="D16:D18"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="G10:H10"/>
-    <mergeCell ref="G11:H11"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="C16:C18"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="L10:M10"/>
-    <mergeCell ref="L11:M11"/>
-    <mergeCell ref="K20:L20"/>
-    <mergeCell ref="B37:E41"/>
-    <mergeCell ref="G16:G18"/>
-    <mergeCell ref="I16:I18"/>
-    <mergeCell ref="J16:L17"/>
-    <mergeCell ref="D31:E31"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="G31:H31"/>
-    <mergeCell ref="C24:C25"/>
+    <mergeCell ref="M16:N17"/>
+    <mergeCell ref="I12:K12"/>
+    <mergeCell ref="I27:K27"/>
+    <mergeCell ref="L27:M27"/>
+    <mergeCell ref="K21:L21"/>
+    <mergeCell ref="N24:N25"/>
+    <mergeCell ref="I24:K25"/>
+    <mergeCell ref="I26:K26"/>
+    <mergeCell ref="L26:M26"/>
+    <mergeCell ref="B15:N15"/>
+    <mergeCell ref="L12:M12"/>
+    <mergeCell ref="K18:L18"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="H24:H25"/>
+    <mergeCell ref="H16:H18"/>
+    <mergeCell ref="K19:L19"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="I13:K13"/>
+    <mergeCell ref="I30:J30"/>
+    <mergeCell ref="K31:L31"/>
+    <mergeCell ref="I31:J31"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="L24:M25"/>
+    <mergeCell ref="L28:M28"/>
     <mergeCell ref="E24:E25"/>
-    <mergeCell ref="F24:F25"/>
-    <mergeCell ref="B30:E30"/>
-    <mergeCell ref="G30:H30"/>
-    <mergeCell ref="H28:J28"/>
+    <mergeCell ref="D24:D25"/>
+    <mergeCell ref="B23:N23"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E26:E28" xr:uid="{B316A799-CF60-4C99-A88E-2204076E38E6}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F26:F28" xr:uid="{B316A799-CF60-4C99-A88E-2204076E38E6}">
       <formula1>"กล่อง, เม็ด, ไวอัล, แอมพูล, ขวด, box, tablet, vial, ampoul, bottle"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2751,7 +2760,7 @@
       <c r="B2" t="s">
         <v>77</v>
       </c>
-      <c r="C2" s="120"/>
+      <c r="C2" s="117"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
@@ -2760,7 +2769,7 @@
       <c r="B3" t="s">
         <v>79</v>
       </c>
-      <c r="C3" s="121"/>
+      <c r="C3" s="118"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
@@ -2769,7 +2778,7 @@
       <c r="B4" t="s">
         <v>80</v>
       </c>
-      <c r="C4" s="121"/>
+      <c r="C4" s="118"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
@@ -2778,7 +2787,7 @@
       <c r="B5" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="121"/>
+      <c r="C5" s="118"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
@@ -2787,7 +2796,7 @@
       <c r="B6" t="s">
         <v>20</v>
       </c>
-      <c r="C6" s="122"/>
+      <c r="C6" s="119"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
@@ -3464,17 +3473,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <SharedWithUsers xmlns="1444eecc-14bb-4066-abe6-ce6de21d9439">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3675,20 +3679,23 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <SharedWithUsers xmlns="1444eecc-14bb-4066-abe6-ce6de21d9439">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7EBE950A-5812-419E-B174-6A5D9B8E0414}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A00E6A9-20DD-4842-9306-307EB080AF2E}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="1444eecc-14bb-4066-abe6-ce6de21d9439"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -3713,9 +3720,11 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A00E6A9-20DD-4842-9306-307EB080AF2E}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7EBE950A-5812-419E-B174-6A5D9B8E0414}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="1444eecc-14bb-4066-abe6-ce6de21d9439"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Excel template should display Quotation delivery channels in each row instead of comma separated values
</commit_message>
<xml_diff>
--- a/srv/xlsx-templates/TH - Quotation Template.xlsx
+++ b/srv/xlsx-templates/TH - Quotation Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27726"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EHMHV\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vasub\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{798E66B4-719A-4816-A196-14D9CAC1A823}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D28421B1-1281-4B0D-A2CA-04A2854EF551}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19200" windowHeight="9020" xr2:uid="{F5CC2154-27BB-4652-B61E-D913F0CC6809}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{F5CC2154-27BB-4652-B61E-D913F0CC6809}"/>
   </bookViews>
   <sheets>
     <sheet name="Quotation" sheetId="3" r:id="rId1"/>
@@ -456,18 +456,9 @@
     <t>${offerValidation.DeliveryDue}</t>
   </si>
   <si>
-    <t>${offerValidation.QuotationDeliverymethod}</t>
-  </si>
-  <si>
     <t>${offerValidation.TENDER_SUBMITTED_BY}</t>
   </si>
   <si>
-    <t>${offerValidation.QuotationRecipientcontact}</t>
-  </si>
-  <si>
-    <t>${offerValidation.QuotationRecipientname}</t>
-  </si>
-  <si>
     <t>Receiver Information (Name)</t>
   </si>
   <si>
@@ -490,6 +481,15 @@
   </si>
   <si>
     <t>${table:offerProductValidation.TenderAnnouncementReference}</t>
+  </si>
+  <si>
+    <t>${table:quotationDelevery.QuotationDeliverymethod}</t>
+  </si>
+  <si>
+    <t>${table:quotationDelevery.QuotationRecipientname}</t>
+  </si>
+  <si>
+    <t>${table:quotationDelevery.QuotationRecipientcontact}</t>
   </si>
 </sst>
 </file>
@@ -497,8 +497,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="164" formatCode="#\.###\.###.00"/>
+    <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="#\.###\.###.00"/>
   </numFmts>
   <fonts count="13" x14ac:knownFonts="1">
     <font>
@@ -851,7 +851,7 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="125">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -863,7 +863,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -874,8 +874,8 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="5" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="43" fontId="5" fillId="0" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -917,7 +917,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="43" fontId="5" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
@@ -965,197 +965,206 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="43" fontId="5" fillId="0" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="6" fillId="0" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1168,15 +1177,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1215,16 +1215,16 @@
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="#\.###\.###.00"/>
+      <numFmt numFmtId="165" formatCode="#\.###\.###.00"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="#\.###\.###.00"/>
+      <numFmt numFmtId="165" formatCode="#\.###\.###.00"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="#\.###\.###.00"/>
+      <numFmt numFmtId="165" formatCode="#\.###\.###.00"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="#\.###\.###.00"/>
+      <numFmt numFmtId="165" formatCode="#\.###\.###.00"/>
     </dxf>
     <dxf>
       <font>
@@ -1748,46 +1748,46 @@
       <c r="B3" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="86" t="s">
+      <c r="C3" s="59" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="87"/>
-      <c r="E3" s="87"/>
-      <c r="F3" s="87"/>
-      <c r="G3" s="88"/>
+      <c r="D3" s="60"/>
+      <c r="E3" s="60"/>
+      <c r="F3" s="60"/>
+      <c r="G3" s="61"/>
       <c r="H3" s="10"/>
       <c r="I3" s="25" t="s">
         <v>2</v>
       </c>
-      <c r="J3" s="86" t="s">
+      <c r="J3" s="59" t="s">
         <v>3</v>
       </c>
-      <c r="K3" s="87"/>
-      <c r="L3" s="87"/>
-      <c r="M3" s="88"/>
+      <c r="K3" s="60"/>
+      <c r="L3" s="60"/>
+      <c r="M3" s="61"/>
       <c r="N3" s="10"/>
     </row>
     <row r="4" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B4" s="26" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="80" t="s">
+      <c r="C4" s="62" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="89"/>
-      <c r="E4" s="89"/>
-      <c r="F4" s="89"/>
-      <c r="G4" s="81"/>
+      <c r="D4" s="63"/>
+      <c r="E4" s="63"/>
+      <c r="F4" s="63"/>
+      <c r="G4" s="64"/>
       <c r="H4" s="10"/>
       <c r="I4" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="J4" s="95" t="s">
+      <c r="J4" s="70" t="s">
         <v>6</v>
       </c>
-      <c r="K4" s="96"/>
-      <c r="L4" s="96"/>
-      <c r="M4" s="97"/>
+      <c r="K4" s="71"/>
+      <c r="L4" s="71"/>
+      <c r="M4" s="72"/>
       <c r="N4" s="10"/>
     </row>
     <row r="5" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -1836,151 +1836,151 @@
       <c r="N7" s="10"/>
     </row>
     <row r="8" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B8" s="90" t="s">
+      <c r="B8" s="65" t="s">
         <v>133</v>
       </c>
-      <c r="C8" s="91"/>
-      <c r="D8" s="91"/>
-      <c r="E8" s="91"/>
-      <c r="F8" s="91"/>
-      <c r="G8" s="91"/>
-      <c r="H8" s="91"/>
-      <c r="I8" s="91"/>
-      <c r="J8" s="91"/>
-      <c r="K8" s="91"/>
-      <c r="L8" s="91"/>
-      <c r="M8" s="91"/>
-      <c r="N8" s="92"/>
+      <c r="C8" s="66"/>
+      <c r="D8" s="66"/>
+      <c r="E8" s="66"/>
+      <c r="F8" s="66"/>
+      <c r="G8" s="66"/>
+      <c r="H8" s="66"/>
+      <c r="I8" s="66"/>
+      <c r="J8" s="66"/>
+      <c r="K8" s="66"/>
+      <c r="L8" s="66"/>
+      <c r="M8" s="66"/>
+      <c r="N8" s="67"/>
     </row>
     <row r="9" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B9" s="98" t="s">
+      <c r="B9" s="73" t="s">
         <v>7</v>
       </c>
-      <c r="C9" s="99"/>
-      <c r="D9" s="78" t="s">
+      <c r="C9" s="74"/>
+      <c r="D9" s="81" t="s">
         <v>8</v>
       </c>
-      <c r="E9" s="78"/>
+      <c r="E9" s="81"/>
       <c r="F9" s="38"/>
-      <c r="G9" s="84" t="s">
+      <c r="G9" s="85" t="s">
         <v>9</v>
       </c>
-      <c r="H9" s="85"/>
-      <c r="I9" s="101" t="s">
+      <c r="H9" s="86"/>
+      <c r="I9" s="77" t="s">
         <v>10</v>
       </c>
-      <c r="J9" s="101"/>
-      <c r="K9" s="102"/>
-      <c r="L9" s="93" t="s">
+      <c r="J9" s="77"/>
+      <c r="K9" s="78"/>
+      <c r="L9" s="68" t="s">
         <v>11</v>
       </c>
-      <c r="M9" s="94"/>
+      <c r="M9" s="69"/>
       <c r="N9" s="48" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="10" spans="2:14" ht="26.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="76" t="s">
+      <c r="B10" s="75" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="77"/>
-      <c r="D10" s="79" t="str">
+      <c r="C10" s="76"/>
+      <c r="D10" s="82" t="str">
         <f>Settings!A14</f>
         <v>${offerValidation.CUSTOMER_CODE}</v>
       </c>
-      <c r="E10" s="79"/>
+      <c r="E10" s="82"/>
       <c r="F10" s="38"/>
-      <c r="G10" s="82" t="s">
+      <c r="G10" s="83" t="s">
         <v>13</v>
       </c>
-      <c r="H10" s="82"/>
-      <c r="I10" s="103" t="s">
+      <c r="H10" s="83"/>
+      <c r="I10" s="79" t="s">
         <v>14</v>
       </c>
-      <c r="J10" s="103"/>
-      <c r="K10" s="104"/>
-      <c r="L10" s="53" t="s">
+      <c r="J10" s="79"/>
+      <c r="K10" s="80"/>
+      <c r="L10" s="89" t="s">
         <v>15</v>
       </c>
-      <c r="M10" s="54"/>
+      <c r="M10" s="90"/>
       <c r="N10" s="48" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="11" spans="2:14" ht="26.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="76" t="s">
+      <c r="B11" s="75" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="77"/>
-      <c r="D11" s="80" t="str">
+      <c r="C11" s="76"/>
+      <c r="D11" s="62" t="str">
         <f>Settings!A9</f>
         <v>${offerValidation.INSTITUTENAME}</v>
       </c>
-      <c r="E11" s="81"/>
+      <c r="E11" s="64"/>
       <c r="F11" s="38"/>
-      <c r="G11" s="83" t="s">
+      <c r="G11" s="84" t="s">
         <v>17</v>
       </c>
-      <c r="H11" s="83"/>
-      <c r="I11" s="103" t="s">
+      <c r="H11" s="84"/>
+      <c r="I11" s="79" t="s">
         <v>18</v>
       </c>
-      <c r="J11" s="103"/>
-      <c r="K11" s="104"/>
-      <c r="L11" s="53" t="s">
+      <c r="J11" s="79"/>
+      <c r="K11" s="80"/>
+      <c r="L11" s="89" t="s">
         <v>19</v>
       </c>
-      <c r="M11" s="54"/>
+      <c r="M11" s="90"/>
       <c r="N11" s="48" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="12" spans="2:14" ht="26" x14ac:dyDescent="0.35">
-      <c r="B12" s="76" t="s">
+      <c r="B12" s="75" t="s">
         <v>20</v>
       </c>
-      <c r="C12" s="77"/>
-      <c r="D12" s="74" t="s">
+      <c r="C12" s="76"/>
+      <c r="D12" s="87" t="s">
         <v>21</v>
       </c>
-      <c r="E12" s="75"/>
+      <c r="E12" s="88"/>
       <c r="F12" s="10"/>
-      <c r="G12" s="112" t="s">
+      <c r="G12" s="92" t="s">
         <v>22</v>
       </c>
-      <c r="H12" s="112"/>
-      <c r="I12" s="105" t="s">
+      <c r="H12" s="92"/>
+      <c r="I12" s="94" t="s">
         <v>23</v>
       </c>
-      <c r="J12" s="105"/>
-      <c r="K12" s="106"/>
-      <c r="L12" s="53" t="s">
+      <c r="J12" s="94"/>
+      <c r="K12" s="95"/>
+      <c r="L12" s="89" t="s">
         <v>15</v>
       </c>
-      <c r="M12" s="54"/>
+      <c r="M12" s="90"/>
       <c r="N12" s="48" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="13" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B13" s="76" t="s">
+      <c r="B13" s="75" t="s">
         <v>24</v>
       </c>
-      <c r="C13" s="77"/>
-      <c r="D13" s="74" t="s">
+      <c r="C13" s="76"/>
+      <c r="D13" s="87" t="s">
         <v>25</v>
       </c>
-      <c r="E13" s="75"/>
+      <c r="E13" s="88"/>
       <c r="F13" s="10"/>
-      <c r="G13" s="112" t="s">
+      <c r="G13" s="92" t="s">
         <v>124</v>
       </c>
-      <c r="H13" s="112"/>
-      <c r="I13" s="105" t="s">
+      <c r="H13" s="92"/>
+      <c r="I13" s="94" t="s">
         <v>134</v>
       </c>
-      <c r="J13" s="105"/>
-      <c r="K13" s="106"/>
+      <c r="J13" s="94"/>
+      <c r="K13" s="95"/>
     </row>
     <row r="14" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B14" s="10"/>
@@ -1995,88 +1995,88 @@
       <c r="K14" s="10"/>
     </row>
     <row r="15" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B15" s="90" t="s">
+      <c r="B15" s="65" t="s">
         <v>26</v>
       </c>
-      <c r="C15" s="91"/>
-      <c r="D15" s="91"/>
-      <c r="E15" s="91"/>
-      <c r="F15" s="91"/>
-      <c r="G15" s="91"/>
-      <c r="H15" s="91"/>
-      <c r="I15" s="91"/>
-      <c r="J15" s="91"/>
-      <c r="K15" s="91"/>
-      <c r="L15" s="91"/>
-      <c r="M15" s="91"/>
-      <c r="N15" s="92"/>
+      <c r="C15" s="66"/>
+      <c r="D15" s="66"/>
+      <c r="E15" s="66"/>
+      <c r="F15" s="66"/>
+      <c r="G15" s="66"/>
+      <c r="H15" s="66"/>
+      <c r="I15" s="66"/>
+      <c r="J15" s="66"/>
+      <c r="K15" s="66"/>
+      <c r="L15" s="66"/>
+      <c r="M15" s="66"/>
+      <c r="N15" s="67"/>
     </row>
     <row r="16" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B16" s="100" t="s">
+      <c r="B16" s="54" t="s">
         <v>27</v>
       </c>
-      <c r="C16" s="65" t="s">
+      <c r="C16" s="56" t="s">
         <v>28</v>
       </c>
-      <c r="D16" s="65" t="s">
+      <c r="D16" s="56" t="s">
         <v>29</v>
       </c>
-      <c r="E16" s="65" t="s">
+      <c r="E16" s="56" t="s">
         <v>30</v>
       </c>
-      <c r="F16" s="65" t="s">
+      <c r="F16" s="56" t="s">
         <v>31</v>
       </c>
-      <c r="G16" s="65" t="s">
+      <c r="G16" s="56" t="s">
         <v>32</v>
       </c>
-      <c r="H16" s="113" t="s">
+      <c r="H16" s="93" t="s">
         <v>33</v>
       </c>
-      <c r="I16" s="65" t="s">
+      <c r="I16" s="56" t="s">
         <v>34</v>
       </c>
-      <c r="J16" s="65" t="s">
+      <c r="J16" s="56" t="s">
         <v>35</v>
       </c>
-      <c r="K16" s="65"/>
-      <c r="L16" s="65"/>
-      <c r="M16" s="65" t="s">
+      <c r="K16" s="56"/>
+      <c r="L16" s="56"/>
+      <c r="M16" s="56" t="s">
         <v>36</v>
       </c>
-      <c r="N16" s="65"/>
+      <c r="N16" s="56"/>
     </row>
     <row r="17" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="B17" s="100"/>
-      <c r="C17" s="65"/>
-      <c r="D17" s="65"/>
-      <c r="E17" s="65"/>
-      <c r="F17" s="65"/>
-      <c r="G17" s="65"/>
-      <c r="H17" s="114"/>
-      <c r="I17" s="65"/>
-      <c r="J17" s="65"/>
-      <c r="K17" s="65"/>
-      <c r="L17" s="65"/>
-      <c r="M17" s="65"/>
-      <c r="N17" s="65"/>
+      <c r="B17" s="54"/>
+      <c r="C17" s="56"/>
+      <c r="D17" s="56"/>
+      <c r="E17" s="56"/>
+      <c r="F17" s="56"/>
+      <c r="G17" s="56"/>
+      <c r="H17" s="58"/>
+      <c r="I17" s="56"/>
+      <c r="J17" s="56"/>
+      <c r="K17" s="56"/>
+      <c r="L17" s="56"/>
+      <c r="M17" s="56"/>
+      <c r="N17" s="56"/>
     </row>
     <row r="18" spans="2:15" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="100"/>
-      <c r="C18" s="65"/>
-      <c r="D18" s="65"/>
-      <c r="E18" s="65"/>
-      <c r="F18" s="65"/>
-      <c r="G18" s="65"/>
-      <c r="H18" s="69"/>
-      <c r="I18" s="65"/>
+      <c r="B18" s="54"/>
+      <c r="C18" s="56"/>
+      <c r="D18" s="56"/>
+      <c r="E18" s="56"/>
+      <c r="F18" s="56"/>
+      <c r="G18" s="56"/>
+      <c r="H18" s="55"/>
+      <c r="I18" s="56"/>
       <c r="J18" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="K18" s="111" t="s">
+      <c r="K18" s="91" t="s">
         <v>38</v>
       </c>
-      <c r="L18" s="111"/>
+      <c r="L18" s="91"/>
       <c r="M18" s="11" t="s">
         <v>37</v>
       </c>
@@ -2112,10 +2112,10 @@
       <c r="J19" s="36" t="s">
         <v>47</v>
       </c>
-      <c r="K19" s="115" t="s">
+      <c r="K19" s="118" t="s">
         <v>48</v>
       </c>
-      <c r="L19" s="115"/>
+      <c r="L19" s="118"/>
       <c r="M19" s="39" t="s">
         <v>49</v>
       </c>
@@ -2134,8 +2134,8 @@
       <c r="H20" s="13"/>
       <c r="I20" s="12"/>
       <c r="J20" s="15"/>
-      <c r="K20" s="55"/>
-      <c r="L20" s="55"/>
+      <c r="K20" s="117"/>
+      <c r="L20" s="117"/>
       <c r="M20" s="14"/>
       <c r="N20" s="35"/>
     </row>
@@ -2149,10 +2149,10 @@
       <c r="H21" s="13"/>
       <c r="I21" s="12"/>
       <c r="J21" s="15"/>
-      <c r="K21" s="110" t="s">
+      <c r="K21" s="114" t="s">
         <v>51</v>
       </c>
-      <c r="L21" s="110"/>
+      <c r="L21" s="114"/>
       <c r="M21" s="36" t="s">
         <v>52</v>
       </c>
@@ -2176,72 +2176,72 @@
       <c r="N22" s="10"/>
     </row>
     <row r="23" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="B23" s="121" t="s">
+      <c r="B23" s="51" t="s">
         <v>54</v>
       </c>
-      <c r="C23" s="121"/>
-      <c r="D23" s="121"/>
-      <c r="E23" s="121"/>
-      <c r="F23" s="121"/>
-      <c r="G23" s="121"/>
-      <c r="H23" s="121"/>
-      <c r="I23" s="121"/>
-      <c r="J23" s="121"/>
-      <c r="K23" s="121"/>
-      <c r="L23" s="121"/>
-      <c r="M23" s="121"/>
-      <c r="N23" s="121"/>
+      <c r="C23" s="51"/>
+      <c r="D23" s="51"/>
+      <c r="E23" s="51"/>
+      <c r="F23" s="51"/>
+      <c r="G23" s="51"/>
+      <c r="H23" s="51"/>
+      <c r="I23" s="51"/>
+      <c r="J23" s="51"/>
+      <c r="K23" s="51"/>
+      <c r="L23" s="51"/>
+      <c r="M23" s="51"/>
+      <c r="N23" s="51"/>
     </row>
     <row r="24" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="B24" s="120" t="s">
+      <c r="B24" s="53" t="s">
         <v>27</v>
       </c>
-      <c r="C24" s="69" t="s">
+      <c r="C24" s="55" t="s">
         <v>28</v>
       </c>
-      <c r="D24" s="114" t="s">
+      <c r="D24" s="58" t="s">
         <v>125</v>
       </c>
-      <c r="E24" s="114" t="s">
+      <c r="E24" s="58" t="s">
         <v>126</v>
       </c>
-      <c r="F24" s="69" t="s">
+      <c r="F24" s="55" t="s">
         <v>55</v>
       </c>
-      <c r="G24" s="69" t="s">
+      <c r="G24" s="55" t="s">
         <v>57</v>
       </c>
-      <c r="H24" s="69" t="s">
+      <c r="H24" s="55" t="s">
         <v>58</v>
       </c>
-      <c r="I24" s="69" t="s">
+      <c r="I24" s="55" t="s">
         <v>56</v>
       </c>
-      <c r="J24" s="69"/>
-      <c r="K24" s="69"/>
-      <c r="L24" s="69" t="s">
+      <c r="J24" s="55"/>
+      <c r="K24" s="55"/>
+      <c r="L24" s="55" t="s">
         <v>59</v>
       </c>
-      <c r="M24" s="69"/>
-      <c r="N24" s="69" t="s">
+      <c r="M24" s="55"/>
+      <c r="N24" s="55" t="s">
         <v>60</v>
       </c>
       <c r="O24" s="10"/>
     </row>
     <row r="25" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="B25" s="100"/>
-      <c r="C25" s="65"/>
-      <c r="D25" s="69"/>
-      <c r="E25" s="69"/>
-      <c r="F25" s="65"/>
-      <c r="G25" s="65"/>
-      <c r="H25" s="65"/>
-      <c r="I25" s="65"/>
-      <c r="J25" s="65"/>
-      <c r="K25" s="65"/>
-      <c r="L25" s="65"/>
-      <c r="M25" s="65"/>
-      <c r="N25" s="65"/>
+      <c r="B25" s="54"/>
+      <c r="C25" s="56"/>
+      <c r="D25" s="55"/>
+      <c r="E25" s="55"/>
+      <c r="F25" s="56"/>
+      <c r="G25" s="56"/>
+      <c r="H25" s="56"/>
+      <c r="I25" s="56"/>
+      <c r="J25" s="56"/>
+      <c r="K25" s="56"/>
+      <c r="L25" s="56"/>
+      <c r="M25" s="56"/>
+      <c r="N25" s="56"/>
       <c r="O25" s="10"/>
     </row>
     <row r="26" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -2252,10 +2252,10 @@
         <v>123</v>
       </c>
       <c r="D26" s="36" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="E26" s="36" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="F26" s="40"/>
       <c r="G26" s="50" t="s">
@@ -2264,15 +2264,15 @@
       <c r="H26" s="50" t="s">
         <v>63</v>
       </c>
-      <c r="I26" s="66" t="s">
+      <c r="I26" s="57" t="s">
         <v>61</v>
       </c>
-      <c r="J26" s="66"/>
-      <c r="K26" s="66"/>
-      <c r="L26" s="66" t="s">
+      <c r="J26" s="57"/>
+      <c r="K26" s="57"/>
+      <c r="L26" s="57" t="s">
         <v>64</v>
       </c>
-      <c r="M26" s="66"/>
+      <c r="M26" s="57"/>
       <c r="N26" s="16" t="s">
         <v>65</v>
       </c>
@@ -2286,11 +2286,11 @@
       <c r="F27" s="16"/>
       <c r="G27" s="16"/>
       <c r="H27" s="16"/>
-      <c r="I27" s="107"/>
-      <c r="J27" s="108"/>
-      <c r="K27" s="109"/>
-      <c r="L27" s="66"/>
-      <c r="M27" s="66"/>
+      <c r="I27" s="111"/>
+      <c r="J27" s="112"/>
+      <c r="K27" s="113"/>
+      <c r="L27" s="57"/>
+      <c r="M27" s="57"/>
       <c r="N27" s="16"/>
       <c r="O27" s="10"/>
     </row>
@@ -2302,11 +2302,11 @@
       <c r="F28" s="16"/>
       <c r="G28" s="16"/>
       <c r="H28" s="16"/>
-      <c r="I28" s="73"/>
-      <c r="J28" s="73"/>
-      <c r="K28" s="73"/>
-      <c r="L28" s="66"/>
-      <c r="M28" s="66"/>
+      <c r="I28" s="110"/>
+      <c r="J28" s="110"/>
+      <c r="K28" s="110"/>
+      <c r="L28" s="57"/>
+      <c r="M28" s="57"/>
       <c r="N28" s="16"/>
       <c r="O28" s="10"/>
     </row>
@@ -2326,21 +2326,21 @@
       <c r="N29" s="10"/>
     </row>
     <row r="30" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B30" s="70" t="s">
+      <c r="B30" s="107" t="s">
         <v>66</v>
       </c>
-      <c r="C30" s="70"/>
-      <c r="D30" s="70"/>
-      <c r="E30" s="70"/>
+      <c r="C30" s="107"/>
+      <c r="D30" s="107"/>
+      <c r="E30" s="107"/>
       <c r="F30" s="18"/>
-      <c r="G30" s="71" t="s">
+      <c r="G30" s="108" t="s">
         <v>67</v>
       </c>
-      <c r="H30" s="72"/>
-      <c r="I30" s="116" t="s">
-        <v>143</v>
-      </c>
-      <c r="J30" s="117"/>
+      <c r="H30" s="109"/>
+      <c r="I30" s="119" t="s">
+        <v>140</v>
+      </c>
+      <c r="J30" s="120"/>
       <c r="K30" s="26" t="s">
         <v>15</v>
       </c>
@@ -2353,23 +2353,23 @@
         <v>68</v>
       </c>
       <c r="C31" s="20"/>
-      <c r="D31" s="66" t="s">
+      <c r="D31" s="57" t="s">
+        <v>145</v>
+      </c>
+      <c r="E31" s="57"/>
+      <c r="F31" s="10"/>
+      <c r="G31" s="105" t="s">
         <v>148</v>
       </c>
-      <c r="E31" s="66"/>
-      <c r="F31" s="10"/>
-      <c r="G31" s="67" t="s">
-        <v>139</v>
-      </c>
-      <c r="H31" s="68"/>
-      <c r="I31" s="119" t="s">
-        <v>142</v>
-      </c>
-      <c r="J31" s="119"/>
-      <c r="K31" s="118" t="s">
-        <v>141</v>
-      </c>
-      <c r="L31" s="75"/>
+      <c r="H31" s="106"/>
+      <c r="I31" s="52" t="s">
+        <v>149</v>
+      </c>
+      <c r="J31" s="52"/>
+      <c r="K31" s="121" t="s">
+        <v>150</v>
+      </c>
+      <c r="L31" s="88"/>
       <c r="M31" s="10"/>
       <c r="N31" s="10"/>
     </row>
@@ -2378,10 +2378,10 @@
         <v>69</v>
       </c>
       <c r="C32" s="20"/>
-      <c r="D32" s="66" t="s">
-        <v>149</v>
-      </c>
-      <c r="E32" s="66"/>
+      <c r="D32" s="57" t="s">
+        <v>146</v>
+      </c>
+      <c r="E32" s="57"/>
       <c r="F32" s="10"/>
       <c r="G32" s="10"/>
       <c r="H32" s="10"/>
@@ -2398,10 +2398,10 @@
       </c>
       <c r="C33" s="20"/>
       <c r="D33" s="16" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="E33" s="16" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="F33" s="10"/>
       <c r="G33" s="10"/>
@@ -2422,7 +2422,7 @@
         <v>138</v>
       </c>
       <c r="E34" s="16" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="F34" s="10"/>
       <c r="G34" s="10"/>
@@ -2455,52 +2455,52 @@
       <c r="D36" s="45"/>
       <c r="E36" s="46"/>
       <c r="F36" s="28"/>
-      <c r="G36" s="51" t="s">
+      <c r="G36" s="115" t="s">
         <v>127</v>
       </c>
-      <c r="H36" s="52"/>
+      <c r="H36" s="116"/>
       <c r="I36" s="47" t="s">
         <v>130</v>
       </c>
       <c r="J36" s="28"/>
     </row>
     <row r="37" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B37" s="56" t="s">
+      <c r="B37" s="96" t="s">
         <v>73</v>
       </c>
-      <c r="C37" s="57"/>
-      <c r="D37" s="57"/>
-      <c r="E37" s="58"/>
+      <c r="C37" s="97"/>
+      <c r="D37" s="97"/>
+      <c r="E37" s="98"/>
       <c r="F37" s="28"/>
-      <c r="G37" s="51" t="s">
+      <c r="G37" s="115" t="s">
         <v>128</v>
       </c>
-      <c r="H37" s="52"/>
+      <c r="H37" s="116"/>
       <c r="I37" s="47" t="s">
         <v>131</v>
       </c>
       <c r="J37" s="28"/>
     </row>
     <row r="38" spans="2:14" ht="26" x14ac:dyDescent="0.35">
-      <c r="B38" s="59"/>
-      <c r="C38" s="60"/>
-      <c r="D38" s="60"/>
-      <c r="E38" s="61"/>
+      <c r="B38" s="99"/>
+      <c r="C38" s="100"/>
+      <c r="D38" s="100"/>
+      <c r="E38" s="101"/>
       <c r="F38" s="28"/>
-      <c r="G38" s="51" t="s">
+      <c r="G38" s="115" t="s">
         <v>129</v>
       </c>
-      <c r="H38" s="52"/>
+      <c r="H38" s="116"/>
       <c r="I38" s="49" t="s">
         <v>132</v>
       </c>
       <c r="J38" s="28"/>
     </row>
     <row r="39" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B39" s="59"/>
-      <c r="C39" s="60"/>
-      <c r="D39" s="60"/>
-      <c r="E39" s="61"/>
+      <c r="B39" s="99"/>
+      <c r="C39" s="100"/>
+      <c r="D39" s="100"/>
+      <c r="E39" s="101"/>
       <c r="F39" s="28"/>
       <c r="G39" s="28"/>
       <c r="H39" s="28"/>
@@ -2508,10 +2508,10 @@
       <c r="J39" s="28"/>
     </row>
     <row r="40" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B40" s="59"/>
-      <c r="C40" s="60"/>
-      <c r="D40" s="60"/>
-      <c r="E40" s="61"/>
+      <c r="B40" s="99"/>
+      <c r="C40" s="100"/>
+      <c r="D40" s="100"/>
+      <c r="E40" s="101"/>
       <c r="F40" s="28"/>
       <c r="G40" s="28"/>
       <c r="H40" s="10"/>
@@ -2519,10 +2519,10 @@
       <c r="J40" s="28"/>
     </row>
     <row r="41" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B41" s="62"/>
-      <c r="C41" s="63"/>
-      <c r="D41" s="63"/>
-      <c r="E41" s="64"/>
+      <c r="B41" s="102"/>
+      <c r="C41" s="103"/>
+      <c r="D41" s="103"/>
+      <c r="E41" s="104"/>
       <c r="F41" s="28"/>
       <c r="G41" s="28"/>
       <c r="H41" s="10"/>
@@ -2624,13 +2624,56 @@
     </row>
   </sheetData>
   <mergeCells count="73">
-    <mergeCell ref="B23:N23"/>
-    <mergeCell ref="I31:J31"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="L24:M25"/>
-    <mergeCell ref="L28:M28"/>
-    <mergeCell ref="E24:E25"/>
-    <mergeCell ref="D24:D25"/>
+    <mergeCell ref="G36:H36"/>
+    <mergeCell ref="G37:H37"/>
+    <mergeCell ref="G38:H38"/>
+    <mergeCell ref="L10:M10"/>
+    <mergeCell ref="L11:M11"/>
+    <mergeCell ref="K20:L20"/>
+    <mergeCell ref="M16:N17"/>
+    <mergeCell ref="I12:K12"/>
+    <mergeCell ref="N24:N25"/>
+    <mergeCell ref="I24:K25"/>
+    <mergeCell ref="I26:K26"/>
+    <mergeCell ref="L26:M26"/>
+    <mergeCell ref="H24:H25"/>
+    <mergeCell ref="K19:L19"/>
+    <mergeCell ref="I30:J30"/>
+    <mergeCell ref="K31:L31"/>
+    <mergeCell ref="B37:E41"/>
+    <mergeCell ref="G16:G18"/>
+    <mergeCell ref="I16:I18"/>
+    <mergeCell ref="J16:L17"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="G31:H31"/>
+    <mergeCell ref="C24:C25"/>
+    <mergeCell ref="F24:F25"/>
+    <mergeCell ref="G24:G25"/>
+    <mergeCell ref="B30:E30"/>
+    <mergeCell ref="G30:H30"/>
+    <mergeCell ref="I28:K28"/>
+    <mergeCell ref="I27:K27"/>
+    <mergeCell ref="L27:M27"/>
+    <mergeCell ref="K21:L21"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="C16:C18"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B15:N15"/>
+    <mergeCell ref="L12:M12"/>
+    <mergeCell ref="K18:L18"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="H16:H18"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="I13:K13"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="G10:H10"/>
+    <mergeCell ref="G11:H11"/>
+    <mergeCell ref="G9:H9"/>
     <mergeCell ref="C3:G3"/>
     <mergeCell ref="C4:G4"/>
     <mergeCell ref="F16:F18"/>
@@ -2647,56 +2690,13 @@
     <mergeCell ref="I10:K10"/>
     <mergeCell ref="I11:K11"/>
     <mergeCell ref="D16:D18"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="G10:H10"/>
-    <mergeCell ref="G11:H11"/>
-    <mergeCell ref="G9:H9"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="C16:C18"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B15:N15"/>
-    <mergeCell ref="L12:M12"/>
-    <mergeCell ref="K18:L18"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="H16:H18"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="I13:K13"/>
-    <mergeCell ref="B37:E41"/>
-    <mergeCell ref="G16:G18"/>
-    <mergeCell ref="I16:I18"/>
-    <mergeCell ref="J16:L17"/>
-    <mergeCell ref="D31:E31"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="G31:H31"/>
-    <mergeCell ref="C24:C25"/>
-    <mergeCell ref="F24:F25"/>
-    <mergeCell ref="G24:G25"/>
-    <mergeCell ref="B30:E30"/>
-    <mergeCell ref="G30:H30"/>
-    <mergeCell ref="I28:K28"/>
-    <mergeCell ref="I27:K27"/>
-    <mergeCell ref="L27:M27"/>
-    <mergeCell ref="K21:L21"/>
-    <mergeCell ref="G36:H36"/>
-    <mergeCell ref="G37:H37"/>
-    <mergeCell ref="G38:H38"/>
-    <mergeCell ref="L10:M10"/>
-    <mergeCell ref="L11:M11"/>
-    <mergeCell ref="K20:L20"/>
-    <mergeCell ref="M16:N17"/>
-    <mergeCell ref="I12:K12"/>
-    <mergeCell ref="N24:N25"/>
-    <mergeCell ref="I24:K25"/>
-    <mergeCell ref="I26:K26"/>
-    <mergeCell ref="L26:M26"/>
-    <mergeCell ref="H24:H25"/>
-    <mergeCell ref="K19:L19"/>
-    <mergeCell ref="I30:J30"/>
-    <mergeCell ref="K31:L31"/>
+    <mergeCell ref="B23:N23"/>
+    <mergeCell ref="I31:J31"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="L24:M25"/>
+    <mergeCell ref="L28:M28"/>
+    <mergeCell ref="E24:E25"/>
+    <mergeCell ref="D24:D25"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F26:F28" xr:uid="{B316A799-CF60-4C99-A88E-2204076E38E6}">
@@ -3473,17 +3473,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <SharedWithUsers xmlns="1444eecc-14bb-4066-abe6-ce6de21d9439">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3684,20 +3679,23 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <SharedWithUsers xmlns="1444eecc-14bb-4066-abe6-ce6de21d9439">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7EBE950A-5812-419E-B174-6A5D9B8E0414}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A00E6A9-20DD-4842-9306-307EB080AF2E}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="1444eecc-14bb-4066-abe6-ce6de21d9439"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -3722,9 +3720,11 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A00E6A9-20DD-4842-9306-307EB080AF2E}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7EBE950A-5812-419E-B174-6A5D9B8E0414}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="1444eecc-14bb-4066-abe6-ce6de21d9439"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Lock cells of qoutation doc
</commit_message>
<xml_diff>
--- a/srv/xlsx-templates/TH - Quotation Template.xlsx
+++ b/srv/xlsx-templates/TH - Quotation Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vasub\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bayergroup-my.sharepoint.com/personal/vasudevan_mariyappan_ext_bayer_com/Documents/Personal Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D28421B1-1281-4B0D-A2CA-04A2854EF551}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{9305F03F-A89F-496F-BCF7-3E23A8B36088}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F180EBD1-5883-4B92-BEA4-F8EE346F8F84}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{F5CC2154-27BB-4652-B61E-D913F0CC6809}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19200" windowHeight="9020" xr2:uid="{F5CC2154-27BB-4652-B61E-D913F0CC6809}"/>
   </bookViews>
   <sheets>
     <sheet name="Quotation" sheetId="3" r:id="rId1"/>
@@ -497,8 +497,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="#\.###\.###.00"/>
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="#\.###\.###.00"/>
   </numFmts>
   <fonts count="13" x14ac:knownFonts="1">
     <font>
@@ -601,7 +601,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -623,6 +623,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="2" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -851,9 +857,9 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="125">
+  <cellXfs count="135">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -863,19 +869,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="5" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="5" fillId="0" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -917,21 +920,15 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="5" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -954,21 +951,37 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="4" fontId="5" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="2" fontId="0" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -986,152 +999,170 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1154,7 +1185,7 @@
     <xf numFmtId="49" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="6" fillId="0" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1163,10 +1194,10 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="5" fillId="0" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1175,7 +1206,10 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1215,16 +1249,16 @@
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="165" formatCode="#\.###\.###.00"/>
+      <numFmt numFmtId="164" formatCode="#\.###\.###.00"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="165" formatCode="#\.###\.###.00"/>
+      <numFmt numFmtId="164" formatCode="#\.###\.###.00"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="165" formatCode="#\.###\.###.00"/>
+      <numFmt numFmtId="164" formatCode="#\.###\.###.00"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="165" formatCode="#\.###\.###.00"/>
+      <numFmt numFmtId="164" formatCode="#\.###\.###.00"/>
     </dxf>
     <dxf>
       <font>
@@ -1745,79 +1779,79 @@
       <c r="N2" s="10"/>
     </row>
     <row r="3" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B3" s="25" t="s">
+      <c r="B3" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="59" t="s">
+      <c r="C3" s="63" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="60"/>
-      <c r="E3" s="60"/>
-      <c r="F3" s="60"/>
-      <c r="G3" s="61"/>
+      <c r="D3" s="64"/>
+      <c r="E3" s="64"/>
+      <c r="F3" s="64"/>
+      <c r="G3" s="65"/>
       <c r="H3" s="10"/>
-      <c r="I3" s="25" t="s">
+      <c r="I3" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="J3" s="59" t="s">
+      <c r="J3" s="63" t="s">
         <v>3</v>
       </c>
-      <c r="K3" s="60"/>
-      <c r="L3" s="60"/>
-      <c r="M3" s="61"/>
+      <c r="K3" s="64"/>
+      <c r="L3" s="64"/>
+      <c r="M3" s="65"/>
       <c r="N3" s="10"/>
     </row>
     <row r="4" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="26" t="s">
+      <c r="B4" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="62" t="s">
+      <c r="C4" s="66" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="63"/>
-      <c r="E4" s="63"/>
-      <c r="F4" s="63"/>
-      <c r="G4" s="64"/>
+      <c r="D4" s="67"/>
+      <c r="E4" s="67"/>
+      <c r="F4" s="67"/>
+      <c r="G4" s="68"/>
       <c r="H4" s="10"/>
-      <c r="I4" s="25" t="s">
+      <c r="I4" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="J4" s="70" t="s">
+      <c r="J4" s="74" t="s">
         <v>6</v>
       </c>
-      <c r="K4" s="71"/>
-      <c r="L4" s="71"/>
-      <c r="M4" s="72"/>
+      <c r="K4" s="75"/>
+      <c r="L4" s="75"/>
+      <c r="M4" s="76"/>
       <c r="N4" s="10"/>
     </row>
     <row r="5" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="42"/>
-      <c r="C5" s="42"/>
-      <c r="D5" s="42"/>
-      <c r="E5" s="42"/>
-      <c r="F5" s="42"/>
-      <c r="G5" s="42"/>
+      <c r="B5" s="39"/>
+      <c r="C5" s="39"/>
+      <c r="D5" s="39"/>
+      <c r="E5" s="39"/>
+      <c r="F5" s="39"/>
+      <c r="G5" s="39"/>
       <c r="H5" s="10"/>
       <c r="I5" s="10"/>
-      <c r="J5" s="43"/>
-      <c r="K5" s="43"/>
-      <c r="L5" s="43"/>
-      <c r="M5" s="43"/>
+      <c r="J5" s="40"/>
+      <c r="K5" s="40"/>
+      <c r="L5" s="40"/>
+      <c r="M5" s="40"/>
       <c r="N5" s="10"/>
     </row>
     <row r="6" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="42"/>
-      <c r="C6" s="42"/>
-      <c r="D6" s="42"/>
-      <c r="E6" s="42"/>
-      <c r="F6" s="42"/>
-      <c r="G6" s="42"/>
+      <c r="B6" s="39"/>
+      <c r="C6" s="39"/>
+      <c r="D6" s="39"/>
+      <c r="E6" s="39"/>
+      <c r="F6" s="39"/>
+      <c r="G6" s="39"/>
       <c r="H6" s="10"/>
       <c r="I6" s="10"/>
-      <c r="J6" s="43"/>
-      <c r="K6" s="43"/>
-      <c r="L6" s="43"/>
-      <c r="M6" s="43"/>
+      <c r="J6" s="40"/>
+      <c r="K6" s="40"/>
+      <c r="L6" s="40"/>
+      <c r="M6" s="40"/>
       <c r="N6" s="10"/>
     </row>
     <row r="7" spans="2:14" x14ac:dyDescent="0.35">
@@ -1836,151 +1870,151 @@
       <c r="N7" s="10"/>
     </row>
     <row r="8" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B8" s="65" t="s">
+      <c r="B8" s="69" t="s">
         <v>133</v>
       </c>
-      <c r="C8" s="66"/>
-      <c r="D8" s="66"/>
-      <c r="E8" s="66"/>
-      <c r="F8" s="66"/>
-      <c r="G8" s="66"/>
-      <c r="H8" s="66"/>
-      <c r="I8" s="66"/>
-      <c r="J8" s="66"/>
-      <c r="K8" s="66"/>
-      <c r="L8" s="66"/>
-      <c r="M8" s="66"/>
-      <c r="N8" s="67"/>
+      <c r="C8" s="70"/>
+      <c r="D8" s="70"/>
+      <c r="E8" s="70"/>
+      <c r="F8" s="70"/>
+      <c r="G8" s="70"/>
+      <c r="H8" s="70"/>
+      <c r="I8" s="70"/>
+      <c r="J8" s="70"/>
+      <c r="K8" s="70"/>
+      <c r="L8" s="70"/>
+      <c r="M8" s="70"/>
+      <c r="N8" s="71"/>
     </row>
     <row r="9" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B9" s="73" t="s">
+      <c r="B9" s="77" t="s">
         <v>7</v>
       </c>
-      <c r="C9" s="74"/>
-      <c r="D9" s="81" t="s">
+      <c r="C9" s="78"/>
+      <c r="D9" s="85" t="s">
         <v>8</v>
       </c>
-      <c r="E9" s="81"/>
-      <c r="F9" s="38"/>
-      <c r="G9" s="85" t="s">
+      <c r="E9" s="85"/>
+      <c r="F9" s="36"/>
+      <c r="G9" s="91" t="s">
         <v>9</v>
       </c>
-      <c r="H9" s="86"/>
-      <c r="I9" s="77" t="s">
+      <c r="H9" s="92"/>
+      <c r="I9" s="81" t="s">
         <v>10</v>
       </c>
-      <c r="J9" s="77"/>
-      <c r="K9" s="78"/>
-      <c r="L9" s="68" t="s">
+      <c r="J9" s="81"/>
+      <c r="K9" s="82"/>
+      <c r="L9" s="72" t="s">
         <v>11</v>
       </c>
-      <c r="M9" s="69"/>
-      <c r="N9" s="48" t="s">
+      <c r="M9" s="73"/>
+      <c r="N9" s="44" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="10" spans="2:14" ht="26.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="75" t="s">
+      <c r="B10" s="79" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="76"/>
-      <c r="D10" s="82" t="str">
+      <c r="C10" s="80"/>
+      <c r="D10" s="86" t="str">
         <f>Settings!A14</f>
         <v>${offerValidation.CUSTOMER_CODE}</v>
       </c>
-      <c r="E10" s="82"/>
-      <c r="F10" s="38"/>
-      <c r="G10" s="83" t="s">
+      <c r="E10" s="86"/>
+      <c r="F10" s="36"/>
+      <c r="G10" s="89" t="s">
         <v>13</v>
       </c>
-      <c r="H10" s="83"/>
-      <c r="I10" s="79" t="s">
+      <c r="H10" s="89"/>
+      <c r="I10" s="83" t="s">
         <v>14</v>
       </c>
-      <c r="J10" s="79"/>
-      <c r="K10" s="80"/>
-      <c r="L10" s="89" t="s">
+      <c r="J10" s="83"/>
+      <c r="K10" s="84"/>
+      <c r="L10" s="95" t="s">
         <v>15</v>
       </c>
-      <c r="M10" s="90"/>
-      <c r="N10" s="48" t="s">
+      <c r="M10" s="96"/>
+      <c r="N10" s="44" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="11" spans="2:14" ht="26.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="75" t="s">
+      <c r="B11" s="79" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="76"/>
-      <c r="D11" s="62" t="str">
+      <c r="C11" s="80"/>
+      <c r="D11" s="87" t="str">
         <f>Settings!A9</f>
         <v>${offerValidation.INSTITUTENAME}</v>
       </c>
-      <c r="E11" s="64"/>
-      <c r="F11" s="38"/>
-      <c r="G11" s="84" t="s">
+      <c r="E11" s="88"/>
+      <c r="F11" s="36"/>
+      <c r="G11" s="90" t="s">
         <v>17</v>
       </c>
-      <c r="H11" s="84"/>
-      <c r="I11" s="79" t="s">
+      <c r="H11" s="90"/>
+      <c r="I11" s="83" t="s">
         <v>18</v>
       </c>
-      <c r="J11" s="79"/>
-      <c r="K11" s="80"/>
-      <c r="L11" s="89" t="s">
+      <c r="J11" s="83"/>
+      <c r="K11" s="84"/>
+      <c r="L11" s="95" t="s">
         <v>19</v>
       </c>
-      <c r="M11" s="90"/>
-      <c r="N11" s="48" t="s">
+      <c r="M11" s="96"/>
+      <c r="N11" s="45" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="12" spans="2:14" ht="26" x14ac:dyDescent="0.35">
-      <c r="B12" s="75" t="s">
+      <c r="B12" s="79" t="s">
         <v>20</v>
       </c>
-      <c r="C12" s="76"/>
-      <c r="D12" s="87" t="s">
+      <c r="C12" s="80"/>
+      <c r="D12" s="93" t="s">
         <v>21</v>
       </c>
-      <c r="E12" s="88"/>
+      <c r="E12" s="94"/>
       <c r="F12" s="10"/>
-      <c r="G12" s="92" t="s">
+      <c r="G12" s="98" t="s">
         <v>22</v>
       </c>
-      <c r="H12" s="92"/>
-      <c r="I12" s="94" t="s">
+      <c r="H12" s="98"/>
+      <c r="I12" s="101" t="s">
         <v>23</v>
       </c>
-      <c r="J12" s="94"/>
-      <c r="K12" s="95"/>
-      <c r="L12" s="89" t="s">
+      <c r="J12" s="101"/>
+      <c r="K12" s="102"/>
+      <c r="L12" s="95" t="s">
         <v>15</v>
       </c>
-      <c r="M12" s="90"/>
-      <c r="N12" s="48" t="s">
+      <c r="M12" s="96"/>
+      <c r="N12" s="45" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="13" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B13" s="75" t="s">
+      <c r="B13" s="79" t="s">
         <v>24</v>
       </c>
-      <c r="C13" s="76"/>
-      <c r="D13" s="87" t="s">
+      <c r="C13" s="80"/>
+      <c r="D13" s="93" t="s">
         <v>25</v>
       </c>
-      <c r="E13" s="88"/>
+      <c r="E13" s="94"/>
       <c r="F13" s="10"/>
-      <c r="G13" s="92" t="s">
+      <c r="G13" s="98" t="s">
         <v>124</v>
       </c>
-      <c r="H13" s="92"/>
-      <c r="I13" s="94" t="s">
+      <c r="H13" s="98"/>
+      <c r="I13" s="101" t="s">
         <v>134</v>
       </c>
-      <c r="J13" s="94"/>
-      <c r="K13" s="95"/>
+      <c r="J13" s="101"/>
+      <c r="K13" s="102"/>
     </row>
     <row r="14" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B14" s="10"/>
@@ -1995,168 +2029,168 @@
       <c r="K14" s="10"/>
     </row>
     <row r="15" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B15" s="65" t="s">
+      <c r="B15" s="69" t="s">
         <v>26</v>
       </c>
-      <c r="C15" s="66"/>
-      <c r="D15" s="66"/>
-      <c r="E15" s="66"/>
-      <c r="F15" s="66"/>
-      <c r="G15" s="66"/>
-      <c r="H15" s="66"/>
-      <c r="I15" s="66"/>
-      <c r="J15" s="66"/>
-      <c r="K15" s="66"/>
-      <c r="L15" s="66"/>
-      <c r="M15" s="66"/>
-      <c r="N15" s="67"/>
+      <c r="C15" s="70"/>
+      <c r="D15" s="70"/>
+      <c r="E15" s="70"/>
+      <c r="F15" s="70"/>
+      <c r="G15" s="70"/>
+      <c r="H15" s="70"/>
+      <c r="I15" s="70"/>
+      <c r="J15" s="70"/>
+      <c r="K15" s="70"/>
+      <c r="L15" s="70"/>
+      <c r="M15" s="70"/>
+      <c r="N15" s="71"/>
     </row>
     <row r="16" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B16" s="54" t="s">
+      <c r="B16" s="57" t="s">
         <v>27</v>
       </c>
-      <c r="C16" s="56" t="s">
+      <c r="C16" s="59" t="s">
         <v>28</v>
       </c>
-      <c r="D16" s="56" t="s">
+      <c r="D16" s="59" t="s">
         <v>29</v>
       </c>
-      <c r="E16" s="56" t="s">
+      <c r="E16" s="59" t="s">
         <v>30</v>
       </c>
-      <c r="F16" s="56" t="s">
+      <c r="F16" s="59" t="s">
         <v>31</v>
       </c>
-      <c r="G16" s="56" t="s">
+      <c r="G16" s="59" t="s">
         <v>32</v>
       </c>
-      <c r="H16" s="93" t="s">
+      <c r="H16" s="99" t="s">
         <v>33</v>
       </c>
-      <c r="I16" s="56" t="s">
+      <c r="I16" s="59" t="s">
         <v>34</v>
       </c>
-      <c r="J16" s="56" t="s">
+      <c r="J16" s="59" t="s">
         <v>35</v>
       </c>
-      <c r="K16" s="56"/>
-      <c r="L16" s="56"/>
-      <c r="M16" s="56" t="s">
+      <c r="K16" s="59"/>
+      <c r="L16" s="59"/>
+      <c r="M16" s="59" t="s">
         <v>36</v>
       </c>
-      <c r="N16" s="56"/>
+      <c r="N16" s="59"/>
     </row>
     <row r="17" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="B17" s="54"/>
-      <c r="C17" s="56"/>
-      <c r="D17" s="56"/>
-      <c r="E17" s="56"/>
-      <c r="F17" s="56"/>
-      <c r="G17" s="56"/>
-      <c r="H17" s="58"/>
-      <c r="I17" s="56"/>
-      <c r="J17" s="56"/>
-      <c r="K17" s="56"/>
-      <c r="L17" s="56"/>
-      <c r="M17" s="56"/>
-      <c r="N17" s="56"/>
+      <c r="B17" s="57"/>
+      <c r="C17" s="59"/>
+      <c r="D17" s="59"/>
+      <c r="E17" s="59"/>
+      <c r="F17" s="59"/>
+      <c r="G17" s="59"/>
+      <c r="H17" s="100"/>
+      <c r="I17" s="59"/>
+      <c r="J17" s="59"/>
+      <c r="K17" s="59"/>
+      <c r="L17" s="59"/>
+      <c r="M17" s="59"/>
+      <c r="N17" s="59"/>
     </row>
     <row r="18" spans="2:15" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="54"/>
-      <c r="C18" s="56"/>
-      <c r="D18" s="56"/>
-      <c r="E18" s="56"/>
-      <c r="F18" s="56"/>
-      <c r="G18" s="56"/>
-      <c r="H18" s="55"/>
-      <c r="I18" s="56"/>
-      <c r="J18" s="11" t="s">
+      <c r="B18" s="57"/>
+      <c r="C18" s="59"/>
+      <c r="D18" s="59"/>
+      <c r="E18" s="59"/>
+      <c r="F18" s="59"/>
+      <c r="G18" s="59"/>
+      <c r="H18" s="58"/>
+      <c r="I18" s="59"/>
+      <c r="J18" s="46" t="s">
         <v>37</v>
       </c>
-      <c r="K18" s="91" t="s">
+      <c r="K18" s="97" t="s">
         <v>38</v>
       </c>
-      <c r="L18" s="91"/>
-      <c r="M18" s="11" t="s">
+      <c r="L18" s="97"/>
+      <c r="M18" s="46" t="s">
         <v>37</v>
       </c>
-      <c r="N18" s="11" t="s">
+      <c r="N18" s="46" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="19" spans="2:15" ht="29" x14ac:dyDescent="0.35">
-      <c r="B19" s="24" t="s">
+      <c r="B19" s="23" t="s">
         <v>39</v>
       </c>
-      <c r="C19" s="24" t="s">
+      <c r="C19" s="23" t="s">
         <v>123</v>
       </c>
-      <c r="D19" s="37" t="s">
+      <c r="D19" s="48" t="s">
         <v>41</v>
       </c>
-      <c r="E19" s="37" t="s">
+      <c r="E19" s="48" t="s">
         <v>42</v>
       </c>
-      <c r="F19" s="36" t="s">
+      <c r="F19" s="47" t="s">
         <v>43</v>
       </c>
-      <c r="G19" s="36" t="s">
+      <c r="G19" s="47" t="s">
         <v>44</v>
       </c>
-      <c r="H19" s="36" t="s">
+      <c r="H19" s="35" t="s">
         <v>45</v>
       </c>
-      <c r="I19" s="36" t="s">
+      <c r="I19" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="J19" s="36" t="s">
+      <c r="J19" s="47" t="s">
         <v>47</v>
       </c>
-      <c r="K19" s="118" t="s">
+      <c r="K19" s="127" t="s">
         <v>48</v>
       </c>
-      <c r="L19" s="118"/>
-      <c r="M19" s="39" t="s">
+      <c r="L19" s="127"/>
+      <c r="M19" s="53" t="s">
         <v>49</v>
       </c>
-      <c r="N19" s="39" t="s">
+      <c r="N19" s="53" t="s">
         <v>50</v>
       </c>
-      <c r="O19" s="30"/>
+      <c r="O19" s="29"/>
     </row>
     <row r="20" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="B20" s="12"/>
-      <c r="C20" s="12"/>
-      <c r="D20" s="12"/>
-      <c r="E20" s="29"/>
-      <c r="F20" s="12"/>
-      <c r="G20" s="24"/>
-      <c r="H20" s="13"/>
-      <c r="I20" s="12"/>
-      <c r="J20" s="15"/>
-      <c r="K20" s="117"/>
-      <c r="L20" s="117"/>
-      <c r="M20" s="14"/>
-      <c r="N20" s="35"/>
+      <c r="B20" s="11"/>
+      <c r="C20" s="11"/>
+      <c r="D20" s="11"/>
+      <c r="E20" s="28"/>
+      <c r="F20" s="11"/>
+      <c r="G20" s="23"/>
+      <c r="H20" s="12"/>
+      <c r="I20" s="11"/>
+      <c r="J20" s="14"/>
+      <c r="K20" s="126"/>
+      <c r="L20" s="126"/>
+      <c r="M20" s="13"/>
+      <c r="N20" s="34"/>
     </row>
     <row r="21" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="B21" s="12"/>
-      <c r="C21" s="12"/>
-      <c r="D21" s="12"/>
-      <c r="E21" s="29"/>
-      <c r="F21" s="12"/>
-      <c r="G21" s="24"/>
-      <c r="H21" s="13"/>
-      <c r="I21" s="12"/>
-      <c r="J21" s="15"/>
-      <c r="K21" s="114" t="s">
+      <c r="B21" s="11"/>
+      <c r="C21" s="11"/>
+      <c r="D21" s="11"/>
+      <c r="E21" s="28"/>
+      <c r="F21" s="11"/>
+      <c r="G21" s="23"/>
+      <c r="H21" s="12"/>
+      <c r="I21" s="11"/>
+      <c r="J21" s="14"/>
+      <c r="K21" s="123" t="s">
         <v>51</v>
       </c>
-      <c r="L21" s="114"/>
-      <c r="M21" s="36" t="s">
+      <c r="L21" s="123"/>
+      <c r="M21" s="35" t="s">
         <v>52</v>
       </c>
-      <c r="N21" s="36" t="s">
+      <c r="N21" s="35" t="s">
         <v>53</v>
       </c>
     </row>
@@ -2176,148 +2210,148 @@
       <c r="N22" s="10"/>
     </row>
     <row r="23" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="B23" s="51" t="s">
+      <c r="B23" s="54" t="s">
         <v>54</v>
       </c>
-      <c r="C23" s="51"/>
-      <c r="D23" s="51"/>
-      <c r="E23" s="51"/>
-      <c r="F23" s="51"/>
-      <c r="G23" s="51"/>
-      <c r="H23" s="51"/>
-      <c r="I23" s="51"/>
-      <c r="J23" s="51"/>
-      <c r="K23" s="51"/>
-      <c r="L23" s="51"/>
-      <c r="M23" s="51"/>
-      <c r="N23" s="51"/>
+      <c r="C23" s="54"/>
+      <c r="D23" s="54"/>
+      <c r="E23" s="54"/>
+      <c r="F23" s="54"/>
+      <c r="G23" s="54"/>
+      <c r="H23" s="54"/>
+      <c r="I23" s="54"/>
+      <c r="J23" s="54"/>
+      <c r="K23" s="54"/>
+      <c r="L23" s="54"/>
+      <c r="M23" s="54"/>
+      <c r="N23" s="54"/>
     </row>
     <row r="24" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="B24" s="53" t="s">
+      <c r="B24" s="56" t="s">
         <v>27</v>
       </c>
-      <c r="C24" s="55" t="s">
+      <c r="C24" s="58" t="s">
         <v>28</v>
       </c>
-      <c r="D24" s="58" t="s">
+      <c r="D24" s="61" t="s">
         <v>125</v>
       </c>
-      <c r="E24" s="58" t="s">
+      <c r="E24" s="61" t="s">
         <v>126</v>
       </c>
-      <c r="F24" s="55" t="s">
+      <c r="F24" s="58" t="s">
         <v>55</v>
       </c>
-      <c r="G24" s="55" t="s">
+      <c r="G24" s="62" t="s">
         <v>57</v>
       </c>
-      <c r="H24" s="55" t="s">
+      <c r="H24" s="62" t="s">
         <v>58</v>
       </c>
-      <c r="I24" s="55" t="s">
+      <c r="I24" s="62" t="s">
         <v>56</v>
       </c>
-      <c r="J24" s="55"/>
-      <c r="K24" s="55"/>
-      <c r="L24" s="55" t="s">
+      <c r="J24" s="62"/>
+      <c r="K24" s="62"/>
+      <c r="L24" s="58" t="s">
         <v>59</v>
       </c>
-      <c r="M24" s="55"/>
-      <c r="N24" s="55" t="s">
+      <c r="M24" s="58"/>
+      <c r="N24" s="58" t="s">
         <v>60</v>
       </c>
       <c r="O24" s="10"/>
     </row>
     <row r="25" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="B25" s="54"/>
-      <c r="C25" s="56"/>
-      <c r="D25" s="55"/>
-      <c r="E25" s="55"/>
-      <c r="F25" s="56"/>
-      <c r="G25" s="56"/>
-      <c r="H25" s="56"/>
-      <c r="I25" s="56"/>
-      <c r="J25" s="56"/>
-      <c r="K25" s="56"/>
-      <c r="L25" s="56"/>
-      <c r="M25" s="56"/>
-      <c r="N25" s="56"/>
+      <c r="B25" s="57"/>
+      <c r="C25" s="59"/>
+      <c r="D25" s="62"/>
+      <c r="E25" s="62"/>
+      <c r="F25" s="59"/>
+      <c r="G25" s="115"/>
+      <c r="H25" s="115"/>
+      <c r="I25" s="115"/>
+      <c r="J25" s="115"/>
+      <c r="K25" s="115"/>
+      <c r="L25" s="59"/>
+      <c r="M25" s="59"/>
+      <c r="N25" s="59"/>
       <c r="O25" s="10"/>
     </row>
     <row r="26" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B26" s="12" t="s">
+      <c r="B26" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="C26" s="36" t="s">
+      <c r="C26" s="35" t="s">
         <v>123</v>
       </c>
-      <c r="D26" s="36" t="s">
+      <c r="D26" s="47" t="s">
         <v>147</v>
       </c>
-      <c r="E26" s="36" t="s">
+      <c r="E26" s="47" t="s">
         <v>141</v>
       </c>
-      <c r="F26" s="40"/>
-      <c r="G26" s="50" t="s">
+      <c r="F26" s="37"/>
+      <c r="G26" s="49" t="s">
         <v>62</v>
       </c>
-      <c r="H26" s="50" t="s">
+      <c r="H26" s="49" t="s">
         <v>63</v>
       </c>
-      <c r="I26" s="57" t="s">
+      <c r="I26" s="112" t="s">
         <v>61</v>
       </c>
-      <c r="J26" s="57"/>
-      <c r="K26" s="57"/>
-      <c r="L26" s="57" t="s">
+      <c r="J26" s="112"/>
+      <c r="K26" s="112"/>
+      <c r="L26" s="60" t="s">
         <v>64</v>
       </c>
-      <c r="M26" s="57"/>
-      <c r="N26" s="16" t="s">
+      <c r="M26" s="60"/>
+      <c r="N26" s="15" t="s">
         <v>65</v>
       </c>
       <c r="O26" s="10"/>
     </row>
     <row r="27" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="B27" s="16"/>
-      <c r="C27" s="16"/>
-      <c r="D27" s="16"/>
-      <c r="E27" s="16"/>
-      <c r="F27" s="16"/>
-      <c r="G27" s="16"/>
-      <c r="H27" s="16"/>
-      <c r="I27" s="111"/>
-      <c r="J27" s="112"/>
-      <c r="K27" s="113"/>
-      <c r="L27" s="57"/>
-      <c r="M27" s="57"/>
-      <c r="N27" s="16"/>
+      <c r="B27" s="15"/>
+      <c r="C27" s="15"/>
+      <c r="D27" s="15"/>
+      <c r="E27" s="15"/>
+      <c r="F27" s="15"/>
+      <c r="G27" s="15"/>
+      <c r="H27" s="15"/>
+      <c r="I27" s="120"/>
+      <c r="J27" s="121"/>
+      <c r="K27" s="122"/>
+      <c r="L27" s="60"/>
+      <c r="M27" s="60"/>
+      <c r="N27" s="15"/>
       <c r="O27" s="10"/>
     </row>
     <row r="28" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="B28" s="16"/>
-      <c r="C28" s="16"/>
-      <c r="D28" s="16"/>
-      <c r="E28" s="16"/>
-      <c r="F28" s="16"/>
-      <c r="G28" s="16"/>
-      <c r="H28" s="16"/>
-      <c r="I28" s="110"/>
-      <c r="J28" s="110"/>
-      <c r="K28" s="110"/>
-      <c r="L28" s="57"/>
-      <c r="M28" s="57"/>
-      <c r="N28" s="16"/>
+      <c r="B28" s="15"/>
+      <c r="C28" s="15"/>
+      <c r="D28" s="15"/>
+      <c r="E28" s="15"/>
+      <c r="F28" s="15"/>
+      <c r="G28" s="15"/>
+      <c r="H28" s="15"/>
+      <c r="I28" s="119"/>
+      <c r="J28" s="119"/>
+      <c r="K28" s="119"/>
+      <c r="L28" s="60"/>
+      <c r="M28" s="60"/>
+      <c r="N28" s="15"/>
       <c r="O28" s="10"/>
     </row>
     <row r="29" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B29" s="10"/>
       <c r="C29" s="10"/>
-      <c r="D29" s="17"/>
+      <c r="D29" s="16"/>
       <c r="E29" s="10"/>
       <c r="F29" s="10"/>
       <c r="G29" s="10"/>
-      <c r="H29" s="17"/>
+      <c r="H29" s="16"/>
       <c r="I29" s="10"/>
       <c r="J29" s="10"/>
       <c r="K29" s="10"/>
@@ -2326,62 +2360,62 @@
       <c r="N29" s="10"/>
     </row>
     <row r="30" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B30" s="107" t="s">
+      <c r="B30" s="116" t="s">
         <v>66</v>
       </c>
-      <c r="C30" s="107"/>
-      <c r="D30" s="107"/>
-      <c r="E30" s="107"/>
-      <c r="F30" s="18"/>
-      <c r="G30" s="108" t="s">
+      <c r="C30" s="116"/>
+      <c r="D30" s="116"/>
+      <c r="E30" s="116"/>
+      <c r="F30" s="17"/>
+      <c r="G30" s="117" t="s">
         <v>67</v>
       </c>
-      <c r="H30" s="109"/>
-      <c r="I30" s="119" t="s">
+      <c r="H30" s="118"/>
+      <c r="I30" s="128" t="s">
         <v>140</v>
       </c>
-      <c r="J30" s="120"/>
-      <c r="K30" s="26" t="s">
+      <c r="J30" s="129"/>
+      <c r="K30" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="L30" s="26"/>
+      <c r="L30" s="25"/>
       <c r="M30" s="10"/>
       <c r="N30" s="10"/>
     </row>
     <row r="31" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="B31" s="19" t="s">
+      <c r="B31" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="C31" s="20"/>
-      <c r="D31" s="57" t="s">
+      <c r="C31" s="19"/>
+      <c r="D31" s="112" t="s">
         <v>145</v>
       </c>
-      <c r="E31" s="57"/>
+      <c r="E31" s="112"/>
       <c r="F31" s="10"/>
-      <c r="G31" s="105" t="s">
+      <c r="G31" s="113" t="s">
         <v>148</v>
       </c>
-      <c r="H31" s="106"/>
-      <c r="I31" s="52" t="s">
+      <c r="H31" s="114"/>
+      <c r="I31" s="55" t="s">
         <v>149</v>
       </c>
-      <c r="J31" s="52"/>
-      <c r="K31" s="121" t="s">
+      <c r="J31" s="55"/>
+      <c r="K31" s="130" t="s">
         <v>150</v>
       </c>
-      <c r="L31" s="88"/>
+      <c r="L31" s="131"/>
       <c r="M31" s="10"/>
       <c r="N31" s="10"/>
     </row>
     <row r="32" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="B32" s="19" t="s">
+      <c r="B32" s="18" t="s">
         <v>69</v>
       </c>
-      <c r="C32" s="20"/>
-      <c r="D32" s="57" t="s">
+      <c r="C32" s="19"/>
+      <c r="D32" s="112" t="s">
         <v>146</v>
       </c>
-      <c r="E32" s="57"/>
+      <c r="E32" s="112"/>
       <c r="F32" s="10"/>
       <c r="G32" s="10"/>
       <c r="H32" s="10"/>
@@ -2393,14 +2427,14 @@
       <c r="N32" s="10"/>
     </row>
     <row r="33" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B33" s="19" t="s">
+      <c r="B33" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="C33" s="20"/>
-      <c r="D33" s="16" t="s">
+      <c r="C33" s="19"/>
+      <c r="D33" s="50" t="s">
         <v>142</v>
       </c>
-      <c r="E33" s="16" t="s">
+      <c r="E33" s="50" t="s">
         <v>143</v>
       </c>
       <c r="F33" s="10"/>
@@ -2414,14 +2448,14 @@
       <c r="N33" s="10"/>
     </row>
     <row r="34" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B34" s="21" t="s">
+      <c r="B34" s="20" t="s">
         <v>71</v>
       </c>
-      <c r="C34" s="22"/>
-      <c r="D34" s="16" t="s">
+      <c r="C34" s="21"/>
+      <c r="D34" s="50" t="s">
         <v>138</v>
       </c>
-      <c r="E34" s="16" t="s">
+      <c r="E34" s="50" t="s">
         <v>144</v>
       </c>
       <c r="F34" s="10"/>
@@ -2448,181 +2482,182 @@
       <c r="N35" s="10"/>
     </row>
     <row r="36" spans="2:14" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B36" s="44" t="s">
+      <c r="B36" s="41" t="s">
         <v>72</v>
       </c>
-      <c r="C36" s="45"/>
-      <c r="D36" s="45"/>
-      <c r="E36" s="46"/>
-      <c r="F36" s="28"/>
-      <c r="G36" s="115" t="s">
+      <c r="C36" s="42"/>
+      <c r="D36" s="42"/>
+      <c r="E36" s="43"/>
+      <c r="F36" s="27"/>
+      <c r="G36" s="124" t="s">
         <v>127</v>
       </c>
-      <c r="H36" s="116"/>
-      <c r="I36" s="47" t="s">
+      <c r="H36" s="125"/>
+      <c r="I36" s="51" t="s">
         <v>130</v>
       </c>
-      <c r="J36" s="28"/>
+      <c r="J36" s="27"/>
     </row>
     <row r="37" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B37" s="96" t="s">
+      <c r="B37" s="103" t="s">
         <v>73</v>
       </c>
-      <c r="C37" s="97"/>
-      <c r="D37" s="97"/>
-      <c r="E37" s="98"/>
-      <c r="F37" s="28"/>
-      <c r="G37" s="115" t="s">
+      <c r="C37" s="104"/>
+      <c r="D37" s="104"/>
+      <c r="E37" s="105"/>
+      <c r="F37" s="27"/>
+      <c r="G37" s="124" t="s">
         <v>128</v>
       </c>
-      <c r="H37" s="116"/>
-      <c r="I37" s="47" t="s">
+      <c r="H37" s="125"/>
+      <c r="I37" s="51" t="s">
         <v>131</v>
       </c>
-      <c r="J37" s="28"/>
+      <c r="J37" s="27"/>
     </row>
     <row r="38" spans="2:14" ht="26" x14ac:dyDescent="0.35">
-      <c r="B38" s="99"/>
-      <c r="C38" s="100"/>
-      <c r="D38" s="100"/>
-      <c r="E38" s="101"/>
-      <c r="F38" s="28"/>
-      <c r="G38" s="115" t="s">
+      <c r="B38" s="106"/>
+      <c r="C38" s="107"/>
+      <c r="D38" s="107"/>
+      <c r="E38" s="108"/>
+      <c r="F38" s="27"/>
+      <c r="G38" s="124" t="s">
         <v>129</v>
       </c>
-      <c r="H38" s="116"/>
-      <c r="I38" s="49" t="s">
+      <c r="H38" s="125"/>
+      <c r="I38" s="52" t="s">
         <v>132</v>
       </c>
-      <c r="J38" s="28"/>
+      <c r="J38" s="27"/>
     </row>
     <row r="39" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B39" s="99"/>
-      <c r="C39" s="100"/>
-      <c r="D39" s="100"/>
-      <c r="E39" s="101"/>
-      <c r="F39" s="28"/>
-      <c r="G39" s="28"/>
-      <c r="H39" s="28"/>
-      <c r="I39" s="28"/>
-      <c r="J39" s="28"/>
+      <c r="B39" s="106"/>
+      <c r="C39" s="107"/>
+      <c r="D39" s="107"/>
+      <c r="E39" s="108"/>
+      <c r="F39" s="27"/>
+      <c r="G39" s="27"/>
+      <c r="H39" s="27"/>
+      <c r="I39" s="27"/>
+      <c r="J39" s="27"/>
     </row>
     <row r="40" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B40" s="99"/>
-      <c r="C40" s="100"/>
-      <c r="D40" s="100"/>
-      <c r="E40" s="101"/>
-      <c r="F40" s="28"/>
-      <c r="G40" s="28"/>
+      <c r="B40" s="106"/>
+      <c r="C40" s="107"/>
+      <c r="D40" s="107"/>
+      <c r="E40" s="108"/>
+      <c r="F40" s="27"/>
+      <c r="G40" s="27"/>
       <c r="H40" s="10"/>
-      <c r="I40" s="28"/>
-      <c r="J40" s="28"/>
+      <c r="I40" s="27"/>
+      <c r="J40" s="27"/>
     </row>
     <row r="41" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B41" s="102"/>
-      <c r="C41" s="103"/>
-      <c r="D41" s="103"/>
-      <c r="E41" s="104"/>
-      <c r="F41" s="28"/>
-      <c r="G41" s="28"/>
+      <c r="B41" s="109"/>
+      <c r="C41" s="110"/>
+      <c r="D41" s="110"/>
+      <c r="E41" s="111"/>
+      <c r="F41" s="27"/>
+      <c r="G41" s="27"/>
       <c r="H41" s="10"/>
-      <c r="I41" s="28"/>
-      <c r="J41" s="28"/>
+      <c r="I41" s="27"/>
+      <c r="J41" s="27"/>
     </row>
     <row r="42" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B42" s="28"/>
-      <c r="C42" s="28"/>
-      <c r="D42" s="28"/>
-      <c r="E42" s="28"/>
-      <c r="F42" s="28"/>
+      <c r="B42" s="27"/>
+      <c r="C42" s="27"/>
+      <c r="D42" s="27"/>
+      <c r="E42" s="27"/>
+      <c r="F42" s="27"/>
       <c r="H42" s="10"/>
       <c r="I42" s="10"/>
       <c r="J42" s="10"/>
     </row>
     <row r="43" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B43" s="28"/>
-      <c r="C43" s="28"/>
-      <c r="D43" s="28"/>
-      <c r="E43" s="28"/>
-      <c r="F43" s="28"/>
+      <c r="B43" s="27"/>
+      <c r="C43" s="27"/>
+      <c r="D43" s="27"/>
+      <c r="E43" s="27"/>
+      <c r="F43" s="27"/>
       <c r="H43" s="10"/>
       <c r="I43" s="10"/>
       <c r="J43" s="10"/>
     </row>
     <row r="44" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B44" s="28"/>
-      <c r="C44" s="28"/>
-      <c r="D44" s="28"/>
-      <c r="E44" s="28"/>
-      <c r="H44" s="23"/>
+      <c r="B44" s="27"/>
+      <c r="C44" s="27"/>
+      <c r="D44" s="27"/>
+      <c r="E44" s="27"/>
+      <c r="H44" s="22"/>
       <c r="I44" s="10"/>
       <c r="J44" s="10"/>
       <c r="K44" s="10"/>
     </row>
     <row r="45" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B45" s="28"/>
-      <c r="C45" s="28"/>
-      <c r="D45" s="28"/>
-      <c r="E45" s="28"/>
-      <c r="H45" s="23"/>
+      <c r="B45" s="27"/>
+      <c r="C45" s="27"/>
+      <c r="D45" s="27"/>
+      <c r="E45" s="27"/>
+      <c r="H45" s="22"/>
       <c r="I45" s="10"/>
       <c r="J45" s="10"/>
       <c r="K45" s="10"/>
     </row>
     <row r="46" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B46" s="28"/>
-      <c r="C46" s="28"/>
-      <c r="D46" s="28"/>
-      <c r="E46" s="28"/>
-      <c r="H46" s="23"/>
-      <c r="I46" s="23"/>
-      <c r="J46" s="23"/>
+      <c r="B46" s="27"/>
+      <c r="C46" s="27"/>
+      <c r="D46" s="27"/>
+      <c r="E46" s="27"/>
+      <c r="H46" s="22"/>
+      <c r="I46" s="22"/>
+      <c r="J46" s="22"/>
     </row>
     <row r="47" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B47" s="28"/>
-      <c r="C47" s="28"/>
-      <c r="D47" s="28"/>
-      <c r="E47" s="28"/>
-      <c r="H47" s="17"/>
-      <c r="I47" s="23"/>
-      <c r="J47" s="23"/>
+      <c r="B47" s="27"/>
+      <c r="C47" s="27"/>
+      <c r="D47" s="27"/>
+      <c r="E47" s="27"/>
+      <c r="H47" s="16"/>
+      <c r="I47" s="22"/>
+      <c r="J47" s="22"/>
     </row>
     <row r="48" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B48" s="28"/>
-      <c r="C48" s="28"/>
-      <c r="D48" s="28"/>
-      <c r="E48" s="28"/>
-      <c r="G48" s="28"/>
-      <c r="I48" s="23"/>
-      <c r="J48" s="23"/>
+      <c r="B48" s="27"/>
+      <c r="C48" s="27"/>
+      <c r="D48" s="27"/>
+      <c r="E48" s="27"/>
+      <c r="G48" s="27"/>
+      <c r="I48" s="22"/>
+      <c r="J48" s="22"/>
     </row>
     <row r="49" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B49" s="28"/>
-      <c r="C49" s="28"/>
-      <c r="D49" s="28"/>
-      <c r="E49" s="28"/>
-      <c r="G49" s="28"/>
+      <c r="B49" s="27"/>
+      <c r="C49" s="27"/>
+      <c r="D49" s="27"/>
+      <c r="E49" s="27"/>
+      <c r="G49" s="27"/>
       <c r="I49" s="10"/>
       <c r="J49" s="10"/>
     </row>
     <row r="50" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B50" s="28"/>
-      <c r="C50" s="28"/>
-      <c r="D50" s="28"/>
-      <c r="E50" s="28"/>
-      <c r="F50" s="28"/>
+      <c r="B50" s="27"/>
+      <c r="C50" s="27"/>
+      <c r="D50" s="27"/>
+      <c r="E50" s="27"/>
+      <c r="F50" s="27"/>
     </row>
     <row r="51" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B51" s="28"/>
-      <c r="C51" s="28"/>
-      <c r="D51" s="28"/>
-      <c r="E51" s="28"/>
-      <c r="F51" s="28"/>
+      <c r="B51" s="27"/>
+      <c r="C51" s="27"/>
+      <c r="D51" s="27"/>
+      <c r="E51" s="27"/>
+      <c r="F51" s="27"/>
     </row>
     <row r="53" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="J53" s="41"/>
+      <c r="J53" s="38"/>
     </row>
   </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
   <mergeCells count="73">
     <mergeCell ref="G36:H36"/>
     <mergeCell ref="G37:H37"/>
@@ -2720,7 +2755,7 @@
   <cols>
     <col min="1" max="1" width="43.54296875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="50.26953125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="50.26953125" style="24" customWidth="1"/>
+    <col min="3" max="3" width="50.26953125" style="23" customWidth="1"/>
     <col min="4" max="4" width="47.26953125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="36.7265625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="46.7265625" bestFit="1" customWidth="1"/>
@@ -2751,7 +2786,7 @@
       <c r="B1" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="C1" s="32"/>
+      <c r="C1" s="31"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
@@ -2760,7 +2795,7 @@
       <c r="B2" t="s">
         <v>77</v>
       </c>
-      <c r="C2" s="122"/>
+      <c r="C2" s="132"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
@@ -2769,7 +2804,7 @@
       <c r="B3" t="s">
         <v>79</v>
       </c>
-      <c r="C3" s="123"/>
+      <c r="C3" s="133"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
@@ -2778,7 +2813,7 @@
       <c r="B4" t="s">
         <v>80</v>
       </c>
-      <c r="C4" s="123"/>
+      <c r="C4" s="133"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
@@ -2787,7 +2822,7 @@
       <c r="B5" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="123"/>
+      <c r="C5" s="133"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
@@ -2796,7 +2831,7 @@
       <c r="B6" t="s">
         <v>20</v>
       </c>
-      <c r="C6" s="124"/>
+      <c r="C6" s="134"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
@@ -2871,8 +2906,8 @@
       </c>
     </row>
     <row r="17" spans="1:27" x14ac:dyDescent="0.35">
-      <c r="B17" s="31"/>
-      <c r="C17" s="27"/>
+      <c r="B17" s="30"/>
+      <c r="C17" s="26"/>
     </row>
     <row r="18" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
@@ -2886,7 +2921,7 @@
       <c r="B19" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="C19" s="33" t="s">
+      <c r="C19" s="32" t="s">
         <v>91</v>
       </c>
       <c r="D19" s="2" t="s">
@@ -2969,7 +3004,7 @@
       <c r="B20" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="C20" s="24" t="s">
+      <c r="C20" s="23" t="s">
         <v>42</v>
       </c>
       <c r="D20" t="s">
@@ -3018,13 +3053,13 @@
         <f>IF(E20&gt;0,IF(E20="Unit",CONCATENATE(Settings!Q20," ",Settings!E20,"s"),CONCATENATE((Settings!Q20/Settings!M20)," ",Settings!E20,"s")),"")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="S20" s="34" t="s">
+      <c r="S20" s="33" t="s">
         <v>119</v>
       </c>
-      <c r="T20" s="34" t="s">
+      <c r="T20" s="33" t="s">
         <v>120</v>
       </c>
-      <c r="U20" s="34" t="s">
+      <c r="U20" s="33" t="s">
         <v>121</v>
       </c>
       <c r="V20" t="s">
@@ -3473,15 +3508,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010075F372E8CCA016418A193AD921508903" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="f5e922417d740f1a527805650dc2dfa9">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="399317f3-0083-4d0b-9572-12af99626311" xmlns:ns3="1444eecc-14bb-4066-abe6-ce6de21d9439" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="078d79524add6eac9b94134ca637184e" ns2:_="" ns3:_="">
     <xsd:import namespace="399317f3-0083-4d0b-9572-12af99626311"/>
@@ -3678,7 +3704,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <SharedWithUsers xmlns="1444eecc-14bb-4066-abe6-ce6de21d9439">
@@ -3692,15 +3718,16 @@
 </p:properties>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A00E6A9-20DD-4842-9306-307EB080AF2E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8CF88A1C-AA0D-4F8F-A0FD-6F3FAFCA9DC0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3719,7 +3746,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7EBE950A-5812-419E-B174-6A5D9B8E0414}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -3727,4 +3754,12 @@
     <ds:schemaRef ds:uri="1444eecc-14bb-4066-abe6-ce6de21d9439"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A00E6A9-20DD-4842-9306-307EB080AF2E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Updated TH quotation document
</commit_message>
<xml_diff>
--- a/srv/xlsx-templates/TH - Quotation Template.xlsx
+++ b/srv/xlsx-templates/TH - Quotation Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\VasudevanMariyappan\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C5085E9-BD17-42E6-AC3D-F10506252C9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50565FD1-E59D-4DD1-A1F7-0766C9C9C756}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1298,7 +1298,7 @@
         <xdr:cNvPr id="2004" name="Object 980" hidden="1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E76A386A-1A85-2AEE-A43A-6CE73AAE8F5A}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{05C99FBB-D800-D544-7D7D-74B95D080779}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1365,7 +1365,7 @@
                   <a14:compatExt spid="_x0000_s2001"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AB95A911-A0CA-33AF-393E-A3EBFAC94803}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D4EDB410-2319-7249-20CA-96044F9E7596}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -1440,7 +1440,7 @@
                   <a14:compatExt spid="_x0000_s2002"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FB4F2458-B52E-71E4-92C6-C490413B2B3B}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B212CE8B-7352-CFC4-FB75-AB0FDCC35DBD}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -1515,7 +1515,7 @@
                   <a14:compatExt spid="_x0000_s2003"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A782C953-43B5-F6F9-A668-6EC1059F2C23}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FEB39E88-9F95-6364-D53E-5111EB02B52B}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>

</xml_diff>